<commit_message>
Remove mezzanine from model; add football-field slide; enrich deck
Model: pref_bal=0 removes mezzanine — OT's $1.0bn is funded by BA equity
injection (equity-down), so returns are read off common-stock FCFE (Ke)
rather than mezz DSCR. Regenerated FCFF_model_lines.xlsx.

Deck (now 5 slides, SK earnings template via HTML→PNG, Space Grotesk
hero numbers per the handoff guideline):
- New P4 Football Field (BA consolidated): DCF / EV-EBITDA / NAV ranges,
  conclusion band $3.0-4.0bn, equity-return callout
- P1 cover: drop the funding-need panel (lives on P2 now)
- P2: 2x2 KPI cards (capacity / existing debt / retrofit / ASP)
- P5: indicative engagement timeline strip to fill whitespace
- installed Space Grotesk + Noto Serif KR/IBM Plex fonts for rendering

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKBA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKOT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SKBA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SKOT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Consolidated" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,13 +491,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -521,7 +521,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -545,7 +545,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -576,14 +576,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -652,9 +652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>자체 전극·ex-AMPC EBITDA 9% (메자닌 $1bn 적격)</t>
+          <t>자체 전극·ex-AMPC EBITDA 9% (지분 수익률 기준)</t>
         </is>
       </c>
       <c r="D47" s="19" t="n">
@@ -4203,22 +4203,22 @@
     <row r="108">
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>SKOT · 우선주/메자닌 ($mm) ★</t>
+          <t>SKOT · 메자닌 ($mm) — 제거 ★</t>
         </is>
       </c>
       <c r="C108" s="18" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>링펜싱 격리 조달</t>
+          <t>메자닌 제거: OT는 BA 증자(equity-down)로 자금조달</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>SKOT · 메자닌 배당률 ★</t>
+          <t>SKOT · 메자닌 배당률 (inert) ★</t>
         </is>
       </c>
       <c r="C109" s="19" t="n">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="D109" s="8" t="inlineStr">
         <is>
-          <t>(B)키커 부여→10%에서 인하</t>
+          <t>메자닌 제거로 미사용 (bal=0)</t>
         </is>
       </c>
     </row>
@@ -9423,7 +9423,7 @@
     <row r="50">
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>※ 메자닌 구조: (A)만기 2032 단축 (B)배당 7%+키커 (C)AMPC창내 amortizing → DSCR 개선 · DOE 이자만 · 각 SPV non-recourse</t>
+          <t>※ 메자닌 제거: OT 소요 $1bn은 BA 증자(equity-down)로 조달 → OT 신규부채·DSCR 불요. 수익률은 보통주 FCFE(Ke)로 평가. DOE 이자만·각 SPV non-recourse.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Net debt = $9bn (DOE 4 + BA 5); football field equity bridge (verified)
Redefined net debt to BA-consolidated DOE $4bn + BA standalone $5bn = $9bn
and recalculated (LibreOffice Calc, total_errors=0):
  Platform EV 3,576 · Equity(DCF, EV-netdebt) -5,424 · Equity(FCFE) +708
  · NAV 5,000  ($mm)

Football field P4: replaced the KPI row with an EV→Equity bridge
(platform EV 3.6 / -net debt 9.0 / FCFE +0.7 / DCF -5.4) and rewrote the
callout — platform EV << debt, so equity is thin and only positive on the
interest-only (principal-unpaid) FCFE basis; margin is the lever. DCF base
marker updated 3.45 -> 3.58. Docs + CLAUDE.md base case synced; deck PDF
re-exported.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -3977,10 +3977,90 @@
     <t xml:space="preserve">Terminal growth (TGR) ★</t>
   </si>
   <si>
-    <t xml:space="preserve">Net debt incl. DOE loan ($mm) ★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV→Equity</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Net debt = DOE $4bn + BA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단독 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$5bn ($mm) ★</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BA</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연결</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: OT DOE 4,000 + BA </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단독 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5,000</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Mid-year convention</t>
@@ -10307,8 +10387,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="26245628"/>
-        <c:axId val="47548902"/>
+        <c:axId val="51000699"/>
+        <c:axId val="98545226"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10453,11 +10533,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="26245628"/>
-        <c:axId val="47548902"/>
+        <c:axId val="51000699"/>
+        <c:axId val="98545226"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26245628"/>
+        <c:axId val="51000699"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10489,7 +10569,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47548902"/>
+        <c:crossAx val="98545226"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10497,7 +10577,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47548902"/>
+        <c:axId val="98545226"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10539,7 +10619,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26245628"/>
+        <c:crossAx val="51000699"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13534,7 +13614,7 @@
         <v>125</v>
       </c>
       <c r="C93" s="19" t="n">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>126</v>
@@ -18641,7 +18721,7 @@
       </c>
       <c r="D63" s="38" t="n">
         <f aca="false">-Assumptions!$C$93</f>
-        <v>-6000</v>
+        <v>-9000</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18650,7 +18730,7 @@
       </c>
       <c r="D64" s="74" t="n">
         <f aca="false">D62-Assumptions!$C$93</f>
-        <v>-2424.31707534089</v>
+        <v>-5424.31707534089</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18712,7 +18792,7 @@
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-2424.31707534089</v>
+        <v>-5424.31707534089</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18761,7 +18841,7 @@
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-2424.31707534089</v>
+        <v>-5424.31707534089</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18770,7 +18850,7 @@
       </c>
       <c r="D81" s="76" t="n">
         <f aca="false">(Assumptions!$C$118+Assumptions!$C$119)-D64</f>
-        <v>7424.31707534089</v>
+        <v>10424.3170753409</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Grant-first funding mix (grant 10 / equity 30 / non-recourse debt 60)
Model: grant stays 10% (capex_grant); new non-recourse debt set to 60%
of growth capex (ba_debt=852 @6.5%); removed the HoldCo credit layer
(hc_mezz/ba_hc/ot_hc=0); equity is the 30% residual. Net debt updated to
9,852 (DOE 4,000 + BA 5,000 + new 852). Recalc total_errors=0.

Lower debt (85%->60%) cuts the interest drag, so FCFE equity improves
+708 -> +1,123 ($mm); DCF-bridge equity -6,276 (EV 3,576 - net debt
9,852). Deck: P3 flow pills now show the 10/30/60 mix amounts; football
field equity bridge + callout updated. Docs synced; pptx/PDF re-exported.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -3977,20 +3977,25 @@
     <t xml:space="preserve">Terminal growth (TGR) ★</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Net debt = DOE $4bn + BA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+    <t xml:space="preserve">Net debt ($mm) ★</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DOE 4,000 + BA </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -3998,68 +4003,35 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">$5bn ($mm) ★</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">BA</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">연결</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: OT DOE 4,000 + BA </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단독 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5,000</t>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5,000 + </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신규 비소구부채 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">852</t>
     </r>
   </si>
   <si>
@@ -4448,7 +4420,37 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">공통 조달 → 양 공장 후순위 출자</t>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그랜트우선 구조</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: HoldCo </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">크레딧 레이어 제거</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4509,84 +4511,75 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">SKBA · project debt ($mm) ★</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개조 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">capex </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">조달</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SKBA · project debt </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이자율 ★</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DOE-clean → </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">저리</t>
-    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신규 비소구부채 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">($mm) ★</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그랜트우선</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: growth capex $1.42bn × 60% (BA </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일괄조달</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">비소구부채 이자율 ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비소구 → 소폭 가산</t>
   </si>
   <si>
     <r>
@@ -4625,21 +4618,31 @@
         <i val="true"/>
         <sz val="8"/>
         <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">HoldCo </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">우산 배분</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그랜트우선 구조</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제거</t>
     </r>
   </si>
   <si>
@@ -5211,42 +5214,84 @@
         <i val="true"/>
         <sz val="8"/>
         <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">waiver </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전제</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·DOE </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">비담보 형태</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그랜트우선 구조</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제거 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(OT</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BA </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">증자</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -10387,8 +10432,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="51000699"/>
-        <c:axId val="98545226"/>
+        <c:axId val="63956033"/>
+        <c:axId val="150070"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10533,11 +10578,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="51000699"/>
-        <c:axId val="98545226"/>
+        <c:axId val="63956033"/>
+        <c:axId val="150070"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="51000699"/>
+        <c:axId val="63956033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10569,7 +10614,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98545226"/>
+        <c:crossAx val="150070"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10577,7 +10622,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98545226"/>
+        <c:axId val="150070"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10619,7 +10664,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51000699"/>
+        <c:crossAx val="63956033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13614,7 +13659,7 @@
         <v>125</v>
       </c>
       <c r="C93" s="19" t="n">
-        <v>9000</v>
+        <v>9852</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>126</v>
@@ -13659,7 +13704,7 @@
         <v>131</v>
       </c>
       <c r="C99" s="19" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>132</v>
@@ -13682,24 +13727,24 @@
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="21" t="s">
+      <c r="B102" s="18" t="s">
         <v>136</v>
       </c>
       <c r="C102" s="19" t="n">
-        <v>400</v>
+        <v>852</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B103" s="21" t="s">
+      <c r="B103" s="18" t="s">
         <v>138</v>
       </c>
       <c r="C103" s="20" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D103" s="10" t="s">
+        <v>0.065</v>
+      </c>
+      <c r="D103" s="8" t="s">
         <v>139</v>
       </c>
     </row>
@@ -13708,9 +13753,9 @@
         <v>140</v>
       </c>
       <c r="C104" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="D104" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D104" s="8" t="s">
         <v>141</v>
       </c>
     </row>
@@ -13801,9 +13846,9 @@
         <v>157</v>
       </c>
       <c r="C113" s="19" t="n">
-        <v>500</v>
-      </c>
-      <c r="D113" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D113" s="8" t="s">
         <v>158</v>
       </c>
     </row>
@@ -17675,43 +17720,43 @@
       </c>
       <c r="D32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="E32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="G32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="H32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="I32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="J32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="K32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="L32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
       <c r="M32" s="38" t="n">
         <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
-        <v>-24</v>
+        <v>-55.38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17720,43 +17765,43 @@
       </c>
       <c r="D33" s="38" t="n">
         <f aca="false">-D32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="E33" s="38" t="n">
         <f aca="false">-E32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="F33" s="38" t="n">
         <f aca="false">-F32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="G33" s="38" t="n">
         <f aca="false">-G32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="H33" s="38" t="n">
         <f aca="false">-H32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="I33" s="38" t="n">
         <f aca="false">-I32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="J33" s="38" t="n">
         <f aca="false">-J32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="K33" s="38" t="n">
         <f aca="false">-K32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="L33" s="38" t="n">
         <f aca="false">-L32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
       <c r="M33" s="38" t="n">
         <f aca="false">-M32*Assumptions!$C$86</f>
-        <v>5.52</v>
+        <v>12.7374</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17765,43 +17810,43 @@
       </c>
       <c r="D34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="E34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="F34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="G34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="H34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="I34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="J34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="K34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="L34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
       <c r="M34" s="38" t="n">
         <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
-        <v>-27</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17810,43 +17855,43 @@
       </c>
       <c r="D35" s="56" t="n">
         <f aca="false">D26+D32+D33+D34</f>
-        <v>-225.48</v>
+        <v>-222.6426</v>
       </c>
       <c r="E35" s="56" t="n">
         <f aca="false">E26+E32+E33+E34</f>
-        <v>-57.5931159999998</v>
+        <v>-54.7557159999998</v>
       </c>
       <c r="F35" s="56" t="n">
         <f aca="false">F26+F32+F33+F34</f>
-        <v>352.4555304</v>
+        <v>355.2929304</v>
       </c>
       <c r="G35" s="56" t="n">
         <f aca="false">G26+G32+G33+G34</f>
-        <v>592.68489936</v>
+        <v>595.52229936</v>
       </c>
       <c r="H35" s="56" t="n">
         <f aca="false">H26+H32+H33+H34</f>
-        <v>530.080132512</v>
+        <v>532.917532512</v>
       </c>
       <c r="I35" s="56" t="n">
         <f aca="false">I26+I32+I33+I34</f>
-        <v>410.469088032</v>
+        <v>413.306488032</v>
       </c>
       <c r="J35" s="56" t="n">
         <f aca="false">J26+J32+J33+J34</f>
-        <v>253.65639888</v>
+        <v>256.49379888</v>
       </c>
       <c r="K35" s="56" t="n">
         <f aca="false">K26+K32+K33+K34</f>
-        <v>84.0216647999998</v>
+        <v>86.8590647999998</v>
       </c>
       <c r="L35" s="56" t="n">
         <f aca="false">L26+L32+L33+L34</f>
-        <v>82.31637072</v>
+        <v>85.15377072</v>
       </c>
       <c r="M35" s="56" t="n">
         <f aca="false">M26+M32+M33+M34</f>
-        <v>80.6110766399998</v>
+        <v>83.4484766399998</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18125,43 +18170,43 @@
       </c>
       <c r="D42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="E42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="F42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="G42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="H42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="I42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="J42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="K42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="L42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
       <c r="M42" s="38" t="n">
         <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
-        <v>-45</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18170,43 +18215,43 @@
       </c>
       <c r="D43" s="56" t="n">
         <f aca="false">D27+D36+D37+D41+D40+D42</f>
-        <v>-379</v>
+        <v>-334</v>
       </c>
       <c r="E43" s="56" t="n">
         <f aca="false">E27+E36+E37+E41+E40+E42</f>
-        <v>-649</v>
+        <v>-604</v>
       </c>
       <c r="F43" s="56" t="n">
         <f aca="false">F27+F36+F37+F41+F40+F42</f>
-        <v>-208.64384712</v>
+        <v>-163.64384712</v>
       </c>
       <c r="G43" s="56" t="n">
         <f aca="false">G27+G36+G37+G41+G40+G42</f>
-        <v>382.94207864</v>
+        <v>427.94207864</v>
       </c>
       <c r="H43" s="56" t="n">
         <f aca="false">H27+H36+H37+H41+H40+H42</f>
-        <v>398.76989296</v>
+        <v>443.76989296</v>
       </c>
       <c r="I43" s="56" t="n">
         <f aca="false">I27+I36+I37+I41+I40+I42</f>
-        <v>304.91428576</v>
+        <v>349.91428576</v>
       </c>
       <c r="J43" s="56" t="n">
         <f aca="false">J27+J36+J37+J41+J40+J42</f>
-        <v>136.22980936</v>
+        <v>181.22980936</v>
       </c>
       <c r="K43" s="56" t="n">
         <f aca="false">K27+K36+K37+K41+K40+K42</f>
-        <v>-66.9185924</v>
+        <v>-21.9185924</v>
       </c>
       <c r="L43" s="56" t="n">
         <f aca="false">L27+L36+L37+L41+L40+L42</f>
-        <v>-68.4482741600006</v>
+        <v>-23.4482741600006</v>
       </c>
       <c r="M43" s="56" t="n">
         <f aca="false">M27+M36+M37+M41+M40+M42</f>
-        <v>-69.9779559199998</v>
+        <v>-24.9779559199998</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18350,43 +18395,43 @@
       </c>
       <c r="D47" s="59" t="n">
         <f aca="false">D35+D43</f>
-        <v>-604.48</v>
+        <v>-556.6426</v>
       </c>
       <c r="E47" s="59" t="n">
         <f aca="false">E35+E43</f>
-        <v>-706.593116</v>
+        <v>-658.755716</v>
       </c>
       <c r="F47" s="59" t="n">
         <f aca="false">F35+F43</f>
-        <v>143.811683280001</v>
+        <v>191.649083280001</v>
       </c>
       <c r="G47" s="59" t="n">
         <f aca="false">G35+G43</f>
-        <v>975.626978</v>
+        <v>1023.464378</v>
       </c>
       <c r="H47" s="59" t="n">
         <f aca="false">H35+H43</f>
-        <v>928.850025472</v>
+        <v>976.687425472</v>
       </c>
       <c r="I47" s="59" t="n">
         <f aca="false">I35+I43</f>
-        <v>715.383373792</v>
+        <v>763.220773792</v>
       </c>
       <c r="J47" s="59" t="n">
         <f aca="false">J35+J43</f>
-        <v>389.886208240001</v>
+        <v>437.723608240001</v>
       </c>
       <c r="K47" s="59" t="n">
         <f aca="false">K35+K43</f>
-        <v>17.1030723999998</v>
+        <v>64.9404723999998</v>
       </c>
       <c r="L47" s="59" t="n">
         <f aca="false">L35+L43</f>
-        <v>13.8680965599995</v>
+        <v>61.7054965599995</v>
       </c>
       <c r="M47" s="59" t="n">
         <f aca="false">M35+M43</f>
-        <v>10.63312072</v>
+        <v>58.47052072</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18440,43 +18485,43 @@
       </c>
       <c r="D49" s="39" t="n">
         <f aca="false">D47*D48</f>
-        <v>-568.646950520517</v>
+        <v>-523.645310051304</v>
       </c>
       <c r="E49" s="39" t="n">
         <f aca="false">E47*E48</f>
-        <v>-588.236185555214</v>
+        <v>-548.41172496299</v>
       </c>
       <c r="F49" s="39" t="n">
         <f aca="false">F47*F48</f>
-        <v>105.949292488738</v>
+        <v>141.192177968582</v>
       </c>
       <c r="G49" s="39" t="n">
         <f aca="false">G47*G48</f>
-        <v>636.076350538275</v>
+        <v>667.264744768226</v>
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">H47*H48</f>
-        <v>535.91091398293</v>
+        <v>563.511262858992</v>
       </c>
       <c r="I49" s="39" t="n">
         <f aca="false">I47*I48</f>
-        <v>365.264447933785</v>
+        <v>389.689535434725</v>
       </c>
       <c r="J49" s="39" t="n">
         <f aca="false">J47*J48</f>
-        <v>176.168391955624</v>
+        <v>197.783513637873</v>
       </c>
       <c r="K49" s="39" t="n">
         <f aca="false">K47*K48</f>
-        <v>6.83889298646469</v>
+        <v>25.967319253941</v>
       </c>
       <c r="L49" s="39" t="n">
         <f aca="false">L47*L48</f>
-        <v>4.90738450465169</v>
+        <v>21.8351953608254</v>
       </c>
       <c r="M49" s="39" t="n">
         <f aca="false">M47*M48</f>
-        <v>3.32977993112107</v>
+        <v>18.3101435206554</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18721,7 +18766,7 @@
       </c>
       <c r="D63" s="38" t="n">
         <f aca="false">-Assumptions!$C$93</f>
-        <v>-9000</v>
+        <v>-9852</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18730,7 +18775,7 @@
       </c>
       <c r="D64" s="74" t="n">
         <f aca="false">D62-Assumptions!$C$93</f>
-        <v>-5424.31707534089</v>
+        <v>-6276.31707534089</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18756,7 +18801,7 @@
       </c>
       <c r="D69" s="38" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>677.562318245858</v>
+        <v>953.496857789527</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18765,7 +18810,7 @@
       </c>
       <c r="D70" s="38" t="n">
         <f aca="false">M47*(1+Assumptions!$C$92)/(Assumptions!$C$91-Assumptions!$C$92)</f>
-        <v>98.5980284945457</v>
+        <v>542.181192130909</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18774,7 +18819,7 @@
       </c>
       <c r="D71" s="38" t="n">
         <f aca="false">D70*1/(1+Assumptions!$C$91)^((10)-Assumptions!$C$94)</f>
-        <v>30.8761411794863</v>
+        <v>169.784967191531</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18783,7 +18828,7 @@
       </c>
       <c r="D72" s="73" t="n">
         <f aca="false">D69+D71</f>
-        <v>708.438459425344</v>
+        <v>1123.28182498106</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18792,7 +18837,7 @@
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-5424.31707534089</v>
+        <v>-6276.31707534089</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18841,7 +18886,7 @@
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-5424.31707534089</v>
+        <v>-6276.31707534089</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18850,7 +18895,7 @@
       </c>
       <c r="D81" s="76" t="n">
         <f aca="false">(Assumptions!$C$118+Assumptions!$C$119)-D64</f>
-        <v>10424.3170753409</v>
+        <v>11276.3170753409</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Net debt = $6.4bn (BA 3.7 + OT 2.6); refresh P4 chain + final check
Model netdebt 9,852 -> 6,400. Recalc total_errors=0: EV 3,576, Equity(DCF)
-2,824, Equity(FCFE) +1,123 ($mm). P4 reverse-valuation refreshed with the
$6.4bn net debt: min equity $2.1 -> min EV $8.6 -> min multiple ~19x ->
required ex-AMPC EBITDA ~22.5% (sweep confirmed EV@23%=8,751; fit
EV≈370·M+249). Margin gauge/callout updated. P2 stale EV 3.45 -> 3.6bn.
Docs + CLAUDE.md synced. Final cross-check: chain arithmetic ties to the
slide; P2 shows gross borrowings ($9bn) vs P4 net debt ($6.4bn) by design
(gap = cash). pptx/PDF re-exported.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -3989,49 +3989,28 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">DOE 4,000 + BA </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단독 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5,000 + </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">신규 비소구부채 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">852</t>
+      <t xml:space="preserve">BA/OT </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">합산 순차입금 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= BA 3,700 + OT 2,600</t>
     </r>
   </si>
   <si>
@@ -10432,8 +10411,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="63956033"/>
-        <c:axId val="150070"/>
+        <c:axId val="94752096"/>
+        <c:axId val="24120652"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10578,11 +10557,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="63956033"/>
-        <c:axId val="150070"/>
+        <c:axId val="94752096"/>
+        <c:axId val="24120652"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63956033"/>
+        <c:axId val="94752096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10614,7 +10593,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="150070"/>
+        <c:crossAx val="24120652"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10622,7 +10601,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="150070"/>
+        <c:axId val="24120652"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10664,7 +10643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63956033"/>
+        <c:crossAx val="94752096"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13659,7 +13638,7 @@
         <v>125</v>
       </c>
       <c r="C93" s="19" t="n">
-        <v>9852</v>
+        <v>6400</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>126</v>
@@ -18766,7 +18745,7 @@
       </c>
       <c r="D63" s="38" t="n">
         <f aca="false">-Assumptions!$C$93</f>
-        <v>-9852</v>
+        <v>-6400</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18775,7 +18754,7 @@
       </c>
       <c r="D64" s="74" t="n">
         <f aca="false">D62-Assumptions!$C$93</f>
-        <v>-6276.31707534089</v>
+        <v>-2824.31707534089</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18837,7 +18816,7 @@
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-6276.31707534089</v>
+        <v>-2824.31707534089</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18886,7 +18865,7 @@
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-6276.31707534089</v>
+        <v>-2824.31707534089</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18895,7 +18874,7 @@
       </c>
       <c r="D81" s="76" t="n">
         <f aca="false">(Assumptions!$C$118+Assumptions!$C$119)-D64</f>
-        <v>11276.3170753409</v>
+        <v>7824.31707534089</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
model+deck: SKBA pre-SOP 기저 EBITDA floor($0.2bn) + 조달 시나리오 역산
모델 (build_model3.py)
- SKBA 기저 EBITDA를 pre-SOP floor로 반영: MAX(0, 200-(gp+sga))
  → 2026 ex-AMPC EBITDA $200mm, run-rate(2030-32) $442mm 유지(개조분)
- NOL/tax carryforward는 기존대로 반영(TCJA 80% 한도) — 명시
- extract.py: 재계산+핵심값 추출 헬퍼
- scenarios.py: 조달 시나리오(그랜트/CoC 희석) → implied 멀티플 + 3x3 민감도

덱 (gen_funding_edit.js, 편집형)
- S2: run-rate EBITDA 442, DCF EV 4.0bn, 기저 EBITDA(pre-SOP) $0.2bn
- S4: 역산을 조달 시나리오로 재구성 — BASE 19.3x → ①/② 17.7x → ①+② 16.6x
  peer 8~13x 밴드 대비 위치 바(레버 -2.7x), 잔여 갭은 마진(~22%)이 결정

문서: CLAUDE.md·펀딩구조_v2 검산표/역산표 동기화

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="285">
   <si>
     <t xml:space="preserve">US LFP/ESS CELL PLATFORM — LINE-LEVEL FINANCIAL PROJECTION</t>
   </si>
@@ -3635,6 +3635,123 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SKBA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기저 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EBITDA floor (pre-SOP, $mm/yr) ★</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">양산 전</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(2026~) </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기존 사업 하한 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개조분이 이보다 크면 미적용</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(run-rate </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유지</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Net working capital (% rev) ★</t>
   </si>
   <si>
@@ -6277,6 +6394,46 @@
   </si>
   <si>
     <t xml:space="preserve">D&amp;A</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기저 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EBITDA floor </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보정 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(pre-SOP)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">EBIT (pre-AMPC)</t>
@@ -10411,8 +10568,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="94752096"/>
-        <c:axId val="24120652"/>
+        <c:axId val="38045476"/>
+        <c:axId val="76172954"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10515,19 +10672,19 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="1">
-                  <c:v>-360</c:v>
+                  <c:v>-168.58636</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-462.113116</c:v>
+                  <c:v>-340.279684</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>388.291683280001</c:v>
+                  <c:v>436.14279688</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1220.106978</c:v>
+                  <c:v>1242.57192264</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1173.330025472</c:v>
+                  <c:v>1176.49565696</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>959.863373792</c:v>
@@ -10536,13 +10693,13 @@
                   <c:v>634.366208240001</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>261.5830724</c:v>
+                  <c:v>262.3508516</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>258.34809656</c:v>
+                  <c:v>261.737009839999</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>255.11312072</c:v>
+                  <c:v>261.12316808</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10557,11 +10714,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94752096"/>
-        <c:axId val="24120652"/>
+        <c:axId val="38045476"/>
+        <c:axId val="76172954"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94752096"/>
+        <c:axId val="38045476"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10593,7 +10750,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24120652"/>
+        <c:crossAx val="76172954"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10601,7 +10758,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24120652"/>
+        <c:axId val="76172954"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10643,7 +10800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94752096"/>
+        <c:crossAx val="38045476"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10910,7 +11067,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:M122"/>
+  <dimension ref="B1:M123"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -13558,27 +13715,27 @@
       <c r="B85" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="C85" s="20" t="n">
-        <v>0.15</v>
+      <c r="C85" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C86" s="20" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="D86" s="10" t="s">
-        <v>114</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C87" s="19" t="n">
-        <v>4000</v>
+      <c r="C87" s="20" t="n">
+        <v>0.23</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>116</v>
@@ -13589,9 +13746,9 @@
         <v>117</v>
       </c>
       <c r="C88" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D88" s="8" t="s">
+        <v>4000</v>
+      </c>
+      <c r="D88" s="10" t="s">
         <v>118</v>
       </c>
     </row>
@@ -13599,10 +13756,10 @@
       <c r="B89" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="C89" s="20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D89" s="10" t="s">
+      <c r="C89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="8" t="s">
         <v>120</v>
       </c>
     </row>
@@ -13611,18 +13768,18 @@
         <v>121</v>
       </c>
       <c r="C90" s="20" t="n">
-        <v>0.105</v>
+        <v>0.8</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C91" s="20" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="D91" s="8" t="s">
-        <v>123</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13630,62 +13787,62 @@
         <v>124</v>
       </c>
       <c r="C92" s="20" t="n">
-        <v>0.02</v>
+        <v>0.13</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C93" s="19" t="n">
-        <v>6400</v>
-      </c>
-      <c r="D93" s="10" t="s">
         <v>126</v>
+      </c>
+      <c r="C93" s="20" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C94" s="45" t="n">
+      <c r="C94" s="19" t="n">
+        <v>6400</v>
+      </c>
+      <c r="D94" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B95" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C95" s="45" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B96" s="46" t="s">
-        <v>128</v>
-      </c>
-      <c r="C96" s="13"/>
-      <c r="D96" s="13"/>
-      <c r="E96" s="13"/>
-      <c r="F96" s="13"/>
-      <c r="G96" s="13"/>
-      <c r="H96" s="13"/>
-      <c r="I96" s="13"/>
-      <c r="J96" s="13"/>
-      <c r="K96" s="13"/>
-      <c r="L96" s="13"/>
-      <c r="M96" s="13"/>
-    </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B97" s="14" t="s">
-        <v>129</v>
-      </c>
+      <c r="B97" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="C97" s="13"/>
+      <c r="D97" s="13"/>
+      <c r="E97" s="13"/>
+      <c r="F97" s="13"/>
+      <c r="G97" s="13"/>
+      <c r="H97" s="13"/>
+      <c r="I97" s="13"/>
+      <c r="J97" s="13"/>
+      <c r="K97" s="13"/>
+      <c r="L97" s="13"/>
+      <c r="M97" s="13"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B98" s="47" t="s">
-        <v>130</v>
+      <c r="B98" s="14" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B99" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="C99" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D99" s="8" t="s">
+      <c r="B99" s="47" t="s">
         <v>132</v>
       </c>
     </row>
@@ -13693,26 +13850,26 @@
       <c r="B100" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="C100" s="20" t="n">
-        <v>0.09</v>
+      <c r="C100" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="48" t="s">
+      <c r="B101" s="21" t="s">
         <v>135</v>
       </c>
+      <c r="C101" s="20" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="C102" s="19" t="n">
-        <v>852</v>
-      </c>
-      <c r="D102" s="8" t="s">
+      <c r="B102" s="48" t="s">
         <v>137</v>
       </c>
     </row>
@@ -13720,37 +13877,37 @@
       <c r="B103" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="C103" s="20" t="n">
-        <v>0.065</v>
+      <c r="C103" s="19" t="n">
+        <v>852</v>
       </c>
       <c r="D103" s="8" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B104" s="21" t="s">
+      <c r="B104" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="C104" s="19" t="n">
-        <v>0</v>
+      <c r="C104" s="20" t="n">
+        <v>0.065</v>
       </c>
       <c r="D104" s="8" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B105" s="47" t="s">
+      <c r="B105" s="21" t="s">
         <v>142</v>
       </c>
+      <c r="C105" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" s="8" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C106" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D106" s="8" t="s">
+      <c r="B106" s="47" t="s">
         <v>144</v>
       </c>
     </row>
@@ -13758,8 +13915,8 @@
       <c r="B107" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="C107" s="20" t="n">
-        <v>0.05</v>
+      <c r="C107" s="19" t="n">
+        <v>4000</v>
       </c>
       <c r="D107" s="8" t="s">
         <v>146</v>
@@ -13769,8 +13926,8 @@
       <c r="B108" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C108" s="19" t="n">
-        <v>0</v>
+      <c r="C108" s="20" t="n">
+        <v>0.05</v>
       </c>
       <c r="D108" s="8" t="s">
         <v>148</v>
@@ -13780,8 +13937,8 @@
       <c r="B109" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C109" s="20" t="n">
-        <v>0.07</v>
+      <c r="C109" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D109" s="8" t="s">
         <v>150</v>
@@ -13791,10 +13948,10 @@
       <c r="B110" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="C110" s="49" t="n">
-        <v>2029</v>
-      </c>
-      <c r="D110" s="10" t="s">
+      <c r="C110" s="20" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D110" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -13803,7 +13960,7 @@
         <v>153</v>
       </c>
       <c r="C111" s="49" t="n">
-        <v>2032</v>
+        <v>2029</v>
       </c>
       <c r="D111" s="10" t="s">
         <v>154</v>
@@ -13813,8 +13970,8 @@
       <c r="B112" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="C112" s="20" t="n">
-        <v>0.05</v>
+      <c r="C112" s="49" t="n">
+        <v>2032</v>
       </c>
       <c r="D112" s="10" t="s">
         <v>156</v>
@@ -13824,31 +13981,31 @@
       <c r="B113" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="C113" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D113" s="8" t="s">
+      <c r="C113" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D113" s="10" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B115" s="10" t="s">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B114" s="21" t="s">
         <v>159</v>
+      </c>
+      <c r="C114" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="8" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B118" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="C118" s="50" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D118" s="8" t="s">
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B117" s="10" t="s">
         <v>162</v>
       </c>
     </row>
@@ -13856,21 +14013,32 @@
       <c r="B119" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="C119" s="19" t="n">
-        <v>3000</v>
+      <c r="C119" s="50" t="n">
+        <v>2000</v>
       </c>
       <c r="D119" s="8" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B121" s="10" t="s">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B120" s="21" t="s">
         <v>165</v>
       </c>
+      <c r="C120" s="19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B122" s="51" t="s">
-        <v>166</v>
+      <c r="B122" s="10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B123" s="51" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -13889,7 +14057,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:M37"/>
+  <dimension ref="B1:M38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -13900,17 +14068,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="53" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="32" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
@@ -13926,7 +14094,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="17" t="s">
@@ -13962,7 +14130,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D6" s="54" t="n">
         <f aca="false">Assumptions!D45</f>
@@ -14007,7 +14175,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D7" s="38" t="n">
         <f aca="false">Assumptions!D46</f>
@@ -14052,7 +14220,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="55" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D8" s="56" t="n">
         <f aca="false">D6*D7</f>
@@ -14097,7 +14265,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D9" s="38" t="n">
         <f aca="false">-(Assumptions!D43*Assumptions!D49+Assumptions!D44*Assumptions!D50)</f>
@@ -14142,7 +14310,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="32" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
@@ -14158,7 +14326,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="17" t="s">
@@ -14194,7 +14362,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="55" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D12" s="56" t="n">
         <f aca="false">D8+D9</f>
@@ -14239,7 +14407,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D13" s="38" t="n">
         <f aca="false">-D8*Assumptions!$C$81</f>
@@ -14284,7 +14452,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D14" s="38" t="n">
         <f aca="false">Assumptions!D53</f>
@@ -14329,7 +14497,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D15" s="38" t="n">
         <f aca="false">-D14*Assumptions!$C$82</f>
@@ -14373,910 +14541,955 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="55" t="s">
-        <v>180</v>
-      </c>
-      <c r="D16" s="56" t="n">
-        <f aca="false">D12+D13+D15</f>
-        <v>-13.34</v>
-      </c>
-      <c r="E16" s="56" t="n">
-        <f aca="false">E12+E13+E15</f>
-        <v>46.9460000000001</v>
-      </c>
-      <c r="F16" s="56" t="n">
-        <f aca="false">F12+F13+F15</f>
-        <v>121.8276</v>
-      </c>
-      <c r="G16" s="56" t="n">
-        <f aca="false">G12+G13+G15</f>
-        <v>148.43784</v>
-      </c>
-      <c r="H16" s="56" t="n">
-        <f aca="false">H12+H13+H15</f>
-        <v>168.667728</v>
-      </c>
-      <c r="I16" s="56" t="n">
-        <f aca="false">I12+I13+I15</f>
+      <c r="B16" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="D16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(D12+D13))</f>
+        <v>200</v>
+      </c>
+      <c r="E16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(E12+E13))</f>
+        <v>127.708</v>
+      </c>
+      <c r="F16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(F12+F13))</f>
+        <v>50.1583999999997</v>
+      </c>
+      <c r="G16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(G12+G13))</f>
+        <v>23.54816</v>
+      </c>
+      <c r="H16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(H12+H13))</f>
+        <v>3.31827199999995</v>
+      </c>
+      <c r="I16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(I12+I13))</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(J12+J13))</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(K12+K13))</f>
+        <v>0.804800000000256</v>
+      </c>
+      <c r="L16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(L12+L13))</f>
+        <v>3.55231999999992</v>
+      </c>
+      <c r="M16" s="38" t="n">
+        <f aca="false">MAX(0,Assumptions!$C$85-(M12+M13))</f>
+        <v>6.29984000000027</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="55" t="s">
+        <v>183</v>
+      </c>
+      <c r="D17" s="56" t="n">
+        <f aca="false">D12+D13+D15+D16</f>
+        <v>186.66</v>
+      </c>
+      <c r="E17" s="56" t="n">
+        <f aca="false">E12+E13+E15+E16</f>
+        <v>174.654</v>
+      </c>
+      <c r="F17" s="56" t="n">
+        <f aca="false">F12+F13+F15+F16</f>
+        <v>171.986</v>
+      </c>
+      <c r="G17" s="56" t="n">
+        <f aca="false">G12+G13+G15+G16</f>
+        <v>171.986</v>
+      </c>
+      <c r="H17" s="56" t="n">
+        <f aca="false">H12+H13+H15+H16</f>
+        <v>171.986</v>
+      </c>
+      <c r="I17" s="56" t="n">
+        <f aca="false">I12+I13+I15+I16</f>
         <v>174.654608</v>
       </c>
-      <c r="J16" s="56" t="n">
-        <f aca="false">J12+J13+J15</f>
+      <c r="J17" s="56" t="n">
+        <f aca="false">J12+J13+J15+J16</f>
         <v>173.92872</v>
       </c>
-      <c r="K16" s="56" t="n">
-        <f aca="false">K12+K13+K15</f>
-        <v>171.1812</v>
-      </c>
-      <c r="L16" s="56" t="n">
-        <f aca="false">L12+L13+L15</f>
-        <v>168.43368</v>
-      </c>
-      <c r="M16" s="56" t="n">
-        <f aca="false">M12+M13+M15</f>
-        <v>165.68616</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="D17" s="57" t="n">
-        <f aca="false">IF(D8=0,0,D16/D8)</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="57" t="n">
-        <f aca="false">IF(E8=0,0,E16/E8)</f>
-        <v>0.064939412383113</v>
-      </c>
-      <c r="F17" s="57" t="n">
-        <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.0741494826536825</v>
-      </c>
-      <c r="G17" s="57" t="n">
-        <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.0762721667283266</v>
-      </c>
-      <c r="H17" s="57" t="n">
-        <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.0774836862647096</v>
-      </c>
-      <c r="I17" s="57" t="n">
-        <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.0776565201121746</v>
-      </c>
-      <c r="J17" s="57" t="n">
-        <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.0775149745432765</v>
-      </c>
-      <c r="K17" s="57" t="n">
-        <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0773427672955974</v>
-      </c>
-      <c r="L17" s="57" t="n">
-        <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0771657430619695</v>
-      </c>
-      <c r="M17" s="57" t="n">
-        <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0769836968642668</v>
+      <c r="K17" s="56" t="n">
+        <f aca="false">K12+K13+K15+K16</f>
+        <v>171.986</v>
+      </c>
+      <c r="L17" s="56" t="n">
+        <f aca="false">L12+L13+L15+L16</f>
+        <v>171.986</v>
+      </c>
+      <c r="M17" s="56" t="n">
+        <f aca="false">M12+M13+M15+M16</f>
+        <v>171.986</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>182</v>
-      </c>
-      <c r="D18" s="38" t="n">
+        <v>184</v>
+      </c>
+      <c r="D18" s="57" t="n">
+        <f aca="false">IF(D8=0,0,D17/D8)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="57" t="n">
+        <f aca="false">IF(E8=0,0,E17/E8)</f>
+        <v>0.241595197255575</v>
+      </c>
+      <c r="F18" s="57" t="n">
+        <f aca="false">IF(F8=0,0,F17/F8)</f>
+        <v>0.104678027997565</v>
+      </c>
+      <c r="G18" s="57" t="n">
+        <f aca="false">IF(G8=0,0,G17/G8)</f>
+        <v>0.0883719735273564</v>
+      </c>
+      <c r="H18" s="57" t="n">
+        <f aca="false">IF(H8=0,0,H17/H8)</f>
+        <v>0.0790080558026034</v>
+      </c>
+      <c r="I18" s="57" t="n">
+        <f aca="false">IF(I8=0,0,I17/I8)</f>
+        <v>0.0776565201121746</v>
+      </c>
+      <c r="J18" s="57" t="n">
+        <f aca="false">IF(J8=0,0,J17/J8)</f>
+        <v>0.0775149745432765</v>
+      </c>
+      <c r="K18" s="57" t="n">
+        <f aca="false">IF(K8=0,0,K17/K8)</f>
+        <v>0.0777063905154341</v>
+      </c>
+      <c r="L18" s="57" t="n">
+        <f aca="false">IF(L8=0,0,L17/L8)</f>
+        <v>0.0787931931799856</v>
+      </c>
+      <c r="M18" s="57" t="n">
+        <f aca="false">IF(M8=0,0,M17/M8)</f>
+        <v>0.079910827125801</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D19" s="38" t="n">
         <f aca="false">(Assumptions!D45)*Assumptions!D8</f>
         <v>0</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="E19" s="38" t="n">
         <f aca="false">(Assumptions!E45)*Assumptions!E8</f>
         <v>209.88</v>
       </c>
-      <c r="F18" s="38" t="n">
+      <c r="F19" s="38" t="n">
         <f aca="false">(Assumptions!F45)*Assumptions!F8</f>
         <v>477</v>
       </c>
-      <c r="G18" s="38" t="n">
+      <c r="G19" s="38" t="n">
         <f aca="false">(Assumptions!G45)*Assumptions!G8</f>
         <v>572.4</v>
       </c>
-      <c r="H18" s="38" t="n">
+      <c r="H19" s="38" t="n">
         <f aca="false">(Assumptions!H45)*Assumptions!H8</f>
         <v>486.54</v>
       </c>
-      <c r="I18" s="38" t="n">
+      <c r="I19" s="38" t="n">
         <f aca="false">(Assumptions!I45)*Assumptions!I8</f>
         <v>339.624</v>
       </c>
-      <c r="J18" s="38" t="n">
+      <c r="J19" s="38" t="n">
         <f aca="false">(Assumptions!J45)*Assumptions!J8</f>
         <v>171.72</v>
       </c>
-      <c r="K18" s="38" t="n">
+      <c r="K19" s="38" t="n">
         <f aca="false">(Assumptions!K45)*Assumptions!K8</f>
         <v>0</v>
       </c>
-      <c r="L18" s="38" t="n">
+      <c r="L19" s="38" t="n">
         <f aca="false">(Assumptions!L45)*Assumptions!L8</f>
         <v>0</v>
       </c>
-      <c r="M18" s="38" t="n">
+      <c r="M19" s="38" t="n">
         <f aca="false">(Assumptions!M45)*Assumptions!M8</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="55" t="s">
-        <v>183</v>
-      </c>
-      <c r="D19" s="56" t="n">
-        <f aca="false">D16+D18</f>
-        <v>-13.34</v>
-      </c>
-      <c r="E19" s="56" t="n">
-        <f aca="false">E16+E18</f>
-        <v>256.826</v>
-      </c>
-      <c r="F19" s="56" t="n">
-        <f aca="false">F16+F18</f>
-        <v>598.8276</v>
-      </c>
-      <c r="G19" s="56" t="n">
-        <f aca="false">G16+G18</f>
-        <v>720.83784</v>
-      </c>
-      <c r="H19" s="56" t="n">
-        <f aca="false">H16+H18</f>
-        <v>655.207728</v>
-      </c>
-      <c r="I19" s="56" t="n">
-        <f aca="false">I16+I18</f>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="55" t="s">
+        <v>186</v>
+      </c>
+      <c r="D20" s="56" t="n">
+        <f aca="false">D17+D19</f>
+        <v>186.66</v>
+      </c>
+      <c r="E20" s="56" t="n">
+        <f aca="false">E17+E19</f>
+        <v>384.534</v>
+      </c>
+      <c r="F20" s="56" t="n">
+        <f aca="false">F17+F19</f>
+        <v>648.986</v>
+      </c>
+      <c r="G20" s="56" t="n">
+        <f aca="false">G17+G19</f>
+        <v>744.386</v>
+      </c>
+      <c r="H20" s="56" t="n">
+        <f aca="false">H17+H19</f>
+        <v>658.526</v>
+      </c>
+      <c r="I20" s="56" t="n">
+        <f aca="false">I17+I19</f>
         <v>514.278608</v>
       </c>
-      <c r="J19" s="56" t="n">
-        <f aca="false">J16+J18</f>
+      <c r="J20" s="56" t="n">
+        <f aca="false">J17+J19</f>
         <v>345.64872</v>
       </c>
-      <c r="K19" s="56" t="n">
-        <f aca="false">K16+K18</f>
-        <v>171.1812</v>
-      </c>
-      <c r="L19" s="56" t="n">
-        <f aca="false">L16+L18</f>
-        <v>168.43368</v>
-      </c>
-      <c r="M19" s="56" t="n">
-        <f aca="false">M16+M18</f>
-        <v>165.68616</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="32" t="s">
-        <v>184</v>
-      </c>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
+      <c r="K20" s="56" t="n">
+        <f aca="false">K17+K19</f>
+        <v>171.986</v>
+      </c>
+      <c r="L20" s="56" t="n">
+        <f aca="false">L17+L19</f>
+        <v>171.986</v>
+      </c>
+      <c r="M20" s="56" t="n">
+        <f aca="false">M17+M19</f>
+        <v>171.986</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="17" t="s">
+      <c r="B22" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E23" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F23" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="G23" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H23" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="17" t="s">
+      <c r="I23" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="J22" s="17" t="s">
+      <c r="J23" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="K23" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="L23" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="M22" s="17" t="s">
+      <c r="M23" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="18" t="s">
-        <v>185</v>
-      </c>
-      <c r="D23" s="38" t="n">
-        <f aca="false">MAX(0,D16)</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="38" t="n">
-        <f aca="false">MAX(0,E16)</f>
-        <v>46.9460000000001</v>
-      </c>
-      <c r="F23" s="38" t="n">
-        <f aca="false">MAX(0,F16)</f>
-        <v>121.8276</v>
-      </c>
-      <c r="G23" s="38" t="n">
-        <f aca="false">MAX(0,G16)</f>
-        <v>148.43784</v>
-      </c>
-      <c r="H23" s="38" t="n">
-        <f aca="false">MAX(0,H16)</f>
-        <v>168.667728</v>
-      </c>
-      <c r="I23" s="38" t="n">
-        <f aca="false">MAX(0,I16)</f>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" s="38" t="n">
+        <f aca="false">MAX(0,D17)</f>
+        <v>186.66</v>
+      </c>
+      <c r="E24" s="38" t="n">
+        <f aca="false">MAX(0,E17)</f>
+        <v>174.654</v>
+      </c>
+      <c r="F24" s="38" t="n">
+        <f aca="false">MAX(0,F17)</f>
+        <v>171.986</v>
+      </c>
+      <c r="G24" s="38" t="n">
+        <f aca="false">MAX(0,G17)</f>
+        <v>171.986</v>
+      </c>
+      <c r="H24" s="38" t="n">
+        <f aca="false">MAX(0,H17)</f>
+        <v>171.986</v>
+      </c>
+      <c r="I24" s="38" t="n">
+        <f aca="false">MAX(0,I17)</f>
         <v>174.654608</v>
       </c>
-      <c r="J23" s="38" t="n">
-        <f aca="false">MAX(0,J16)</f>
+      <c r="J24" s="38" t="n">
+        <f aca="false">MAX(0,J17)</f>
         <v>173.92872</v>
       </c>
-      <c r="K23" s="38" t="n">
-        <f aca="false">MAX(0,K16)</f>
-        <v>171.1812</v>
-      </c>
-      <c r="L23" s="38" t="n">
-        <f aca="false">MAX(0,L16)</f>
-        <v>168.43368</v>
-      </c>
-      <c r="M23" s="38" t="n">
-        <f aca="false">MAX(0,M16)</f>
-        <v>165.68616</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="D24" s="38" t="n">
-        <f aca="false">Assumptions!$C$87</f>
-        <v>4000</v>
-      </c>
-      <c r="E24" s="38" t="n">
-        <f aca="false">D27</f>
-        <v>4013.34</v>
-      </c>
-      <c r="F24" s="38" t="n">
-        <f aca="false">E27</f>
-        <v>3975.7832</v>
-      </c>
-      <c r="G24" s="38" t="n">
-        <f aca="false">F27</f>
-        <v>3878.32112</v>
-      </c>
-      <c r="H24" s="38" t="n">
-        <f aca="false">G27</f>
-        <v>3759.570848</v>
-      </c>
-      <c r="I24" s="38" t="n">
-        <f aca="false">H27</f>
-        <v>3624.6366656</v>
-      </c>
-      <c r="J24" s="38" t="n">
-        <f aca="false">I27</f>
-        <v>3484.9129792</v>
-      </c>
       <c r="K24" s="38" t="n">
-        <f aca="false">J27</f>
-        <v>3345.7700032</v>
+        <f aca="false">MAX(0,K17)</f>
+        <v>171.986</v>
       </c>
       <c r="L24" s="38" t="n">
-        <f aca="false">K27</f>
-        <v>3208.8250432</v>
+        <f aca="false">MAX(0,L17)</f>
+        <v>171.986</v>
       </c>
       <c r="M24" s="38" t="n">
-        <f aca="false">L27</f>
-        <v>3074.0780992</v>
+        <f aca="false">MAX(0,M17)</f>
+        <v>171.986</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D25" s="38" t="n">
-        <f aca="false">MIN(D24,D23*Assumptions!$C$89)</f>
-        <v>0</v>
+        <f aca="false">Assumptions!$C$88</f>
+        <v>4000</v>
       </c>
       <c r="E25" s="38" t="n">
-        <f aca="false">MIN(E24,E23*Assumptions!$C$89)</f>
-        <v>37.5568000000001</v>
+        <f aca="false">D28</f>
+        <v>3850.672</v>
       </c>
       <c r="F25" s="38" t="n">
-        <f aca="false">MIN(F24,F23*Assumptions!$C$89)</f>
-        <v>97.4620800000003</v>
+        <f aca="false">E28</f>
+        <v>3710.9488</v>
       </c>
       <c r="G25" s="38" t="n">
-        <f aca="false">MIN(G24,G23*Assumptions!$C$89)</f>
-        <v>118.750272</v>
+        <f aca="false">F28</f>
+        <v>3573.36</v>
       </c>
       <c r="H25" s="38" t="n">
-        <f aca="false">MIN(H24,H23*Assumptions!$C$89)</f>
-        <v>134.9341824</v>
+        <f aca="false">G28</f>
+        <v>3435.7712</v>
       </c>
       <c r="I25" s="38" t="n">
-        <f aca="false">MIN(I24,I23*Assumptions!$C$89)</f>
-        <v>139.7236864</v>
+        <f aca="false">H28</f>
+        <v>3298.1824</v>
       </c>
       <c r="J25" s="38" t="n">
-        <f aca="false">MIN(J24,J23*Assumptions!$C$89)</f>
-        <v>139.142976</v>
+        <f aca="false">I28</f>
+        <v>3158.4587136</v>
       </c>
       <c r="K25" s="38" t="n">
-        <f aca="false">MIN(K24,K23*Assumptions!$C$89)</f>
-        <v>136.94496</v>
+        <f aca="false">J28</f>
+        <v>3019.3157376</v>
       </c>
       <c r="L25" s="38" t="n">
-        <f aca="false">MIN(L24,L23*Assumptions!$C$89)</f>
-        <v>134.746944</v>
+        <f aca="false">K28</f>
+        <v>2881.7269376</v>
       </c>
       <c r="M25" s="38" t="n">
-        <f aca="false">MIN(M24,M23*Assumptions!$C$89)</f>
-        <v>132.548928</v>
+        <f aca="false">L28</f>
+        <v>2744.1381376</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D26" s="38" t="n">
-        <f aca="false">MAX(0,-D16)</f>
-        <v>13.34</v>
+        <f aca="false">MIN(D25,D24*Assumptions!$C$90)</f>
+        <v>149.328</v>
       </c>
       <c r="E26" s="38" t="n">
-        <f aca="false">MAX(0,-E16)</f>
-        <v>0</v>
+        <f aca="false">MIN(E25,E24*Assumptions!$C$90)</f>
+        <v>139.7232</v>
       </c>
       <c r="F26" s="38" t="n">
-        <f aca="false">MAX(0,-F16)</f>
-        <v>0</v>
+        <f aca="false">MIN(F25,F24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
       <c r="G26" s="38" t="n">
-        <f aca="false">MAX(0,-G16)</f>
-        <v>0</v>
+        <f aca="false">MIN(G25,G24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
       <c r="H26" s="38" t="n">
-        <f aca="false">MAX(0,-H16)</f>
-        <v>0</v>
+        <f aca="false">MIN(H25,H24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
       <c r="I26" s="38" t="n">
-        <f aca="false">MAX(0,-I16)</f>
-        <v>0</v>
+        <f aca="false">MIN(I25,I24*Assumptions!$C$90)</f>
+        <v>139.7236864</v>
       </c>
       <c r="J26" s="38" t="n">
-        <f aca="false">MAX(0,-J16)</f>
-        <v>0</v>
+        <f aca="false">MIN(J25,J24*Assumptions!$C$90)</f>
+        <v>139.142976</v>
       </c>
       <c r="K26" s="38" t="n">
-        <f aca="false">MAX(0,-K16)</f>
-        <v>0</v>
+        <f aca="false">MIN(K25,K24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
       <c r="L26" s="38" t="n">
-        <f aca="false">MAX(0,-L16)</f>
-        <v>0</v>
+        <f aca="false">MIN(L25,L24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
       <c r="M26" s="38" t="n">
-        <f aca="false">MAX(0,-M16)</f>
-        <v>0</v>
+        <f aca="false">MIN(M25,M24*Assumptions!$C$90)</f>
+        <v>137.5888</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D27" s="38" t="n">
-        <f aca="false">D24-D25+D26</f>
-        <v>4013.34</v>
+        <f aca="false">MAX(0,-D17)</f>
+        <v>0</v>
       </c>
       <c r="E27" s="38" t="n">
-        <f aca="false">E24-E25+E26</f>
-        <v>3975.7832</v>
+        <f aca="false">MAX(0,-E17)</f>
+        <v>0</v>
       </c>
       <c r="F27" s="38" t="n">
-        <f aca="false">F24-F25+F26</f>
-        <v>3878.32112</v>
+        <f aca="false">MAX(0,-F17)</f>
+        <v>0</v>
       </c>
       <c r="G27" s="38" t="n">
-        <f aca="false">G24-G25+G26</f>
-        <v>3759.570848</v>
+        <f aca="false">MAX(0,-G17)</f>
+        <v>0</v>
       </c>
       <c r="H27" s="38" t="n">
-        <f aca="false">H24-H25+H26</f>
-        <v>3624.6366656</v>
+        <f aca="false">MAX(0,-H17)</f>
+        <v>0</v>
       </c>
       <c r="I27" s="38" t="n">
-        <f aca="false">I24-I25+I26</f>
-        <v>3484.9129792</v>
+        <f aca="false">MAX(0,-I17)</f>
+        <v>0</v>
       </c>
       <c r="J27" s="38" t="n">
-        <f aca="false">J24-J25+J26</f>
-        <v>3345.7700032</v>
+        <f aca="false">MAX(0,-J17)</f>
+        <v>0</v>
       </c>
       <c r="K27" s="38" t="n">
-        <f aca="false">K24-K25+K26</f>
-        <v>3208.8250432</v>
+        <f aca="false">MAX(0,-K17)</f>
+        <v>0</v>
       </c>
       <c r="L27" s="38" t="n">
-        <f aca="false">L24-L25+L26</f>
-        <v>3074.0780992</v>
+        <f aca="false">MAX(0,-L17)</f>
+        <v>0</v>
       </c>
       <c r="M27" s="38" t="n">
-        <f aca="false">M24-M25+M26</f>
-        <v>2941.5291712</v>
+        <f aca="false">MAX(0,-M17)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="18" t="s">
-        <v>190</v>
+      <c r="B28" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="D28" s="38" t="n">
-        <f aca="false">D23-D25</f>
-        <v>0</v>
+        <f aca="false">D25-D26+D27</f>
+        <v>3850.672</v>
       </c>
       <c r="E28" s="38" t="n">
-        <f aca="false">E23-E25</f>
-        <v>9.38920000000002</v>
+        <f aca="false">E25-E26+E27</f>
+        <v>3710.9488</v>
       </c>
       <c r="F28" s="38" t="n">
-        <f aca="false">F23-F25</f>
-        <v>24.3655200000001</v>
+        <f aca="false">F25-F26+F27</f>
+        <v>3573.36</v>
       </c>
       <c r="G28" s="38" t="n">
-        <f aca="false">G23-G25</f>
-        <v>29.687568</v>
+        <f aca="false">G25-G26+G27</f>
+        <v>3435.7712</v>
       </c>
       <c r="H28" s="38" t="n">
-        <f aca="false">H23-H25</f>
-        <v>33.7335456</v>
+        <f aca="false">H25-H26+H27</f>
+        <v>3298.1824</v>
       </c>
       <c r="I28" s="38" t="n">
-        <f aca="false">I23-I25</f>
-        <v>34.9309216</v>
+        <f aca="false">I25-I26+I27</f>
+        <v>3158.4587136</v>
       </c>
       <c r="J28" s="38" t="n">
-        <f aca="false">J23-J25</f>
-        <v>34.785744</v>
+        <f aca="false">J25-J26+J27</f>
+        <v>3019.3157376</v>
       </c>
       <c r="K28" s="38" t="n">
-        <f aca="false">K23-K25</f>
-        <v>34.23624</v>
+        <f aca="false">K25-K26+K27</f>
+        <v>2881.7269376</v>
       </c>
       <c r="L28" s="38" t="n">
-        <f aca="false">L23-L25</f>
-        <v>33.686736</v>
+        <f aca="false">L25-L26+L27</f>
+        <v>2744.1381376</v>
       </c>
       <c r="M28" s="38" t="n">
-        <f aca="false">M23-M25</f>
-        <v>33.1372319999999</v>
+        <f aca="false">M25-M26+M27</f>
+        <v>2606.5493376</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="18" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D29" s="38" t="n">
-        <f aca="false">-D28*Assumptions!$C$86</f>
-        <v>-0</v>
+        <f aca="false">D24-D26</f>
+        <v>37.332</v>
       </c>
       <c r="E29" s="38" t="n">
-        <f aca="false">-E28*Assumptions!$C$86</f>
-        <v>-2.159516</v>
+        <f aca="false">E24-E26</f>
+        <v>34.9308</v>
       </c>
       <c r="F29" s="38" t="n">
-        <f aca="false">-F28*Assumptions!$C$86</f>
-        <v>-5.60406960000001</v>
+        <f aca="false">F24-F26</f>
+        <v>34.3972</v>
       </c>
       <c r="G29" s="38" t="n">
-        <f aca="false">-G28*Assumptions!$C$86</f>
-        <v>-6.82814064</v>
+        <f aca="false">G24-G26</f>
+        <v>34.3972</v>
       </c>
       <c r="H29" s="38" t="n">
-        <f aca="false">-H28*Assumptions!$C$86</f>
-        <v>-7.758715488</v>
+        <f aca="false">H24-H26</f>
+        <v>34.3972</v>
       </c>
       <c r="I29" s="38" t="n">
-        <f aca="false">-I28*Assumptions!$C$86</f>
+        <f aca="false">I24-I26</f>
+        <v>34.9309216</v>
+      </c>
+      <c r="J29" s="38" t="n">
+        <f aca="false">J24-J26</f>
+        <v>34.785744</v>
+      </c>
+      <c r="K29" s="38" t="n">
+        <f aca="false">K24-K26</f>
+        <v>34.3972</v>
+      </c>
+      <c r="L29" s="38" t="n">
+        <f aca="false">L24-L26</f>
+        <v>34.3972</v>
+      </c>
+      <c r="M29" s="38" t="n">
+        <f aca="false">M24-M26</f>
+        <v>34.3972</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="D30" s="38" t="n">
+        <f aca="false">-D29*Assumptions!$C$87</f>
+        <v>-8.58636</v>
+      </c>
+      <c r="E30" s="38" t="n">
+        <f aca="false">-E29*Assumptions!$C$87</f>
+        <v>-8.034084</v>
+      </c>
+      <c r="F30" s="38" t="n">
+        <f aca="false">-F29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+      <c r="G30" s="38" t="n">
+        <f aca="false">-G29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+      <c r="H30" s="38" t="n">
+        <f aca="false">-H29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+      <c r="I30" s="38" t="n">
+        <f aca="false">-I29*Assumptions!$C$87</f>
         <v>-8.034111968</v>
       </c>
-      <c r="J29" s="38" t="n">
-        <f aca="false">-J28*Assumptions!$C$86</f>
+      <c r="J30" s="38" t="n">
+        <f aca="false">-J29*Assumptions!$C$87</f>
         <v>-8.00072112000001</v>
       </c>
-      <c r="K29" s="38" t="n">
-        <f aca="false">-K28*Assumptions!$C$86</f>
-        <v>-7.87433519999999</v>
-      </c>
-      <c r="L29" s="38" t="n">
-        <f aca="false">-L28*Assumptions!$C$86</f>
-        <v>-7.74794928</v>
-      </c>
-      <c r="M29" s="38" t="n">
-        <f aca="false">-M28*Assumptions!$C$86</f>
-        <v>-7.62156335999998</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="55" t="s">
-        <v>192</v>
-      </c>
-      <c r="D30" s="56" t="n">
-        <f aca="false">D19+D29</f>
-        <v>-13.34</v>
-      </c>
-      <c r="E30" s="56" t="n">
-        <f aca="false">E19+E29</f>
-        <v>254.666484</v>
-      </c>
-      <c r="F30" s="56" t="n">
-        <f aca="false">F19+F29</f>
-        <v>593.2235304</v>
-      </c>
-      <c r="G30" s="56" t="n">
-        <f aca="false">G19+G29</f>
-        <v>714.00969936</v>
-      </c>
-      <c r="H30" s="56" t="n">
-        <f aca="false">H19+H29</f>
-        <v>647.449012512</v>
-      </c>
-      <c r="I30" s="56" t="n">
-        <f aca="false">I19+I29</f>
+      <c r="K30" s="38" t="n">
+        <f aca="false">-K29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+      <c r="L30" s="38" t="n">
+        <f aca="false">-L29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+      <c r="M30" s="38" t="n">
+        <f aca="false">-M29*Assumptions!$C$87</f>
+        <v>-7.911356</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="55" t="s">
+        <v>195</v>
+      </c>
+      <c r="D31" s="56" t="n">
+        <f aca="false">D20+D30</f>
+        <v>178.07364</v>
+      </c>
+      <c r="E31" s="56" t="n">
+        <f aca="false">E20+E30</f>
+        <v>376.499916</v>
+      </c>
+      <c r="F31" s="56" t="n">
+        <f aca="false">F20+F30</f>
+        <v>641.074644</v>
+      </c>
+      <c r="G31" s="56" t="n">
+        <f aca="false">G20+G30</f>
+        <v>736.474644</v>
+      </c>
+      <c r="H31" s="56" t="n">
+        <f aca="false">H20+H30</f>
+        <v>650.614644</v>
+      </c>
+      <c r="I31" s="56" t="n">
+        <f aca="false">I20+I30</f>
         <v>506.244496032</v>
       </c>
-      <c r="J30" s="56" t="n">
-        <f aca="false">J19+J29</f>
+      <c r="J31" s="56" t="n">
+        <f aca="false">J20+J30</f>
         <v>337.64799888</v>
       </c>
-      <c r="K30" s="56" t="n">
-        <f aca="false">K19+K29</f>
-        <v>163.3068648</v>
-      </c>
-      <c r="L30" s="56" t="n">
-        <f aca="false">L19+L29</f>
-        <v>160.68573072</v>
-      </c>
-      <c r="M30" s="56" t="n">
-        <f aca="false">M19+M29</f>
-        <v>158.06459664</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="D31" s="38" t="n">
+      <c r="K31" s="56" t="n">
+        <f aca="false">K20+K30</f>
+        <v>164.074644</v>
+      </c>
+      <c r="L31" s="56" t="n">
+        <f aca="false">L20+L30</f>
+        <v>164.074644</v>
+      </c>
+      <c r="M31" s="56" t="n">
+        <f aca="false">M20+M30</f>
+        <v>164.074644</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="D32" s="38" t="n">
         <f aca="false">-D15</f>
         <v>13.34</v>
       </c>
-      <c r="E31" s="38" t="n">
+      <c r="E32" s="38" t="n">
         <f aca="false">-E15</f>
         <v>25.346</v>
       </c>
-      <c r="F31" s="38" t="n">
+      <c r="F32" s="38" t="n">
         <f aca="false">-F15</f>
         <v>28.014</v>
       </c>
-      <c r="G31" s="38" t="n">
+      <c r="G32" s="38" t="n">
         <f aca="false">-G15</f>
         <v>28.014</v>
       </c>
-      <c r="H31" s="38" t="n">
+      <c r="H32" s="38" t="n">
         <f aca="false">-H15</f>
         <v>28.014</v>
       </c>
-      <c r="I31" s="38" t="n">
+      <c r="I32" s="38" t="n">
         <f aca="false">-I15</f>
         <v>28.014</v>
       </c>
-      <c r="J31" s="38" t="n">
+      <c r="J32" s="38" t="n">
         <f aca="false">-J15</f>
         <v>28.014</v>
       </c>
-      <c r="K31" s="38" t="n">
+      <c r="K32" s="38" t="n">
         <f aca="false">-K15</f>
         <v>28.014</v>
       </c>
-      <c r="L31" s="38" t="n">
+      <c r="L32" s="38" t="n">
         <f aca="false">-L15</f>
         <v>28.014</v>
       </c>
-      <c r="M31" s="38" t="n">
+      <c r="M32" s="38" t="n">
         <f aca="false">-M15</f>
         <v>28.014</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="D32" s="38" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D33" s="38" t="n">
         <f aca="false">-D8*Assumptions!$C$83</f>
         <v>-0</v>
       </c>
-      <c r="E32" s="38" t="n">
+      <c r="E33" s="38" t="n">
         <f aca="false">-E8*Assumptions!$C$83</f>
         <v>-21.6876</v>
       </c>
-      <c r="F32" s="38" t="n">
+      <c r="F33" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$83</f>
         <v>-49.29</v>
       </c>
-      <c r="G32" s="38" t="n">
+      <c r="G33" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$83</f>
         <v>-58.3848</v>
       </c>
-      <c r="H32" s="38" t="n">
+      <c r="H33" s="38" t="n">
         <f aca="false">-H8*Assumptions!$C$83</f>
         <v>-65.30448</v>
       </c>
-      <c r="I32" s="38" t="n">
+      <c r="I33" s="38" t="n">
         <f aca="false">-I8*Assumptions!$C$83</f>
         <v>-67.471968</v>
       </c>
-      <c r="J32" s="38" t="n">
+      <c r="J33" s="38" t="n">
         <f aca="false">-J8*Assumptions!$C$83</f>
         <v>-67.31424</v>
       </c>
-      <c r="K32" s="38" t="n">
+      <c r="K33" s="38" t="n">
         <f aca="false">-K8*Assumptions!$C$83</f>
         <v>-66.3984</v>
       </c>
-      <c r="L32" s="38" t="n">
+      <c r="L33" s="38" t="n">
         <f aca="false">-L8*Assumptions!$C$83</f>
         <v>-65.48256</v>
       </c>
-      <c r="M32" s="38" t="n">
+      <c r="M33" s="38" t="n">
         <f aca="false">-M8*Assumptions!$C$83</f>
         <v>-64.56672</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="21" t="s">
-        <v>195</v>
-      </c>
-      <c r="D33" s="38" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="D34" s="38" t="n">
         <f aca="false">-Assumptions!D53</f>
         <v>-200</v>
       </c>
-      <c r="E33" s="38" t="n">
+      <c r="E34" s="38" t="n">
         <f aca="false">-Assumptions!E53</f>
         <v>-180</v>
       </c>
-      <c r="F33" s="38" t="n">
+      <c r="F34" s="38" t="n">
         <f aca="false">-Assumptions!F53</f>
         <v>-40</v>
       </c>
-      <c r="G33" s="38" t="n">
+      <c r="G34" s="38" t="n">
         <f aca="false">-Assumptions!G53</f>
         <v>-0</v>
       </c>
-      <c r="H33" s="38" t="n">
+      <c r="H34" s="38" t="n">
         <f aca="false">-Assumptions!H53</f>
         <v>-0</v>
       </c>
-      <c r="I33" s="38" t="n">
+      <c r="I34" s="38" t="n">
         <f aca="false">-Assumptions!I53</f>
         <v>-0</v>
       </c>
-      <c r="J33" s="38" t="n">
+      <c r="J34" s="38" t="n">
         <f aca="false">-Assumptions!J53</f>
         <v>-0</v>
       </c>
-      <c r="K33" s="38" t="n">
+      <c r="K34" s="38" t="n">
         <f aca="false">-Assumptions!K53</f>
         <v>-0</v>
       </c>
-      <c r="L33" s="38" t="n">
+      <c r="L34" s="38" t="n">
         <f aca="false">-Assumptions!L53</f>
         <v>-0</v>
       </c>
-      <c r="M33" s="38" t="n">
+      <c r="M34" s="38" t="n">
         <f aca="false">-Assumptions!M53</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="21" t="s">
-        <v>196</v>
-      </c>
-      <c r="D34" s="38" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="D35" s="38" t="n">
         <f aca="false">Assumptions!D53*Assumptions!$C$84</f>
         <v>20</v>
       </c>
-      <c r="E34" s="38" t="n">
+      <c r="E35" s="38" t="n">
         <f aca="false">Assumptions!E53*Assumptions!$C$84</f>
         <v>18</v>
       </c>
-      <c r="F34" s="38" t="n">
+      <c r="F35" s="38" t="n">
         <f aca="false">Assumptions!F53*Assumptions!$C$84</f>
         <v>4</v>
       </c>
-      <c r="G34" s="38" t="n">
+      <c r="G35" s="38" t="n">
         <f aca="false">Assumptions!G53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="H34" s="38" t="n">
+      <c r="H35" s="38" t="n">
         <f aca="false">Assumptions!H53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="I34" s="38" t="n">
+      <c r="I35" s="38" t="n">
         <f aca="false">Assumptions!I53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="J34" s="38" t="n">
+      <c r="J35" s="38" t="n">
         <f aca="false">Assumptions!J53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="K34" s="38" t="n">
+      <c r="K35" s="38" t="n">
         <f aca="false">Assumptions!K53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="L34" s="38" t="n">
+      <c r="L35" s="38" t="n">
         <f aca="false">Assumptions!L53*Assumptions!$C$84</f>
         <v>0</v>
       </c>
-      <c r="M34" s="38" t="n">
+      <c r="M35" s="38" t="n">
         <f aca="false">Assumptions!M53*Assumptions!$C$84</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="D35" s="38" t="n">
-        <f aca="false">D8*Assumptions!$C$85</f>
-        <v>0</v>
-      </c>
-      <c r="E35" s="38" t="n">
-        <f aca="false">E8*Assumptions!$C$85</f>
-        <v>108.438</v>
-      </c>
-      <c r="F35" s="38" t="n">
-        <f aca="false">F8*Assumptions!$C$85</f>
-        <v>246.45</v>
-      </c>
-      <c r="G35" s="38" t="n">
-        <f aca="false">G8*Assumptions!$C$85</f>
-        <v>291.924</v>
-      </c>
-      <c r="H35" s="38" t="n">
-        <f aca="false">H8*Assumptions!$C$85</f>
-        <v>326.5224</v>
-      </c>
-      <c r="I35" s="38" t="n">
-        <f aca="false">I8*Assumptions!$C$85</f>
-        <v>337.35984</v>
-      </c>
-      <c r="J35" s="38" t="n">
-        <f aca="false">J8*Assumptions!$C$85</f>
-        <v>336.5712</v>
-      </c>
-      <c r="K35" s="38" t="n">
-        <f aca="false">K8*Assumptions!$C$85</f>
-        <v>331.992</v>
-      </c>
-      <c r="L35" s="38" t="n">
-        <f aca="false">L8*Assumptions!$C$85</f>
-        <v>327.4128</v>
-      </c>
-      <c r="M35" s="38" t="n">
-        <f aca="false">M8*Assumptions!$C$85</f>
-        <v>322.8336</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="21" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D36" s="38" t="n">
-        <f aca="false">-D35</f>
+        <f aca="false">D8*Assumptions!$C$86</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="38" t="n">
+        <f aca="false">E8*Assumptions!$C$86</f>
+        <v>108.438</v>
+      </c>
+      <c r="F36" s="38" t="n">
+        <f aca="false">F8*Assumptions!$C$86</f>
+        <v>246.45</v>
+      </c>
+      <c r="G36" s="38" t="n">
+        <f aca="false">G8*Assumptions!$C$86</f>
+        <v>291.924</v>
+      </c>
+      <c r="H36" s="38" t="n">
+        <f aca="false">H8*Assumptions!$C$86</f>
+        <v>326.5224</v>
+      </c>
+      <c r="I36" s="38" t="n">
+        <f aca="false">I8*Assumptions!$C$86</f>
+        <v>337.35984</v>
+      </c>
+      <c r="J36" s="38" t="n">
+        <f aca="false">J8*Assumptions!$C$86</f>
+        <v>336.5712</v>
+      </c>
+      <c r="K36" s="38" t="n">
+        <f aca="false">K8*Assumptions!$C$86</f>
+        <v>331.992</v>
+      </c>
+      <c r="L36" s="38" t="n">
+        <f aca="false">L8*Assumptions!$C$86</f>
+        <v>327.4128</v>
+      </c>
+      <c r="M36" s="38" t="n">
+        <f aca="false">M8*Assumptions!$C$86</f>
+        <v>322.8336</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="D37" s="38" t="n">
+        <f aca="false">-D36</f>
         <v>-0</v>
       </c>
-      <c r="E36" s="38" t="n">
-        <f aca="false">-(E35-D35)</f>
+      <c r="E37" s="38" t="n">
+        <f aca="false">-(E36-D36)</f>
         <v>-108.438</v>
       </c>
-      <c r="F36" s="38" t="n">
-        <f aca="false">-(F35-E35)</f>
+      <c r="F37" s="38" t="n">
+        <f aca="false">-(F36-E36)</f>
         <v>-138.012</v>
       </c>
-      <c r="G36" s="38" t="n">
-        <f aca="false">-(G35-F35)</f>
+      <c r="G37" s="38" t="n">
+        <f aca="false">-(G36-F36)</f>
         <v>-45.474</v>
       </c>
-      <c r="H36" s="38" t="n">
-        <f aca="false">-(H35-G35)</f>
+      <c r="H37" s="38" t="n">
+        <f aca="false">-(H36-G36)</f>
         <v>-34.5984</v>
       </c>
-      <c r="I36" s="38" t="n">
-        <f aca="false">-(I35-H35)</f>
+      <c r="I37" s="38" t="n">
+        <f aca="false">-(I36-H36)</f>
         <v>-10.83744</v>
       </c>
-      <c r="J36" s="38" t="n">
-        <f aca="false">-(J35-I35)</f>
+      <c r="J37" s="38" t="n">
+        <f aca="false">-(J36-I36)</f>
         <v>0.788639999999987</v>
       </c>
-      <c r="K36" s="38" t="n">
-        <f aca="false">-(K35-J35)</f>
+      <c r="K37" s="38" t="n">
+        <f aca="false">-(K36-J36)</f>
         <v>4.57920000000001</v>
       </c>
-      <c r="L36" s="38" t="n">
-        <f aca="false">-(L35-K35)</f>
+      <c r="L37" s="38" t="n">
+        <f aca="false">-(L36-K36)</f>
         <v>4.57919999999996</v>
       </c>
-      <c r="M36" s="38" t="n">
-        <f aca="false">-(M35-L35)</f>
+      <c r="M37" s="38" t="n">
+        <f aca="false">-(M36-L36)</f>
         <v>4.57920000000007</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="58" t="s">
-        <v>199</v>
-      </c>
-      <c r="D37" s="59" t="n">
-        <f aca="false">D30+D31+D32+D33+D34+D36</f>
-        <v>-180</v>
-      </c>
-      <c r="E37" s="59" t="n">
-        <f aca="false">E30+E31+E32+E33+E34+E36</f>
-        <v>-12.1131159999998</v>
-      </c>
-      <c r="F37" s="59" t="n">
-        <f aca="false">F30+F31+F32+F33+F34+F36</f>
-        <v>397.9355304</v>
-      </c>
-      <c r="G37" s="59" t="n">
-        <f aca="false">G30+G31+G32+G33+G34+G36</f>
-        <v>638.16489936</v>
-      </c>
-      <c r="H37" s="59" t="n">
-        <f aca="false">H30+H31+H32+H33+H34+H36</f>
-        <v>575.560132512</v>
-      </c>
-      <c r="I37" s="59" t="n">
-        <f aca="false">I30+I31+I32+I33+I34+I36</f>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="58" t="s">
+        <v>202</v>
+      </c>
+      <c r="D38" s="59" t="n">
+        <f aca="false">D31+D32+D33+D34+D35+D37</f>
+        <v>11.41364</v>
+      </c>
+      <c r="E38" s="59" t="n">
+        <f aca="false">E31+E32+E33+E34+E35+E37</f>
+        <v>109.720316</v>
+      </c>
+      <c r="F38" s="59" t="n">
+        <f aca="false">F31+F32+F33+F34+F35+F37</f>
+        <v>445.786644</v>
+      </c>
+      <c r="G38" s="59" t="n">
+        <f aca="false">G31+G32+G33+G34+G35+G37</f>
+        <v>660.629844</v>
+      </c>
+      <c r="H38" s="59" t="n">
+        <f aca="false">H31+H32+H33+H34+H35+H37</f>
+        <v>578.725764</v>
+      </c>
+      <c r="I38" s="59" t="n">
+        <f aca="false">I31+I32+I33+I34+I35+I37</f>
         <v>455.949088032</v>
       </c>
-      <c r="J37" s="59" t="n">
-        <f aca="false">J30+J31+J32+J33+J34+J36</f>
+      <c r="J38" s="59" t="n">
+        <f aca="false">J31+J32+J33+J34+J35+J37</f>
         <v>299.13639888</v>
       </c>
-      <c r="K37" s="59" t="n">
-        <f aca="false">K30+K31+K32+K33+K34+K36</f>
-        <v>129.5016648</v>
-      </c>
-      <c r="L37" s="59" t="n">
-        <f aca="false">L30+L31+L32+L33+L34+L36</f>
-        <v>127.79637072</v>
-      </c>
-      <c r="M37" s="59" t="n">
-        <f aca="false">M30+M31+M32+M33+M34+M36</f>
-        <v>126.09107664</v>
+      <c r="K38" s="59" t="n">
+        <f aca="false">K31+K32+K33+K34+K35+K37</f>
+        <v>130.269444</v>
+      </c>
+      <c r="L38" s="59" t="n">
+        <f aca="false">L31+L32+L33+L34+L35+L37</f>
+        <v>131.185284</v>
+      </c>
+      <c r="M38" s="59" t="n">
+        <f aca="false">M31+M32+M33+M34+M35+M37</f>
+        <v>132.101124</v>
       </c>
     </row>
   </sheetData>
@@ -15306,17 +15519,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="52" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="53" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="12" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -15332,7 +15545,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="17" t="s">
@@ -15368,7 +15581,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="18" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D6" s="60" t="n">
         <f aca="false">Assumptions!D69*Assumptions!D72</f>
@@ -15413,7 +15626,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="18" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D7" s="60" t="n">
         <f aca="false">Assumptions!D70*Assumptions!D75</f>
@@ -15458,7 +15671,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="55" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D8" s="56" t="n">
         <f aca="false">D6+D7</f>
@@ -15503,7 +15716,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D9" s="38" t="n">
         <f aca="false">-(Assumptions!D69*Assumptions!D74+Assumptions!D70*Assumptions!D77)</f>
@@ -15548,7 +15761,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -15564,7 +15777,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="17" t="s">
@@ -15600,7 +15813,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="55" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D12" s="56" t="n">
         <f aca="false">D8+D9</f>
@@ -15645,7 +15858,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D13" s="38" t="n">
         <f aca="false">-D8*Assumptions!$C$81</f>
@@ -15690,7 +15903,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D14" s="38" t="n">
         <f aca="false">Assumptions!D78</f>
@@ -15735,7 +15948,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D15" s="38" t="n">
         <f aca="false">-D14*Assumptions!$C$82</f>
@@ -15780,7 +15993,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="55" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D16" s="56" t="n">
         <f aca="false">D12+D13+D15</f>
@@ -15825,7 +16038,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D17" s="57" t="n">
         <f aca="false">IF(D8=0,0,D16/D8)</f>
@@ -15870,7 +16083,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D18" s="38" t="n">
         <f aca="false">(Assumptions!D69+Assumptions!D70)*Assumptions!D8</f>
@@ -15915,7 +16128,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="55" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D19" s="56" t="n">
         <f aca="false">D16+D18</f>
@@ -15960,7 +16173,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="12" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
@@ -15976,7 +16189,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C22" s="16"/>
       <c r="D22" s="17" t="s">
@@ -16012,7 +16225,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="18" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D23" s="38" t="n">
         <f aca="false">MAX(0,D16)</f>
@@ -16057,10 +16270,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="21" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D24" s="38" t="n">
-        <f aca="false">Assumptions!$C$88</f>
+        <f aca="false">Assumptions!$C$89</f>
         <v>0</v>
       </c>
       <c r="E24" s="38" t="n">
@@ -16102,52 +16315,52 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="21" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D25" s="38" t="n">
-        <f aca="false">MIN(D24,D23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(D24,D23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="E25" s="38" t="n">
-        <f aca="false">MIN(E24,E23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(E24,E23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="F25" s="38" t="n">
-        <f aca="false">MIN(F24,F23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(F24,F23*Assumptions!$C$90)</f>
         <v>36.0717760000002</v>
       </c>
       <c r="G25" s="38" t="n">
-        <f aca="false">MIN(G24,G23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(G24,G23*Assumptions!$C$90)</f>
         <v>23.9582239999998</v>
       </c>
       <c r="H25" s="38" t="n">
-        <f aca="false">MIN(H24,H23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(H24,H23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="I25" s="38" t="n">
-        <f aca="false">MIN(I24,I23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(I24,I23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="J25" s="38" t="n">
-        <f aca="false">MIN(J24,J23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(J24,J23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="K25" s="38" t="n">
-        <f aca="false">MIN(K24,K23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(K24,K23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="L25" s="38" t="n">
-        <f aca="false">MIN(L24,L23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(L24,L23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
       <c r="M25" s="38" t="n">
-        <f aca="false">MIN(M24,M23*Assumptions!$C$89)</f>
+        <f aca="false">MIN(M24,M23*Assumptions!$C$90)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="21" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D26" s="38" t="n">
         <f aca="false">MAX(0,-D16)</f>
@@ -16192,7 +16405,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="21" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D27" s="38" t="n">
         <f aca="false">D24-D25+D26</f>
@@ -16237,7 +16450,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="18" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D28" s="38" t="n">
         <f aca="false">D23-D25</f>
@@ -16282,52 +16495,52 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="18" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D29" s="38" t="n">
-        <f aca="false">-D28*Assumptions!$C$86</f>
+        <f aca="false">-D28*Assumptions!$C$87</f>
         <v>-0</v>
       </c>
       <c r="E29" s="38" t="n">
-        <f aca="false">-E28*Assumptions!$C$86</f>
+        <f aca="false">-E28*Assumptions!$C$87</f>
         <v>-0</v>
       </c>
       <c r="F29" s="38" t="n">
-        <f aca="false">-F28*Assumptions!$C$86</f>
+        <f aca="false">-F28*Assumptions!$C$87</f>
         <v>-2.07412712000001</v>
       </c>
       <c r="G29" s="38" t="n">
-        <f aca="false">-G28*Assumptions!$C$86</f>
+        <f aca="false">-G28*Assumptions!$C$87</f>
         <v>-19.0312653600001</v>
       </c>
       <c r="H29" s="38" t="n">
-        <f aca="false">-H28*Assumptions!$C$86</f>
+        <f aca="false">-H28*Assumptions!$C$87</f>
         <v>-34.75521904</v>
       </c>
       <c r="I29" s="38" t="n">
-        <f aca="false">-I28*Assumptions!$C$86</f>
+        <f aca="false">-I28*Assumptions!$C$87</f>
         <v>-41.1535062400001</v>
       </c>
       <c r="J29" s="38" t="n">
-        <f aca="false">-J28*Assumptions!$C$86</f>
+        <f aca="false">-J28*Assumptions!$C$87</f>
         <v>-43.8787026400001</v>
       </c>
       <c r="K29" s="38" t="n">
-        <f aca="false">-K28*Assumptions!$C$86</f>
+        <f aca="false">-K28*Assumptions!$C$87</f>
         <v>-43.0729924</v>
       </c>
       <c r="L29" s="38" t="n">
-        <f aca="false">-L28*Assumptions!$C$86</f>
+        <f aca="false">-L28*Assumptions!$C$87</f>
         <v>-42.2672821599998</v>
       </c>
       <c r="M29" s="38" t="n">
-        <f aca="false">-M28*Assumptions!$C$86</f>
+        <f aca="false">-M28*Assumptions!$C$87</f>
         <v>-41.4615719200001</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="55" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D30" s="56" t="n">
         <f aca="false">D19+D29</f>
@@ -16372,7 +16585,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="21" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D31" s="38" t="n">
         <f aca="false">-D15</f>
@@ -16417,7 +16630,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="21" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D32" s="38" t="n">
         <f aca="false">-D8*Assumptions!$C$83</f>
@@ -16462,7 +16675,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="21" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D33" s="38" t="n">
         <f aca="false">-Assumptions!D78</f>
@@ -16507,7 +16720,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="21" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D34" s="38" t="n">
         <f aca="false">Assumptions!D78*Assumptions!$C$84</f>
@@ -16552,52 +16765,52 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="21" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D35" s="38" t="n">
-        <f aca="false">D8*Assumptions!$C$85</f>
+        <f aca="false">D8*Assumptions!$C$86</f>
         <v>0</v>
       </c>
       <c r="E35" s="38" t="n">
-        <f aca="false">E8*Assumptions!$C$85</f>
+        <f aca="false">E8*Assumptions!$C$86</f>
         <v>0</v>
       </c>
       <c r="F35" s="38" t="n">
-        <f aca="false">F8*Assumptions!$C$85</f>
+        <f aca="false">F8*Assumptions!$C$86</f>
         <v>186.3162</v>
       </c>
       <c r="G35" s="38" t="n">
-        <f aca="false">G8*Assumptions!$C$85</f>
+        <f aca="false">G8*Assumptions!$C$86</f>
         <v>289.00476</v>
       </c>
       <c r="H35" s="38" t="n">
-        <f aca="false">H8*Assumptions!$C$85</f>
+        <f aca="false">H8*Assumptions!$C$86</f>
         <v>363.01608</v>
       </c>
       <c r="I35" s="38" t="n">
-        <f aca="false">I8*Assumptions!$C$85</f>
+        <f aca="false">I8*Assumptions!$C$86</f>
         <v>409.38048</v>
       </c>
       <c r="J35" s="38" t="n">
-        <f aca="false">J8*Assumptions!$C$85</f>
+        <f aca="false">J8*Assumptions!$C$86</f>
         <v>429.12828</v>
       </c>
       <c r="K35" s="38" t="n">
-        <f aca="false">K8*Assumptions!$C$85</f>
+        <f aca="false">K8*Assumptions!$C$86</f>
         <v>423.2898</v>
       </c>
       <c r="L35" s="38" t="n">
-        <f aca="false">L8*Assumptions!$C$85</f>
+        <f aca="false">L8*Assumptions!$C$86</f>
         <v>417.45132</v>
       </c>
       <c r="M35" s="38" t="n">
-        <f aca="false">M8*Assumptions!$C$85</f>
+        <f aca="false">M8*Assumptions!$C$86</f>
         <v>411.61284</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="21" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D36" s="38" t="n">
         <f aca="false">-D35</f>
@@ -16642,7 +16855,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="58" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D37" s="59" t="n">
         <f aca="false">D30+D31+D32+D33+D34+D36</f>
@@ -16712,17 +16925,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="53" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="43" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C4" s="44"/>
       <c r="D4" s="44"/>
@@ -16738,7 +16951,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="17" t="s">
@@ -16774,7 +16987,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="61" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D6" s="62" t="n">
         <f aca="false">SKBA!D8</f>
@@ -16819,7 +17032,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="63" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D7" s="64" t="n">
         <f aca="false">SKOT!D8</f>
@@ -16864,7 +17077,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="55" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D8" s="56" t="n">
         <f aca="false">D6+D7</f>
@@ -16909,7 +17122,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D9" s="54" t="n">
         <f aca="false">SKBA!D6+Assumptions!D69+Assumptions!D70</f>
@@ -16954,7 +17167,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="43" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
@@ -16970,7 +17183,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="17" t="s">
@@ -17006,52 +17219,52 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D13" s="38" t="n">
-        <f aca="false">SKBA!D16+SKOT!D16</f>
-        <v>-26.68</v>
+        <f aca="false">SKBA!D17+SKOT!D16</f>
+        <v>173.32</v>
       </c>
       <c r="E13" s="38" t="n">
-        <f aca="false">SKBA!E16+SKOT!E16</f>
-        <v>0.256000000000093</v>
+        <f aca="false">SKBA!E17+SKOT!E16</f>
+        <v>127.964</v>
       </c>
       <c r="F13" s="38" t="n">
-        <f aca="false">SKBA!F16+SKOT!F16</f>
-        <v>166.917320000001</v>
+        <f aca="false">SKBA!F17+SKOT!F16</f>
+        <v>217.07572</v>
       </c>
       <c r="G13" s="38" t="n">
-        <f aca="false">SKBA!G16+SKOT!G16</f>
-        <v>255.140696</v>
+        <f aca="false">SKBA!G17+SKOT!G16</f>
+        <v>278.688856</v>
       </c>
       <c r="H13" s="38" t="n">
-        <f aca="false">SKBA!H16+SKOT!H16</f>
-        <v>319.777376</v>
+        <f aca="false">SKBA!H17+SKOT!H16</f>
+        <v>323.095648</v>
       </c>
       <c r="I13" s="38" t="n">
-        <f aca="false">SKBA!I16+SKOT!I16</f>
+        <f aca="false">SKBA!I17+SKOT!I16</f>
         <v>353.582896</v>
       </c>
       <c r="J13" s="38" t="n">
-        <f aca="false">SKBA!J16+SKOT!J16</f>
+        <f aca="false">SKBA!J17+SKOT!J16</f>
         <v>364.705688</v>
       </c>
       <c r="K13" s="38" t="n">
-        <f aca="false">SKBA!K16+SKOT!K16</f>
-        <v>358.45508</v>
+        <f aca="false">SKBA!K17+SKOT!K16</f>
+        <v>359.25988</v>
       </c>
       <c r="L13" s="38" t="n">
-        <f aca="false">SKBA!L16+SKOT!L16</f>
-        <v>352.204471999999</v>
+        <f aca="false">SKBA!L17+SKOT!L16</f>
+        <v>355.756791999999</v>
       </c>
       <c r="M13" s="38" t="n">
-        <f aca="false">SKBA!M16+SKOT!M16</f>
-        <v>345.953864</v>
+        <f aca="false">SKBA!M17+SKOT!M16</f>
+        <v>352.253704</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D14" s="57" t="n">
         <f aca="false">IF(D8=0,0,D13/D8)</f>
@@ -17059,19 +17272,19 @@
       </c>
       <c r="E14" s="57" t="n">
         <f aca="false">IF(E8=0,0,E13/E8)</f>
-        <v>0.000354119404636879</v>
+        <v>0.177009904277098</v>
       </c>
       <c r="F14" s="57" t="n">
         <f aca="false">IF(F8=0,0,F13/F8)</f>
-        <v>0.057854790877846</v>
+        <v>0.0752400672695789</v>
       </c>
       <c r="G14" s="57" t="n">
         <f aca="false">IF(G8=0,0,G13/G8)</f>
-        <v>0.0658791697625712</v>
+        <v>0.0719594746867068</v>
       </c>
       <c r="H14" s="57" t="n">
         <f aca="false">IF(H8=0,0,H13/H8)</f>
-        <v>0.0695633496770187</v>
+        <v>0.0702851959763</v>
       </c>
       <c r="I14" s="57" t="n">
         <f aca="false">IF(I8=0,0,I13/I8)</f>
@@ -17083,110 +17296,110 @@
       </c>
       <c r="K14" s="57" t="n">
         <f aca="false">IF(K8=0,0,K13/K8)</f>
-        <v>0.0711896698689151</v>
+        <v>0.0713495042512609</v>
       </c>
       <c r="L14" s="57" t="n">
         <f aca="false">IF(L8=0,0,L13/L8)</f>
-        <v>0.0709265883286201</v>
+        <v>0.071641951017858</v>
       </c>
       <c r="M14" s="57" t="n">
         <f aca="false">IF(M8=0,0,M13/M8)</f>
-        <v>0.0706560434822177</v>
+        <v>0.0719426941466284</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D15" s="38" t="n">
-        <f aca="false">SKBA!D18+SKOT!D18</f>
+        <f aca="false">SKBA!D19+SKOT!D18</f>
         <v>0</v>
       </c>
       <c r="E15" s="38" t="n">
-        <f aca="false">SKBA!E18+SKOT!E18</f>
+        <f aca="false">SKBA!E19+SKOT!E18</f>
         <v>209.88</v>
       </c>
       <c r="F15" s="38" t="n">
-        <f aca="false">SKBA!F18+SKOT!F18</f>
+        <f aca="false">SKBA!F19+SKOT!F18</f>
         <v>851.22</v>
       </c>
       <c r="G15" s="38" t="n">
-        <f aca="false">SKBA!G18+SKOT!G18</f>
+        <f aca="false">SKBA!G19+SKOT!G18</f>
         <v>1160.46</v>
       </c>
       <c r="H15" s="38" t="n">
-        <f aca="false">SKBA!H18+SKOT!H18</f>
+        <f aca="false">SKBA!H19+SKOT!H18</f>
         <v>1047.87</v>
       </c>
       <c r="I15" s="38" t="n">
-        <f aca="false">SKBA!I18+SKOT!I18</f>
+        <f aca="false">SKBA!I19+SKOT!I18</f>
         <v>767.304</v>
       </c>
       <c r="J15" s="38" t="n">
-        <f aca="false">SKBA!J18+SKOT!J18</f>
+        <f aca="false">SKBA!J19+SKOT!J18</f>
         <v>398.925</v>
       </c>
       <c r="K15" s="38" t="n">
-        <f aca="false">SKBA!K18+SKOT!K18</f>
+        <f aca="false">SKBA!K19+SKOT!K18</f>
         <v>0</v>
       </c>
       <c r="L15" s="38" t="n">
-        <f aca="false">SKBA!L18+SKOT!L18</f>
+        <f aca="false">SKBA!L19+SKOT!L18</f>
         <v>0</v>
       </c>
       <c r="M15" s="38" t="n">
-        <f aca="false">SKBA!M18+SKOT!M18</f>
+        <f aca="false">SKBA!M19+SKOT!M18</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="55" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D16" s="56" t="n">
-        <f aca="false">SKBA!D19+SKOT!D19</f>
-        <v>-26.68</v>
+        <f aca="false">SKBA!D20+SKOT!D19</f>
+        <v>173.32</v>
       </c>
       <c r="E16" s="56" t="n">
-        <f aca="false">SKBA!E19+SKOT!E19</f>
-        <v>210.136</v>
+        <f aca="false">SKBA!E20+SKOT!E19</f>
+        <v>337.844</v>
       </c>
       <c r="F16" s="56" t="n">
-        <f aca="false">SKBA!F19+SKOT!F19</f>
-        <v>1018.13732</v>
+        <f aca="false">SKBA!F20+SKOT!F19</f>
+        <v>1068.29572</v>
       </c>
       <c r="G16" s="56" t="n">
-        <f aca="false">SKBA!G19+SKOT!G19</f>
-        <v>1415.600696</v>
+        <f aca="false">SKBA!G20+SKOT!G19</f>
+        <v>1439.148856</v>
       </c>
       <c r="H16" s="56" t="n">
-        <f aca="false">SKBA!H19+SKOT!H19</f>
-        <v>1367.647376</v>
+        <f aca="false">SKBA!H20+SKOT!H19</f>
+        <v>1370.965648</v>
       </c>
       <c r="I16" s="56" t="n">
-        <f aca="false">SKBA!I19+SKOT!I19</f>
+        <f aca="false">SKBA!I20+SKOT!I19</f>
         <v>1120.886896</v>
       </c>
       <c r="J16" s="56" t="n">
-        <f aca="false">SKBA!J19+SKOT!J19</f>
+        <f aca="false">SKBA!J20+SKOT!J19</f>
         <v>763.630688</v>
       </c>
       <c r="K16" s="56" t="n">
-        <f aca="false">SKBA!K19+SKOT!K19</f>
-        <v>358.45508</v>
+        <f aca="false">SKBA!K20+SKOT!K19</f>
+        <v>359.25988</v>
       </c>
       <c r="L16" s="56" t="n">
-        <f aca="false">SKBA!L19+SKOT!L19</f>
-        <v>352.204471999999</v>
+        <f aca="false">SKBA!L20+SKOT!L19</f>
+        <v>355.756791999999</v>
       </c>
       <c r="M16" s="56" t="n">
-        <f aca="false">SKBA!M19+SKOT!M19</f>
-        <v>345.953864</v>
+        <f aca="false">SKBA!M20+SKOT!M19</f>
+        <v>352.253704</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D17" s="57" t="n">
         <f aca="false">IF(D8=0,0,D16/D8)</f>
@@ -17194,19 +17407,19 @@
       </c>
       <c r="E17" s="57" t="n">
         <f aca="false">IF(E8=0,0,E16/E8)</f>
-        <v>0.290676700049798</v>
+        <v>0.46733248492226</v>
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.352894006047607</v>
+        <v>0.37027928243934</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.365518320008808</v>
+        <v>0.371598624932944</v>
       </c>
       <c r="H17" s="57" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.297513644778751</v>
+        <v>0.298235491078032</v>
       </c>
       <c r="I17" s="57" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
@@ -17218,20 +17431,20 @@
       </c>
       <c r="K17" s="57" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0711896698689151</v>
+        <v>0.0713495042512609</v>
       </c>
       <c r="L17" s="57" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0709265883286201</v>
+        <v>0.071641951017858</v>
       </c>
       <c r="M17" s="57" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0706560434822177</v>
+        <v>0.0719426941466284</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D18" s="38" t="n">
         <f aca="false">-(SKBA!D15+SKOT!D15)</f>
@@ -17276,27 +17489,27 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="55" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D19" s="56" t="n">
         <f aca="false">D16+D18</f>
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E19" s="56" t="n">
         <f aca="false">E16+E18</f>
-        <v>282.172</v>
+        <v>409.88</v>
       </c>
       <c r="F19" s="56" t="n">
         <f aca="false">F16+F18</f>
-        <v>1112.85132</v>
+        <v>1163.00972</v>
       </c>
       <c r="G19" s="56" t="n">
         <f aca="false">G16+G18</f>
-        <v>1510.314696</v>
+        <v>1533.862856</v>
       </c>
       <c r="H19" s="56" t="n">
         <f aca="false">H16+H18</f>
-        <v>1462.361376</v>
+        <v>1465.679648</v>
       </c>
       <c r="I19" s="56" t="n">
         <f aca="false">I16+I18</f>
@@ -17308,20 +17521,20 @@
       </c>
       <c r="K19" s="56" t="n">
         <f aca="false">K16+K18</f>
-        <v>453.16908</v>
+        <v>453.97388</v>
       </c>
       <c r="L19" s="56" t="n">
         <f aca="false">L16+L18</f>
-        <v>446.918471999999</v>
+        <v>450.470791999999</v>
       </c>
       <c r="M19" s="56" t="n">
         <f aca="false">M16+M18</f>
-        <v>440.667864</v>
+        <v>446.967704</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D20" s="57" t="n">
         <f aca="false">IF(D8=0,0,D19/D8)</f>
@@ -17329,19 +17542,19 @@
       </c>
       <c r="E20" s="57" t="n">
         <f aca="false">IF(E8=0,0,E19/E8)</f>
-        <v>0.390322580645161</v>
+        <v>0.566978365517623</v>
       </c>
       <c r="F20" s="57" t="n">
         <f aca="false">IF(F8=0,0,F19/F8)</f>
-        <v>0.385722586468167</v>
+        <v>0.4031078628599</v>
       </c>
       <c r="G20" s="57" t="n">
         <f aca="false">IF(G8=0,0,G19/G8)</f>
-        <v>0.389974158621446</v>
+        <v>0.396054463545582</v>
       </c>
       <c r="H20" s="57" t="n">
         <f aca="false">IF(H8=0,0,H19/H8)</f>
-        <v>0.318117426020952</v>
+        <v>0.318839272320234</v>
       </c>
       <c r="I20" s="57" t="n">
         <f aca="false">IF(I8=0,0,I19/I8)</f>
@@ -17353,40 +17566,40 @@
       </c>
       <c r="K20" s="57" t="n">
         <f aca="false">IF(K8=0,0,K19/K8)</f>
-        <v>0.09</v>
+        <v>0.0901598343823458</v>
       </c>
       <c r="L20" s="57" t="n">
         <f aca="false">IF(L8=0,0,L19/L8)</f>
-        <v>0.0899999999999999</v>
+        <v>0.0907153626892377</v>
       </c>
       <c r="M20" s="57" t="n">
         <f aca="false">IF(M8=0,0,M19/M8)</f>
-        <v>0.09</v>
+        <v>0.0912866506644107</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="65" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D21" s="39" t="n">
         <f aca="false">D19-D15</f>
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E21" s="39" t="n">
         <f aca="false">E19-E15</f>
-        <v>72.2920000000001</v>
+        <v>200</v>
       </c>
       <c r="F21" s="39" t="n">
         <f aca="false">F19-F15</f>
-        <v>261.631320000001</v>
+        <v>311.78972</v>
       </c>
       <c r="G21" s="39" t="n">
         <f aca="false">G19-G15</f>
-        <v>349.854696</v>
+        <v>373.402856</v>
       </c>
       <c r="H21" s="39" t="n">
         <f aca="false">H19-H15</f>
-        <v>414.491376</v>
+        <v>417.809648</v>
       </c>
       <c r="I21" s="39" t="n">
         <f aca="false">I19-I15</f>
@@ -17398,20 +17611,20 @@
       </c>
       <c r="K21" s="39" t="n">
         <f aca="false">K19-K15</f>
-        <v>453.16908</v>
+        <v>453.97388</v>
       </c>
       <c r="L21" s="39" t="n">
         <f aca="false">L19-L15</f>
-        <v>446.918471999999</v>
+        <v>450.470791999999</v>
       </c>
       <c r="M21" s="39" t="n">
         <f aca="false">M19-M15</f>
-        <v>440.667864</v>
+        <v>446.967704</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="21" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D22" s="57" t="n">
         <f aca="false">IF(D8=0,0,D21/D8)</f>
@@ -17419,19 +17632,19 @@
       </c>
       <c r="E22" s="57" t="n">
         <f aca="false">IF(E8=0,0,E21/E8)</f>
-        <v>0.1</v>
+        <v>0.276655784872462</v>
       </c>
       <c r="F22" s="57" t="n">
         <f aca="false">IF(F8=0,0,F21/F8)</f>
-        <v>0.0906833712984057</v>
+        <v>0.108068647690139</v>
       </c>
       <c r="G22" s="57" t="n">
         <f aca="false">IF(G8=0,0,G21/G8)</f>
-        <v>0.0903350083752094</v>
+        <v>0.096415313299345</v>
       </c>
       <c r="H22" s="57" t="n">
         <f aca="false">IF(H8=0,0,H21/H8)</f>
-        <v>0.0901671309192201</v>
+        <v>0.0908889772185013</v>
       </c>
       <c r="I22" s="57" t="n">
         <f aca="false">IF(I8=0,0,I21/I8)</f>
@@ -17443,20 +17656,20 @@
       </c>
       <c r="K22" s="57" t="n">
         <f aca="false">IF(K8=0,0,K21/K8)</f>
-        <v>0.09</v>
+        <v>0.0901598343823458</v>
       </c>
       <c r="L22" s="57" t="n">
         <f aca="false">IF(L8=0,0,L21/L8)</f>
-        <v>0.0899999999999999</v>
+        <v>0.0907153626892377</v>
       </c>
       <c r="M22" s="57" t="n">
         <f aca="false">IF(M8=0,0,M21/M8)</f>
-        <v>0.09</v>
+        <v>0.0912866506644107</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="43" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C24" s="44"/>
       <c r="D24" s="44"/>
@@ -17472,7 +17685,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="17" t="s">
@@ -17508,52 +17721,52 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="21" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D26" s="66" t="n">
-        <f aca="false">SKBA!D37</f>
-        <v>-180</v>
+        <f aca="false">SKBA!D38</f>
+        <v>11.41364</v>
       </c>
       <c r="E26" s="66" t="n">
-        <f aca="false">SKBA!E37</f>
-        <v>-12.1131159999998</v>
+        <f aca="false">SKBA!E38</f>
+        <v>109.720316</v>
       </c>
       <c r="F26" s="66" t="n">
-        <f aca="false">SKBA!F37</f>
-        <v>397.9355304</v>
+        <f aca="false">SKBA!F38</f>
+        <v>445.786644</v>
       </c>
       <c r="G26" s="66" t="n">
-        <f aca="false">SKBA!G37</f>
-        <v>638.16489936</v>
+        <f aca="false">SKBA!G38</f>
+        <v>660.629844</v>
       </c>
       <c r="H26" s="66" t="n">
-        <f aca="false">SKBA!H37</f>
-        <v>575.560132512</v>
+        <f aca="false">SKBA!H38</f>
+        <v>578.725764</v>
       </c>
       <c r="I26" s="66" t="n">
-        <f aca="false">SKBA!I37</f>
+        <f aca="false">SKBA!I38</f>
         <v>455.949088032</v>
       </c>
       <c r="J26" s="66" t="n">
-        <f aca="false">SKBA!J37</f>
+        <f aca="false">SKBA!J38</f>
         <v>299.13639888</v>
       </c>
       <c r="K26" s="66" t="n">
-        <f aca="false">SKBA!K37</f>
-        <v>129.5016648</v>
+        <f aca="false">SKBA!K38</f>
+        <v>130.269444</v>
       </c>
       <c r="L26" s="66" t="n">
-        <f aca="false">SKBA!L37</f>
-        <v>127.79637072</v>
+        <f aca="false">SKBA!L38</f>
+        <v>131.185284</v>
       </c>
       <c r="M26" s="66" t="n">
-        <f aca="false">SKBA!M37</f>
-        <v>126.09107664</v>
+        <f aca="false">SKBA!M38</f>
+        <v>132.101124</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="21" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D27" s="66" t="n">
         <f aca="false">SKOT!D37</f>
@@ -17598,27 +17811,27 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="58" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D28" s="59" t="n">
         <f aca="false">D26+D27</f>
-        <v>-360</v>
+        <v>-168.58636</v>
       </c>
       <c r="E28" s="59" t="n">
         <f aca="false">E26+E27</f>
-        <v>-462.113116</v>
+        <v>-340.279684</v>
       </c>
       <c r="F28" s="59" t="n">
         <f aca="false">F26+F27</f>
-        <v>388.291683280001</v>
+        <v>436.14279688</v>
       </c>
       <c r="G28" s="59" t="n">
         <f aca="false">G26+G27</f>
-        <v>1220.106978</v>
+        <v>1242.57192264</v>
       </c>
       <c r="H28" s="59" t="n">
         <f aca="false">H26+H27</f>
-        <v>1173.330025472</v>
+        <v>1176.49565696</v>
       </c>
       <c r="I28" s="59" t="n">
         <f aca="false">I26+I27</f>
@@ -17630,20 +17843,20 @@
       </c>
       <c r="K28" s="59" t="n">
         <f aca="false">K26+K27</f>
-        <v>261.5830724</v>
+        <v>262.3508516</v>
       </c>
       <c r="L28" s="59" t="n">
         <f aca="false">L26+L27</f>
-        <v>258.34809656</v>
+        <v>261.737009839999</v>
       </c>
       <c r="M28" s="59" t="n">
         <f aca="false">M26+M27</f>
-        <v>255.11312072</v>
+        <v>261.12316808</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="4" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -17659,7 +17872,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="17" t="s">
@@ -17695,162 +17908,162 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="21" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="E32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="F32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="G32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="H32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="I32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="J32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="K32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="L32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
       <c r="M32" s="38" t="n">
-        <f aca="false">-Assumptions!$C$102*Assumptions!$C$103</f>
+        <f aca="false">-Assumptions!$C$103*Assumptions!$C$104</f>
         <v>-55.38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="21" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D33" s="38" t="n">
-        <f aca="false">-D32*Assumptions!$C$86</f>
+        <f aca="false">-D32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="E33" s="38" t="n">
-        <f aca="false">-E32*Assumptions!$C$86</f>
+        <f aca="false">-E32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="F33" s="38" t="n">
-        <f aca="false">-F32*Assumptions!$C$86</f>
+        <f aca="false">-F32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="G33" s="38" t="n">
-        <f aca="false">-G32*Assumptions!$C$86</f>
+        <f aca="false">-G32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="H33" s="38" t="n">
-        <f aca="false">-H32*Assumptions!$C$86</f>
+        <f aca="false">-H32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="I33" s="38" t="n">
-        <f aca="false">-I32*Assumptions!$C$86</f>
+        <f aca="false">-I32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="J33" s="38" t="n">
-        <f aca="false">-J32*Assumptions!$C$86</f>
+        <f aca="false">-J32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="K33" s="38" t="n">
-        <f aca="false">-K32*Assumptions!$C$86</f>
+        <f aca="false">-K32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="L33" s="38" t="n">
-        <f aca="false">-L32*Assumptions!$C$86</f>
+        <f aca="false">-L32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
       <c r="M33" s="38" t="n">
-        <f aca="false">-M32*Assumptions!$C$86</f>
+        <f aca="false">-M32*Assumptions!$C$87</f>
         <v>12.7374</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="21" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="E34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="F34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="G34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="H34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="I34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="J34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="K34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="L34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="M34" s="38" t="n">
-        <f aca="false">-Assumptions!$C$104*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$105*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="55" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D35" s="56" t="n">
         <f aca="false">D26+D32+D33+D34</f>
-        <v>-222.6426</v>
+        <v>-31.22896</v>
       </c>
       <c r="E35" s="56" t="n">
         <f aca="false">E26+E32+E33+E34</f>
-        <v>-54.7557159999998</v>
+        <v>67.077716</v>
       </c>
       <c r="F35" s="56" t="n">
         <f aca="false">F26+F32+F33+F34</f>
-        <v>355.2929304</v>
+        <v>403.144044</v>
       </c>
       <c r="G35" s="56" t="n">
         <f aca="false">G26+G32+G33+G34</f>
-        <v>595.52229936</v>
+        <v>617.987244</v>
       </c>
       <c r="H35" s="56" t="n">
         <f aca="false">H26+H32+H33+H34</f>
-        <v>532.917532512</v>
+        <v>536.083164</v>
       </c>
       <c r="I35" s="56" t="n">
         <f aca="false">I26+I32+I33+I34</f>
@@ -17862,335 +18075,335 @@
       </c>
       <c r="K35" s="56" t="n">
         <f aca="false">K26+K32+K33+K34</f>
-        <v>86.8590647999998</v>
+        <v>87.626844</v>
       </c>
       <c r="L35" s="56" t="n">
         <f aca="false">L26+L32+L33+L34</f>
-        <v>85.15377072</v>
+        <v>88.542684</v>
       </c>
       <c r="M35" s="56" t="n">
         <f aca="false">M26+M32+M33+M34</f>
-        <v>83.4484766399998</v>
+        <v>89.4585240000001</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="21" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="E36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="F36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="G36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="H36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="I36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="J36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="K36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="L36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
       <c r="M36" s="38" t="n">
-        <f aca="false">-Assumptions!$C$106*Assumptions!$C$107</f>
+        <f aca="false">-Assumptions!$C$107*Assumptions!$C$108</f>
         <v>-200</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="21" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D37" s="38" t="n">
-        <f aca="false">-D36*Assumptions!$C$86</f>
+        <f aca="false">-D36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="E37" s="38" t="n">
-        <f aca="false">-E36*Assumptions!$C$86</f>
+        <f aca="false">-E36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="F37" s="38" t="n">
-        <f aca="false">-F36*Assumptions!$C$86</f>
+        <f aca="false">-F36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="G37" s="38" t="n">
-        <f aca="false">-G36*Assumptions!$C$86</f>
+        <f aca="false">-G36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="H37" s="38" t="n">
-        <f aca="false">-H36*Assumptions!$C$86</f>
+        <f aca="false">-H36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="I37" s="38" t="n">
-        <f aca="false">-I36*Assumptions!$C$86</f>
+        <f aca="false">-I36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="J37" s="38" t="n">
-        <f aca="false">-J36*Assumptions!$C$86</f>
+        <f aca="false">-J36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="K37" s="38" t="n">
-        <f aca="false">-K36*Assumptions!$C$86</f>
+        <f aca="false">-K36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="L37" s="38" t="n">
-        <f aca="false">-L36*Assumptions!$C$86</f>
+        <f aca="false">-L36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
       <c r="M37" s="38" t="n">
-        <f aca="false">-M36*Assumptions!$C$86</f>
+        <f aca="false">-M36*Assumptions!$C$87</f>
         <v>46</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="18" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="E38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="F38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="G38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="H38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="I38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="J38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="K38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="L38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
       <c r="M38" s="38" t="n">
-        <f aca="false">Assumptions!$C$108/(Assumptions!$C$111-Assumptions!$C$110+1)</f>
+        <f aca="false">Assumptions!$C$109/(Assumptions!$C$112-Assumptions!$C$111+1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="18" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-D38*MAX(0,MIN((2026)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-D38*MAX(0,MIN((2026)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="E39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-E38*MAX(0,MIN((2027)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-E38*MAX(0,MIN((2027)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="F39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-F38*MAX(0,MIN((2028)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-F38*MAX(0,MIN((2028)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="G39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-G38*MAX(0,MIN((2029)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-G38*MAX(0,MIN((2029)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="H39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-H38*MAX(0,MIN((2030)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-H38*MAX(0,MIN((2030)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="I39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-I38*MAX(0,MIN((2031)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-I38*MAX(0,MIN((2031)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="J39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-J38*MAX(0,MIN((2032)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-J38*MAX(0,MIN((2032)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="K39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-K38*MAX(0,MIN((2033)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-K38*MAX(0,MIN((2033)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="L39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-L38*MAX(0,MIN((2034)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-L38*MAX(0,MIN((2034)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
       <c r="M39" s="38" t="n">
-        <f aca="false">MAX(0,Assumptions!$C$108-M38*MAX(0,MIN((2035)-Assumptions!$C$110,Assumptions!$C$111-Assumptions!$C$110+1)))</f>
+        <f aca="false">MAX(0,Assumptions!$C$109-M38*MAX(0,MIN((2035)-Assumptions!$C$111,Assumptions!$C$112-Assumptions!$C$111+1)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="18" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D40" s="38" t="n">
-        <f aca="false">-IF(AND((2026)&gt;=Assumptions!$C$110,(2026)&lt;=Assumptions!$C$111),MIN(D39,D38),0)</f>
+        <f aca="false">-IF(AND((2026)&gt;=Assumptions!$C$111,(2026)&lt;=Assumptions!$C$112),MIN(D39,D38),0)</f>
         <v>-0</v>
       </c>
       <c r="E40" s="38" t="n">
-        <f aca="false">-IF(AND((2027)&gt;=Assumptions!$C$110,(2027)&lt;=Assumptions!$C$111),MIN(E39,E38),0)</f>
+        <f aca="false">-IF(AND((2027)&gt;=Assumptions!$C$111,(2027)&lt;=Assumptions!$C$112),MIN(E39,E38),0)</f>
         <v>-0</v>
       </c>
       <c r="F40" s="38" t="n">
-        <f aca="false">-IF(AND((2028)&gt;=Assumptions!$C$110,(2028)&lt;=Assumptions!$C$111),MIN(F39,F38),0)</f>
+        <f aca="false">-IF(AND((2028)&gt;=Assumptions!$C$111,(2028)&lt;=Assumptions!$C$112),MIN(F39,F38),0)</f>
         <v>-0</v>
       </c>
       <c r="G40" s="38" t="n">
-        <f aca="false">-IF(AND((2029)&gt;=Assumptions!$C$110,(2029)&lt;=Assumptions!$C$111),MIN(G39,G38),0)</f>
+        <f aca="false">-IF(AND((2029)&gt;=Assumptions!$C$111,(2029)&lt;=Assumptions!$C$112),MIN(G39,G38),0)</f>
         <v>-0</v>
       </c>
       <c r="H40" s="38" t="n">
-        <f aca="false">-IF(AND((2030)&gt;=Assumptions!$C$110,(2030)&lt;=Assumptions!$C$111),MIN(H39,H38),0)</f>
+        <f aca="false">-IF(AND((2030)&gt;=Assumptions!$C$111,(2030)&lt;=Assumptions!$C$112),MIN(H39,H38),0)</f>
         <v>-0</v>
       </c>
       <c r="I40" s="38" t="n">
-        <f aca="false">-IF(AND((2031)&gt;=Assumptions!$C$110,(2031)&lt;=Assumptions!$C$111),MIN(I39,I38),0)</f>
+        <f aca="false">-IF(AND((2031)&gt;=Assumptions!$C$111,(2031)&lt;=Assumptions!$C$112),MIN(I39,I38),0)</f>
         <v>-0</v>
       </c>
       <c r="J40" s="38" t="n">
-        <f aca="false">-IF(AND((2032)&gt;=Assumptions!$C$110,(2032)&lt;=Assumptions!$C$111),MIN(J39,J38),0)</f>
+        <f aca="false">-IF(AND((2032)&gt;=Assumptions!$C$111,(2032)&lt;=Assumptions!$C$112),MIN(J39,J38),0)</f>
         <v>-0</v>
       </c>
       <c r="K40" s="38" t="n">
-        <f aca="false">-IF(AND((2033)&gt;=Assumptions!$C$110,(2033)&lt;=Assumptions!$C$111),MIN(K39,K38),0)</f>
+        <f aca="false">-IF(AND((2033)&gt;=Assumptions!$C$111,(2033)&lt;=Assumptions!$C$112),MIN(K39,K38),0)</f>
         <v>-0</v>
       </c>
       <c r="L40" s="38" t="n">
-        <f aca="false">-IF(AND((2034)&gt;=Assumptions!$C$110,(2034)&lt;=Assumptions!$C$111),MIN(L39,L38),0)</f>
+        <f aca="false">-IF(AND((2034)&gt;=Assumptions!$C$111,(2034)&lt;=Assumptions!$C$112),MIN(L39,L38),0)</f>
         <v>-0</v>
       </c>
       <c r="M40" s="38" t="n">
-        <f aca="false">-IF(AND((2035)&gt;=Assumptions!$C$110,(2035)&lt;=Assumptions!$C$111),MIN(M39,M38),0)</f>
+        <f aca="false">-IF(AND((2035)&gt;=Assumptions!$C$111,(2035)&lt;=Assumptions!$C$112),MIN(M39,M38),0)</f>
         <v>-0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="21" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D41" s="38" t="n">
-        <f aca="false">-D39*Assumptions!$C$109</f>
+        <f aca="false">-D39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="E41" s="38" t="n">
-        <f aca="false">-E39*Assumptions!$C$109</f>
+        <f aca="false">-E39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="F41" s="38" t="n">
-        <f aca="false">-F39*Assumptions!$C$109</f>
+        <f aca="false">-F39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="G41" s="38" t="n">
-        <f aca="false">-G39*Assumptions!$C$109</f>
+        <f aca="false">-G39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="H41" s="38" t="n">
-        <f aca="false">-H39*Assumptions!$C$109</f>
+        <f aca="false">-H39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="I41" s="38" t="n">
-        <f aca="false">-I39*Assumptions!$C$109</f>
+        <f aca="false">-I39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="J41" s="38" t="n">
-        <f aca="false">-J39*Assumptions!$C$109</f>
+        <f aca="false">-J39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="K41" s="38" t="n">
-        <f aca="false">-K39*Assumptions!$C$109</f>
+        <f aca="false">-K39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="L41" s="38" t="n">
-        <f aca="false">-L39*Assumptions!$C$109</f>
+        <f aca="false">-L39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
       <c r="M41" s="38" t="n">
-        <f aca="false">-M39*Assumptions!$C$109</f>
+        <f aca="false">-M39*Assumptions!$C$110</f>
         <v>-0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="21" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="E42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="F42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="G42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="H42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="I42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="J42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="K42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="L42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
       <c r="M42" s="38" t="n">
-        <f aca="false">-Assumptions!$C$113*Assumptions!$C$100</f>
+        <f aca="false">-Assumptions!$C$114*Assumptions!$C$101</f>
         <v>-0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="55" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D43" s="56" t="n">
         <f aca="false">D27+D36+D37+D41+D40+D42</f>
@@ -18235,7 +18448,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="21" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D44" s="66" t="n">
         <f aca="false">SKOT!D19-SKOT!D15+SKOT!D32</f>
@@ -18280,7 +18493,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="18" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D45" s="38" t="n">
         <f aca="false">-D36-D41-D40</f>
@@ -18325,7 +18538,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="21" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D46" s="67" t="n">
         <f aca="false">IF(D45=0,0,D44/D45)</f>
@@ -18370,27 +18583,27 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="68" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D47" s="59" t="n">
         <f aca="false">D35+D43</f>
-        <v>-556.6426</v>
+        <v>-365.22896</v>
       </c>
       <c r="E47" s="59" t="n">
         <f aca="false">E35+E43</f>
-        <v>-658.755716</v>
+        <v>-536.922284</v>
       </c>
       <c r="F47" s="59" t="n">
         <f aca="false">F35+F43</f>
-        <v>191.649083280001</v>
+        <v>239.50019688</v>
       </c>
       <c r="G47" s="59" t="n">
         <f aca="false">G35+G43</f>
-        <v>1023.464378</v>
+        <v>1045.92932264</v>
       </c>
       <c r="H47" s="59" t="n">
         <f aca="false">H35+H43</f>
-        <v>976.687425472</v>
+        <v>979.85305696</v>
       </c>
       <c r="I47" s="59" t="n">
         <f aca="false">I35+I43</f>
@@ -18402,85 +18615,85 @@
       </c>
       <c r="K47" s="59" t="n">
         <f aca="false">K35+K43</f>
-        <v>64.9404723999998</v>
+        <v>65.7082516000001</v>
       </c>
       <c r="L47" s="59" t="n">
         <f aca="false">L35+L43</f>
-        <v>61.7054965599995</v>
+        <v>65.0944098399994</v>
       </c>
       <c r="M47" s="59" t="n">
         <f aca="false">M35+M43</f>
-        <v>58.47052072</v>
+        <v>64.4805680800003</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="21" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((1)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((1)-Assumptions!$C$95)</f>
         <v>0.940720868383597</v>
       </c>
       <c r="E48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((2)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((2)-Assumptions!$C$95)</f>
         <v>0.832496343702299</v>
       </c>
       <c r="F48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((3)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((3)-Assumptions!$C$95)</f>
         <v>0.736722428055132</v>
       </c>
       <c r="G48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((4)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((4)-Assumptions!$C$95)</f>
         <v>0.651966750491267</v>
       </c>
       <c r="H48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((5)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((5)-Assumptions!$C$95)</f>
         <v>0.576961726098466</v>
       </c>
       <c r="I48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((6)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((6)-Assumptions!$C$95)</f>
         <v>0.510585598317227</v>
       </c>
       <c r="J48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((7)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((7)-Assumptions!$C$95)</f>
         <v>0.451845662227634</v>
       </c>
       <c r="K48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((8)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((8)-Assumptions!$C$95)</f>
         <v>0.399863417900562</v>
       </c>
       <c r="L48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((9)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((9)-Assumptions!$C$95)</f>
         <v>0.353861431770408</v>
       </c>
       <c r="M48" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$91)^((10)-Assumptions!$C$94)</f>
+        <f aca="false">1/(1+Assumptions!$C$92)^((10)-Assumptions!$C$95)</f>
         <v>0.313151709531335</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="65" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D49" s="39" t="n">
         <f aca="false">D47*D48</f>
-        <v>-523.645310051304</v>
+        <v>-343.578504410038</v>
       </c>
       <c r="E49" s="39" t="n">
         <f aca="false">E47*E48</f>
-        <v>-548.41172496299</v>
+        <v>-446.985838282287</v>
       </c>
       <c r="F49" s="39" t="n">
         <f aca="false">F47*F48</f>
-        <v>141.192177968582</v>
+        <v>176.445166565116</v>
       </c>
       <c r="G49" s="39" t="n">
         <f aca="false">G47*G48</f>
-        <v>667.264744768226</v>
+        <v>681.911141725133</v>
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">H47*H48</f>
-        <v>563.511262858992</v>
+        <v>565.337711066501</v>
       </c>
       <c r="I49" s="39" t="n">
         <f aca="false">I47*I48</f>
@@ -18492,25 +18705,25 @@
       </c>
       <c r="K49" s="39" t="n">
         <f aca="false">K47*K48</f>
-        <v>25.967319253941</v>
+        <v>26.2743260690461</v>
       </c>
       <c r="L49" s="39" t="n">
         <f aca="false">L47*L48</f>
-        <v>21.8351953608254</v>
+        <v>23.034401066232</v>
       </c>
       <c r="M49" s="39" t="n">
         <f aca="false">M47*M48</f>
-        <v>18.3101435206554</v>
+        <v>20.1922001258037</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -18526,7 +18739,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C53" s="16"/>
       <c r="D53" s="17" t="s">
@@ -18562,117 +18775,117 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="21" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D54" s="70" t="n">
-        <f aca="false">(1)-Assumptions!$C$94</f>
+        <f aca="false">(1)-Assumptions!$C$95</f>
         <v>0.5</v>
       </c>
       <c r="E54" s="70" t="n">
-        <f aca="false">(2)-Assumptions!$C$94</f>
+        <f aca="false">(2)-Assumptions!$C$95</f>
         <v>1.5</v>
       </c>
       <c r="F54" s="70" t="n">
-        <f aca="false">(3)-Assumptions!$C$94</f>
+        <f aca="false">(3)-Assumptions!$C$95</f>
         <v>2.5</v>
       </c>
       <c r="G54" s="70" t="n">
-        <f aca="false">(4)-Assumptions!$C$94</f>
+        <f aca="false">(4)-Assumptions!$C$95</f>
         <v>3.5</v>
       </c>
       <c r="H54" s="70" t="n">
-        <f aca="false">(5)-Assumptions!$C$94</f>
+        <f aca="false">(5)-Assumptions!$C$95</f>
         <v>4.5</v>
       </c>
       <c r="I54" s="70" t="n">
-        <f aca="false">(6)-Assumptions!$C$94</f>
+        <f aca="false">(6)-Assumptions!$C$95</f>
         <v>5.5</v>
       </c>
       <c r="J54" s="70" t="n">
-        <f aca="false">(7)-Assumptions!$C$94</f>
+        <f aca="false">(7)-Assumptions!$C$95</f>
         <v>6.5</v>
       </c>
       <c r="K54" s="70" t="n">
-        <f aca="false">(8)-Assumptions!$C$94</f>
+        <f aca="false">(8)-Assumptions!$C$95</f>
         <v>7.5</v>
       </c>
       <c r="L54" s="70" t="n">
-        <f aca="false">(9)-Assumptions!$C$94</f>
+        <f aca="false">(9)-Assumptions!$C$95</f>
         <v>8.5</v>
       </c>
       <c r="M54" s="70" t="n">
-        <f aca="false">(10)-Assumptions!$C$94</f>
+        <f aca="false">(10)-Assumptions!$C$95</f>
         <v>9.5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="21" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^D54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^D54</f>
         <v>0.951302988308988</v>
       </c>
       <c r="E55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^E54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^E54</f>
         <v>0.860907681727591</v>
       </c>
       <c r="F55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^F54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^F54</f>
         <v>0.77910197441411</v>
       </c>
       <c r="G55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^G54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^G54</f>
         <v>0.705069660103267</v>
       </c>
       <c r="H55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^H54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^H54</f>
         <v>0.638072090591192</v>
       </c>
       <c r="I55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^I54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^I54</f>
         <v>0.577440805964879</v>
       </c>
       <c r="J55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^J54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^J54</f>
         <v>0.522570865126588</v>
       </c>
       <c r="K55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^K54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^K54</f>
         <v>0.47291481006931</v>
       </c>
       <c r="L55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^L54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^L54</f>
         <v>0.427977203682634</v>
       </c>
       <c r="M55" s="69" t="n">
-        <f aca="false">1/(1+Assumptions!$C$90)^M54</f>
+        <f aca="false">1/(1+Assumptions!$C$91)^M54</f>
         <v>0.387309686590619</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="65" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D56" s="39" t="n">
         <f aca="false">D28*D55</f>
-        <v>-342.469075791236</v>
+        <v>-160.376708056135</v>
       </c>
       <c r="E56" s="39" t="n">
         <f aca="false">E28*E55</f>
-        <v>-397.836731391473</v>
+        <v>-292.949393891437</v>
       </c>
       <c r="F56" s="39" t="n">
         <f aca="false">F28*F55</f>
-        <v>302.518817092027</v>
+        <v>339.7997141757</v>
       </c>
       <c r="G56" s="39" t="n">
         <f aca="false">G28*G55</f>
-        <v>860.260412268084</v>
+        <v>876.099763149647</v>
       </c>
       <c r="H56" s="39" t="n">
         <f aca="false">H28*H55</f>
-        <v>748.669142306335</v>
+        <v>750.689043407925</v>
       </c>
       <c r="I56" s="39" t="n">
         <f aca="false">I28*I55</f>
@@ -18684,20 +18897,20 @@
       </c>
       <c r="K56" s="39" t="n">
         <f aca="false">K28*K55</f>
-        <v>123.706509001392</v>
+        <v>124.069603155936</v>
       </c>
       <c r="L56" s="39" t="n">
         <f aca="false">L28*L55</f>
-        <v>110.56709594248</v>
+        <v>112.017473571577</v>
       </c>
       <c r="M56" s="39" t="n">
         <f aca="false">M28*M55</f>
-        <v>98.8077828312179</v>
+        <v>101.135532390614</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="71" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -18705,70 +18918,70 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="21" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D59" s="38" t="n">
         <f aca="false">SUM(D56:M56)</f>
-        <v>2389.9895306845</v>
+        <v>2736.2506063295</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="21" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D60" s="38" t="n">
-        <f aca="false">M28*(1+Assumptions!$C$92)/(Assumptions!$C$90-Assumptions!$C$92)</f>
-        <v>3061.35744864</v>
+        <f aca="false">M28*(1+Assumptions!$C$93)/(Assumptions!$C$91-Assumptions!$C$93)</f>
+        <v>3133.47801696</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="21" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D61" s="38" t="n">
         <f aca="false">D60*M55</f>
-        <v>1185.69339397461</v>
+        <v>1213.62638868737</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="72" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D62" s="73" t="n">
         <f aca="false">D59+D61</f>
-        <v>3575.68292465911</v>
+        <v>3949.87699501687</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="21" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D63" s="38" t="n">
-        <f aca="false">-Assumptions!$C$93</f>
+        <f aca="false">-Assumptions!$C$94</f>
         <v>-6400</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="71" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D64" s="74" t="n">
-        <f aca="false">D62-Assumptions!$C$93</f>
-        <v>-2824.31707534089</v>
+        <f aca="false">D62-Assumptions!$C$94</f>
+        <v>-2450.12300498313</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D66" s="75" t="n">
         <f aca="false">D61/D62</f>
-        <v>0.331599143144845</v>
+        <v>0.307256755139077</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="71" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
@@ -18776,57 +18989,57 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="21" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D69" s="38" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>953.496857789527</v>
+        <v>1290.1036529981</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="21" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D70" s="38" t="n">
-        <f aca="false">M47*(1+Assumptions!$C$92)/(Assumptions!$C$91-Assumptions!$C$92)</f>
-        <v>542.181192130909</v>
+        <f aca="false">M47*(1+Assumptions!$C$93)/(Assumptions!$C$92-Assumptions!$C$93)</f>
+        <v>597.910722196367</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="21" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D71" s="38" t="n">
-        <f aca="false">D70*1/(1+Assumptions!$C$91)^((10)-Assumptions!$C$94)</f>
-        <v>169.784967191531</v>
+        <f aca="false">D70*1/(1+Assumptions!$C$92)^((10)-Assumptions!$C$95)</f>
+        <v>187.236764802907</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="72" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D72" s="73" t="n">
         <f aca="false">D69+D71</f>
-        <v>1123.28182498106</v>
+        <v>1477.34041780101</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-2824.31707534089</v>
+        <v>-2450.12300498313</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="51" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="43" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C76" s="44"/>
       <c r="D76" s="44"/>
@@ -18834,62 +19047,62 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="21" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D77" s="66" t="n">
-        <f aca="false">Assumptions!$C$118</f>
+        <f aca="false">Assumptions!$C$119</f>
         <v>2000</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="21" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D78" s="66" t="n">
-        <f aca="false">Assumptions!$C$119</f>
+        <f aca="false">Assumptions!$C$120</f>
         <v>3000</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="77" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D79" s="78" t="n">
-        <f aca="false">Assumptions!$C$118+Assumptions!$C$119</f>
+        <f aca="false">Assumptions!$C$119+Assumptions!$C$120</f>
         <v>5000</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="65" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-2824.31707534089</v>
+        <v>-2450.12300498313</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="53" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D81" s="76" t="n">
-        <f aca="false">(Assumptions!$C$118+Assumptions!$C$119)-D64</f>
-        <v>7824.31707534089</v>
+        <f aca="false">(Assumptions!$C$119+Assumptions!$C$120)-D64</f>
+        <v>7450.12300498313</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="51" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="8" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="4" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C85" s="5"/>
       <c r="D85" s="5"/>
@@ -18897,25 +19110,25 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="21" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D86" s="66" t="n">
         <f aca="false">G21</f>
-        <v>349.854696</v>
+        <v>373.402856</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="21" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D87" s="66" t="n">
         <f aca="false">AVERAGE(H21:J21)</f>
-        <v>440.735986666667</v>
+        <v>441.842077333334</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="80" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D88" s="81" t="n">
         <v>8</v>
@@ -18929,60 +19142,60 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G89" s="8" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="82" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D90" s="79" t="n">
         <f aca="false">$D$86*D88</f>
-        <v>2798.837568</v>
+        <v>2987.222848</v>
       </c>
       <c r="E90" s="79" t="n">
         <f aca="false">$D$86*E88</f>
-        <v>3848.401656</v>
+        <v>4107.431416</v>
       </c>
       <c r="F90" s="79" t="n">
         <f aca="false">$D$86*F88</f>
-        <v>4897.965744</v>
+        <v>5227.639984</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="82" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D91" s="79" t="n">
         <f aca="false">$D$87*D88</f>
-        <v>3525.88789333334</v>
+        <v>3534.73661866667</v>
       </c>
       <c r="E91" s="79" t="n">
         <f aca="false">$D$87*E88</f>
-        <v>4848.09585333334</v>
+        <v>4860.26285066667</v>
       </c>
       <c r="F91" s="79" t="n">
         <f aca="false">$D$87*F88</f>
-        <v>6170.30381333334</v>
+        <v>6185.78908266667</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D92" s="76" t="n">
         <f aca="false">D62</f>
-        <v>3575.68292465911</v>
+        <v>3949.87699501687</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="51" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="8" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
model+deck: 가동률 85%/82%(DC수요) 반영 — run-rate EBITDA·시나리오 갱신
- eff 토글 0.80→1.00(히든 해구트 제거 → util곡선=실효 가동률)
- util plateau: BA 85% / OT 82% (run-rate)
  → run-rate ex-AMPC EBITDA $442→$554mm, DCF EV $4.0→$5.0bn, FCFE +2.4bn
  마진 9%·pre-SOP 기저 floor $0.2bn·2026 $200mm 유지
- 역산 시나리오(분모 $554mm): BASE 19.3→15.4x, ①/② 14.1x, ①+② 13.3x
  = peer 상단(13x) 사실상 안착(잔여 +0.3x)
- 덱 S2(가동률/매출/EBITDA/EV KPI)·S4(가정·표·밴드바·결론) 동기화
- CLAUDE.md·펀딩구조_v2 검산표/역산표 갱신

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -295,7 +295,60 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">실제 생산</t>
+      <t xml:space="preserve">실제 생산 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1.0 → util</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">곡선</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실효 가동률</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -10410,31 +10463,31 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>722.92</c:v>
+                  <c:v>903.65</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1643</c:v>
+                  <c:v>2086.61</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1946.16</c:v>
+                  <c:v>2497.572</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2176.816</c:v>
+                  <c:v>2689.008</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2249.0656</c:v>
+                  <c:v>2684.98</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2243.808</c:v>
+                  <c:v>2648.94</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2213.28</c:v>
+                  <c:v>2612.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2182.752</c:v>
+                  <c:v>2576.86</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2152.224</c:v>
+                  <c:v>2540.82</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10539,28 +10592,28 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1242.108</c:v>
+                  <c:v>1552.635</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1926.6984</c:v>
+                  <c:v>2539.7388</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2420.1072</c:v>
+                  <c:v>3241.215</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2729.2032</c:v>
+                  <c:v>3624.723</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2860.8552</c:v>
+                  <c:v>3576.069</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2821.932</c:v>
+                  <c:v>3527.415</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2783.0088</c:v>
+                  <c:v>3478.761</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2744.0856</c:v>
+                  <c:v>3430.107</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10568,8 +10621,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="38045476"/>
-        <c:axId val="76172954"/>
+        <c:axId val="38457199"/>
+        <c:axId val="21383864"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10675,31 +10728,31 @@
                   <c:v>-168.58636</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-340.279684</c:v>
+                  <c:v>-320.341084</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>436.14279688</c:v>
+                  <c:v>576.5144851</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1242.57192264</c:v>
+                  <c:v>1557.91114236</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1176.49565696</c:v>
+                  <c:v>1513.38719486</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>959.863373792</c:v>
+                  <c:v>1225.6047407</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>634.366208240001</c:v>
+                  <c:v>804.5742941</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>262.3508516</c:v>
+                  <c:v>313.9177475</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>261.737009839999</c:v>
+                  <c:v>309.9924509</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>261.12316808</c:v>
+                  <c:v>306.0671543</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10714,11 +10767,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="38045476"/>
-        <c:axId val="76172954"/>
+        <c:axId val="38457199"/>
+        <c:axId val="21383864"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="38045476"/>
+        <c:axId val="38457199"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10750,7 +10803,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76172954"/>
+        <c:crossAx val="21383864"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10758,7 +10811,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76172954"/>
+        <c:axId val="21383864"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10800,7 +10853,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38045476"/>
+        <c:crossAx val="38457199"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11112,7 +11165,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>5</v>
@@ -11868,28 +11921,28 @@
         <v>0.55</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="H31" s="20" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="I31" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="J31" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="K31" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L31" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="M31" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11905,39 +11958,39 @@
       </c>
       <c r="E32" s="37" t="n">
         <f aca="false">E30*E31*$C$6</f>
-        <v>2.332</v>
+        <v>2.915</v>
       </c>
       <c r="F32" s="37" t="n">
         <f aca="false">F30*F31*$C$6</f>
-        <v>2.968</v>
+        <v>3.816</v>
       </c>
       <c r="G32" s="37" t="n">
         <f aca="false">G30*G31*$C$6</f>
-        <v>3.392</v>
+        <v>4.346</v>
       </c>
       <c r="H32" s="37" t="n">
         <f aca="false">H30*H31*$C$6</f>
-        <v>3.7312</v>
+        <v>4.505</v>
       </c>
       <c r="I32" s="37" t="n">
         <f aca="false">I30*I31*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="J32" s="37" t="n">
         <f aca="false">J30*J31*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="K32" s="37" t="n">
         <f aca="false">K30*K31*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="L32" s="37" t="n">
         <f aca="false">L30*L31*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="M32" s="37" t="n">
         <f aca="false">M30*M31*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11989,28 +12042,28 @@
         <v>0.55</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="H34" s="20" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="I34" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="J34" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="K34" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L34" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="M34" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12026,39 +12079,39 @@
       </c>
       <c r="E35" s="37" t="n">
         <f aca="false">E33*E34*$C$6</f>
-        <v>2.332</v>
+        <v>2.915</v>
       </c>
       <c r="F35" s="37" t="n">
         <f aca="false">F33*F34*$C$6</f>
-        <v>2.968</v>
+        <v>3.816</v>
       </c>
       <c r="G35" s="37" t="n">
         <f aca="false">G33*G34*$C$6</f>
-        <v>3.392</v>
+        <v>4.346</v>
       </c>
       <c r="H35" s="37" t="n">
         <f aca="false">H33*H34*$C$6</f>
-        <v>3.7312</v>
+        <v>4.505</v>
       </c>
       <c r="I35" s="37" t="n">
         <f aca="false">I33*I34*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="J35" s="37" t="n">
         <f aca="false">J33*J34*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="K35" s="37" t="n">
         <f aca="false">K33*K34*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="L35" s="37" t="n">
         <f aca="false">L33*L34*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="M35" s="37" t="n">
         <f aca="false">M33*M34*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12118,25 +12171,25 @@
         <v>0.55</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="H38" s="20" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="I38" s="20" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="J38" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="K38" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L38" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="M38" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12156,35 +12209,35 @@
       </c>
       <c r="F39" s="37" t="n">
         <f aca="false">F37*F38*$C$6</f>
-        <v>2.332</v>
+        <v>2.915</v>
       </c>
       <c r="G39" s="37" t="n">
         <f aca="false">G37*G38*$C$6</f>
-        <v>2.968</v>
+        <v>3.816</v>
       </c>
       <c r="H39" s="37" t="n">
         <f aca="false">H37*H38*$C$6</f>
-        <v>3.4768</v>
+        <v>4.399</v>
       </c>
       <c r="I39" s="37" t="n">
         <f aca="false">I37*I38*$C$6</f>
-        <v>3.7312</v>
+        <v>4.505</v>
       </c>
       <c r="J39" s="37" t="n">
         <f aca="false">J37*J38*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="K39" s="37" t="n">
         <f aca="false">K37*K38*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="L39" s="37" t="n">
         <f aca="false">L37*L38*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="M39" s="37" t="n">
         <f aca="false">M37*M38*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12239,25 +12292,25 @@
         <v>0.55</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="H41" s="20" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="I41" s="20" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="J41" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="K41" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L41" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="M41" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12277,35 +12330,35 @@
       </c>
       <c r="F42" s="37" t="n">
         <f aca="false">F40*F41*$C$6</f>
-        <v>2.332</v>
+        <v>2.915</v>
       </c>
       <c r="G42" s="37" t="n">
         <f aca="false">G40*G41*$C$6</f>
-        <v>2.968</v>
+        <v>3.816</v>
       </c>
       <c r="H42" s="37" t="n">
         <f aca="false">H40*H41*$C$6</f>
-        <v>3.4768</v>
+        <v>4.399</v>
       </c>
       <c r="I42" s="37" t="n">
         <f aca="false">I40*I41*$C$6</f>
-        <v>3.7312</v>
+        <v>4.505</v>
       </c>
       <c r="J42" s="37" t="n">
         <f aca="false">J40*J41*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="K42" s="37" t="n">
         <f aca="false">K40*K41*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="L42" s="37" t="n">
         <f aca="false">L40*L41*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
       <c r="M42" s="37" t="n">
         <f aca="false">M40*M41*$C$6</f>
-        <v>3.816</v>
+        <v>4.505</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12321,39 +12374,39 @@
       </c>
       <c r="E43" s="37" t="n">
         <f aca="false">E32+E35</f>
-        <v>4.664</v>
+        <v>5.83</v>
       </c>
       <c r="F43" s="37" t="n">
         <f aca="false">F32+F35</f>
-        <v>5.936</v>
+        <v>7.632</v>
       </c>
       <c r="G43" s="37" t="n">
         <f aca="false">G32+G35</f>
-        <v>6.784</v>
+        <v>8.692</v>
       </c>
       <c r="H43" s="37" t="n">
         <f aca="false">H32+H35</f>
-        <v>7.4624</v>
+        <v>9.01</v>
       </c>
       <c r="I43" s="37" t="n">
         <f aca="false">I32+I35</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="J43" s="37" t="n">
         <f aca="false">J32+J35</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="K43" s="37" t="n">
         <f aca="false">K32+K35</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="L43" s="37" t="n">
         <f aca="false">L32+L35</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="M43" s="37" t="n">
         <f aca="false">M32+M35</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12373,35 +12426,35 @@
       </c>
       <c r="F44" s="37" t="n">
         <f aca="false">F39+F42</f>
-        <v>4.664</v>
+        <v>5.83</v>
       </c>
       <c r="G44" s="37" t="n">
         <f aca="false">G39+G42</f>
-        <v>5.936</v>
+        <v>7.632</v>
       </c>
       <c r="H44" s="37" t="n">
         <f aca="false">H39+H42</f>
-        <v>6.9536</v>
+        <v>8.798</v>
       </c>
       <c r="I44" s="37" t="n">
         <f aca="false">I39+I42</f>
-        <v>7.4624</v>
+        <v>9.01</v>
       </c>
       <c r="J44" s="37" t="n">
         <f aca="false">J39+J42</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="K44" s="37" t="n">
         <f aca="false">K39+K42</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="L44" s="37" t="n">
         <f aca="false">L39+L42</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
       <c r="M44" s="37" t="n">
         <f aca="false">M39+M42</f>
-        <v>7.632</v>
+        <v>9.01</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12417,39 +12470,39 @@
       </c>
       <c r="E45" s="37" t="n">
         <f aca="false">E43+E44</f>
-        <v>4.664</v>
+        <v>5.83</v>
       </c>
       <c r="F45" s="37" t="n">
         <f aca="false">F43+F44</f>
-        <v>10.6</v>
+        <v>13.462</v>
       </c>
       <c r="G45" s="37" t="n">
         <f aca="false">G43+G44</f>
-        <v>12.72</v>
+        <v>16.324</v>
       </c>
       <c r="H45" s="37" t="n">
         <f aca="false">H43+H44</f>
-        <v>14.416</v>
+        <v>17.808</v>
       </c>
       <c r="I45" s="37" t="n">
         <f aca="false">I43+I44</f>
-        <v>15.0944</v>
+        <v>18.02</v>
       </c>
       <c r="J45" s="37" t="n">
         <f aca="false">J43+J44</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="K45" s="37" t="n">
         <f aca="false">K43+K44</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="L45" s="37" t="n">
         <f aca="false">L43+L44</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="M45" s="37" t="n">
         <f aca="false">M43+M44</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12907,13 +12960,13 @@
         <v>0.35</v>
       </c>
       <c r="G60" s="20" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H60" s="20" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I60" s="20" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="J60" s="20" t="n">
         <v>0.85</v>
@@ -12945,35 +12998,35 @@
       </c>
       <c r="F61" s="37" t="n">
         <f aca="false">F59*F60*$C$6</f>
-        <v>3.78</v>
+        <v>4.725</v>
       </c>
       <c r="G61" s="37" t="n">
         <f aca="false">G59*G60*$C$6</f>
-        <v>5.94</v>
+        <v>7.83</v>
       </c>
       <c r="H61" s="37" t="n">
         <f aca="false">H59*H60*$C$6</f>
-        <v>7.56</v>
+        <v>10.125</v>
       </c>
       <c r="I61" s="37" t="n">
         <f aca="false">I59*I60*$C$6</f>
-        <v>8.64</v>
+        <v>11.475</v>
       </c>
       <c r="J61" s="37" t="n">
         <f aca="false">J59*J60*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="K61" s="37" t="n">
         <f aca="false">K59*K60*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="L61" s="37" t="n">
         <f aca="false">L59*L60*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="M61" s="37" t="n">
         <f aca="false">M59*M60*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13028,13 +13081,13 @@
         <v>0.35</v>
       </c>
       <c r="G63" s="20" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H63" s="20" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I63" s="20" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="J63" s="20" t="n">
         <v>0.85</v>
@@ -13066,35 +13119,35 @@
       </c>
       <c r="F64" s="37" t="n">
         <f aca="false">F62*F63*$C$6</f>
-        <v>3.78</v>
+        <v>4.725</v>
       </c>
       <c r="G64" s="37" t="n">
         <f aca="false">G62*G63*$C$6</f>
-        <v>5.94</v>
+        <v>7.83</v>
       </c>
       <c r="H64" s="37" t="n">
         <f aca="false">H62*H63*$C$6</f>
-        <v>7.56</v>
+        <v>10.125</v>
       </c>
       <c r="I64" s="37" t="n">
         <f aca="false">I62*I63*$C$6</f>
-        <v>8.64</v>
+        <v>11.475</v>
       </c>
       <c r="J64" s="37" t="n">
         <f aca="false">J62*J63*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="K64" s="37" t="n">
         <f aca="false">K62*K63*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="L64" s="37" t="n">
         <f aca="false">L62*L63*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
       <c r="M64" s="37" t="n">
         <f aca="false">M62*M63*$C$6</f>
-        <v>9.18</v>
+        <v>11.475</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13154,13 +13207,13 @@
         <v>0.35</v>
       </c>
       <c r="G67" s="20" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H67" s="20" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I67" s="20" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="J67" s="20" t="n">
         <v>0.85</v>
@@ -13192,35 +13245,35 @@
       </c>
       <c r="F68" s="37" t="n">
         <f aca="false">F66*F67*$C$6</f>
-        <v>0.756</v>
+        <v>0.945</v>
       </c>
       <c r="G68" s="37" t="n">
         <f aca="false">G66*G67*$C$6</f>
-        <v>1.188</v>
+        <v>1.566</v>
       </c>
       <c r="H68" s="37" t="n">
         <f aca="false">H66*H67*$C$6</f>
-        <v>1.512</v>
+        <v>2.025</v>
       </c>
       <c r="I68" s="37" t="n">
         <f aca="false">I66*I67*$C$6</f>
-        <v>1.728</v>
+        <v>2.295</v>
       </c>
       <c r="J68" s="37" t="n">
         <f aca="false">J66*J67*$C$6</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="K68" s="37" t="n">
         <f aca="false">K66*K67*$C$6</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="L68" s="37" t="n">
         <f aca="false">L66*L67*$C$6</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="M68" s="37" t="n">
         <f aca="false">M66*M67*$C$6</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13240,35 +13293,35 @@
       </c>
       <c r="F69" s="37" t="n">
         <f aca="false">F61+F64</f>
-        <v>7.56</v>
+        <v>9.45</v>
       </c>
       <c r="G69" s="37" t="n">
         <f aca="false">G61+G64</f>
-        <v>11.88</v>
+        <v>15.66</v>
       </c>
       <c r="H69" s="37" t="n">
         <f aca="false">H61+H64</f>
-        <v>15.12</v>
+        <v>20.25</v>
       </c>
       <c r="I69" s="37" t="n">
         <f aca="false">I61+I64</f>
-        <v>17.28</v>
+        <v>22.95</v>
       </c>
       <c r="J69" s="37" t="n">
         <f aca="false">J61+J64</f>
-        <v>18.36</v>
+        <v>22.95</v>
       </c>
       <c r="K69" s="37" t="n">
         <f aca="false">K61+K64</f>
-        <v>18.36</v>
+        <v>22.95</v>
       </c>
       <c r="L69" s="37" t="n">
         <f aca="false">L61+L64</f>
-        <v>18.36</v>
+        <v>22.95</v>
       </c>
       <c r="M69" s="37" t="n">
         <f aca="false">M61+M64</f>
-        <v>18.36</v>
+        <v>22.95</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13288,35 +13341,35 @@
       </c>
       <c r="F70" s="37" t="n">
         <f aca="false">F68</f>
-        <v>0.756</v>
+        <v>0.945</v>
       </c>
       <c r="G70" s="37" t="n">
         <f aca="false">G68</f>
-        <v>1.188</v>
+        <v>1.566</v>
       </c>
       <c r="H70" s="37" t="n">
         <f aca="false">H68</f>
-        <v>1.512</v>
+        <v>2.025</v>
       </c>
       <c r="I70" s="37" t="n">
         <f aca="false">I68</f>
-        <v>1.728</v>
+        <v>2.295</v>
       </c>
       <c r="J70" s="37" t="n">
         <f aca="false">J68</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="K70" s="37" t="n">
         <f aca="false">K68</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="L70" s="37" t="n">
         <f aca="false">L68</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
       <c r="M70" s="37" t="n">
         <f aca="false">M68</f>
-        <v>1.836</v>
+        <v>2.295</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14138,39 +14191,39 @@
       </c>
       <c r="E6" s="54" t="n">
         <f aca="false">Assumptions!E45</f>
-        <v>4.664</v>
+        <v>5.83</v>
       </c>
       <c r="F6" s="54" t="n">
         <f aca="false">Assumptions!F45</f>
-        <v>10.6</v>
+        <v>13.462</v>
       </c>
       <c r="G6" s="54" t="n">
         <f aca="false">Assumptions!G45</f>
-        <v>12.72</v>
+        <v>16.324</v>
       </c>
       <c r="H6" s="54" t="n">
         <f aca="false">Assumptions!H45</f>
-        <v>14.416</v>
+        <v>17.808</v>
       </c>
       <c r="I6" s="54" t="n">
         <f aca="false">Assumptions!I45</f>
-        <v>15.0944</v>
+        <v>18.02</v>
       </c>
       <c r="J6" s="54" t="n">
         <f aca="false">Assumptions!J45</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="K6" s="54" t="n">
         <f aca="false">Assumptions!K45</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="L6" s="54" t="n">
         <f aca="false">Assumptions!L45</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
       <c r="M6" s="54" t="n">
         <f aca="false">Assumptions!M45</f>
-        <v>15.264</v>
+        <v>18.02</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14228,39 +14281,39 @@
       </c>
       <c r="E8" s="56" t="n">
         <f aca="false">E6*E7</f>
-        <v>722.92</v>
+        <v>903.65</v>
       </c>
       <c r="F8" s="56" t="n">
         <f aca="false">F6*F7</f>
-        <v>1643</v>
+        <v>2086.61</v>
       </c>
       <c r="G8" s="56" t="n">
         <f aca="false">G6*G7</f>
-        <v>1946.16</v>
+        <v>2497.572</v>
       </c>
       <c r="H8" s="56" t="n">
         <f aca="false">H6*H7</f>
-        <v>2176.816</v>
+        <v>2689.008</v>
       </c>
       <c r="I8" s="56" t="n">
         <f aca="false">I6*I7</f>
-        <v>2249.0656</v>
+        <v>2684.98</v>
       </c>
       <c r="J8" s="56" t="n">
         <f aca="false">J6*J7</f>
-        <v>2243.808</v>
+        <v>2648.94</v>
       </c>
       <c r="K8" s="56" t="n">
         <f aca="false">K6*K7</f>
-        <v>2213.28</v>
+        <v>2612.9</v>
       </c>
       <c r="L8" s="56" t="n">
         <f aca="false">L6*L7</f>
-        <v>2182.752</v>
+        <v>2576.86</v>
       </c>
       <c r="M8" s="56" t="n">
         <f aca="false">M6*M7</f>
-        <v>2152.224</v>
+        <v>2540.82</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14273,39 +14326,39 @@
       </c>
       <c r="E9" s="38" t="n">
         <f aca="false">-(Assumptions!E43*Assumptions!E49+Assumptions!E44*Assumptions!E50)</f>
-        <v>-607.2528</v>
+        <v>-759.066</v>
       </c>
       <c r="F9" s="38" t="n">
         <f aca="false">-(Assumptions!F43*Assumptions!F49+Assumptions!F44*Assumptions!F50)</f>
-        <v>-1394.5784</v>
+        <v>-1770.8254</v>
       </c>
       <c r="G9" s="38" t="n">
         <f aca="false">-(Assumptions!G43*Assumptions!G49+Assumptions!G44*Assumptions!G50)</f>
-        <v>-1652.93856</v>
+        <v>-2121.3144</v>
       </c>
       <c r="H9" s="38" t="n">
         <f aca="false">-(Assumptions!H43*Assumptions!H49+Assumptions!H44*Assumptions!H50)</f>
-        <v>-1849.525312</v>
+        <v>-2285.33668</v>
       </c>
       <c r="I9" s="38" t="n">
         <f aca="false">-(Assumptions!I43*Assumptions!I49+Assumptions!I44*Assumptions!I50)</f>
-        <v>-1911.453056</v>
+        <v>-2282.233</v>
       </c>
       <c r="J9" s="38" t="n">
         <f aca="false">-(Assumptions!J43*Assumptions!J49+Assumptions!J44*Assumptions!J50)</f>
-        <v>-1907.2368</v>
+        <v>-2251.599</v>
       </c>
       <c r="K9" s="38" t="n">
         <f aca="false">-(Assumptions!K43*Assumptions!K49+Assumptions!K44*Assumptions!K50)</f>
-        <v>-1881.288</v>
+        <v>-2220.965</v>
       </c>
       <c r="L9" s="38" t="n">
         <f aca="false">-(Assumptions!L43*Assumptions!L49+Assumptions!L44*Assumptions!L50)</f>
-        <v>-1855.3392</v>
+        <v>-2190.331</v>
       </c>
       <c r="M9" s="38" t="n">
         <f aca="false">-(Assumptions!M43*Assumptions!M49+Assumptions!M44*Assumptions!M50)</f>
-        <v>-1829.3904</v>
+        <v>-2159.697</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14370,39 +14423,39 @@
       </c>
       <c r="E12" s="56" t="n">
         <f aca="false">E8+E9</f>
-        <v>115.6672</v>
+        <v>144.584</v>
       </c>
       <c r="F12" s="56" t="n">
         <f aca="false">F8+F9</f>
-        <v>248.4216</v>
+        <v>315.7846</v>
       </c>
       <c r="G12" s="56" t="n">
         <f aca="false">G8+G9</f>
-        <v>293.22144</v>
+        <v>376.2576</v>
       </c>
       <c r="H12" s="56" t="n">
         <f aca="false">H8+H9</f>
-        <v>327.290688</v>
+        <v>403.67132</v>
       </c>
       <c r="I12" s="56" t="n">
         <f aca="false">I8+I9</f>
-        <v>337.612544</v>
+        <v>402.747</v>
       </c>
       <c r="J12" s="56" t="n">
         <f aca="false">J8+J9</f>
-        <v>336.5712</v>
+        <v>397.341</v>
       </c>
       <c r="K12" s="56" t="n">
         <f aca="false">K8+K9</f>
-        <v>331.992</v>
+        <v>391.935</v>
       </c>
       <c r="L12" s="56" t="n">
         <f aca="false">L8+L9</f>
-        <v>327.4128</v>
+        <v>386.529</v>
       </c>
       <c r="M12" s="56" t="n">
         <f aca="false">M8+M9</f>
-        <v>322.8336</v>
+        <v>381.123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14415,39 +14468,39 @@
       </c>
       <c r="E13" s="38" t="n">
         <f aca="false">-E8*Assumptions!$C$81</f>
-        <v>-43.3752</v>
+        <v>-54.219</v>
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$81</f>
-        <v>-98.58</v>
+        <v>-125.1966</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$81</f>
-        <v>-116.7696</v>
+        <v>-149.85432</v>
       </c>
       <c r="H13" s="38" t="n">
         <f aca="false">-H8*Assumptions!$C$81</f>
-        <v>-130.60896</v>
+        <v>-161.34048</v>
       </c>
       <c r="I13" s="38" t="n">
         <f aca="false">-I8*Assumptions!$C$81</f>
-        <v>-134.943936</v>
+        <v>-161.0988</v>
       </c>
       <c r="J13" s="38" t="n">
         <f aca="false">-J8*Assumptions!$C$81</f>
-        <v>-134.62848</v>
+        <v>-158.9364</v>
       </c>
       <c r="K13" s="38" t="n">
         <f aca="false">-K8*Assumptions!$C$81</f>
-        <v>-132.7968</v>
+        <v>-156.774</v>
       </c>
       <c r="L13" s="38" t="n">
         <f aca="false">-L8*Assumptions!$C$81</f>
-        <v>-130.96512</v>
+        <v>-154.6116</v>
       </c>
       <c r="M13" s="38" t="n">
         <f aca="false">-M8*Assumptions!$C$81</f>
-        <v>-129.13344</v>
+        <v>-152.4492</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14550,19 +14603,19 @@
       </c>
       <c r="E16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(E12+E13))</f>
-        <v>127.708</v>
+        <v>109.635</v>
       </c>
       <c r="F16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(F12+F13))</f>
-        <v>50.1583999999997</v>
+        <v>9.41199999999981</v>
       </c>
       <c r="G16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(G12+G13))</f>
-        <v>23.54816</v>
+        <v>0</v>
       </c>
       <c r="H16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(H12+H13))</f>
-        <v>3.31827199999995</v>
+        <v>0</v>
       </c>
       <c r="I16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(I12+I13))</f>
@@ -14574,15 +14627,15 @@
       </c>
       <c r="K16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(K12+K13))</f>
-        <v>0.804800000000256</v>
+        <v>0</v>
       </c>
       <c r="L16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(L12+L13))</f>
-        <v>3.55231999999992</v>
+        <v>0</v>
       </c>
       <c r="M16" s="38" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(M12+M13))</f>
-        <v>6.29984000000027</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14603,31 +14656,31 @@
       </c>
       <c r="G17" s="56" t="n">
         <f aca="false">G12+G13+G15+G16</f>
-        <v>171.986</v>
+        <v>198.38928</v>
       </c>
       <c r="H17" s="56" t="n">
         <f aca="false">H12+H13+H15+H16</f>
-        <v>171.986</v>
+        <v>214.31684</v>
       </c>
       <c r="I17" s="56" t="n">
         <f aca="false">I12+I13+I15+I16</f>
-        <v>174.654608</v>
+        <v>213.6342</v>
       </c>
       <c r="J17" s="56" t="n">
         <f aca="false">J12+J13+J15+J16</f>
-        <v>173.92872</v>
+        <v>210.3906</v>
       </c>
       <c r="K17" s="56" t="n">
         <f aca="false">K12+K13+K15+K16</f>
-        <v>171.986</v>
+        <v>207.147</v>
       </c>
       <c r="L17" s="56" t="n">
         <f aca="false">L12+L13+L15+L16</f>
-        <v>171.986</v>
+        <v>203.9034</v>
       </c>
       <c r="M17" s="56" t="n">
         <f aca="false">M12+M13+M15+M16</f>
-        <v>171.986</v>
+        <v>200.6598</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14640,39 +14693,39 @@
       </c>
       <c r="E18" s="57" t="n">
         <f aca="false">IF(E8=0,0,E17/E8)</f>
-        <v>0.241595197255575</v>
+        <v>0.19327615780446</v>
       </c>
       <c r="F18" s="57" t="n">
         <f aca="false">IF(F8=0,0,F17/F8)</f>
-        <v>0.104678027997565</v>
+        <v>0.0824236440925712</v>
       </c>
       <c r="G18" s="57" t="n">
         <f aca="false">IF(G8=0,0,G17/G8)</f>
-        <v>0.0883719735273564</v>
+        <v>0.079432857190904</v>
       </c>
       <c r="H18" s="57" t="n">
         <f aca="false">IF(H8=0,0,H17/H8)</f>
-        <v>0.0790080558026034</v>
+        <v>0.079701079357146</v>
       </c>
       <c r="I18" s="57" t="n">
         <f aca="false">IF(I8=0,0,I17/I8)</f>
-        <v>0.0776565201121746</v>
+        <v>0.0795664027292569</v>
       </c>
       <c r="J18" s="57" t="n">
         <f aca="false">IF(J8=0,0,J17/J8)</f>
-        <v>0.0775149745432765</v>
+        <v>0.0794244490248929</v>
       </c>
       <c r="K18" s="57" t="n">
         <f aca="false">IF(K8=0,0,K17/K8)</f>
-        <v>0.0777063905154341</v>
+        <v>0.0792785793562708</v>
       </c>
       <c r="L18" s="57" t="n">
         <f aca="false">IF(L8=0,0,L17/L8)</f>
-        <v>0.0787931931799856</v>
+        <v>0.0791286294171977</v>
       </c>
       <c r="M18" s="57" t="n">
         <f aca="false">IF(M8=0,0,M17/M8)</f>
-        <v>0.079910827125801</v>
+        <v>0.0789744255791438</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14685,27 +14738,27 @@
       </c>
       <c r="E19" s="38" t="n">
         <f aca="false">(Assumptions!E45)*Assumptions!E8</f>
-        <v>209.88</v>
+        <v>262.35</v>
       </c>
       <c r="F19" s="38" t="n">
         <f aca="false">(Assumptions!F45)*Assumptions!F8</f>
-        <v>477</v>
+        <v>605.79</v>
       </c>
       <c r="G19" s="38" t="n">
         <f aca="false">(Assumptions!G45)*Assumptions!G8</f>
-        <v>572.4</v>
+        <v>734.58</v>
       </c>
       <c r="H19" s="38" t="n">
         <f aca="false">(Assumptions!H45)*Assumptions!H8</f>
-        <v>486.54</v>
+        <v>601.02</v>
       </c>
       <c r="I19" s="38" t="n">
         <f aca="false">(Assumptions!I45)*Assumptions!I8</f>
-        <v>339.624</v>
+        <v>405.45</v>
       </c>
       <c r="J19" s="38" t="n">
         <f aca="false">(Assumptions!J45)*Assumptions!J8</f>
-        <v>171.72</v>
+        <v>202.725</v>
       </c>
       <c r="K19" s="38" t="n">
         <f aca="false">(Assumptions!K45)*Assumptions!K8</f>
@@ -14730,39 +14783,39 @@
       </c>
       <c r="E20" s="56" t="n">
         <f aca="false">E17+E19</f>
-        <v>384.534</v>
+        <v>437.004</v>
       </c>
       <c r="F20" s="56" t="n">
         <f aca="false">F17+F19</f>
-        <v>648.986</v>
+        <v>777.776</v>
       </c>
       <c r="G20" s="56" t="n">
         <f aca="false">G17+G19</f>
-        <v>744.386</v>
+        <v>932.96928</v>
       </c>
       <c r="H20" s="56" t="n">
         <f aca="false">H17+H19</f>
-        <v>658.526</v>
+        <v>815.33684</v>
       </c>
       <c r="I20" s="56" t="n">
         <f aca="false">I17+I19</f>
-        <v>514.278608</v>
+        <v>619.0842</v>
       </c>
       <c r="J20" s="56" t="n">
         <f aca="false">J17+J19</f>
-        <v>345.64872</v>
+        <v>413.1156</v>
       </c>
       <c r="K20" s="56" t="n">
         <f aca="false">K17+K19</f>
-        <v>171.986</v>
+        <v>207.147</v>
       </c>
       <c r="L20" s="56" t="n">
         <f aca="false">L17+L19</f>
-        <v>171.986</v>
+        <v>203.9034</v>
       </c>
       <c r="M20" s="56" t="n">
         <f aca="false">M17+M19</f>
-        <v>171.986</v>
+        <v>200.6598</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14835,31 +14888,31 @@
       </c>
       <c r="G24" s="38" t="n">
         <f aca="false">MAX(0,G17)</f>
-        <v>171.986</v>
+        <v>198.38928</v>
       </c>
       <c r="H24" s="38" t="n">
         <f aca="false">MAX(0,H17)</f>
-        <v>171.986</v>
+        <v>214.31684</v>
       </c>
       <c r="I24" s="38" t="n">
         <f aca="false">MAX(0,I17)</f>
-        <v>174.654608</v>
+        <v>213.6342</v>
       </c>
       <c r="J24" s="38" t="n">
         <f aca="false">MAX(0,J17)</f>
-        <v>173.92872</v>
+        <v>210.3906</v>
       </c>
       <c r="K24" s="38" t="n">
         <f aca="false">MAX(0,K17)</f>
-        <v>171.986</v>
+        <v>207.147</v>
       </c>
       <c r="L24" s="38" t="n">
         <f aca="false">MAX(0,L17)</f>
-        <v>171.986</v>
+        <v>203.9034</v>
       </c>
       <c r="M24" s="38" t="n">
         <f aca="false">MAX(0,M17)</f>
-        <v>171.986</v>
+        <v>200.6598</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14884,27 +14937,27 @@
       </c>
       <c r="H25" s="38" t="n">
         <f aca="false">G28</f>
-        <v>3435.7712</v>
+        <v>3414.648576</v>
       </c>
       <c r="I25" s="38" t="n">
         <f aca="false">H28</f>
-        <v>3298.1824</v>
+        <v>3243.195104</v>
       </c>
       <c r="J25" s="38" t="n">
         <f aca="false">I28</f>
-        <v>3158.4587136</v>
+        <v>3072.287744</v>
       </c>
       <c r="K25" s="38" t="n">
         <f aca="false">J28</f>
-        <v>3019.3157376</v>
+        <v>2903.975264</v>
       </c>
       <c r="L25" s="38" t="n">
         <f aca="false">K28</f>
-        <v>2881.7269376</v>
+        <v>2738.257664</v>
       </c>
       <c r="M25" s="38" t="n">
         <f aca="false">L28</f>
-        <v>2744.1381376</v>
+        <v>2575.134944</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14925,31 +14978,31 @@
       </c>
       <c r="G26" s="38" t="n">
         <f aca="false">MIN(G25,G24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>158.711424</v>
       </c>
       <c r="H26" s="38" t="n">
         <f aca="false">MIN(H25,H24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>171.453472</v>
       </c>
       <c r="I26" s="38" t="n">
         <f aca="false">MIN(I25,I24*Assumptions!$C$90)</f>
-        <v>139.7236864</v>
+        <v>170.90736</v>
       </c>
       <c r="J26" s="38" t="n">
         <f aca="false">MIN(J25,J24*Assumptions!$C$90)</f>
-        <v>139.142976</v>
+        <v>168.31248</v>
       </c>
       <c r="K26" s="38" t="n">
         <f aca="false">MIN(K25,K24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>165.7176</v>
       </c>
       <c r="L26" s="38" t="n">
         <f aca="false">MIN(L25,L24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>163.12272</v>
       </c>
       <c r="M26" s="38" t="n">
         <f aca="false">MIN(M25,M24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>160.52784</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15015,31 +15068,31 @@
       </c>
       <c r="G28" s="38" t="n">
         <f aca="false">G25-G26+G27</f>
-        <v>3435.7712</v>
+        <v>3414.648576</v>
       </c>
       <c r="H28" s="38" t="n">
         <f aca="false">H25-H26+H27</f>
-        <v>3298.1824</v>
+        <v>3243.195104</v>
       </c>
       <c r="I28" s="38" t="n">
         <f aca="false">I25-I26+I27</f>
-        <v>3158.4587136</v>
+        <v>3072.287744</v>
       </c>
       <c r="J28" s="38" t="n">
         <f aca="false">J25-J26+J27</f>
-        <v>3019.3157376</v>
+        <v>2903.975264</v>
       </c>
       <c r="K28" s="38" t="n">
         <f aca="false">K25-K26+K27</f>
-        <v>2881.7269376</v>
+        <v>2738.257664</v>
       </c>
       <c r="L28" s="38" t="n">
         <f aca="false">L25-L26+L27</f>
-        <v>2744.1381376</v>
+        <v>2575.134944</v>
       </c>
       <c r="M28" s="38" t="n">
         <f aca="false">M25-M26+M27</f>
-        <v>2606.5493376</v>
+        <v>2414.607104</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15060,31 +15113,31 @@
       </c>
       <c r="G29" s="38" t="n">
         <f aca="false">G24-G26</f>
-        <v>34.3972</v>
+        <v>39.6778560000001</v>
       </c>
       <c r="H29" s="38" t="n">
         <f aca="false">H24-H26</f>
-        <v>34.3972</v>
+        <v>42.8633680000001</v>
       </c>
       <c r="I29" s="38" t="n">
         <f aca="false">I24-I26</f>
-        <v>34.9309216</v>
+        <v>42.72684</v>
       </c>
       <c r="J29" s="38" t="n">
         <f aca="false">J24-J26</f>
-        <v>34.785744</v>
+        <v>42.07812</v>
       </c>
       <c r="K29" s="38" t="n">
         <f aca="false">K24-K26</f>
-        <v>34.3972</v>
+        <v>41.4294</v>
       </c>
       <c r="L29" s="38" t="n">
         <f aca="false">L24-L26</f>
-        <v>34.3972</v>
+        <v>40.78068</v>
       </c>
       <c r="M29" s="38" t="n">
         <f aca="false">M24-M26</f>
-        <v>34.3972</v>
+        <v>40.13196</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15105,31 +15158,31 @@
       </c>
       <c r="G30" s="38" t="n">
         <f aca="false">-G29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.12590688000002</v>
       </c>
       <c r="H30" s="38" t="n">
         <f aca="false">-H29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.85857464000002</v>
       </c>
       <c r="I30" s="38" t="n">
         <f aca="false">-I29*Assumptions!$C$87</f>
-        <v>-8.034111968</v>
+        <v>-9.82717320000001</v>
       </c>
       <c r="J30" s="38" t="n">
         <f aca="false">-J29*Assumptions!$C$87</f>
-        <v>-8.00072112000001</v>
+        <v>-9.67796759999999</v>
       </c>
       <c r="K30" s="38" t="n">
         <f aca="false">-K29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.528762</v>
       </c>
       <c r="L30" s="38" t="n">
         <f aca="false">-L29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.3795564</v>
       </c>
       <c r="M30" s="38" t="n">
         <f aca="false">-M29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.2303508</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15142,39 +15195,39 @@
       </c>
       <c r="E31" s="56" t="n">
         <f aca="false">E20+E30</f>
-        <v>376.499916</v>
+        <v>428.969916</v>
       </c>
       <c r="F31" s="56" t="n">
         <f aca="false">F20+F30</f>
-        <v>641.074644</v>
+        <v>769.864644</v>
       </c>
       <c r="G31" s="56" t="n">
         <f aca="false">G20+G30</f>
-        <v>736.474644</v>
+        <v>923.84337312</v>
       </c>
       <c r="H31" s="56" t="n">
         <f aca="false">H20+H30</f>
-        <v>650.614644</v>
+        <v>805.47826536</v>
       </c>
       <c r="I31" s="56" t="n">
         <f aca="false">I20+I30</f>
-        <v>506.244496032</v>
+        <v>609.2570268</v>
       </c>
       <c r="J31" s="56" t="n">
         <f aca="false">J20+J30</f>
-        <v>337.64799888</v>
+        <v>403.4376324</v>
       </c>
       <c r="K31" s="56" t="n">
         <f aca="false">K20+K30</f>
-        <v>164.074644</v>
+        <v>197.618238</v>
       </c>
       <c r="L31" s="56" t="n">
         <f aca="false">L20+L30</f>
-        <v>164.074644</v>
+        <v>194.5238436</v>
       </c>
       <c r="M31" s="56" t="n">
         <f aca="false">M20+M30</f>
-        <v>164.074644</v>
+        <v>191.4294492</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15232,39 +15285,39 @@
       </c>
       <c r="E33" s="38" t="n">
         <f aca="false">-E8*Assumptions!$C$83</f>
-        <v>-21.6876</v>
+        <v>-27.1095</v>
       </c>
       <c r="F33" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$83</f>
-        <v>-49.29</v>
+        <v>-62.5983</v>
       </c>
       <c r="G33" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$83</f>
-        <v>-58.3848</v>
+        <v>-74.92716</v>
       </c>
       <c r="H33" s="38" t="n">
         <f aca="false">-H8*Assumptions!$C$83</f>
-        <v>-65.30448</v>
+        <v>-80.67024</v>
       </c>
       <c r="I33" s="38" t="n">
         <f aca="false">-I8*Assumptions!$C$83</f>
-        <v>-67.471968</v>
+        <v>-80.5494</v>
       </c>
       <c r="J33" s="38" t="n">
         <f aca="false">-J8*Assumptions!$C$83</f>
-        <v>-67.31424</v>
+        <v>-79.4682</v>
       </c>
       <c r="K33" s="38" t="n">
         <f aca="false">-K8*Assumptions!$C$83</f>
-        <v>-66.3984</v>
+        <v>-78.387</v>
       </c>
       <c r="L33" s="38" t="n">
         <f aca="false">-L8*Assumptions!$C$83</f>
-        <v>-65.48256</v>
+        <v>-77.3058</v>
       </c>
       <c r="M33" s="38" t="n">
         <f aca="false">-M8*Assumptions!$C$83</f>
-        <v>-64.56672</v>
+        <v>-76.2246</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15367,39 +15420,39 @@
       </c>
       <c r="E36" s="38" t="n">
         <f aca="false">E8*Assumptions!$C$86</f>
-        <v>108.438</v>
+        <v>135.5475</v>
       </c>
       <c r="F36" s="38" t="n">
         <f aca="false">F8*Assumptions!$C$86</f>
-        <v>246.45</v>
+        <v>312.9915</v>
       </c>
       <c r="G36" s="38" t="n">
         <f aca="false">G8*Assumptions!$C$86</f>
-        <v>291.924</v>
+        <v>374.6358</v>
       </c>
       <c r="H36" s="38" t="n">
         <f aca="false">H8*Assumptions!$C$86</f>
-        <v>326.5224</v>
+        <v>403.3512</v>
       </c>
       <c r="I36" s="38" t="n">
         <f aca="false">I8*Assumptions!$C$86</f>
-        <v>337.35984</v>
+        <v>402.747</v>
       </c>
       <c r="J36" s="38" t="n">
         <f aca="false">J8*Assumptions!$C$86</f>
-        <v>336.5712</v>
+        <v>397.341</v>
       </c>
       <c r="K36" s="38" t="n">
         <f aca="false">K8*Assumptions!$C$86</f>
-        <v>331.992</v>
+        <v>391.935</v>
       </c>
       <c r="L36" s="38" t="n">
         <f aca="false">L8*Assumptions!$C$86</f>
-        <v>327.4128</v>
+        <v>386.529</v>
       </c>
       <c r="M36" s="38" t="n">
         <f aca="false">M8*Assumptions!$C$86</f>
-        <v>322.8336</v>
+        <v>381.123</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15412,39 +15465,39 @@
       </c>
       <c r="E37" s="38" t="n">
         <f aca="false">-(E36-D36)</f>
-        <v>-108.438</v>
+        <v>-135.5475</v>
       </c>
       <c r="F37" s="38" t="n">
         <f aca="false">-(F36-E36)</f>
-        <v>-138.012</v>
+        <v>-177.444</v>
       </c>
       <c r="G37" s="38" t="n">
         <f aca="false">-(G36-F36)</f>
-        <v>-45.474</v>
+        <v>-61.6442999999999</v>
       </c>
       <c r="H37" s="38" t="n">
         <f aca="false">-(H36-G36)</f>
-        <v>-34.5984</v>
+        <v>-28.7154</v>
       </c>
       <c r="I37" s="38" t="n">
         <f aca="false">-(I36-H36)</f>
-        <v>-10.83744</v>
+        <v>0.604199999999935</v>
       </c>
       <c r="J37" s="38" t="n">
         <f aca="false">-(J36-I36)</f>
-        <v>0.788639999999987</v>
+        <v>5.40600000000001</v>
       </c>
       <c r="K37" s="38" t="n">
         <f aca="false">-(K36-J36)</f>
-        <v>4.57920000000001</v>
+        <v>5.40600000000001</v>
       </c>
       <c r="L37" s="38" t="n">
         <f aca="false">-(L36-K36)</f>
-        <v>4.57919999999996</v>
+        <v>5.40600000000001</v>
       </c>
       <c r="M37" s="38" t="n">
         <f aca="false">-(M36-L36)</f>
-        <v>4.57920000000007</v>
+        <v>5.40600000000001</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15457,39 +15510,39 @@
       </c>
       <c r="E38" s="59" t="n">
         <f aca="false">E31+E32+E33+E34+E35+E37</f>
-        <v>109.720316</v>
+        <v>129.658916</v>
       </c>
       <c r="F38" s="59" t="n">
         <f aca="false">F31+F32+F33+F34+F35+F37</f>
-        <v>445.786644</v>
+        <v>521.836344</v>
       </c>
       <c r="G38" s="59" t="n">
         <f aca="false">G31+G32+G33+G34+G35+G37</f>
-        <v>660.629844</v>
+        <v>815.28591312</v>
       </c>
       <c r="H38" s="59" t="n">
         <f aca="false">H31+H32+H33+H34+H35+H37</f>
-        <v>578.725764</v>
+        <v>724.10662536</v>
       </c>
       <c r="I38" s="59" t="n">
         <f aca="false">I31+I32+I33+I34+I35+I37</f>
-        <v>455.949088032</v>
+        <v>557.3258268</v>
       </c>
       <c r="J38" s="59" t="n">
         <f aca="false">J31+J32+J33+J34+J35+J37</f>
-        <v>299.13639888</v>
+        <v>357.3894324</v>
       </c>
       <c r="K38" s="59" t="n">
         <f aca="false">K31+K32+K33+K34+K35+K37</f>
-        <v>130.269444</v>
+        <v>152.651238</v>
       </c>
       <c r="L38" s="59" t="n">
         <f aca="false">L31+L32+L33+L34+L35+L37</f>
-        <v>131.185284</v>
+        <v>150.6380436</v>
       </c>
       <c r="M38" s="59" t="n">
         <f aca="false">M31+M32+M33+M34+M35+M37</f>
-        <v>132.101124</v>
+        <v>148.6248492</v>
       </c>
     </row>
   </sheetData>
@@ -15593,35 +15646,35 @@
       </c>
       <c r="F6" s="60" t="n">
         <f aca="false">Assumptions!F69*Assumptions!F72</f>
-        <v>1124.928</v>
+        <v>1406.16</v>
       </c>
       <c r="G6" s="60" t="n">
         <f aca="false">Assumptions!G69*Assumptions!G72</f>
-        <v>1744.9344</v>
+        <v>2300.1408</v>
       </c>
       <c r="H6" s="60" t="n">
         <f aca="false">Assumptions!H69*Assumptions!H72</f>
-        <v>2191.7952</v>
+        <v>2935.44</v>
       </c>
       <c r="I6" s="60" t="n">
         <f aca="false">Assumptions!I69*Assumptions!I72</f>
-        <v>2471.7312</v>
+        <v>3282.768</v>
       </c>
       <c r="J6" s="60" t="n">
         <f aca="false">Assumptions!J69*Assumptions!J72</f>
-        <v>2590.9632</v>
+        <v>3238.704</v>
       </c>
       <c r="K6" s="60" t="n">
         <f aca="false">Assumptions!K69*Assumptions!K72</f>
-        <v>2555.712</v>
+        <v>3194.64</v>
       </c>
       <c r="L6" s="60" t="n">
         <f aca="false">Assumptions!L69*Assumptions!L72</f>
-        <v>2520.4608</v>
+        <v>3150.576</v>
       </c>
       <c r="M6" s="60" t="n">
         <f aca="false">Assumptions!M69*Assumptions!M72</f>
-        <v>2485.2096</v>
+        <v>3106.512</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15638,35 +15691,35 @@
       </c>
       <c r="F7" s="60" t="n">
         <f aca="false">Assumptions!F70*Assumptions!F75</f>
-        <v>117.18</v>
+        <v>146.475</v>
       </c>
       <c r="G7" s="60" t="n">
         <f aca="false">Assumptions!G70*Assumptions!G75</f>
-        <v>181.764</v>
+        <v>239.598</v>
       </c>
       <c r="H7" s="60" t="n">
         <f aca="false">Assumptions!H70*Assumptions!H75</f>
-        <v>228.312</v>
+        <v>305.775</v>
       </c>
       <c r="I7" s="60" t="n">
         <f aca="false">Assumptions!I70*Assumptions!I75</f>
-        <v>257.472</v>
+        <v>341.955</v>
       </c>
       <c r="J7" s="60" t="n">
         <f aca="false">Assumptions!J70*Assumptions!J75</f>
-        <v>269.892</v>
+        <v>337.365</v>
       </c>
       <c r="K7" s="60" t="n">
         <f aca="false">Assumptions!K70*Assumptions!K75</f>
-        <v>266.22</v>
+        <v>332.775</v>
       </c>
       <c r="L7" s="60" t="n">
         <f aca="false">Assumptions!L70*Assumptions!L75</f>
-        <v>262.548</v>
+        <v>328.185</v>
       </c>
       <c r="M7" s="60" t="n">
         <f aca="false">Assumptions!M70*Assumptions!M75</f>
-        <v>258.876</v>
+        <v>323.595</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15683,35 +15736,35 @@
       </c>
       <c r="F8" s="56" t="n">
         <f aca="false">F6+F7</f>
-        <v>1242.108</v>
+        <v>1552.635</v>
       </c>
       <c r="G8" s="56" t="n">
         <f aca="false">G6+G7</f>
-        <v>1926.6984</v>
+        <v>2539.7388</v>
       </c>
       <c r="H8" s="56" t="n">
         <f aca="false">H6+H7</f>
-        <v>2420.1072</v>
+        <v>3241.215</v>
       </c>
       <c r="I8" s="56" t="n">
         <f aca="false">I6+I7</f>
-        <v>2729.2032</v>
+        <v>3624.723</v>
       </c>
       <c r="J8" s="56" t="n">
         <f aca="false">J6+J7</f>
-        <v>2860.8552</v>
+        <v>3576.069</v>
       </c>
       <c r="K8" s="56" t="n">
         <f aca="false">K6+K7</f>
-        <v>2821.932</v>
+        <v>3527.415</v>
       </c>
       <c r="L8" s="56" t="n">
         <f aca="false">L6+L7</f>
-        <v>2783.0088</v>
+        <v>3478.761</v>
       </c>
       <c r="M8" s="56" t="n">
         <f aca="false">M6+M7</f>
-        <v>2744.0856</v>
+        <v>3430.107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15728,35 +15781,35 @@
       </c>
       <c r="F9" s="38" t="n">
         <f aca="false">-(Assumptions!F69*Assumptions!F74+Assumptions!F70*Assumptions!F77)</f>
-        <v>-1055.7918</v>
+        <v>-1319.73975</v>
       </c>
       <c r="G9" s="38" t="n">
         <f aca="false">-(Assumptions!G69*Assumptions!G74+Assumptions!G70*Assumptions!G77)</f>
-        <v>-1637.69364</v>
+        <v>-2158.77798</v>
       </c>
       <c r="H9" s="38" t="n">
         <f aca="false">-(Assumptions!H69*Assumptions!H74+Assumptions!H70*Assumptions!H77)</f>
-        <v>-2057.09112</v>
+        <v>-2755.03275</v>
       </c>
       <c r="I9" s="38" t="n">
         <f aca="false">-(Assumptions!I69*Assumptions!I74+Assumptions!I70*Assumptions!I77)</f>
-        <v>-2319.82272</v>
+        <v>-3081.01455</v>
       </c>
       <c r="J9" s="38" t="n">
         <f aca="false">-(Assumptions!J69*Assumptions!J74+Assumptions!J70*Assumptions!J77)</f>
-        <v>-2431.72692</v>
+        <v>-3039.65865</v>
       </c>
       <c r="K9" s="38" t="n">
         <f aca="false">-(Assumptions!K69*Assumptions!K74+Assumptions!K70*Assumptions!K77)</f>
-        <v>-2398.6422</v>
+        <v>-2998.30275</v>
       </c>
       <c r="L9" s="38" t="n">
         <f aca="false">-(Assumptions!L69*Assumptions!L74+Assumptions!L70*Assumptions!L77)</f>
-        <v>-2365.55748</v>
+        <v>-2956.94685</v>
       </c>
       <c r="M9" s="38" t="n">
         <f aca="false">-(Assumptions!M69*Assumptions!M74+Assumptions!M70*Assumptions!M77)</f>
-        <v>-2332.47276</v>
+        <v>-2915.59095</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15825,35 +15878,35 @@
       </c>
       <c r="F12" s="56" t="n">
         <f aca="false">F8+F9</f>
-        <v>186.3162</v>
+        <v>232.89525</v>
       </c>
       <c r="G12" s="56" t="n">
         <f aca="false">G8+G9</f>
-        <v>289.00476</v>
+        <v>380.96082</v>
       </c>
       <c r="H12" s="56" t="n">
         <f aca="false">H8+H9</f>
-        <v>363.01608</v>
+        <v>486.18225</v>
       </c>
       <c r="I12" s="56" t="n">
         <f aca="false">I8+I9</f>
-        <v>409.38048</v>
+        <v>543.70845</v>
       </c>
       <c r="J12" s="56" t="n">
         <f aca="false">J8+J9</f>
-        <v>429.12828</v>
+        <v>536.410350000001</v>
       </c>
       <c r="K12" s="56" t="n">
         <f aca="false">K8+K9</f>
-        <v>423.2898</v>
+        <v>529.11225</v>
       </c>
       <c r="L12" s="56" t="n">
         <f aca="false">L8+L9</f>
-        <v>417.451319999999</v>
+        <v>521.81415</v>
       </c>
       <c r="M12" s="56" t="n">
         <f aca="false">M8+M9</f>
-        <v>411.61284</v>
+        <v>514.51605</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15870,35 +15923,35 @@
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$81</f>
-        <v>-74.52648</v>
+        <v>-93.1581</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$81</f>
-        <v>-115.601904</v>
+        <v>-152.384328</v>
       </c>
       <c r="H13" s="38" t="n">
         <f aca="false">-H8*Assumptions!$C$81</f>
-        <v>-145.206432</v>
+        <v>-194.4729</v>
       </c>
       <c r="I13" s="38" t="n">
         <f aca="false">-I8*Assumptions!$C$81</f>
-        <v>-163.752192</v>
+        <v>-217.48338</v>
       </c>
       <c r="J13" s="38" t="n">
         <f aca="false">-J8*Assumptions!$C$81</f>
-        <v>-171.651312</v>
+        <v>-214.56414</v>
       </c>
       <c r="K13" s="38" t="n">
         <f aca="false">-K8*Assumptions!$C$81</f>
-        <v>-169.31592</v>
+        <v>-211.6449</v>
       </c>
       <c r="L13" s="38" t="n">
         <f aca="false">-L8*Assumptions!$C$81</f>
-        <v>-166.980528</v>
+        <v>-208.72566</v>
       </c>
       <c r="M13" s="38" t="n">
         <f aca="false">-M8*Assumptions!$C$81</f>
-        <v>-164.645136</v>
+        <v>-205.80642</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16005,35 +16058,35 @@
       </c>
       <c r="F16" s="56" t="n">
         <f aca="false">F12+F13+F15</f>
-        <v>45.0897200000002</v>
+        <v>73.0371499999999</v>
       </c>
       <c r="G16" s="56" t="n">
         <f aca="false">G12+G13+G15</f>
-        <v>106.702856</v>
+        <v>161.876492</v>
       </c>
       <c r="H16" s="56" t="n">
         <f aca="false">H12+H13+H15</f>
-        <v>151.109648</v>
+        <v>225.00935</v>
       </c>
       <c r="I16" s="56" t="n">
         <f aca="false">I12+I13+I15</f>
-        <v>178.928288</v>
+        <v>259.52507</v>
       </c>
       <c r="J16" s="56" t="n">
         <f aca="false">J12+J13+J15</f>
-        <v>190.776968</v>
+        <v>255.146210000001</v>
       </c>
       <c r="K16" s="56" t="n">
         <f aca="false">K12+K13+K15</f>
-        <v>187.27388</v>
+        <v>250.76735</v>
       </c>
       <c r="L16" s="56" t="n">
         <f aca="false">L12+L13+L15</f>
-        <v>183.770791999999</v>
+        <v>246.38849</v>
       </c>
       <c r="M16" s="56" t="n">
         <f aca="false">M12+M13+M15</f>
-        <v>180.267704</v>
+        <v>242.00963</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16050,35 +16103,35 @@
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.0363009657775332</v>
+        <v>0.0470407726220264</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.0553811930294851</v>
+        <v>0.0637374567809886</v>
       </c>
       <c r="H17" s="57" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.0624392374023762</v>
+        <v>0.0694212972604409</v>
       </c>
       <c r="I17" s="57" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.065560632495228</v>
+        <v>0.0715985938787598</v>
       </c>
       <c r="J17" s="57" t="n">
         <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.0666852932647554</v>
+        <v>0.0713482346118043</v>
       </c>
       <c r="K17" s="57" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0663637111028898</v>
+        <v>0.0710909688823118</v>
       </c>
       <c r="L17" s="57" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0660331336357971</v>
+        <v>0.0708265069086379</v>
       </c>
       <c r="M17" s="57" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0656931780845322</v>
+        <v>0.0705545424676257</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16095,23 +16148,23 @@
       </c>
       <c r="F18" s="38" t="n">
         <f aca="false">(Assumptions!F69+Assumptions!F70)*Assumptions!F8</f>
-        <v>374.22</v>
+        <v>467.775</v>
       </c>
       <c r="G18" s="38" t="n">
         <f aca="false">(Assumptions!G69+Assumptions!G70)*Assumptions!G8</f>
-        <v>588.06</v>
+        <v>775.17</v>
       </c>
       <c r="H18" s="38" t="n">
         <f aca="false">(Assumptions!H69+Assumptions!H70)*Assumptions!H8</f>
-        <v>561.33</v>
+        <v>751.78125</v>
       </c>
       <c r="I18" s="38" t="n">
         <f aca="false">(Assumptions!I69+Assumptions!I70)*Assumptions!I8</f>
-        <v>427.68</v>
+        <v>568.0125</v>
       </c>
       <c r="J18" s="38" t="n">
         <f aca="false">(Assumptions!J69+Assumptions!J70)*Assumptions!J8</f>
-        <v>227.205</v>
+        <v>284.00625</v>
       </c>
       <c r="K18" s="38" t="n">
         <f aca="false">(Assumptions!K69+Assumptions!K70)*Assumptions!K8</f>
@@ -16140,35 +16193,35 @@
       </c>
       <c r="F19" s="56" t="n">
         <f aca="false">F16+F18</f>
-        <v>419.30972</v>
+        <v>540.81215</v>
       </c>
       <c r="G19" s="56" t="n">
         <f aca="false">G16+G18</f>
-        <v>694.762856</v>
+        <v>937.046492</v>
       </c>
       <c r="H19" s="56" t="n">
         <f aca="false">H16+H18</f>
-        <v>712.439648</v>
+        <v>976.7906</v>
       </c>
       <c r="I19" s="56" t="n">
         <f aca="false">I16+I18</f>
-        <v>606.608288</v>
+        <v>827.53757</v>
       </c>
       <c r="J19" s="56" t="n">
         <f aca="false">J16+J18</f>
-        <v>417.981968</v>
+        <v>539.152460000001</v>
       </c>
       <c r="K19" s="56" t="n">
         <f aca="false">K16+K18</f>
-        <v>187.27388</v>
+        <v>250.76735</v>
       </c>
       <c r="L19" s="56" t="n">
         <f aca="false">L16+L18</f>
-        <v>183.770791999999</v>
+        <v>246.38849</v>
       </c>
       <c r="M19" s="56" t="n">
         <f aca="false">M16+M18</f>
-        <v>180.267704</v>
+        <v>242.00963</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16237,35 +16290,35 @@
       </c>
       <c r="F23" s="38" t="n">
         <f aca="false">MAX(0,F16)</f>
-        <v>45.0897200000002</v>
+        <v>73.0371499999999</v>
       </c>
       <c r="G23" s="38" t="n">
         <f aca="false">MAX(0,G16)</f>
-        <v>106.702856</v>
+        <v>161.876492</v>
       </c>
       <c r="H23" s="38" t="n">
         <f aca="false">MAX(0,H16)</f>
-        <v>151.109648</v>
+        <v>225.00935</v>
       </c>
       <c r="I23" s="38" t="n">
         <f aca="false">MAX(0,I16)</f>
-        <v>178.928288</v>
+        <v>259.52507</v>
       </c>
       <c r="J23" s="38" t="n">
         <f aca="false">MAX(0,J16)</f>
-        <v>190.776968</v>
+        <v>255.146210000001</v>
       </c>
       <c r="K23" s="38" t="n">
         <f aca="false">MAX(0,K16)</f>
-        <v>187.27388</v>
+        <v>250.76735</v>
       </c>
       <c r="L23" s="38" t="n">
         <f aca="false">MAX(0,L16)</f>
-        <v>183.770791999999</v>
+        <v>246.38849</v>
       </c>
       <c r="M23" s="38" t="n">
         <f aca="false">MAX(0,M16)</f>
-        <v>180.267704</v>
+        <v>242.00963</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16286,7 +16339,7 @@
       </c>
       <c r="G24" s="38" t="n">
         <f aca="false">F27</f>
-        <v>23.9582239999998</v>
+        <v>1.60028000000011</v>
       </c>
       <c r="H24" s="38" t="n">
         <f aca="false">G27</f>
@@ -16327,11 +16380,11 @@
       </c>
       <c r="F25" s="38" t="n">
         <f aca="false">MIN(F24,F23*Assumptions!$C$90)</f>
-        <v>36.0717760000002</v>
+        <v>58.4297199999999</v>
       </c>
       <c r="G25" s="38" t="n">
         <f aca="false">MIN(G24,G23*Assumptions!$C$90)</f>
-        <v>23.9582239999998</v>
+        <v>1.60028000000011</v>
       </c>
       <c r="H25" s="38" t="n">
         <f aca="false">MIN(H24,H23*Assumptions!$C$90)</f>
@@ -16417,7 +16470,7 @@
       </c>
       <c r="F27" s="38" t="n">
         <f aca="false">F24-F25+F26</f>
-        <v>23.9582239999998</v>
+        <v>1.60028000000011</v>
       </c>
       <c r="G27" s="38" t="n">
         <f aca="false">G24-G25+G26</f>
@@ -16462,35 +16515,35 @@
       </c>
       <c r="F28" s="38" t="n">
         <f aca="false">F23-F25</f>
-        <v>9.01794400000004</v>
+        <v>14.60743</v>
       </c>
       <c r="G28" s="38" t="n">
         <f aca="false">G23-G25</f>
-        <v>82.7446320000002</v>
+        <v>160.276212</v>
       </c>
       <c r="H28" s="38" t="n">
         <f aca="false">H23-H25</f>
-        <v>151.109648</v>
+        <v>225.00935</v>
       </c>
       <c r="I28" s="38" t="n">
         <f aca="false">I23-I25</f>
-        <v>178.928288</v>
+        <v>259.52507</v>
       </c>
       <c r="J28" s="38" t="n">
         <f aca="false">J23-J25</f>
-        <v>190.776968</v>
+        <v>255.146210000001</v>
       </c>
       <c r="K28" s="38" t="n">
         <f aca="false">K23-K25</f>
-        <v>187.27388</v>
+        <v>250.76735</v>
       </c>
       <c r="L28" s="38" t="n">
         <f aca="false">L23-L25</f>
-        <v>183.770791999999</v>
+        <v>246.38849</v>
       </c>
       <c r="M28" s="38" t="n">
         <f aca="false">M23-M25</f>
-        <v>180.267704</v>
+        <v>242.00963</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16507,35 +16560,35 @@
       </c>
       <c r="F29" s="38" t="n">
         <f aca="false">-F28*Assumptions!$C$87</f>
-        <v>-2.07412712000001</v>
+        <v>-3.35970889999999</v>
       </c>
       <c r="G29" s="38" t="n">
         <f aca="false">-G28*Assumptions!$C$87</f>
-        <v>-19.0312653600001</v>
+        <v>-36.8635287599999</v>
       </c>
       <c r="H29" s="38" t="n">
         <f aca="false">-H28*Assumptions!$C$87</f>
-        <v>-34.75521904</v>
+        <v>-51.7521505</v>
       </c>
       <c r="I29" s="38" t="n">
         <f aca="false">-I28*Assumptions!$C$87</f>
-        <v>-41.1535062400001</v>
+        <v>-59.6907660999999</v>
       </c>
       <c r="J29" s="38" t="n">
         <f aca="false">-J28*Assumptions!$C$87</f>
-        <v>-43.8787026400001</v>
+        <v>-58.6836283000001</v>
       </c>
       <c r="K29" s="38" t="n">
         <f aca="false">-K28*Assumptions!$C$87</f>
-        <v>-43.0729924</v>
+        <v>-57.6764904999999</v>
       </c>
       <c r="L29" s="38" t="n">
         <f aca="false">-L28*Assumptions!$C$87</f>
-        <v>-42.2672821599998</v>
+        <v>-56.6693527000001</v>
       </c>
       <c r="M29" s="38" t="n">
         <f aca="false">-M28*Assumptions!$C$87</f>
-        <v>-41.4615719200001</v>
+        <v>-55.6622149</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16552,35 +16605,35 @@
       </c>
       <c r="F30" s="56" t="n">
         <f aca="false">F19+F29</f>
-        <v>417.23559288</v>
+        <v>537.4524411</v>
       </c>
       <c r="G30" s="56" t="n">
         <f aca="false">G19+G29</f>
-        <v>675.73159064</v>
+        <v>900.18296324</v>
       </c>
       <c r="H30" s="56" t="n">
         <f aca="false">H19+H29</f>
-        <v>677.68442896</v>
+        <v>925.0384495</v>
       </c>
       <c r="I30" s="56" t="n">
         <f aca="false">I19+I29</f>
-        <v>565.45478176</v>
+        <v>767.8468039</v>
       </c>
       <c r="J30" s="56" t="n">
         <f aca="false">J19+J29</f>
-        <v>374.10326536</v>
+        <v>480.4688317</v>
       </c>
       <c r="K30" s="56" t="n">
         <f aca="false">K19+K29</f>
-        <v>144.2008876</v>
+        <v>193.0908595</v>
       </c>
       <c r="L30" s="56" t="n">
         <f aca="false">L19+L29</f>
-        <v>141.503509839999</v>
+        <v>189.7191373</v>
       </c>
       <c r="M30" s="56" t="n">
         <f aca="false">M19+M29</f>
-        <v>138.80613208</v>
+        <v>186.3474151</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16642,35 +16695,35 @@
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$83</f>
-        <v>-37.26324</v>
+        <v>-46.57905</v>
       </c>
       <c r="G32" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$83</f>
-        <v>-57.800952</v>
+        <v>-76.192164</v>
       </c>
       <c r="H32" s="38" t="n">
         <f aca="false">-H8*Assumptions!$C$83</f>
-        <v>-72.603216</v>
+        <v>-97.23645</v>
       </c>
       <c r="I32" s="38" t="n">
         <f aca="false">-I8*Assumptions!$C$83</f>
-        <v>-81.876096</v>
+        <v>-108.74169</v>
       </c>
       <c r="J32" s="38" t="n">
         <f aca="false">-J8*Assumptions!$C$83</f>
-        <v>-85.825656</v>
+        <v>-107.28207</v>
       </c>
       <c r="K32" s="38" t="n">
         <f aca="false">-K8*Assumptions!$C$83</f>
-        <v>-84.65796</v>
+        <v>-105.82245</v>
       </c>
       <c r="L32" s="38" t="n">
         <f aca="false">-L8*Assumptions!$C$83</f>
-        <v>-83.490264</v>
+        <v>-104.36283</v>
       </c>
       <c r="M32" s="38" t="n">
         <f aca="false">-M8*Assumptions!$C$83</f>
-        <v>-82.322568</v>
+        <v>-102.90321</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16777,35 +16830,35 @@
       </c>
       <c r="F35" s="38" t="n">
         <f aca="false">F8*Assumptions!$C$86</f>
-        <v>186.3162</v>
+        <v>232.89525</v>
       </c>
       <c r="G35" s="38" t="n">
         <f aca="false">G8*Assumptions!$C$86</f>
-        <v>289.00476</v>
+        <v>380.96082</v>
       </c>
       <c r="H35" s="38" t="n">
         <f aca="false">H8*Assumptions!$C$86</f>
-        <v>363.01608</v>
+        <v>486.18225</v>
       </c>
       <c r="I35" s="38" t="n">
         <f aca="false">I8*Assumptions!$C$86</f>
-        <v>409.38048</v>
+        <v>543.70845</v>
       </c>
       <c r="J35" s="38" t="n">
         <f aca="false">J8*Assumptions!$C$86</f>
-        <v>429.12828</v>
+        <v>536.41035</v>
       </c>
       <c r="K35" s="38" t="n">
         <f aca="false">K8*Assumptions!$C$86</f>
-        <v>423.2898</v>
+        <v>529.11225</v>
       </c>
       <c r="L35" s="38" t="n">
         <f aca="false">L8*Assumptions!$C$86</f>
-        <v>417.45132</v>
+        <v>521.81415</v>
       </c>
       <c r="M35" s="38" t="n">
         <f aca="false">M8*Assumptions!$C$86</f>
-        <v>411.61284</v>
+        <v>514.51605</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16822,35 +16875,35 @@
       </c>
       <c r="F36" s="38" t="n">
         <f aca="false">-(F35-E35)</f>
-        <v>-186.3162</v>
+        <v>-232.89525</v>
       </c>
       <c r="G36" s="38" t="n">
         <f aca="false">-(G35-F35)</f>
-        <v>-102.68856</v>
+        <v>-148.06557</v>
       </c>
       <c r="H36" s="38" t="n">
         <f aca="false">-(H35-G35)</f>
-        <v>-74.01132</v>
+        <v>-105.22143</v>
       </c>
       <c r="I36" s="38" t="n">
         <f aca="false">-(I35-H35)</f>
-        <v>-46.3644</v>
+        <v>-57.5261999999999</v>
       </c>
       <c r="J36" s="38" t="n">
         <f aca="false">-(J35-I35)</f>
-        <v>-19.7477999999999</v>
+        <v>7.29809999999986</v>
       </c>
       <c r="K36" s="38" t="n">
         <f aca="false">-(K35-J35)</f>
-        <v>5.83848</v>
+        <v>7.29810000000009</v>
       </c>
       <c r="L36" s="38" t="n">
         <f aca="false">-(L35-K35)</f>
-        <v>5.83848</v>
+        <v>7.29809999999998</v>
       </c>
       <c r="M36" s="38" t="n">
         <f aca="false">-(M35-L35)</f>
-        <v>5.83848</v>
+        <v>7.29809999999998</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16867,35 +16920,35 @@
       </c>
       <c r="F37" s="59" t="n">
         <f aca="false">F30+F31+F32+F33+F34+F36</f>
-        <v>-9.64384711999981</v>
+        <v>54.6781411</v>
       </c>
       <c r="G37" s="59" t="n">
         <f aca="false">G30+G31+G32+G33+G34+G36</f>
-        <v>581.94207864</v>
+        <v>742.62522924</v>
       </c>
       <c r="H37" s="59" t="n">
         <f aca="false">H30+H31+H32+H33+H34+H36</f>
-        <v>597.76989296</v>
+        <v>789.2805695</v>
       </c>
       <c r="I37" s="59" t="n">
         <f aca="false">I30+I31+I32+I33+I34+I36</f>
-        <v>503.91428576</v>
+        <v>668.2789139</v>
       </c>
       <c r="J37" s="59" t="n">
         <f aca="false">J30+J31+J32+J33+J34+J36</f>
-        <v>335.22980936</v>
+        <v>447.1848617</v>
       </c>
       <c r="K37" s="59" t="n">
         <f aca="false">K30+K31+K32+K33+K34+K36</f>
-        <v>132.0814076</v>
+        <v>161.2665095</v>
       </c>
       <c r="L37" s="59" t="n">
         <f aca="false">L30+L31+L32+L33+L34+L36</f>
-        <v>130.551725839999</v>
+        <v>159.3544073</v>
       </c>
       <c r="M37" s="59" t="n">
         <f aca="false">M30+M31+M32+M33+M34+M36</f>
-        <v>129.02204408</v>
+        <v>157.4423051</v>
       </c>
     </row>
   </sheetData>
@@ -16995,39 +17048,39 @@
       </c>
       <c r="E6" s="62" t="n">
         <f aca="false">SKBA!E8</f>
-        <v>722.92</v>
+        <v>903.65</v>
       </c>
       <c r="F6" s="62" t="n">
         <f aca="false">SKBA!F8</f>
-        <v>1643</v>
+        <v>2086.61</v>
       </c>
       <c r="G6" s="62" t="n">
         <f aca="false">SKBA!G8</f>
-        <v>1946.16</v>
+        <v>2497.572</v>
       </c>
       <c r="H6" s="62" t="n">
         <f aca="false">SKBA!H8</f>
-        <v>2176.816</v>
+        <v>2689.008</v>
       </c>
       <c r="I6" s="62" t="n">
         <f aca="false">SKBA!I8</f>
-        <v>2249.0656</v>
+        <v>2684.98</v>
       </c>
       <c r="J6" s="62" t="n">
         <f aca="false">SKBA!J8</f>
-        <v>2243.808</v>
+        <v>2648.94</v>
       </c>
       <c r="K6" s="62" t="n">
         <f aca="false">SKBA!K8</f>
-        <v>2213.28</v>
+        <v>2612.9</v>
       </c>
       <c r="L6" s="62" t="n">
         <f aca="false">SKBA!L8</f>
-        <v>2182.752</v>
+        <v>2576.86</v>
       </c>
       <c r="M6" s="62" t="n">
         <f aca="false">SKBA!M8</f>
-        <v>2152.224</v>
+        <v>2540.82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17044,35 +17097,35 @@
       </c>
       <c r="F7" s="64" t="n">
         <f aca="false">SKOT!F8</f>
-        <v>1242.108</v>
+        <v>1552.635</v>
       </c>
       <c r="G7" s="64" t="n">
         <f aca="false">SKOT!G8</f>
-        <v>1926.6984</v>
+        <v>2539.7388</v>
       </c>
       <c r="H7" s="64" t="n">
         <f aca="false">SKOT!H8</f>
-        <v>2420.1072</v>
+        <v>3241.215</v>
       </c>
       <c r="I7" s="64" t="n">
         <f aca="false">SKOT!I8</f>
-        <v>2729.2032</v>
+        <v>3624.723</v>
       </c>
       <c r="J7" s="64" t="n">
         <f aca="false">SKOT!J8</f>
-        <v>2860.8552</v>
+        <v>3576.069</v>
       </c>
       <c r="K7" s="64" t="n">
         <f aca="false">SKOT!K8</f>
-        <v>2821.932</v>
+        <v>3527.415</v>
       </c>
       <c r="L7" s="64" t="n">
         <f aca="false">SKOT!L8</f>
-        <v>2783.0088</v>
+        <v>3478.761</v>
       </c>
       <c r="M7" s="64" t="n">
         <f aca="false">SKOT!M8</f>
-        <v>2744.0856</v>
+        <v>3430.107</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17085,39 +17138,39 @@
       </c>
       <c r="E8" s="56" t="n">
         <f aca="false">E6+E7</f>
-        <v>722.92</v>
+        <v>903.65</v>
       </c>
       <c r="F8" s="56" t="n">
         <f aca="false">F6+F7</f>
-        <v>2885.108</v>
+        <v>3639.245</v>
       </c>
       <c r="G8" s="56" t="n">
         <f aca="false">G6+G7</f>
-        <v>3872.8584</v>
+        <v>5037.3108</v>
       </c>
       <c r="H8" s="56" t="n">
         <f aca="false">H6+H7</f>
-        <v>4596.9232</v>
+        <v>5930.223</v>
       </c>
       <c r="I8" s="56" t="n">
         <f aca="false">I6+I7</f>
-        <v>4978.2688</v>
+        <v>6309.703</v>
       </c>
       <c r="J8" s="56" t="n">
         <f aca="false">J6+J7</f>
-        <v>5104.6632</v>
+        <v>6225.009</v>
       </c>
       <c r="K8" s="56" t="n">
         <f aca="false">K6+K7</f>
-        <v>5035.212</v>
+        <v>6140.315</v>
       </c>
       <c r="L8" s="56" t="n">
         <f aca="false">L6+L7</f>
-        <v>4965.7608</v>
+        <v>6055.621</v>
       </c>
       <c r="M8" s="56" t="n">
         <f aca="false">M6+M7</f>
-        <v>4896.3096</v>
+        <v>5970.927</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17130,39 +17183,39 @@
       </c>
       <c r="E9" s="54" t="n">
         <f aca="false">SKBA!E6+Assumptions!E69+Assumptions!E70</f>
-        <v>4.664</v>
+        <v>5.83</v>
       </c>
       <c r="F9" s="54" t="n">
         <f aca="false">SKBA!F6+Assumptions!F69+Assumptions!F70</f>
-        <v>18.916</v>
+        <v>23.857</v>
       </c>
       <c r="G9" s="54" t="n">
         <f aca="false">SKBA!G6+Assumptions!G69+Assumptions!G70</f>
-        <v>25.788</v>
+        <v>33.55</v>
       </c>
       <c r="H9" s="54" t="n">
         <f aca="false">SKBA!H6+Assumptions!H69+Assumptions!H70</f>
-        <v>31.048</v>
+        <v>40.083</v>
       </c>
       <c r="I9" s="54" t="n">
         <f aca="false">SKBA!I6+Assumptions!I69+Assumptions!I70</f>
-        <v>34.1024</v>
+        <v>43.265</v>
       </c>
       <c r="J9" s="54" t="n">
         <f aca="false">SKBA!J6+Assumptions!J69+Assumptions!J70</f>
-        <v>35.46</v>
+        <v>43.265</v>
       </c>
       <c r="K9" s="54" t="n">
         <f aca="false">SKBA!K6+Assumptions!K69+Assumptions!K70</f>
-        <v>35.46</v>
+        <v>43.265</v>
       </c>
       <c r="L9" s="54" t="n">
         <f aca="false">SKBA!L6+Assumptions!L69+Assumptions!L70</f>
-        <v>35.46</v>
+        <v>43.265</v>
       </c>
       <c r="M9" s="54" t="n">
         <f aca="false">SKBA!M6+Assumptions!M69+Assumptions!M70</f>
-        <v>35.46</v>
+        <v>43.265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17231,35 +17284,35 @@
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">SKBA!F17+SKOT!F16</f>
-        <v>217.07572</v>
+        <v>245.02315</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">SKBA!G17+SKOT!G16</f>
-        <v>278.688856</v>
+        <v>360.265772</v>
       </c>
       <c r="H13" s="38" t="n">
         <f aca="false">SKBA!H17+SKOT!H16</f>
-        <v>323.095648</v>
+        <v>439.32619</v>
       </c>
       <c r="I13" s="38" t="n">
         <f aca="false">SKBA!I17+SKOT!I16</f>
-        <v>353.582896</v>
+        <v>473.15927</v>
       </c>
       <c r="J13" s="38" t="n">
         <f aca="false">SKBA!J17+SKOT!J16</f>
-        <v>364.705688</v>
+        <v>465.53681</v>
       </c>
       <c r="K13" s="38" t="n">
         <f aca="false">SKBA!K17+SKOT!K16</f>
-        <v>359.25988</v>
+        <v>457.91435</v>
       </c>
       <c r="L13" s="38" t="n">
         <f aca="false">SKBA!L17+SKOT!L16</f>
-        <v>355.756791999999</v>
+        <v>450.29189</v>
       </c>
       <c r="M13" s="38" t="n">
         <f aca="false">SKBA!M17+SKOT!M16</f>
-        <v>352.253704</v>
+        <v>442.66943</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17272,39 +17325,39 @@
       </c>
       <c r="E14" s="57" t="n">
         <f aca="false">IF(E8=0,0,E13/E8)</f>
-        <v>0.177009904277098</v>
+        <v>0.141607923421679</v>
       </c>
       <c r="F14" s="57" t="n">
         <f aca="false">IF(F8=0,0,F13/F8)</f>
-        <v>0.0752400672695789</v>
+        <v>0.0673280172123613</v>
       </c>
       <c r="G14" s="57" t="n">
         <f aca="false">IF(G8=0,0,G13/G8)</f>
-        <v>0.0719594746867068</v>
+        <v>0.0715194647112106</v>
       </c>
       <c r="H14" s="57" t="n">
         <f aca="false">IF(H8=0,0,H13/H8)</f>
-        <v>0.0702851959763</v>
+        <v>0.0740825749723072</v>
       </c>
       <c r="I14" s="57" t="n">
         <f aca="false">IF(I8=0,0,I13/I8)</f>
-        <v>0.0710252720785186</v>
+        <v>0.0749891508364181</v>
       </c>
       <c r="J14" s="57" t="n">
         <f aca="false">IF(J8=0,0,J13/J8)</f>
-        <v>0.0714455927278416</v>
+        <v>0.0747849215960974</v>
       </c>
       <c r="K14" s="57" t="n">
         <f aca="false">IF(K8=0,0,K13/K8)</f>
-        <v>0.0713495042512609</v>
+        <v>0.0745750584456986</v>
       </c>
       <c r="L14" s="57" t="n">
         <f aca="false">IF(L8=0,0,L13/L8)</f>
-        <v>0.071641951017858</v>
+        <v>0.0743593249973868</v>
       </c>
       <c r="M14" s="57" t="n">
         <f aca="false">IF(M8=0,0,M13/M8)</f>
-        <v>0.0719426941466284</v>
+        <v>0.0741374714512504</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17317,27 +17370,27 @@
       </c>
       <c r="E15" s="38" t="n">
         <f aca="false">SKBA!E19+SKOT!E18</f>
-        <v>209.88</v>
+        <v>262.35</v>
       </c>
       <c r="F15" s="38" t="n">
         <f aca="false">SKBA!F19+SKOT!F18</f>
-        <v>851.22</v>
+        <v>1073.565</v>
       </c>
       <c r="G15" s="38" t="n">
         <f aca="false">SKBA!G19+SKOT!G18</f>
-        <v>1160.46</v>
+        <v>1509.75</v>
       </c>
       <c r="H15" s="38" t="n">
         <f aca="false">SKBA!H19+SKOT!H18</f>
-        <v>1047.87</v>
+        <v>1352.80125</v>
       </c>
       <c r="I15" s="38" t="n">
         <f aca="false">SKBA!I19+SKOT!I18</f>
-        <v>767.304</v>
+        <v>973.4625</v>
       </c>
       <c r="J15" s="38" t="n">
         <f aca="false">SKBA!J19+SKOT!J18</f>
-        <v>398.925</v>
+        <v>486.73125</v>
       </c>
       <c r="K15" s="38" t="n">
         <f aca="false">SKBA!K19+SKOT!K18</f>
@@ -17362,39 +17415,39 @@
       </c>
       <c r="E16" s="56" t="n">
         <f aca="false">SKBA!E20+SKOT!E19</f>
-        <v>337.844</v>
+        <v>390.314</v>
       </c>
       <c r="F16" s="56" t="n">
         <f aca="false">SKBA!F20+SKOT!F19</f>
-        <v>1068.29572</v>
+        <v>1318.58815</v>
       </c>
       <c r="G16" s="56" t="n">
         <f aca="false">SKBA!G20+SKOT!G19</f>
-        <v>1439.148856</v>
+        <v>1870.015772</v>
       </c>
       <c r="H16" s="56" t="n">
         <f aca="false">SKBA!H20+SKOT!H19</f>
-        <v>1370.965648</v>
+        <v>1792.12744</v>
       </c>
       <c r="I16" s="56" t="n">
         <f aca="false">SKBA!I20+SKOT!I19</f>
-        <v>1120.886896</v>
+        <v>1446.62177</v>
       </c>
       <c r="J16" s="56" t="n">
         <f aca="false">SKBA!J20+SKOT!J19</f>
-        <v>763.630688</v>
+        <v>952.26806</v>
       </c>
       <c r="K16" s="56" t="n">
         <f aca="false">SKBA!K20+SKOT!K19</f>
-        <v>359.25988</v>
+        <v>457.91435</v>
       </c>
       <c r="L16" s="56" t="n">
         <f aca="false">SKBA!L20+SKOT!L19</f>
-        <v>355.756791999999</v>
+        <v>450.29189</v>
       </c>
       <c r="M16" s="56" t="n">
         <f aca="false">SKBA!M20+SKOT!M19</f>
-        <v>352.253704</v>
+        <v>442.66943</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17407,39 +17460,39 @@
       </c>
       <c r="E17" s="57" t="n">
         <f aca="false">IF(E8=0,0,E16/E8)</f>
-        <v>0.46733248492226</v>
+        <v>0.43193050406684</v>
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.37027928243934</v>
+        <v>0.362324644260004</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.371598624932944</v>
+        <v>0.371232954694795</v>
       </c>
       <c r="H17" s="57" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.298235491078032</v>
+        <v>0.302202369118328</v>
       </c>
       <c r="I17" s="57" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.225155961044129</v>
+        <v>0.229269391919081</v>
       </c>
       <c r="J17" s="57" t="n">
         <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.149594725074124</v>
+        <v>0.152974567586971</v>
       </c>
       <c r="K17" s="57" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0713495042512609</v>
+        <v>0.0745750584456986</v>
       </c>
       <c r="L17" s="57" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.071641951017858</v>
+        <v>0.0743593249973868</v>
       </c>
       <c r="M17" s="57" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0719426941466284</v>
+        <v>0.0741374714512504</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17497,39 +17550,39 @@
       </c>
       <c r="E19" s="56" t="n">
         <f aca="false">E16+E18</f>
-        <v>409.88</v>
+        <v>462.35</v>
       </c>
       <c r="F19" s="56" t="n">
         <f aca="false">F16+F18</f>
-        <v>1163.00972</v>
+        <v>1413.30215</v>
       </c>
       <c r="G19" s="56" t="n">
         <f aca="false">G16+G18</f>
-        <v>1533.862856</v>
+        <v>1964.729772</v>
       </c>
       <c r="H19" s="56" t="n">
         <f aca="false">H16+H18</f>
-        <v>1465.679648</v>
+        <v>1886.84144</v>
       </c>
       <c r="I19" s="56" t="n">
         <f aca="false">I16+I18</f>
-        <v>1215.600896</v>
+        <v>1541.33577</v>
       </c>
       <c r="J19" s="56" t="n">
         <f aca="false">J16+J18</f>
-        <v>858.344688</v>
+        <v>1046.98206</v>
       </c>
       <c r="K19" s="56" t="n">
         <f aca="false">K16+K18</f>
-        <v>453.97388</v>
+        <v>552.62835</v>
       </c>
       <c r="L19" s="56" t="n">
         <f aca="false">L16+L18</f>
-        <v>450.470791999999</v>
+        <v>545.00589</v>
       </c>
       <c r="M19" s="56" t="n">
         <f aca="false">M16+M18</f>
-        <v>446.967704</v>
+        <v>537.38343</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17542,39 +17595,39 @@
       </c>
       <c r="E20" s="57" t="n">
         <f aca="false">IF(E8=0,0,E19/E8)</f>
-        <v>0.566978365517623</v>
+        <v>0.511647208543131</v>
       </c>
       <c r="F20" s="57" t="n">
         <f aca="false">IF(F8=0,0,F19/F8)</f>
-        <v>0.4031078628599</v>
+        <v>0.388350372123888</v>
       </c>
       <c r="G20" s="57" t="n">
         <f aca="false">IF(G8=0,0,G19/G8)</f>
-        <v>0.396054463545582</v>
+        <v>0.390035447485194</v>
       </c>
       <c r="H20" s="57" t="n">
         <f aca="false">IF(H8=0,0,H19/H8)</f>
-        <v>0.318839272320234</v>
+        <v>0.318173775252634</v>
       </c>
       <c r="I20" s="57" t="n">
         <f aca="false">IF(I8=0,0,I19/I8)</f>
-        <v>0.24418145038693</v>
+        <v>0.244280241082663</v>
       </c>
       <c r="J20" s="57" t="n">
         <f aca="false">IF(J8=0,0,J19/J8)</f>
-        <v>0.168149132346283</v>
+        <v>0.168189645990873</v>
       </c>
       <c r="K20" s="57" t="n">
         <f aca="false">IF(K8=0,0,K19/K8)</f>
-        <v>0.0901598343823458</v>
+        <v>0.0899999999999999</v>
       </c>
       <c r="L20" s="57" t="n">
         <f aca="false">IF(L8=0,0,L19/L8)</f>
-        <v>0.0907153626892377</v>
+        <v>0.09</v>
       </c>
       <c r="M20" s="57" t="n">
         <f aca="false">IF(M8=0,0,M19/M8)</f>
-        <v>0.0912866506644107</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17591,35 +17644,35 @@
       </c>
       <c r="F21" s="39" t="n">
         <f aca="false">F19-F15</f>
-        <v>311.78972</v>
+        <v>339.73715</v>
       </c>
       <c r="G21" s="39" t="n">
         <f aca="false">G19-G15</f>
-        <v>373.402856</v>
+        <v>454.979772</v>
       </c>
       <c r="H21" s="39" t="n">
         <f aca="false">H19-H15</f>
-        <v>417.809648</v>
+        <v>534.04019</v>
       </c>
       <c r="I21" s="39" t="n">
         <f aca="false">I19-I15</f>
-        <v>448.296896</v>
+        <v>567.87327</v>
       </c>
       <c r="J21" s="39" t="n">
         <f aca="false">J19-J15</f>
-        <v>459.419688</v>
+        <v>560.25081</v>
       </c>
       <c r="K21" s="39" t="n">
         <f aca="false">K19-K15</f>
-        <v>453.97388</v>
+        <v>552.62835</v>
       </c>
       <c r="L21" s="39" t="n">
         <f aca="false">L19-L15</f>
-        <v>450.470791999999</v>
+        <v>545.00589</v>
       </c>
       <c r="M21" s="39" t="n">
         <f aca="false">M19-M15</f>
-        <v>446.967704</v>
+        <v>537.38343</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17632,23 +17685,23 @@
       </c>
       <c r="E22" s="57" t="n">
         <f aca="false">IF(E8=0,0,E21/E8)</f>
-        <v>0.276655784872462</v>
+        <v>0.221324627897969</v>
       </c>
       <c r="F22" s="57" t="n">
         <f aca="false">IF(F8=0,0,F21/F8)</f>
-        <v>0.108068647690139</v>
+        <v>0.0933537450762451</v>
       </c>
       <c r="G22" s="57" t="n">
         <f aca="false">IF(G8=0,0,G21/G8)</f>
-        <v>0.096415313299345</v>
+        <v>0.0903219575016098</v>
       </c>
       <c r="H22" s="57" t="n">
         <f aca="false">IF(H8=0,0,H21/H8)</f>
-        <v>0.0908889772185013</v>
+        <v>0.0900539811066127</v>
       </c>
       <c r="I22" s="57" t="n">
         <f aca="false">IF(I8=0,0,I21/I8)</f>
-        <v>0.0900507614213199</v>
+        <v>0.09</v>
       </c>
       <c r="J22" s="57" t="n">
         <f aca="false">IF(J8=0,0,J21/J8)</f>
@@ -17656,15 +17709,15 @@
       </c>
       <c r="K22" s="57" t="n">
         <f aca="false">IF(K8=0,0,K21/K8)</f>
-        <v>0.0901598343823458</v>
+        <v>0.0899999999999999</v>
       </c>
       <c r="L22" s="57" t="n">
         <f aca="false">IF(L8=0,0,L21/L8)</f>
-        <v>0.0907153626892377</v>
+        <v>0.09</v>
       </c>
       <c r="M22" s="57" t="n">
         <f aca="false">IF(M8=0,0,M21/M8)</f>
-        <v>0.0912866506644107</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17729,39 +17782,39 @@
       </c>
       <c r="E26" s="66" t="n">
         <f aca="false">SKBA!E38</f>
-        <v>109.720316</v>
+        <v>129.658916</v>
       </c>
       <c r="F26" s="66" t="n">
         <f aca="false">SKBA!F38</f>
-        <v>445.786644</v>
+        <v>521.836344</v>
       </c>
       <c r="G26" s="66" t="n">
         <f aca="false">SKBA!G38</f>
-        <v>660.629844</v>
+        <v>815.28591312</v>
       </c>
       <c r="H26" s="66" t="n">
         <f aca="false">SKBA!H38</f>
-        <v>578.725764</v>
+        <v>724.10662536</v>
       </c>
       <c r="I26" s="66" t="n">
         <f aca="false">SKBA!I38</f>
-        <v>455.949088032</v>
+        <v>557.3258268</v>
       </c>
       <c r="J26" s="66" t="n">
         <f aca="false">SKBA!J38</f>
-        <v>299.13639888</v>
+        <v>357.3894324</v>
       </c>
       <c r="K26" s="66" t="n">
         <f aca="false">SKBA!K38</f>
-        <v>130.269444</v>
+        <v>152.651238</v>
       </c>
       <c r="L26" s="66" t="n">
         <f aca="false">SKBA!L38</f>
-        <v>131.185284</v>
+        <v>150.6380436</v>
       </c>
       <c r="M26" s="66" t="n">
         <f aca="false">SKBA!M38</f>
-        <v>132.101124</v>
+        <v>148.6248492</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17778,35 +17831,35 @@
       </c>
       <c r="F27" s="66" t="n">
         <f aca="false">SKOT!F37</f>
-        <v>-9.64384711999981</v>
+        <v>54.6781411</v>
       </c>
       <c r="G27" s="66" t="n">
         <f aca="false">SKOT!G37</f>
-        <v>581.94207864</v>
+        <v>742.62522924</v>
       </c>
       <c r="H27" s="66" t="n">
         <f aca="false">SKOT!H37</f>
-        <v>597.76989296</v>
+        <v>789.2805695</v>
       </c>
       <c r="I27" s="66" t="n">
         <f aca="false">SKOT!I37</f>
-        <v>503.91428576</v>
+        <v>668.2789139</v>
       </c>
       <c r="J27" s="66" t="n">
         <f aca="false">SKOT!J37</f>
-        <v>335.22980936</v>
+        <v>447.1848617</v>
       </c>
       <c r="K27" s="66" t="n">
         <f aca="false">SKOT!K37</f>
-        <v>132.0814076</v>
+        <v>161.2665095</v>
       </c>
       <c r="L27" s="66" t="n">
         <f aca="false">SKOT!L37</f>
-        <v>130.551725839999</v>
+        <v>159.3544073</v>
       </c>
       <c r="M27" s="66" t="n">
         <f aca="false">SKOT!M37</f>
-        <v>129.02204408</v>
+        <v>157.4423051</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17819,39 +17872,39 @@
       </c>
       <c r="E28" s="59" t="n">
         <f aca="false">E26+E27</f>
-        <v>-340.279684</v>
+        <v>-320.341084</v>
       </c>
       <c r="F28" s="59" t="n">
         <f aca="false">F26+F27</f>
-        <v>436.14279688</v>
+        <v>576.5144851</v>
       </c>
       <c r="G28" s="59" t="n">
         <f aca="false">G26+G27</f>
-        <v>1242.57192264</v>
+        <v>1557.91114236</v>
       </c>
       <c r="H28" s="59" t="n">
         <f aca="false">H26+H27</f>
-        <v>1176.49565696</v>
+        <v>1513.38719486</v>
       </c>
       <c r="I28" s="59" t="n">
         <f aca="false">I26+I27</f>
-        <v>959.863373792</v>
+        <v>1225.6047407</v>
       </c>
       <c r="J28" s="59" t="n">
         <f aca="false">J26+J27</f>
-        <v>634.366208240001</v>
+        <v>804.5742941</v>
       </c>
       <c r="K28" s="59" t="n">
         <f aca="false">K26+K27</f>
-        <v>262.3508516</v>
+        <v>313.9177475</v>
       </c>
       <c r="L28" s="59" t="n">
         <f aca="false">L26+L27</f>
-        <v>261.737009839999</v>
+        <v>309.9924509</v>
       </c>
       <c r="M28" s="59" t="n">
         <f aca="false">M26+M27</f>
-        <v>261.12316808</v>
+        <v>306.0671543</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18051,39 +18104,39 @@
       </c>
       <c r="E35" s="56" t="n">
         <f aca="false">E26+E32+E33+E34</f>
-        <v>67.077716</v>
+        <v>87.016316</v>
       </c>
       <c r="F35" s="56" t="n">
         <f aca="false">F26+F32+F33+F34</f>
-        <v>403.144044</v>
+        <v>479.193744</v>
       </c>
       <c r="G35" s="56" t="n">
         <f aca="false">G26+G32+G33+G34</f>
-        <v>617.987244</v>
+        <v>772.64331312</v>
       </c>
       <c r="H35" s="56" t="n">
         <f aca="false">H26+H32+H33+H34</f>
-        <v>536.083164</v>
+        <v>681.46402536</v>
       </c>
       <c r="I35" s="56" t="n">
         <f aca="false">I26+I32+I33+I34</f>
-        <v>413.306488032</v>
+        <v>514.6832268</v>
       </c>
       <c r="J35" s="56" t="n">
         <f aca="false">J26+J32+J33+J34</f>
-        <v>256.49379888</v>
+        <v>314.7468324</v>
       </c>
       <c r="K35" s="56" t="n">
         <f aca="false">K26+K32+K33+K34</f>
-        <v>87.626844</v>
+        <v>110.008638</v>
       </c>
       <c r="L35" s="56" t="n">
         <f aca="false">L26+L32+L33+L34</f>
-        <v>88.542684</v>
+        <v>107.9954436</v>
       </c>
       <c r="M35" s="56" t="n">
         <f aca="false">M26+M32+M33+M34</f>
-        <v>89.4585240000001</v>
+        <v>105.9822492</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18415,35 +18468,35 @@
       </c>
       <c r="F43" s="56" t="n">
         <f aca="false">F27+F36+F37+F41+F40+F42</f>
-        <v>-163.64384712</v>
+        <v>-99.3218589000001</v>
       </c>
       <c r="G43" s="56" t="n">
         <f aca="false">G27+G36+G37+G41+G40+G42</f>
-        <v>427.94207864</v>
+        <v>588.62522924</v>
       </c>
       <c r="H43" s="56" t="n">
         <f aca="false">H27+H36+H37+H41+H40+H42</f>
-        <v>443.76989296</v>
+        <v>635.2805695</v>
       </c>
       <c r="I43" s="56" t="n">
         <f aca="false">I27+I36+I37+I41+I40+I42</f>
-        <v>349.91428576</v>
+        <v>514.2789139</v>
       </c>
       <c r="J43" s="56" t="n">
         <f aca="false">J27+J36+J37+J41+J40+J42</f>
-        <v>181.22980936</v>
+        <v>293.1848617</v>
       </c>
       <c r="K43" s="56" t="n">
         <f aca="false">K27+K36+K37+K41+K40+K42</f>
-        <v>-21.9185924</v>
+        <v>7.2665094999999</v>
       </c>
       <c r="L43" s="56" t="n">
         <f aca="false">L27+L36+L37+L41+L40+L42</f>
-        <v>-23.4482741600006</v>
+        <v>5.35440730000016</v>
       </c>
       <c r="M43" s="56" t="n">
         <f aca="false">M27+M36+M37+M41+M40+M42</f>
-        <v>-24.9779559199998</v>
+        <v>3.44230510000011</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18460,35 +18513,35 @@
       </c>
       <c r="F44" s="66" t="n">
         <f aca="false">SKOT!F19-SKOT!F15+SKOT!F32</f>
-        <v>448.74648</v>
+        <v>560.9331</v>
       </c>
       <c r="G44" s="66" t="n">
         <f aca="false">SKOT!G19-SKOT!G15+SKOT!G32</f>
-        <v>703.661904</v>
+        <v>927.554328</v>
       </c>
       <c r="H44" s="66" t="n">
         <f aca="false">SKOT!H19-SKOT!H15+SKOT!H32</f>
-        <v>706.536432</v>
+        <v>946.25415</v>
       </c>
       <c r="I44" s="66" t="n">
         <f aca="false">SKOT!I19-SKOT!I15+SKOT!I32</f>
-        <v>591.432192</v>
+        <v>785.49588</v>
       </c>
       <c r="J44" s="66" t="n">
         <f aca="false">SKOT!J19-SKOT!J15+SKOT!J32</f>
-        <v>398.856312</v>
+        <v>498.570390000001</v>
       </c>
       <c r="K44" s="66" t="n">
         <f aca="false">SKOT!K19-SKOT!K15+SKOT!K32</f>
-        <v>169.31592</v>
+        <v>211.6449</v>
       </c>
       <c r="L44" s="66" t="n">
         <f aca="false">SKOT!L19-SKOT!L15+SKOT!L32</f>
-        <v>166.980527999999</v>
+        <v>208.72566</v>
       </c>
       <c r="M44" s="66" t="n">
         <f aca="false">SKOT!M19-SKOT!M15+SKOT!M32</f>
-        <v>164.645136</v>
+        <v>205.80642</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18550,35 +18603,35 @@
       </c>
       <c r="F46" s="67" t="n">
         <f aca="false">IF(F45=0,0,F44/F45)</f>
-        <v>2.2437324</v>
+        <v>2.8046655</v>
       </c>
       <c r="G46" s="67" t="n">
         <f aca="false">IF(G45=0,0,G44/G45)</f>
-        <v>3.51830952</v>
+        <v>4.63777164</v>
       </c>
       <c r="H46" s="67" t="n">
         <f aca="false">IF(H45=0,0,H44/H45)</f>
-        <v>3.53268216</v>
+        <v>4.73127075</v>
       </c>
       <c r="I46" s="67" t="n">
         <f aca="false">IF(I45=0,0,I44/I45)</f>
-        <v>2.95716096</v>
+        <v>3.9274794</v>
       </c>
       <c r="J46" s="67" t="n">
         <f aca="false">IF(J45=0,0,J44/J45)</f>
-        <v>1.99428156</v>
+        <v>2.49285195</v>
       </c>
       <c r="K46" s="67" t="n">
         <f aca="false">IF(K45=0,0,K44/K45)</f>
-        <v>0.8465796</v>
+        <v>1.0582245</v>
       </c>
       <c r="L46" s="67" t="n">
         <f aca="false">IF(L45=0,0,L44/L45)</f>
-        <v>0.834902639999996</v>
+        <v>1.0436283</v>
       </c>
       <c r="M46" s="67" t="n">
         <f aca="false">IF(M45=0,0,M44/M45)</f>
-        <v>0.823225680000001</v>
+        <v>1.0290321</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18591,39 +18644,39 @@
       </c>
       <c r="E47" s="59" t="n">
         <f aca="false">E35+E43</f>
-        <v>-536.922284</v>
+        <v>-516.983684</v>
       </c>
       <c r="F47" s="59" t="n">
         <f aca="false">F35+F43</f>
-        <v>239.50019688</v>
+        <v>379.8718851</v>
       </c>
       <c r="G47" s="59" t="n">
         <f aca="false">G35+G43</f>
-        <v>1045.92932264</v>
+        <v>1361.26854236</v>
       </c>
       <c r="H47" s="59" t="n">
         <f aca="false">H35+H43</f>
-        <v>979.85305696</v>
+        <v>1316.74459486</v>
       </c>
       <c r="I47" s="59" t="n">
         <f aca="false">I35+I43</f>
-        <v>763.220773792</v>
+        <v>1028.9621407</v>
       </c>
       <c r="J47" s="59" t="n">
         <f aca="false">J35+J43</f>
-        <v>437.723608240001</v>
+        <v>607.9316941</v>
       </c>
       <c r="K47" s="59" t="n">
         <f aca="false">K35+K43</f>
-        <v>65.7082516000001</v>
+        <v>117.2751475</v>
       </c>
       <c r="L47" s="59" t="n">
         <f aca="false">L35+L43</f>
-        <v>65.0944098399994</v>
+        <v>113.3498509</v>
       </c>
       <c r="M47" s="59" t="n">
         <f aca="false">M35+M43</f>
-        <v>64.4805680800003</v>
+        <v>109.4245543</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18681,39 +18734,39 @@
       </c>
       <c r="E49" s="39" t="n">
         <f aca="false">E47*E48</f>
-        <v>-446.985838282287</v>
+        <v>-430.387026683745</v>
       </c>
       <c r="F49" s="39" t="n">
         <f aca="false">F47*F48</f>
-        <v>176.445166565116</v>
+        <v>279.860137540752</v>
       </c>
       <c r="G49" s="39" t="n">
         <f aca="false">G47*G48</f>
-        <v>681.911141725133</v>
+        <v>887.501828108433</v>
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">H47*H48</f>
-        <v>565.337711066501</v>
+        <v>759.711234281252</v>
       </c>
       <c r="I49" s="39" t="n">
         <f aca="false">I47*I48</f>
-        <v>389.689535434725</v>
+        <v>525.373250255084</v>
       </c>
       <c r="J49" s="39" t="n">
         <f aca="false">J47*J48</f>
-        <v>197.783513637873</v>
+        <v>274.691298909782</v>
       </c>
       <c r="K49" s="39" t="n">
         <f aca="false">K47*K48</f>
-        <v>26.2743260690461</v>
+        <v>46.8940413141424</v>
       </c>
       <c r="L49" s="39" t="n">
         <f aca="false">L47*L48</f>
-        <v>23.034401066232</v>
+        <v>40.1101405304364</v>
       </c>
       <c r="M49" s="39" t="n">
         <f aca="false">M47*M48</f>
-        <v>20.1922001258037</v>
+        <v>34.2664862437495</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18873,39 +18926,39 @@
       </c>
       <c r="E56" s="39" t="n">
         <f aca="false">E28*E55</f>
-        <v>-292.949393891437</v>
+        <v>-275.784099988544</v>
       </c>
       <c r="F56" s="39" t="n">
         <f aca="false">F28*F55</f>
-        <v>339.7997141757</v>
+        <v>449.163573619744</v>
       </c>
       <c r="G56" s="39" t="n">
         <f aca="false">G28*G55</f>
-        <v>876.099763149647</v>
+        <v>1098.43587961486</v>
       </c>
       <c r="H56" s="39" t="n">
         <f aca="false">H28*H55</f>
-        <v>750.689043407925</v>
+        <v>965.650131298259</v>
       </c>
       <c r="I56" s="39" t="n">
         <f aca="false">I28*I55</f>
-        <v>554.264280178621</v>
+        <v>707.714189264185</v>
       </c>
       <c r="J56" s="39" t="n">
         <f aca="false">J28*J55</f>
-        <v>331.50129824705</v>
+        <v>420.447084926451</v>
       </c>
       <c r="K56" s="39" t="n">
         <f aca="false">K28*K55</f>
-        <v>124.069603155936</v>
+        <v>148.456351936348</v>
       </c>
       <c r="L56" s="39" t="n">
         <f aca="false">L28*L55</f>
-        <v>112.017473571577</v>
+        <v>132.669702298908</v>
       </c>
       <c r="M56" s="39" t="n">
         <f aca="false">M28*M55</f>
-        <v>101.135532390614</v>
+        <v>118.542773607616</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18922,7 +18975,7 @@
       </c>
       <c r="D59" s="38" t="n">
         <f aca="false">SUM(D56:M56)</f>
-        <v>2736.2506063295</v>
+        <v>3604.91887852169</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18931,7 +18984,7 @@
       </c>
       <c r="D60" s="38" t="n">
         <f aca="false">M28*(1+Assumptions!$C$93)/(Assumptions!$C$91-Assumptions!$C$93)</f>
-        <v>3133.47801696</v>
+        <v>3672.8058516</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18940,7 +18993,7 @@
       </c>
       <c r="D61" s="38" t="n">
         <f aca="false">D60*M55</f>
-        <v>1213.62638868737</v>
+        <v>1422.51328329139</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18949,7 +19002,7 @@
       </c>
       <c r="D62" s="73" t="n">
         <f aca="false">D59+D61</f>
-        <v>3949.87699501687</v>
+        <v>5027.43216181308</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18967,7 +19020,7 @@
       </c>
       <c r="D64" s="74" t="n">
         <f aca="false">D62-Assumptions!$C$94</f>
-        <v>-2450.12300498313</v>
+        <v>-1372.56783818692</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18976,7 +19029,7 @@
       </c>
       <c r="D66" s="75" t="n">
         <f aca="false">D61/D62</f>
-        <v>0.307256755139077</v>
+        <v>0.282950269144632</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18993,7 +19046,7 @@
       </c>
       <c r="D69" s="38" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>1290.1036529981</v>
+        <v>2074.44288608985</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19002,7 +19055,7 @@
       </c>
       <c r="D70" s="38" t="n">
         <f aca="false">M47*(1+Assumptions!$C$93)/(Assumptions!$C$92-Assumptions!$C$93)</f>
-        <v>597.910722196367</v>
+        <v>1014.66404896364</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19011,7 +19064,7 @@
       </c>
       <c r="D71" s="38" t="n">
         <f aca="false">D70*1/(1+Assumptions!$C$92)^((10)-Assumptions!$C$95)</f>
-        <v>187.236764802907</v>
+        <v>317.743781532949</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19020,7 +19073,7 @@
       </c>
       <c r="D72" s="73" t="n">
         <f aca="false">D69+D71</f>
-        <v>1477.34041780101</v>
+        <v>2392.1866676228</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19029,7 +19082,7 @@
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-2450.12300498313</v>
+        <v>-1372.56783818692</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19078,7 +19131,7 @@
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-2450.12300498313</v>
+        <v>-1372.56783818692</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19087,7 +19140,7 @@
       </c>
       <c r="D81" s="76" t="n">
         <f aca="false">(Assumptions!$C$119+Assumptions!$C$120)-D64</f>
-        <v>7450.12300498313</v>
+        <v>6372.56783818692</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19114,7 +19167,7 @@
       </c>
       <c r="D86" s="66" t="n">
         <f aca="false">G21</f>
-        <v>373.402856</v>
+        <v>454.979772</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19123,7 +19176,7 @@
       </c>
       <c r="D87" s="66" t="n">
         <f aca="false">AVERAGE(H21:J21)</f>
-        <v>441.842077333334</v>
+        <v>554.054756666667</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19151,15 +19204,15 @@
       </c>
       <c r="D90" s="79" t="n">
         <f aca="false">$D$86*D88</f>
-        <v>2987.222848</v>
+        <v>3639.838176</v>
       </c>
       <c r="E90" s="79" t="n">
         <f aca="false">$D$86*E88</f>
-        <v>4107.431416</v>
+        <v>5004.777492</v>
       </c>
       <c r="F90" s="79" t="n">
         <f aca="false">$D$86*F88</f>
-        <v>5227.639984</v>
+        <v>6369.716808</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19168,15 +19221,15 @@
       </c>
       <c r="D91" s="79" t="n">
         <f aca="false">$D$87*D88</f>
-        <v>3534.73661866667</v>
+        <v>4432.43805333333</v>
       </c>
       <c r="E91" s="79" t="n">
         <f aca="false">$D$87*E88</f>
-        <v>4860.26285066667</v>
+        <v>6094.60232333333</v>
       </c>
       <c r="F91" s="79" t="n">
         <f aca="false">$D$87*F88</f>
-        <v>6185.78908266667</v>
+        <v>7756.76659333334</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19185,7 +19238,7 @@
       </c>
       <c r="D92" s="76" t="n">
         <f aca="false">D62</f>
-        <v>3949.87699501687</v>
+        <v>5027.43216181308</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
model+deck: OT SOP '28H2 + 시나리오 필요EBITDA% 열 + AMPC 밸류 기여 별도표시
- OT SOP를 '28 하반기로 조정: ot_util_28 2028 .35→.18(반년)
  → run-rate $554mm·멀티플 불변, EV $5.0→$4.8bn, PV(AMPC) $3.8→$3.6bn
- S4 조달 시나리오 표에 '필요 EBITDA%(→13x)' 열 추가(민감도):
  10.7/9.8/9.8/9.1/8.7% (현 9% 대비 — 최대결합만 충족)
- S2에 AMPC 밸류 분해 박스 추가: DCF EV $4.8bn = ex-AMPC $1.2bn
  + AMPC PV $3.6bn(75%, 2033 소멸) → 멀티플엔 ex-AMPC만
- S2 OT SOP '28 하반기 표기, EV KPI 4.8
- CLAUDE.md·펀딩구조_v2 검산표(AMPC 분해)·역산표 동기화

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -10592,7 +10592,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1552.635</c:v>
+                  <c:v>798.498</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2539.7388</c:v>
@@ -10621,8 +10621,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="38457199"/>
-        <c:axId val="21383864"/>
+        <c:axId val="51287968"/>
+        <c:axId val="40349939"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -10731,10 +10731,10 @@
                   <c:v>-320.341084</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>576.5144851</c:v>
+                  <c:v>420.30394228</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1557.91114236</c:v>
+                  <c:v>1457.27910108</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1513.38719486</c:v>
@@ -10767,11 +10767,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="38457199"/>
-        <c:axId val="21383864"/>
+        <c:axId val="51287968"/>
+        <c:axId val="40349939"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="38457199"/>
+        <c:axId val="51287968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10803,7 +10803,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21383864"/>
+        <c:crossAx val="40349939"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10811,7 +10811,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21383864"/>
+        <c:axId val="40349939"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10853,7 +10853,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38457199"/>
+        <c:crossAx val="51287968"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12957,7 +12957,7 @@
         <v>0</v>
       </c>
       <c r="F60" s="20" t="n">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="G60" s="20" t="n">
         <v>0.58</v>
@@ -12998,7 +12998,7 @@
       </c>
       <c r="F61" s="37" t="n">
         <f aca="false">F59*F60*$C$6</f>
-        <v>4.725</v>
+        <v>2.43</v>
       </c>
       <c r="G61" s="37" t="n">
         <f aca="false">G59*G60*$C$6</f>
@@ -13078,7 +13078,7 @@
         <v>0</v>
       </c>
       <c r="F63" s="20" t="n">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="G63" s="20" t="n">
         <v>0.58</v>
@@ -13119,7 +13119,7 @@
       </c>
       <c r="F64" s="37" t="n">
         <f aca="false">F62*F63*$C$6</f>
-        <v>4.725</v>
+        <v>2.43</v>
       </c>
       <c r="G64" s="37" t="n">
         <f aca="false">G62*G63*$C$6</f>
@@ -13204,7 +13204,7 @@
         <v>0</v>
       </c>
       <c r="F67" s="20" t="n">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="G67" s="20" t="n">
         <v>0.58</v>
@@ -13245,7 +13245,7 @@
       </c>
       <c r="F68" s="37" t="n">
         <f aca="false">F66*F67*$C$6</f>
-        <v>0.945</v>
+        <v>0.486</v>
       </c>
       <c r="G68" s="37" t="n">
         <f aca="false">G66*G67*$C$6</f>
@@ -13293,7 +13293,7 @@
       </c>
       <c r="F69" s="37" t="n">
         <f aca="false">F61+F64</f>
-        <v>9.45</v>
+        <v>4.86</v>
       </c>
       <c r="G69" s="37" t="n">
         <f aca="false">G61+G64</f>
@@ -13341,7 +13341,7 @@
       </c>
       <c r="F70" s="37" t="n">
         <f aca="false">F68</f>
-        <v>0.945</v>
+        <v>0.486</v>
       </c>
       <c r="G70" s="37" t="n">
         <f aca="false">G68</f>
@@ -15646,7 +15646,7 @@
       </c>
       <c r="F6" s="60" t="n">
         <f aca="false">Assumptions!F69*Assumptions!F72</f>
-        <v>1406.16</v>
+        <v>723.168</v>
       </c>
       <c r="G6" s="60" t="n">
         <f aca="false">Assumptions!G69*Assumptions!G72</f>
@@ -15691,7 +15691,7 @@
       </c>
       <c r="F7" s="60" t="n">
         <f aca="false">Assumptions!F70*Assumptions!F75</f>
-        <v>146.475</v>
+        <v>75.33</v>
       </c>
       <c r="G7" s="60" t="n">
         <f aca="false">Assumptions!G70*Assumptions!G75</f>
@@ -15736,7 +15736,7 @@
       </c>
       <c r="F8" s="56" t="n">
         <f aca="false">F6+F7</f>
-        <v>1552.635</v>
+        <v>798.498</v>
       </c>
       <c r="G8" s="56" t="n">
         <f aca="false">G6+G7</f>
@@ -15781,7 +15781,7 @@
       </c>
       <c r="F9" s="38" t="n">
         <f aca="false">-(Assumptions!F69*Assumptions!F74+Assumptions!F70*Assumptions!F77)</f>
-        <v>-1319.73975</v>
+        <v>-678.7233</v>
       </c>
       <c r="G9" s="38" t="n">
         <f aca="false">-(Assumptions!G69*Assumptions!G74+Assumptions!G70*Assumptions!G77)</f>
@@ -15878,7 +15878,7 @@
       </c>
       <c r="F12" s="56" t="n">
         <f aca="false">F8+F9</f>
-        <v>232.89525</v>
+        <v>119.7747</v>
       </c>
       <c r="G12" s="56" t="n">
         <f aca="false">G8+G9</f>
@@ -15923,7 +15923,7 @@
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$81</f>
-        <v>-93.1581</v>
+        <v>-47.90988</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$81</f>
@@ -16058,7 +16058,7 @@
       </c>
       <c r="F16" s="56" t="n">
         <f aca="false">F12+F13+F15</f>
-        <v>73.0371499999999</v>
+        <v>5.16482000000008</v>
       </c>
       <c r="G16" s="56" t="n">
         <f aca="false">G12+G13+G15</f>
@@ -16103,7 +16103,7 @@
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.0470407726220264</v>
+        <v>0.0064681689872737</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
@@ -16148,7 +16148,7 @@
       </c>
       <c r="F18" s="38" t="n">
         <f aca="false">(Assumptions!F69+Assumptions!F70)*Assumptions!F8</f>
-        <v>467.775</v>
+        <v>240.57</v>
       </c>
       <c r="G18" s="38" t="n">
         <f aca="false">(Assumptions!G69+Assumptions!G70)*Assumptions!G8</f>
@@ -16193,7 +16193,7 @@
       </c>
       <c r="F19" s="56" t="n">
         <f aca="false">F16+F18</f>
-        <v>540.81215</v>
+        <v>245.73482</v>
       </c>
       <c r="G19" s="56" t="n">
         <f aca="false">G16+G18</f>
@@ -16290,7 +16290,7 @@
       </c>
       <c r="F23" s="38" t="n">
         <f aca="false">MAX(0,F16)</f>
-        <v>73.0371499999999</v>
+        <v>5.16482000000008</v>
       </c>
       <c r="G23" s="38" t="n">
         <f aca="false">MAX(0,G16)</f>
@@ -16339,7 +16339,7 @@
       </c>
       <c r="G24" s="38" t="n">
         <f aca="false">F27</f>
-        <v>1.60028000000011</v>
+        <v>55.8981439999999</v>
       </c>
       <c r="H24" s="38" t="n">
         <f aca="false">G27</f>
@@ -16380,11 +16380,11 @@
       </c>
       <c r="F25" s="38" t="n">
         <f aca="false">MIN(F24,F23*Assumptions!$C$90)</f>
-        <v>58.4297199999999</v>
+        <v>4.13185600000006</v>
       </c>
       <c r="G25" s="38" t="n">
         <f aca="false">MIN(G24,G23*Assumptions!$C$90)</f>
-        <v>1.60028000000011</v>
+        <v>55.8981439999999</v>
       </c>
       <c r="H25" s="38" t="n">
         <f aca="false">MIN(H24,H23*Assumptions!$C$90)</f>
@@ -16470,7 +16470,7 @@
       </c>
       <c r="F27" s="38" t="n">
         <f aca="false">F24-F25+F26</f>
-        <v>1.60028000000011</v>
+        <v>55.8981439999999</v>
       </c>
       <c r="G27" s="38" t="n">
         <f aca="false">G24-G25+G26</f>
@@ -16515,11 +16515,11 @@
       </c>
       <c r="F28" s="38" t="n">
         <f aca="false">F23-F25</f>
-        <v>14.60743</v>
+        <v>1.03296400000001</v>
       </c>
       <c r="G28" s="38" t="n">
         <f aca="false">G23-G25</f>
-        <v>160.276212</v>
+        <v>105.978348</v>
       </c>
       <c r="H28" s="38" t="n">
         <f aca="false">H23-H25</f>
@@ -16560,11 +16560,11 @@
       </c>
       <c r="F29" s="38" t="n">
         <f aca="false">-F28*Assumptions!$C$87</f>
-        <v>-3.35970889999999</v>
+        <v>-0.237581720000003</v>
       </c>
       <c r="G29" s="38" t="n">
         <f aca="false">-G28*Assumptions!$C$87</f>
-        <v>-36.8635287599999</v>
+        <v>-24.37502004</v>
       </c>
       <c r="H29" s="38" t="n">
         <f aca="false">-H28*Assumptions!$C$87</f>
@@ -16605,11 +16605,11 @@
       </c>
       <c r="F30" s="56" t="n">
         <f aca="false">F19+F29</f>
-        <v>537.4524411</v>
+        <v>245.49723828</v>
       </c>
       <c r="G30" s="56" t="n">
         <f aca="false">G19+G29</f>
-        <v>900.18296324</v>
+        <v>912.67147196</v>
       </c>
       <c r="H30" s="56" t="n">
         <f aca="false">H19+H29</f>
@@ -16695,7 +16695,7 @@
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">-F8*Assumptions!$C$83</f>
-        <v>-46.57905</v>
+        <v>-23.95494</v>
       </c>
       <c r="G32" s="38" t="n">
         <f aca="false">-G8*Assumptions!$C$83</f>
@@ -16830,7 +16830,7 @@
       </c>
       <c r="F35" s="38" t="n">
         <f aca="false">F8*Assumptions!$C$86</f>
-        <v>232.89525</v>
+        <v>119.7747</v>
       </c>
       <c r="G35" s="38" t="n">
         <f aca="false">G8*Assumptions!$C$86</f>
@@ -16875,11 +16875,11 @@
       </c>
       <c r="F36" s="38" t="n">
         <f aca="false">-(F35-E35)</f>
-        <v>-232.89525</v>
+        <v>-119.7747</v>
       </c>
       <c r="G36" s="38" t="n">
         <f aca="false">-(G35-F35)</f>
-        <v>-148.06557</v>
+        <v>-261.18612</v>
       </c>
       <c r="H36" s="38" t="n">
         <f aca="false">-(H35-G35)</f>
@@ -16920,11 +16920,11 @@
       </c>
       <c r="F37" s="59" t="n">
         <f aca="false">F30+F31+F32+F33+F34+F36</f>
-        <v>54.6781411</v>
+        <v>-101.53240172</v>
       </c>
       <c r="G37" s="59" t="n">
         <f aca="false">G30+G31+G32+G33+G34+G36</f>
-        <v>742.62522924</v>
+        <v>641.99318796</v>
       </c>
       <c r="H37" s="59" t="n">
         <f aca="false">H30+H31+H32+H33+H34+H36</f>
@@ -17097,7 +17097,7 @@
       </c>
       <c r="F7" s="64" t="n">
         <f aca="false">SKOT!F8</f>
-        <v>1552.635</v>
+        <v>798.498</v>
       </c>
       <c r="G7" s="64" t="n">
         <f aca="false">SKOT!G8</f>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="F8" s="56" t="n">
         <f aca="false">F6+F7</f>
-        <v>3639.245</v>
+        <v>2885.108</v>
       </c>
       <c r="G8" s="56" t="n">
         <f aca="false">G6+G7</f>
@@ -17187,7 +17187,7 @@
       </c>
       <c r="F9" s="54" t="n">
         <f aca="false">SKBA!F6+Assumptions!F69+Assumptions!F70</f>
-        <v>23.857</v>
+        <v>18.808</v>
       </c>
       <c r="G9" s="54" t="n">
         <f aca="false">SKBA!G6+Assumptions!G69+Assumptions!G70</f>
@@ -17284,7 +17284,7 @@
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">SKBA!F17+SKOT!F16</f>
-        <v>245.02315</v>
+        <v>177.15082</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">SKBA!G17+SKOT!G16</f>
@@ -17329,7 +17329,7 @@
       </c>
       <c r="F14" s="57" t="n">
         <f aca="false">IF(F8=0,0,F13/F8)</f>
-        <v>0.0673280172123613</v>
+        <v>0.0614017984768681</v>
       </c>
       <c r="G14" s="57" t="n">
         <f aca="false">IF(G8=0,0,G13/G8)</f>
@@ -17374,7 +17374,7 @@
       </c>
       <c r="F15" s="38" t="n">
         <f aca="false">SKBA!F19+SKOT!F18</f>
-        <v>1073.565</v>
+        <v>846.36</v>
       </c>
       <c r="G15" s="38" t="n">
         <f aca="false">SKBA!G19+SKOT!G18</f>
@@ -17419,7 +17419,7 @@
       </c>
       <c r="F16" s="56" t="n">
         <f aca="false">SKBA!F20+SKOT!F19</f>
-        <v>1318.58815</v>
+        <v>1023.51082</v>
       </c>
       <c r="G16" s="56" t="n">
         <f aca="false">SKBA!G20+SKOT!G19</f>
@@ -17464,7 +17464,7 @@
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.362324644260004</v>
+        <v>0.354756501316415</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
@@ -17554,7 +17554,7 @@
       </c>
       <c r="F19" s="56" t="n">
         <f aca="false">F16+F18</f>
-        <v>1413.30215</v>
+        <v>1118.22482</v>
       </c>
       <c r="G19" s="56" t="n">
         <f aca="false">G16+G18</f>
@@ -17599,7 +17599,7 @@
       </c>
       <c r="F20" s="57" t="n">
         <f aca="false">IF(F8=0,0,F19/F8)</f>
-        <v>0.388350372123888</v>
+        <v>0.387585081736975</v>
       </c>
       <c r="G20" s="57" t="n">
         <f aca="false">IF(G8=0,0,G19/G8)</f>
@@ -17644,7 +17644,7 @@
       </c>
       <c r="F21" s="39" t="n">
         <f aca="false">F19-F15</f>
-        <v>339.73715</v>
+        <v>271.86482</v>
       </c>
       <c r="G21" s="39" t="n">
         <f aca="false">G19-G15</f>
@@ -17689,7 +17689,7 @@
       </c>
       <c r="F22" s="57" t="n">
         <f aca="false">IF(F8=0,0,F21/F8)</f>
-        <v>0.0933537450762451</v>
+        <v>0.0942303788974278</v>
       </c>
       <c r="G22" s="57" t="n">
         <f aca="false">IF(G8=0,0,G21/G8)</f>
@@ -17831,11 +17831,11 @@
       </c>
       <c r="F27" s="66" t="n">
         <f aca="false">SKOT!F37</f>
-        <v>54.6781411</v>
+        <v>-101.53240172</v>
       </c>
       <c r="G27" s="66" t="n">
         <f aca="false">SKOT!G37</f>
-        <v>742.62522924</v>
+        <v>641.99318796</v>
       </c>
       <c r="H27" s="66" t="n">
         <f aca="false">SKOT!H37</f>
@@ -17876,11 +17876,11 @@
       </c>
       <c r="F28" s="59" t="n">
         <f aca="false">F26+F27</f>
-        <v>576.5144851</v>
+        <v>420.30394228</v>
       </c>
       <c r="G28" s="59" t="n">
         <f aca="false">G26+G27</f>
-        <v>1557.91114236</v>
+        <v>1457.27910108</v>
       </c>
       <c r="H28" s="59" t="n">
         <f aca="false">H26+H27</f>
@@ -18468,11 +18468,11 @@
       </c>
       <c r="F43" s="56" t="n">
         <f aca="false">F27+F36+F37+F41+F40+F42</f>
-        <v>-99.3218589000001</v>
+        <v>-255.53240172</v>
       </c>
       <c r="G43" s="56" t="n">
         <f aca="false">G27+G36+G37+G41+G40+G42</f>
-        <v>588.62522924</v>
+        <v>487.99318796</v>
       </c>
       <c r="H43" s="56" t="n">
         <f aca="false">H27+H36+H37+H41+H40+H42</f>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="F44" s="66" t="n">
         <f aca="false">SKOT!F19-SKOT!F15+SKOT!F32</f>
-        <v>560.9331</v>
+        <v>288.47988</v>
       </c>
       <c r="G44" s="66" t="n">
         <f aca="false">SKOT!G19-SKOT!G15+SKOT!G32</f>
@@ -18603,7 +18603,7 @@
       </c>
       <c r="F46" s="67" t="n">
         <f aca="false">IF(F45=0,0,F44/F45)</f>
-        <v>2.8046655</v>
+        <v>1.4423994</v>
       </c>
       <c r="G46" s="67" t="n">
         <f aca="false">IF(G45=0,0,G44/G45)</f>
@@ -18648,11 +18648,11 @@
       </c>
       <c r="F47" s="59" t="n">
         <f aca="false">F35+F43</f>
-        <v>379.8718851</v>
+        <v>223.66134228</v>
       </c>
       <c r="G47" s="59" t="n">
         <f aca="false">G35+G43</f>
-        <v>1361.26854236</v>
+        <v>1260.63650108</v>
       </c>
       <c r="H47" s="59" t="n">
         <f aca="false">H35+H43</f>
@@ -18738,11 +18738,11 @@
       </c>
       <c r="F49" s="39" t="n">
         <f aca="false">F47*F48</f>
-        <v>279.860137540752</v>
+        <v>164.776327146591</v>
       </c>
       <c r="G49" s="39" t="n">
         <f aca="false">G47*G48</f>
-        <v>887.501828108433</v>
+        <v>821.893083159808</v>
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">H47*H48</f>
@@ -18930,11 +18930,11 @@
       </c>
       <c r="F56" s="39" t="n">
         <f aca="false">F28*F55</f>
-        <v>449.163573619744</v>
+        <v>327.459631284382</v>
       </c>
       <c r="G56" s="39" t="n">
         <f aca="false">G28*G55</f>
-        <v>1098.43587961486</v>
+        <v>1027.48328047407</v>
       </c>
       <c r="H56" s="39" t="n">
         <f aca="false">H28*H55</f>
@@ -18975,7 +18975,7 @@
       </c>
       <c r="D59" s="38" t="n">
         <f aca="false">SUM(D56:M56)</f>
-        <v>3604.91887852169</v>
+        <v>3412.26233704554</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19002,7 +19002,7 @@
       </c>
       <c r="D62" s="73" t="n">
         <f aca="false">D59+D61</f>
-        <v>5027.43216181308</v>
+        <v>4834.77562033693</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19020,7 +19020,7 @@
       </c>
       <c r="D64" s="74" t="n">
         <f aca="false">D62-Assumptions!$C$94</f>
-        <v>-1372.56783818692</v>
+        <v>-1565.22437966307</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19029,7 +19029,7 @@
       </c>
       <c r="D66" s="75" t="n">
         <f aca="false">D61/D62</f>
-        <v>0.282950269144632</v>
+        <v>0.294225295028739</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19046,7 +19046,7 @@
       </c>
       <c r="D69" s="38" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>2074.44288608985</v>
+        <v>1893.75033074706</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19073,7 +19073,7 @@
       </c>
       <c r="D72" s="73" t="n">
         <f aca="false">D69+D71</f>
-        <v>2392.1866676228</v>
+        <v>2211.49411228001</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19082,7 +19082,7 @@
       </c>
       <c r="D73" s="76" t="n">
         <f aca="false">D64</f>
-        <v>-1372.56783818692</v>
+        <v>-1565.22437966307</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19131,7 +19131,7 @@
       </c>
       <c r="D80" s="79" t="n">
         <f aca="false">D64</f>
-        <v>-1372.56783818692</v>
+        <v>-1565.22437966307</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="D81" s="76" t="n">
         <f aca="false">(Assumptions!$C$119+Assumptions!$C$120)-D64</f>
-        <v>6372.56783818692</v>
+        <v>6565.22437966307</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19238,7 +19238,7 @@
       </c>
       <c r="D92" s="76" t="n">
         <f aca="false">D62</f>
-        <v>5027.43216181308</v>
+        <v>4834.77562033693</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
BA 개조 규모 11 → 18 GWh (개조비 $1.4bn 유지)
- BA 4라인 2.75×4 → 4.5×4 = 18.0 GWh, 개조 capex $0.4bn 그대로
- run-rate ex-AMPC EBITDA $438→$518mm (BA 205 + OT 313)
- EV $3.5→$4.4bn · AMPC PV $3.3bn(76%) · ex-AMPC EV $1.1bn · FCFE +$1.9bn
- 역산 필요 BASE 16.5x → 최대결합 13.5x (2029E 20.3~16.6x)
  최대결합(13.5x)만 정상화 peer(13~15x) 하단 진입, BASE는 초과
  필요EBITDA%(→13x) 11.4~9.3% · DCF 내재 8.5x(run)/10.5x(2029E)
- 덱 S2/S4/S5 전 수치·peer 밴드바·결론 갱신 · Multiples 자동 · 문서 동기화

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -1909,7 +1909,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2.75×4 = 11 GWh </t>
+      <t xml:space="preserve">4.5×4 = 18 GWh </t>
     </r>
     <r>
       <rPr>
@@ -2068,7 +2068,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2.75GW · </t>
+      <t xml:space="preserve">4.5GW · </t>
     </r>
     <r>
       <rPr>
@@ -2273,7 +2273,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· 2.75×2)</t>
+      <t xml:space="preserve">· 4.5×2)</t>
     </r>
   </si>
   <si>
@@ -12985,31 +12985,31 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>468.875</c:v>
+                  <c:v>767.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1082.675</c:v>
+                  <c:v>1771.65</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1295.91</c:v>
+                  <c:v>2120.58</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1395.24</c:v>
+                  <c:v>2283.12</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1393.15</c:v>
+                  <c:v>2279.7</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1374.45</c:v>
+                  <c:v>2249.1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1355.75</c:v>
+                  <c:v>2218.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1337.05</c:v>
+                  <c:v>2187.9</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1318.35</c:v>
+                  <c:v>2157.3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13147,8 +13147,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="33283378"/>
-        <c:axId val="99552927"/>
+        <c:axId val="16082118"/>
+        <c:axId val="10905176"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -13258,31 +13258,31 @@
                   <c:v>-168.58636</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-368.306584</c:v>
+                  <c:v>-335.389084</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>244.33099228</c:v>
+                  <c:v>365.09674228</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1065.63890556</c:v>
+                  <c:v>1334.41158876</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1165.6162793</c:v>
+                  <c:v>1404.2825939</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>958.0774169</c:v>
+                  <c:v>1141.6745999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>633.2427827</c:v>
+                  <c:v>750.8232317</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>241.0923485</c:v>
+                  <c:v>291.0705635</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>238.1356643</c:v>
+                  <c:v>287.4491453</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>235.1789801</c:v>
+                  <c:v>283.8277271</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13297,11 +13297,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="33283378"/>
-        <c:axId val="99552927"/>
+        <c:axId val="16082118"/>
+        <c:axId val="10905176"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="33283378"/>
+        <c:axId val="16082118"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13333,7 +13333,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99552927"/>
+        <c:crossAx val="10905176"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13341,7 +13341,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="99552927"/>
+        <c:axId val="10905176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13383,7 +13383,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33283378"/>
+        <c:crossAx val="16082118"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14413,31 +14413,31 @@
         <v>0</v>
       </c>
       <c r="E30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="F30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="G30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="H30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="I30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="J30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="K30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="L30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="M30" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14488,39 +14488,39 @@
       </c>
       <c r="E32" s="38" t="n">
         <f aca="false">E30*E31*$C$6</f>
-        <v>1.5125</v>
+        <v>2.475</v>
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">F30*F31*$C$6</f>
-        <v>1.98</v>
+        <v>3.24</v>
       </c>
       <c r="G32" s="38" t="n">
         <f aca="false">G30*G31*$C$6</f>
-        <v>2.255</v>
+        <v>3.69</v>
       </c>
       <c r="H32" s="38" t="n">
         <f aca="false">H30*H31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="I32" s="38" t="n">
         <f aca="false">I30*I31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="J32" s="38" t="n">
         <f aca="false">J30*J31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="K32" s="38" t="n">
         <f aca="false">K30*K31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="L32" s="38" t="n">
         <f aca="false">L30*L31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="M32" s="38" t="n">
         <f aca="false">M30*M31*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14534,31 +14534,31 @@
         <v>0</v>
       </c>
       <c r="E33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="F33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="G33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="H33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="I33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="J33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="K33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="L33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="M33" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14609,39 +14609,39 @@
       </c>
       <c r="E35" s="38" t="n">
         <f aca="false">E33*E34*$C$6</f>
-        <v>1.5125</v>
+        <v>2.475</v>
       </c>
       <c r="F35" s="38" t="n">
         <f aca="false">F33*F34*$C$6</f>
-        <v>1.98</v>
+        <v>3.24</v>
       </c>
       <c r="G35" s="38" t="n">
         <f aca="false">G33*G34*$C$6</f>
-        <v>2.255</v>
+        <v>3.69</v>
       </c>
       <c r="H35" s="38" t="n">
         <f aca="false">H33*H34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="I35" s="38" t="n">
         <f aca="false">I33*I34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="J35" s="38" t="n">
         <f aca="false">J33*J34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="K35" s="38" t="n">
         <f aca="false">K33*K34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="L35" s="38" t="n">
         <f aca="false">L33*L34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="M35" s="38" t="n">
         <f aca="false">M33*M34*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14663,28 +14663,28 @@
         <v>0</v>
       </c>
       <c r="F37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="G37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="H37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="I37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="J37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="K37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="L37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="M37" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14739,35 +14739,35 @@
       </c>
       <c r="F39" s="38" t="n">
         <f aca="false">F37*F38*$C$6</f>
-        <v>1.5125</v>
+        <v>2.475</v>
       </c>
       <c r="G39" s="38" t="n">
         <f aca="false">G37*G38*$C$6</f>
-        <v>1.98</v>
+        <v>3.24</v>
       </c>
       <c r="H39" s="38" t="n">
         <f aca="false">H37*H38*$C$6</f>
-        <v>2.2825</v>
+        <v>3.735</v>
       </c>
       <c r="I39" s="38" t="n">
         <f aca="false">I37*I38*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="J39" s="38" t="n">
         <f aca="false">J37*J38*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="K39" s="38" t="n">
         <f aca="false">K37*K38*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="L39" s="38" t="n">
         <f aca="false">L37*L38*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="M39" s="38" t="n">
         <f aca="false">M37*M38*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14784,28 +14784,28 @@
         <v>0</v>
       </c>
       <c r="F40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="G40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="H40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="I40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="J40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="K40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="L40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
       <c r="M40" s="37" t="n">
-        <v>2.75</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14860,35 +14860,35 @@
       </c>
       <c r="F42" s="38" t="n">
         <f aca="false">F40*F41*$C$6</f>
-        <v>1.5125</v>
+        <v>2.475</v>
       </c>
       <c r="G42" s="38" t="n">
         <f aca="false">G40*G41*$C$6</f>
-        <v>1.98</v>
+        <v>3.24</v>
       </c>
       <c r="H42" s="38" t="n">
         <f aca="false">H40*H41*$C$6</f>
-        <v>2.2825</v>
+        <v>3.735</v>
       </c>
       <c r="I42" s="38" t="n">
         <f aca="false">I40*I41*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="J42" s="38" t="n">
         <f aca="false">J40*J41*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="K42" s="38" t="n">
         <f aca="false">K40*K41*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="L42" s="38" t="n">
         <f aca="false">L40*L41*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
       <c r="M42" s="38" t="n">
         <f aca="false">M40*M41*$C$6</f>
-        <v>2.3375</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14904,39 +14904,39 @@
       </c>
       <c r="E43" s="38" t="n">
         <f aca="false">E32+E35</f>
-        <v>3.025</v>
+        <v>4.95</v>
       </c>
       <c r="F43" s="38" t="n">
         <f aca="false">F32+F35</f>
-        <v>3.96</v>
+        <v>6.48</v>
       </c>
       <c r="G43" s="38" t="n">
         <f aca="false">G32+G35</f>
-        <v>4.51</v>
+        <v>7.38</v>
       </c>
       <c r="H43" s="38" t="n">
         <f aca="false">H32+H35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="I43" s="38" t="n">
         <f aca="false">I32+I35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="J43" s="38" t="n">
         <f aca="false">J32+J35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="K43" s="38" t="n">
         <f aca="false">K32+K35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="L43" s="38" t="n">
         <f aca="false">L32+L35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="M43" s="38" t="n">
         <f aca="false">M32+M35</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14956,35 +14956,35 @@
       </c>
       <c r="F44" s="38" t="n">
         <f aca="false">F39+F42</f>
-        <v>3.025</v>
+        <v>4.95</v>
       </c>
       <c r="G44" s="38" t="n">
         <f aca="false">G39+G42</f>
-        <v>3.96</v>
+        <v>6.48</v>
       </c>
       <c r="H44" s="38" t="n">
         <f aca="false">H39+H42</f>
-        <v>4.565</v>
+        <v>7.47</v>
       </c>
       <c r="I44" s="38" t="n">
         <f aca="false">I39+I42</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="J44" s="38" t="n">
         <f aca="false">J39+J42</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="K44" s="38" t="n">
         <f aca="false">K39+K42</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="L44" s="38" t="n">
         <f aca="false">L39+L42</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
       <c r="M44" s="38" t="n">
         <f aca="false">M39+M42</f>
-        <v>4.675</v>
+        <v>7.65</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15000,39 +15000,39 @@
       </c>
       <c r="E45" s="38" t="n">
         <f aca="false">E43+E44</f>
-        <v>3.025</v>
+        <v>4.95</v>
       </c>
       <c r="F45" s="38" t="n">
         <f aca="false">F43+F44</f>
-        <v>6.985</v>
+        <v>11.43</v>
       </c>
       <c r="G45" s="38" t="n">
         <f aca="false">G43+G44</f>
-        <v>8.47</v>
+        <v>13.86</v>
       </c>
       <c r="H45" s="38" t="n">
         <f aca="false">H43+H44</f>
-        <v>9.24</v>
+        <v>15.12</v>
       </c>
       <c r="I45" s="38" t="n">
         <f aca="false">I43+I44</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="J45" s="38" t="n">
         <f aca="false">J43+J44</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="K45" s="38" t="n">
         <f aca="false">K43+K44</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="L45" s="38" t="n">
         <f aca="false">L43+L44</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="M45" s="38" t="n">
         <f aca="false">M43+M44</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16721,39 +16721,39 @@
       </c>
       <c r="E6" s="55" t="n">
         <f aca="false">Assumptions!E45</f>
-        <v>3.025</v>
+        <v>4.95</v>
       </c>
       <c r="F6" s="55" t="n">
         <f aca="false">Assumptions!F45</f>
-        <v>6.985</v>
+        <v>11.43</v>
       </c>
       <c r="G6" s="55" t="n">
         <f aca="false">Assumptions!G45</f>
-        <v>8.47</v>
+        <v>13.86</v>
       </c>
       <c r="H6" s="55" t="n">
         <f aca="false">Assumptions!H45</f>
-        <v>9.24</v>
+        <v>15.12</v>
       </c>
       <c r="I6" s="55" t="n">
         <f aca="false">Assumptions!I45</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="J6" s="55" t="n">
         <f aca="false">Assumptions!J45</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="K6" s="55" t="n">
         <f aca="false">Assumptions!K45</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="L6" s="55" t="n">
         <f aca="false">Assumptions!L45</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
       <c r="M6" s="55" t="n">
         <f aca="false">Assumptions!M45</f>
-        <v>9.35</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16811,39 +16811,39 @@
       </c>
       <c r="E8" s="57" t="n">
         <f aca="false">E6*E7</f>
-        <v>468.875</v>
+        <v>767.25</v>
       </c>
       <c r="F8" s="57" t="n">
         <f aca="false">F6*F7</f>
-        <v>1082.675</v>
+        <v>1771.65</v>
       </c>
       <c r="G8" s="57" t="n">
         <f aca="false">G6*G7</f>
-        <v>1295.91</v>
+        <v>2120.58</v>
       </c>
       <c r="H8" s="57" t="n">
         <f aca="false">H6*H7</f>
-        <v>1395.24</v>
+        <v>2283.12</v>
       </c>
       <c r="I8" s="57" t="n">
         <f aca="false">I6*I7</f>
-        <v>1393.15</v>
+        <v>2279.7</v>
       </c>
       <c r="J8" s="57" t="n">
         <f aca="false">J6*J7</f>
-        <v>1374.45</v>
+        <v>2249.1</v>
       </c>
       <c r="K8" s="57" t="n">
         <f aca="false">K6*K7</f>
-        <v>1355.75</v>
+        <v>2218.5</v>
       </c>
       <c r="L8" s="57" t="n">
         <f aca="false">L6*L7</f>
-        <v>1337.05</v>
+        <v>2187.9</v>
       </c>
       <c r="M8" s="57" t="n">
         <f aca="false">M6*M7</f>
-        <v>1318.35</v>
+        <v>2157.3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16856,39 +16856,39 @@
       </c>
       <c r="E9" s="39" t="n">
         <f aca="false">-(Assumptions!E43*Assumptions!E49+Assumptions!E44*Assumptions!E50)</f>
-        <v>-393.855</v>
+        <v>-644.49</v>
       </c>
       <c r="F9" s="39" t="n">
         <f aca="false">-(Assumptions!F43*Assumptions!F49+Assumptions!F44*Assumptions!F50)</f>
-        <v>-918.8245</v>
+        <v>-1503.531</v>
       </c>
       <c r="G9" s="39" t="n">
         <f aca="false">-(Assumptions!G43*Assumptions!G49+Assumptions!G44*Assumptions!G50)</f>
-        <v>-1100.682</v>
+        <v>-1801.116</v>
       </c>
       <c r="H9" s="39" t="n">
         <f aca="false">-(Assumptions!H43*Assumptions!H49+Assumptions!H44*Assumptions!H50)</f>
-        <v>-1185.7879</v>
+        <v>-1940.3802</v>
       </c>
       <c r="I9" s="39" t="n">
         <f aca="false">-(Assumptions!I43*Assumptions!I49+Assumptions!I44*Assumptions!I50)</f>
-        <v>-1184.1775</v>
+        <v>-1937.745</v>
       </c>
       <c r="J9" s="39" t="n">
         <f aca="false">-(Assumptions!J43*Assumptions!J49+Assumptions!J44*Assumptions!J50)</f>
-        <v>-1168.2825</v>
+        <v>-1911.735</v>
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">-(Assumptions!K43*Assumptions!K49+Assumptions!K44*Assumptions!K50)</f>
-        <v>-1152.3875</v>
+        <v>-1885.725</v>
       </c>
       <c r="L9" s="39" t="n">
         <f aca="false">-(Assumptions!L43*Assumptions!L49+Assumptions!L44*Assumptions!L50)</f>
-        <v>-1136.4925</v>
+        <v>-1859.715</v>
       </c>
       <c r="M9" s="39" t="n">
         <f aca="false">-(Assumptions!M43*Assumptions!M49+Assumptions!M44*Assumptions!M50)</f>
-        <v>-1120.5975</v>
+        <v>-1833.705</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16953,39 +16953,39 @@
       </c>
       <c r="E12" s="57" t="n">
         <f aca="false">E8+E9</f>
-        <v>75.02</v>
+        <v>122.76</v>
       </c>
       <c r="F12" s="57" t="n">
         <f aca="false">F8+F9</f>
-        <v>163.8505</v>
+        <v>268.119</v>
       </c>
       <c r="G12" s="57" t="n">
         <f aca="false">G8+G9</f>
-        <v>195.228</v>
+        <v>319.464</v>
       </c>
       <c r="H12" s="57" t="n">
         <f aca="false">H8+H9</f>
-        <v>209.4521</v>
+        <v>342.7398</v>
       </c>
       <c r="I12" s="57" t="n">
         <f aca="false">I8+I9</f>
-        <v>208.9725</v>
+        <v>341.955</v>
       </c>
       <c r="J12" s="57" t="n">
         <f aca="false">J8+J9</f>
-        <v>206.1675</v>
+        <v>337.365</v>
       </c>
       <c r="K12" s="57" t="n">
         <f aca="false">K8+K9</f>
-        <v>203.3625</v>
+        <v>332.775</v>
       </c>
       <c r="L12" s="57" t="n">
         <f aca="false">L8+L9</f>
-        <v>200.5575</v>
+        <v>328.185</v>
       </c>
       <c r="M12" s="57" t="n">
         <f aca="false">M8+M9</f>
-        <v>197.7525</v>
+        <v>323.595</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16998,39 +16998,39 @@
       </c>
       <c r="E13" s="39" t="n">
         <f aca="false">-E8*Assumptions!$C$81</f>
-        <v>-28.1325</v>
+        <v>-46.035</v>
       </c>
       <c r="F13" s="39" t="n">
         <f aca="false">-F8*Assumptions!$C$81</f>
-        <v>-64.9605</v>
+        <v>-106.299</v>
       </c>
       <c r="G13" s="39" t="n">
         <f aca="false">-G8*Assumptions!$C$81</f>
-        <v>-77.7546</v>
+        <v>-127.2348</v>
       </c>
       <c r="H13" s="39" t="n">
         <f aca="false">-H8*Assumptions!$C$81</f>
-        <v>-83.7144</v>
+        <v>-136.9872</v>
       </c>
       <c r="I13" s="39" t="n">
         <f aca="false">-I8*Assumptions!$C$81</f>
-        <v>-83.589</v>
+        <v>-136.782</v>
       </c>
       <c r="J13" s="39" t="n">
         <f aca="false">-J8*Assumptions!$C$81</f>
-        <v>-82.467</v>
+        <v>-134.946</v>
       </c>
       <c r="K13" s="39" t="n">
         <f aca="false">-K8*Assumptions!$C$81</f>
-        <v>-81.345</v>
+        <v>-133.11</v>
       </c>
       <c r="L13" s="39" t="n">
         <f aca="false">-L8*Assumptions!$C$81</f>
-        <v>-80.223</v>
+        <v>-131.274</v>
       </c>
       <c r="M13" s="39" t="n">
         <f aca="false">-M8*Assumptions!$C$81</f>
-        <v>-79.101</v>
+        <v>-129.438</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17133,11 +17133,11 @@
       </c>
       <c r="E16" s="39" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(E12+E13))</f>
-        <v>153.1125</v>
+        <v>123.275</v>
       </c>
       <c r="F16" s="39" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(F12+F13))</f>
-        <v>101.11</v>
+        <v>38.1800000000001</v>
       </c>
       <c r="G16" s="39" t="n">
         <f aca="false">0</f>
@@ -17186,31 +17186,31 @@
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">G12+G13+G15+G16</f>
-        <v>89.4594000000001</v>
+        <v>164.2152</v>
       </c>
       <c r="H17" s="57" t="n">
         <f aca="false">H12+H13+H15+H16</f>
-        <v>97.7237</v>
+        <v>177.7386</v>
       </c>
       <c r="I17" s="57" t="n">
         <f aca="false">I12+I13+I15+I16</f>
-        <v>97.3695000000001</v>
+        <v>177.159</v>
       </c>
       <c r="J17" s="57" t="n">
         <f aca="false">J12+J13+J15+J16</f>
-        <v>95.6865000000003</v>
+        <v>174.405</v>
       </c>
       <c r="K17" s="57" t="n">
         <f aca="false">K12+K13+K15+K16</f>
-        <v>94.0035000000002</v>
+        <v>171.651</v>
       </c>
       <c r="L17" s="57" t="n">
         <f aca="false">L12+L13+L15+L16</f>
-        <v>92.3205000000001</v>
+        <v>168.897</v>
       </c>
       <c r="M17" s="57" t="n">
         <f aca="false">M12+M13+M15+M16</f>
-        <v>90.6375000000001</v>
+        <v>166.143</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17223,39 +17223,39 @@
       </c>
       <c r="E18" s="58" t="n">
         <f aca="false">IF(E8=0,0,E17/E8)</f>
-        <v>0.372495867768595</v>
+        <v>0.227636363636364</v>
       </c>
       <c r="F18" s="58" t="n">
         <f aca="false">IF(F8=0,0,F17/F8)</f>
-        <v>0.158852841342046</v>
+        <v>0.097076736375695</v>
       </c>
       <c r="G18" s="58" t="n">
         <f aca="false">IF(G8=0,0,G17/G8)</f>
-        <v>0.0690321087112532</v>
+        <v>0.0774388139094023</v>
       </c>
       <c r="H18" s="58" t="n">
         <f aca="false">IF(H8=0,0,H17/H8)</f>
-        <v>0.0700407815142915</v>
+        <v>0.0778489961105856</v>
       </c>
       <c r="I18" s="58" t="n">
         <f aca="false">IF(I8=0,0,I17/I8)</f>
-        <v>0.0698916125327496</v>
+        <v>0.0777115409922358</v>
       </c>
       <c r="J18" s="58" t="n">
         <f aca="false">IF(J8=0,0,J17/J8)</f>
-        <v>0.0696180290297939</v>
+        <v>0.0775443510737629</v>
       </c>
       <c r="K18" s="58" t="n">
         <f aca="false">IF(K8=0,0,K17/K8)</f>
-        <v>0.0693368983957221</v>
+        <v>0.0773725490196079</v>
       </c>
       <c r="L18" s="58" t="n">
         <f aca="false">IF(L8=0,0,L17/L8)</f>
-        <v>0.0690479039676902</v>
+        <v>0.0771959413135884</v>
       </c>
       <c r="M18" s="58" t="n">
         <f aca="false">IF(M8=0,0,M17/M8)</f>
-        <v>0.068750711116168</v>
+        <v>0.0770143234598803</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17268,27 +17268,27 @@
       </c>
       <c r="E19" s="39" t="n">
         <f aca="false">(Assumptions!E45)*Assumptions!E8</f>
-        <v>136.125</v>
+        <v>222.75</v>
       </c>
       <c r="F19" s="39" t="n">
         <f aca="false">(Assumptions!F45)*Assumptions!F8</f>
-        <v>314.325</v>
+        <v>514.35</v>
       </c>
       <c r="G19" s="39" t="n">
         <f aca="false">(Assumptions!G45)*Assumptions!G8</f>
-        <v>381.15</v>
+        <v>623.7</v>
       </c>
       <c r="H19" s="39" t="n">
         <f aca="false">(Assumptions!H45)*Assumptions!H8</f>
-        <v>311.85</v>
+        <v>510.3</v>
       </c>
       <c r="I19" s="39" t="n">
         <f aca="false">(Assumptions!I45)*Assumptions!I8</f>
-        <v>210.375</v>
+        <v>344.25</v>
       </c>
       <c r="J19" s="39" t="n">
         <f aca="false">(Assumptions!J45)*Assumptions!J8</f>
-        <v>105.1875</v>
+        <v>172.125</v>
       </c>
       <c r="K19" s="39" t="n">
         <f aca="false">(Assumptions!K45)*Assumptions!K8</f>
@@ -17313,39 +17313,39 @@
       </c>
       <c r="E20" s="57" t="n">
         <f aca="false">E17+E19</f>
-        <v>310.779</v>
+        <v>397.404</v>
       </c>
       <c r="F20" s="57" t="n">
         <f aca="false">F17+F19</f>
-        <v>486.311</v>
+        <v>686.336</v>
       </c>
       <c r="G20" s="57" t="n">
         <f aca="false">G17+G19</f>
-        <v>470.6094</v>
+        <v>787.9152</v>
       </c>
       <c r="H20" s="57" t="n">
         <f aca="false">H17+H19</f>
-        <v>409.5737</v>
+        <v>688.0386</v>
       </c>
       <c r="I20" s="57" t="n">
         <f aca="false">I17+I19</f>
-        <v>307.7445</v>
+        <v>521.409</v>
       </c>
       <c r="J20" s="57" t="n">
         <f aca="false">J17+J19</f>
-        <v>200.874</v>
+        <v>346.53</v>
       </c>
       <c r="K20" s="57" t="n">
         <f aca="false">K17+K19</f>
-        <v>94.0035000000002</v>
+        <v>171.651</v>
       </c>
       <c r="L20" s="57" t="n">
         <f aca="false">L17+L19</f>
-        <v>92.3205000000001</v>
+        <v>168.897</v>
       </c>
       <c r="M20" s="57" t="n">
         <f aca="false">M17+M19</f>
-        <v>90.6375000000001</v>
+        <v>166.143</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17418,31 +17418,31 @@
       </c>
       <c r="G24" s="39" t="n">
         <f aca="false">MAX(0,G17)</f>
-        <v>89.4594000000001</v>
+        <v>164.2152</v>
       </c>
       <c r="H24" s="39" t="n">
         <f aca="false">MAX(0,H17)</f>
-        <v>97.7237</v>
+        <v>177.7386</v>
       </c>
       <c r="I24" s="39" t="n">
         <f aca="false">MAX(0,I17)</f>
-        <v>97.3695000000001</v>
+        <v>177.159</v>
       </c>
       <c r="J24" s="39" t="n">
         <f aca="false">MAX(0,J17)</f>
-        <v>95.6865000000003</v>
+        <v>174.405</v>
       </c>
       <c r="K24" s="39" t="n">
         <f aca="false">MAX(0,K17)</f>
-        <v>94.0035000000002</v>
+        <v>171.651</v>
       </c>
       <c r="L24" s="39" t="n">
         <f aca="false">MAX(0,L17)</f>
-        <v>92.3205000000001</v>
+        <v>168.897</v>
       </c>
       <c r="M24" s="39" t="n">
         <f aca="false">MAX(0,M17)</f>
-        <v>90.6375000000001</v>
+        <v>166.143</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17467,27 +17467,27 @@
       </c>
       <c r="H25" s="39" t="n">
         <f aca="false">G28</f>
-        <v>3501.79248</v>
+        <v>3441.98784</v>
       </c>
       <c r="I25" s="39" t="n">
         <f aca="false">H28</f>
-        <v>3423.61352</v>
+        <v>3299.79696</v>
       </c>
       <c r="J25" s="39" t="n">
         <f aca="false">I28</f>
-        <v>3345.71792</v>
+        <v>3158.06976</v>
       </c>
       <c r="K25" s="39" t="n">
         <f aca="false">J28</f>
-        <v>3269.16872</v>
+        <v>3018.54576</v>
       </c>
       <c r="L25" s="39" t="n">
         <f aca="false">K28</f>
-        <v>3193.96592</v>
+        <v>2881.22496</v>
       </c>
       <c r="M25" s="39" t="n">
         <f aca="false">L28</f>
-        <v>3120.10952</v>
+        <v>2746.10736</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17508,31 +17508,31 @@
       </c>
       <c r="G26" s="39" t="n">
         <f aca="false">MIN(G25,G24*Assumptions!$C$90)</f>
-        <v>71.5675200000001</v>
+        <v>131.37216</v>
       </c>
       <c r="H26" s="39" t="n">
         <f aca="false">MIN(H25,H24*Assumptions!$C$90)</f>
-        <v>78.17896</v>
+        <v>142.19088</v>
       </c>
       <c r="I26" s="39" t="n">
         <f aca="false">MIN(I25,I24*Assumptions!$C$90)</f>
-        <v>77.8956000000001</v>
+        <v>141.7272</v>
       </c>
       <c r="J26" s="39" t="n">
         <f aca="false">MIN(J25,J24*Assumptions!$C$90)</f>
-        <v>76.5492000000002</v>
+        <v>139.524</v>
       </c>
       <c r="K26" s="39" t="n">
         <f aca="false">MIN(K25,K24*Assumptions!$C$90)</f>
-        <v>75.2028000000002</v>
+        <v>137.3208</v>
       </c>
       <c r="L26" s="39" t="n">
         <f aca="false">MIN(L25,L24*Assumptions!$C$90)</f>
-        <v>73.8564000000001</v>
+        <v>135.1176</v>
       </c>
       <c r="M26" s="39" t="n">
         <f aca="false">MIN(M25,M24*Assumptions!$C$90)</f>
-        <v>72.5100000000001</v>
+        <v>132.9144</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17598,31 +17598,31 @@
       </c>
       <c r="G28" s="39" t="n">
         <f aca="false">G25-G26+G27</f>
-        <v>3501.79248</v>
+        <v>3441.98784</v>
       </c>
       <c r="H28" s="39" t="n">
         <f aca="false">H25-H26+H27</f>
-        <v>3423.61352</v>
+        <v>3299.79696</v>
       </c>
       <c r="I28" s="39" t="n">
         <f aca="false">I25-I26+I27</f>
-        <v>3345.71792</v>
+        <v>3158.06976</v>
       </c>
       <c r="J28" s="39" t="n">
         <f aca="false">J25-J26+J27</f>
-        <v>3269.16872</v>
+        <v>3018.54576</v>
       </c>
       <c r="K28" s="39" t="n">
         <f aca="false">K25-K26+K27</f>
-        <v>3193.96592</v>
+        <v>2881.22496</v>
       </c>
       <c r="L28" s="39" t="n">
         <f aca="false">L25-L26+L27</f>
-        <v>3120.10952</v>
+        <v>2746.10736</v>
       </c>
       <c r="M28" s="39" t="n">
         <f aca="false">M25-M26+M27</f>
-        <v>3047.59952</v>
+        <v>2613.19296</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17643,31 +17643,31 @@
       </c>
       <c r="G29" s="39" t="n">
         <f aca="false">G24-G26</f>
-        <v>17.89188</v>
+        <v>32.8430400000001</v>
       </c>
       <c r="H29" s="39" t="n">
         <f aca="false">H24-H26</f>
-        <v>19.54474</v>
+        <v>35.5477200000001</v>
       </c>
       <c r="I29" s="39" t="n">
         <f aca="false">I24-I26</f>
-        <v>19.4739</v>
+        <v>35.4318</v>
       </c>
       <c r="J29" s="39" t="n">
         <f aca="false">J24-J26</f>
-        <v>19.1373000000001</v>
+        <v>34.881</v>
       </c>
       <c r="K29" s="39" t="n">
         <f aca="false">K24-K26</f>
-        <v>18.8007</v>
+        <v>34.3302</v>
       </c>
       <c r="L29" s="39" t="n">
         <f aca="false">L24-L26</f>
-        <v>18.4641</v>
+        <v>33.7794</v>
       </c>
       <c r="M29" s="39" t="n">
         <f aca="false">M24-M26</f>
-        <v>18.1275</v>
+        <v>33.2285999999999</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17688,31 +17688,31 @@
       </c>
       <c r="G30" s="39" t="n">
         <f aca="false">-G29*Assumptions!$C$87</f>
-        <v>-4.1151324</v>
+        <v>-7.55389920000001</v>
       </c>
       <c r="H30" s="39" t="n">
         <f aca="false">-H29*Assumptions!$C$87</f>
-        <v>-4.4952902</v>
+        <v>-8.17597560000001</v>
       </c>
       <c r="I30" s="39" t="n">
         <f aca="false">-I29*Assumptions!$C$87</f>
-        <v>-4.478997</v>
+        <v>-8.149314</v>
       </c>
       <c r="J30" s="39" t="n">
         <f aca="false">-J29*Assumptions!$C$87</f>
-        <v>-4.40157900000001</v>
+        <v>-8.02263000000001</v>
       </c>
       <c r="K30" s="39" t="n">
         <f aca="false">-K29*Assumptions!$C$87</f>
-        <v>-4.32416100000001</v>
+        <v>-7.89594600000001</v>
       </c>
       <c r="L30" s="39" t="n">
         <f aca="false">-L29*Assumptions!$C$87</f>
-        <v>-4.246743</v>
+        <v>-7.769262</v>
       </c>
       <c r="M30" s="39" t="n">
         <f aca="false">-M29*Assumptions!$C$87</f>
-        <v>-4.169325</v>
+        <v>-7.64257799999999</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17725,39 +17725,39 @@
       </c>
       <c r="E31" s="57" t="n">
         <f aca="false">E20+E30</f>
-        <v>302.744916</v>
+        <v>389.369916</v>
       </c>
       <c r="F31" s="57" t="n">
         <f aca="false">F20+F30</f>
-        <v>478.399644</v>
+        <v>678.424644</v>
       </c>
       <c r="G31" s="57" t="n">
         <f aca="false">G20+G30</f>
-        <v>466.4942676</v>
+        <v>780.3613008</v>
       </c>
       <c r="H31" s="57" t="n">
         <f aca="false">H20+H30</f>
-        <v>405.0784098</v>
+        <v>679.8626244</v>
       </c>
       <c r="I31" s="57" t="n">
         <f aca="false">I20+I30</f>
-        <v>303.265503</v>
+        <v>513.259686</v>
       </c>
       <c r="J31" s="57" t="n">
         <f aca="false">J20+J30</f>
-        <v>196.472421</v>
+        <v>338.50737</v>
       </c>
       <c r="K31" s="57" t="n">
         <f aca="false">K20+K30</f>
-        <v>89.6793390000002</v>
+        <v>163.755054</v>
       </c>
       <c r="L31" s="57" t="n">
         <f aca="false">L20+L30</f>
-        <v>88.0737570000001</v>
+        <v>161.127738</v>
       </c>
       <c r="M31" s="57" t="n">
         <f aca="false">M20+M30</f>
-        <v>86.4681750000001</v>
+        <v>158.500422</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17815,39 +17815,39 @@
       </c>
       <c r="E33" s="39" t="n">
         <f aca="false">-E8*Assumptions!$C$83</f>
-        <v>-14.06625</v>
+        <v>-23.0175</v>
       </c>
       <c r="F33" s="39" t="n">
         <f aca="false">-F8*Assumptions!$C$83</f>
-        <v>-32.48025</v>
+        <v>-53.1495</v>
       </c>
       <c r="G33" s="39" t="n">
         <f aca="false">-G8*Assumptions!$C$83</f>
-        <v>-38.8773</v>
+        <v>-63.6174</v>
       </c>
       <c r="H33" s="39" t="n">
         <f aca="false">-H8*Assumptions!$C$83</f>
-        <v>-41.8572</v>
+        <v>-68.4936</v>
       </c>
       <c r="I33" s="39" t="n">
         <f aca="false">-I8*Assumptions!$C$83</f>
-        <v>-41.7945</v>
+        <v>-68.391</v>
       </c>
       <c r="J33" s="39" t="n">
         <f aca="false">-J8*Assumptions!$C$83</f>
-        <v>-41.2335</v>
+        <v>-67.473</v>
       </c>
       <c r="K33" s="39" t="n">
         <f aca="false">-K8*Assumptions!$C$83</f>
-        <v>-40.6725</v>
+        <v>-66.555</v>
       </c>
       <c r="L33" s="39" t="n">
         <f aca="false">-L8*Assumptions!$C$83</f>
-        <v>-40.1115</v>
+        <v>-65.637</v>
       </c>
       <c r="M33" s="39" t="n">
         <f aca="false">-M8*Assumptions!$C$83</f>
-        <v>-39.5505</v>
+        <v>-64.719</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17950,39 +17950,39 @@
       </c>
       <c r="E36" s="39" t="n">
         <f aca="false">E8*Assumptions!$C$86</f>
-        <v>70.33125</v>
+        <v>115.0875</v>
       </c>
       <c r="F36" s="39" t="n">
         <f aca="false">F8*Assumptions!$C$86</f>
-        <v>162.40125</v>
+        <v>265.7475</v>
       </c>
       <c r="G36" s="39" t="n">
         <f aca="false">G8*Assumptions!$C$86</f>
-        <v>194.3865</v>
+        <v>318.087</v>
       </c>
       <c r="H36" s="39" t="n">
         <f aca="false">H8*Assumptions!$C$86</f>
-        <v>209.286</v>
+        <v>342.468</v>
       </c>
       <c r="I36" s="39" t="n">
         <f aca="false">I8*Assumptions!$C$86</f>
-        <v>208.9725</v>
+        <v>341.955</v>
       </c>
       <c r="J36" s="39" t="n">
         <f aca="false">J8*Assumptions!$C$86</f>
-        <v>206.1675</v>
+        <v>337.365</v>
       </c>
       <c r="K36" s="39" t="n">
         <f aca="false">K8*Assumptions!$C$86</f>
-        <v>203.3625</v>
+        <v>332.775</v>
       </c>
       <c r="L36" s="39" t="n">
         <f aca="false">L8*Assumptions!$C$86</f>
-        <v>200.5575</v>
+        <v>328.185</v>
       </c>
       <c r="M36" s="39" t="n">
         <f aca="false">M8*Assumptions!$C$86</f>
-        <v>197.7525</v>
+        <v>323.595</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17995,39 +17995,39 @@
       </c>
       <c r="E37" s="39" t="n">
         <f aca="false">-(E36-D36)</f>
-        <v>-70.33125</v>
+        <v>-115.0875</v>
       </c>
       <c r="F37" s="39" t="n">
         <f aca="false">-(F36-E36)</f>
-        <v>-92.07</v>
+        <v>-150.66</v>
       </c>
       <c r="G37" s="39" t="n">
         <f aca="false">-(G36-F36)</f>
-        <v>-31.98525</v>
+        <v>-52.3395</v>
       </c>
       <c r="H37" s="39" t="n">
         <f aca="false">-(H36-G36)</f>
-        <v>-14.8995</v>
+        <v>-24.381</v>
       </c>
       <c r="I37" s="39" t="n">
         <f aca="false">-(I36-H36)</f>
-        <v>0.313500000000005</v>
+        <v>0.512999999999977</v>
       </c>
       <c r="J37" s="39" t="n">
         <f aca="false">-(J36-I36)</f>
-        <v>2.80499999999998</v>
+        <v>4.59000000000003</v>
       </c>
       <c r="K37" s="39" t="n">
         <f aca="false">-(K36-J36)</f>
-        <v>2.80500000000001</v>
+        <v>4.58999999999998</v>
       </c>
       <c r="L37" s="39" t="n">
         <f aca="false">-(L36-K36)</f>
-        <v>2.80500000000001</v>
+        <v>4.59000000000003</v>
       </c>
       <c r="M37" s="39" t="n">
         <f aca="false">-(M36-L36)</f>
-        <v>2.80500000000001</v>
+        <v>4.58999999999998</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18040,39 +18040,39 @@
       </c>
       <c r="E38" s="60" t="n">
         <f aca="false">E31+E32+E33+E34+E35+E37</f>
-        <v>81.693416</v>
+        <v>114.610916</v>
       </c>
       <c r="F38" s="60" t="n">
         <f aca="false">F31+F32+F33+F34+F35+F37</f>
-        <v>345.863394</v>
+        <v>466.629144</v>
       </c>
       <c r="G38" s="60" t="n">
         <f aca="false">G31+G32+G33+G34+G35+G37</f>
-        <v>423.6457176</v>
+        <v>692.4184008</v>
       </c>
       <c r="H38" s="60" t="n">
         <f aca="false">H31+H32+H33+H34+H35+H37</f>
-        <v>376.3357098</v>
+        <v>615.0020244</v>
       </c>
       <c r="I38" s="60" t="n">
         <f aca="false">I31+I32+I33+I34+I35+I37</f>
-        <v>289.798503</v>
+        <v>473.395686</v>
       </c>
       <c r="J38" s="60" t="n">
         <f aca="false">J31+J32+J33+J34+J35+J37</f>
-        <v>186.057921</v>
+        <v>303.63837</v>
       </c>
       <c r="K38" s="60" t="n">
         <f aca="false">K31+K32+K33+K34+K35+K37</f>
-        <v>79.8258390000002</v>
+        <v>129.804054</v>
       </c>
       <c r="L38" s="60" t="n">
         <f aca="false">L31+L32+L33+L34+L35+L37</f>
-        <v>78.7812570000001</v>
+        <v>128.094738</v>
       </c>
       <c r="M38" s="60" t="n">
         <f aca="false">M31+M32+M33+M34+M35+M37</f>
-        <v>77.7366750000001</v>
+        <v>126.385422</v>
       </c>
     </row>
   </sheetData>
@@ -19578,39 +19578,39 @@
       </c>
       <c r="E6" s="63" t="n">
         <f aca="false">SKBA!E8</f>
-        <v>468.875</v>
+        <v>767.25</v>
       </c>
       <c r="F6" s="63" t="n">
         <f aca="false">SKBA!F8</f>
-        <v>1082.675</v>
+        <v>1771.65</v>
       </c>
       <c r="G6" s="63" t="n">
         <f aca="false">SKBA!G8</f>
-        <v>1295.91</v>
+        <v>2120.58</v>
       </c>
       <c r="H6" s="63" t="n">
         <f aca="false">SKBA!H8</f>
-        <v>1395.24</v>
+        <v>2283.12</v>
       </c>
       <c r="I6" s="63" t="n">
         <f aca="false">SKBA!I8</f>
-        <v>1393.15</v>
+        <v>2279.7</v>
       </c>
       <c r="J6" s="63" t="n">
         <f aca="false">SKBA!J8</f>
-        <v>1374.45</v>
+        <v>2249.1</v>
       </c>
       <c r="K6" s="63" t="n">
         <f aca="false">SKBA!K8</f>
-        <v>1355.75</v>
+        <v>2218.5</v>
       </c>
       <c r="L6" s="63" t="n">
         <f aca="false">SKBA!L8</f>
-        <v>1337.05</v>
+        <v>2187.9</v>
       </c>
       <c r="M6" s="63" t="n">
         <f aca="false">SKBA!M8</f>
-        <v>1318.35</v>
+        <v>2157.3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19668,39 +19668,39 @@
       </c>
       <c r="E8" s="57" t="n">
         <f aca="false">E6+E7</f>
-        <v>468.875</v>
+        <v>767.25</v>
       </c>
       <c r="F8" s="57" t="n">
         <f aca="false">F6+F7</f>
-        <v>1881.173</v>
+        <v>2570.148</v>
       </c>
       <c r="G8" s="57" t="n">
         <f aca="false">G6+G7</f>
-        <v>3835.6488</v>
+        <v>4660.3188</v>
       </c>
       <c r="H8" s="57" t="n">
         <f aca="false">H6+H7</f>
-        <v>4636.455</v>
+        <v>5524.335</v>
       </c>
       <c r="I8" s="57" t="n">
         <f aca="false">I6+I7</f>
-        <v>5017.873</v>
+        <v>5904.423</v>
       </c>
       <c r="J8" s="57" t="n">
         <f aca="false">J6+J7</f>
-        <v>4950.519</v>
+        <v>5825.169</v>
       </c>
       <c r="K8" s="57" t="n">
         <f aca="false">K6+K7</f>
-        <v>4883.165</v>
+        <v>5745.915</v>
       </c>
       <c r="L8" s="57" t="n">
         <f aca="false">L6+L7</f>
-        <v>4815.811</v>
+        <v>5666.661</v>
       </c>
       <c r="M8" s="57" t="n">
         <f aca="false">M6+M7</f>
-        <v>4748.457</v>
+        <v>5587.407</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19713,39 +19713,39 @@
       </c>
       <c r="E9" s="55" t="n">
         <f aca="false">SKBA!E6+Assumptions!E69+Assumptions!E70</f>
-        <v>3.025</v>
+        <v>4.95</v>
       </c>
       <c r="F9" s="55" t="n">
         <f aca="false">SKBA!F6+Assumptions!F69+Assumptions!F70</f>
-        <v>12.331</v>
+        <v>16.776</v>
       </c>
       <c r="G9" s="55" t="n">
         <f aca="false">SKBA!G6+Assumptions!G69+Assumptions!G70</f>
-        <v>25.696</v>
+        <v>31.086</v>
       </c>
       <c r="H9" s="55" t="n">
         <f aca="false">SKBA!H6+Assumptions!H69+Assumptions!H70</f>
-        <v>31.515</v>
+        <v>37.395</v>
       </c>
       <c r="I9" s="55" t="n">
         <f aca="false">SKBA!I6+Assumptions!I69+Assumptions!I70</f>
-        <v>34.595</v>
+        <v>40.545</v>
       </c>
       <c r="J9" s="55" t="n">
         <f aca="false">SKBA!J6+Assumptions!J69+Assumptions!J70</f>
-        <v>34.595</v>
+        <v>40.545</v>
       </c>
       <c r="K9" s="55" t="n">
         <f aca="false">SKBA!K6+Assumptions!K69+Assumptions!K70</f>
-        <v>34.595</v>
+        <v>40.545</v>
       </c>
       <c r="L9" s="55" t="n">
         <f aca="false">SKBA!L6+Assumptions!L69+Assumptions!L70</f>
-        <v>34.595</v>
+        <v>40.545</v>
       </c>
       <c r="M9" s="55" t="n">
         <f aca="false">SKBA!M6+Assumptions!M69+Assumptions!M70</f>
-        <v>34.595</v>
+        <v>40.545</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19818,31 +19818,31 @@
       </c>
       <c r="G13" s="39" t="n">
         <f aca="false">SKBA!G17+SKOT!G16</f>
-        <v>251.335892</v>
+        <v>326.091692</v>
       </c>
       <c r="H13" s="39" t="n">
         <f aca="false">SKBA!H17+SKOT!H16</f>
-        <v>322.73305</v>
+        <v>402.74795</v>
       </c>
       <c r="I13" s="39" t="n">
         <f aca="false">SKBA!I17+SKOT!I16</f>
-        <v>356.89457</v>
+        <v>436.68407</v>
       </c>
       <c r="J13" s="39" t="n">
         <f aca="false">SKBA!J17+SKOT!J16</f>
-        <v>350.832710000001</v>
+        <v>429.551210000001</v>
       </c>
       <c r="K13" s="39" t="n">
         <f aca="false">SKBA!K17+SKOT!K16</f>
-        <v>344.77085</v>
+        <v>422.41835</v>
       </c>
       <c r="L13" s="39" t="n">
         <f aca="false">SKBA!L17+SKOT!L16</f>
-        <v>338.70899</v>
+        <v>415.28549</v>
       </c>
       <c r="M13" s="39" t="n">
         <f aca="false">SKBA!M17+SKOT!M16</f>
-        <v>332.64713</v>
+        <v>408.15263</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19855,39 +19855,39 @@
       </c>
       <c r="E14" s="58" t="n">
         <f aca="false">IF(E8=0,0,E13/E8)</f>
-        <v>0.272917088776326</v>
+        <v>0.166782665363311</v>
       </c>
       <c r="F14" s="58" t="n">
         <f aca="false">IF(F8=0,0,F13/F8)</f>
-        <v>0.0941704032537146</v>
+        <v>0.0689263108583631</v>
       </c>
       <c r="G14" s="58" t="n">
         <f aca="false">IF(G8=0,0,G13/G8)</f>
-        <v>0.0655263047023492</v>
+        <v>0.0699719710162318</v>
       </c>
       <c r="H14" s="58" t="n">
         <f aca="false">IF(H8=0,0,H13/H8)</f>
-        <v>0.0696077175341937</v>
+        <v>0.0729043314715708</v>
       </c>
       <c r="I14" s="58" t="n">
         <f aca="false">IF(I8=0,0,I13/I8)</f>
-        <v>0.0711246717483683</v>
+        <v>0.0739588051194841</v>
       </c>
       <c r="J14" s="58" t="n">
         <f aca="false">IF(J8=0,0,J13/J8)</f>
-        <v>0.0708678645612714</v>
+        <v>0.0737405575700895</v>
       </c>
       <c r="K14" s="58" t="n">
         <f aca="false">IF(K8=0,0,K13/K8)</f>
-        <v>0.0706039730379784</v>
+        <v>0.0735162893986423</v>
       </c>
       <c r="L14" s="58" t="n">
         <f aca="false">IF(L8=0,0,L13/L8)</f>
-        <v>0.0703326999336146</v>
+        <v>0.0732857479916304</v>
       </c>
       <c r="M14" s="58" t="n">
         <f aca="false">IF(M8=0,0,M13/M8)</f>
-        <v>0.0700537311383467</v>
+        <v>0.0730486664028592</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19900,27 +19900,27 @@
       </c>
       <c r="E15" s="39" t="n">
         <f aca="false">SKBA!E19+SKOT!E18</f>
-        <v>136.125</v>
+        <v>222.75</v>
       </c>
       <c r="F15" s="39" t="n">
         <f aca="false">SKBA!F19+SKOT!F18</f>
-        <v>554.895</v>
+        <v>754.92</v>
       </c>
       <c r="G15" s="39" t="n">
         <f aca="false">SKBA!G19+SKOT!G18</f>
-        <v>1156.32</v>
+        <v>1398.87</v>
       </c>
       <c r="H15" s="39" t="n">
         <f aca="false">SKBA!H19+SKOT!H18</f>
-        <v>1063.63125</v>
+        <v>1262.08125</v>
       </c>
       <c r="I15" s="39" t="n">
         <f aca="false">SKBA!I19+SKOT!I18</f>
-        <v>778.3875</v>
+        <v>912.2625</v>
       </c>
       <c r="J15" s="39" t="n">
         <f aca="false">SKBA!J19+SKOT!J18</f>
-        <v>389.19375</v>
+        <v>456.13125</v>
       </c>
       <c r="K15" s="39" t="n">
         <f aca="false">SKBA!K19+SKOT!K18</f>
@@ -19945,39 +19945,39 @@
       </c>
       <c r="E16" s="57" t="n">
         <f aca="false">SKBA!E20+SKOT!E19</f>
-        <v>264.089</v>
+        <v>350.714</v>
       </c>
       <c r="F16" s="57" t="n">
         <f aca="false">SKBA!F20+SKOT!F19</f>
-        <v>732.04582</v>
+        <v>932.07082</v>
       </c>
       <c r="G16" s="57" t="n">
         <f aca="false">SKBA!G20+SKOT!G19</f>
-        <v>1407.655892</v>
+        <v>1724.961692</v>
       </c>
       <c r="H16" s="57" t="n">
         <f aca="false">SKBA!H20+SKOT!H19</f>
-        <v>1386.3643</v>
+        <v>1664.8292</v>
       </c>
       <c r="I16" s="57" t="n">
         <f aca="false">SKBA!I20+SKOT!I19</f>
-        <v>1135.28207</v>
+        <v>1348.94657</v>
       </c>
       <c r="J16" s="57" t="n">
         <f aca="false">SKBA!J20+SKOT!J19</f>
-        <v>740.026460000001</v>
+        <v>885.682460000001</v>
       </c>
       <c r="K16" s="57" t="n">
         <f aca="false">SKBA!K20+SKOT!K19</f>
-        <v>344.77085</v>
+        <v>422.41835</v>
       </c>
       <c r="L16" s="57" t="n">
         <f aca="false">SKBA!L20+SKOT!L19</f>
-        <v>338.70899</v>
+        <v>415.28549</v>
       </c>
       <c r="M16" s="57" t="n">
         <f aca="false">SKBA!M20+SKOT!M19</f>
-        <v>332.64713</v>
+        <v>408.15263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19990,39 +19990,39 @@
       </c>
       <c r="E17" s="58" t="n">
         <f aca="false">IF(E8=0,0,E16/E8)</f>
-        <v>0.563239669421488</v>
+        <v>0.457105246008472</v>
       </c>
       <c r="F17" s="58" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.389143273904101</v>
+        <v>0.362652586543654</v>
       </c>
       <c r="G17" s="58" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.366992904042727</v>
+        <v>0.37013813132269</v>
       </c>
       <c r="H17" s="58" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.299013858648472</v>
+        <v>0.301362824665774</v>
       </c>
       <c r="I17" s="58" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.226247669082099</v>
+        <v>0.228463741503615</v>
       </c>
       <c r="J17" s="58" t="n">
         <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.1494846217134</v>
+        <v>0.152044079751163</v>
       </c>
       <c r="K17" s="58" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0706039730379784</v>
+        <v>0.0735162893986423</v>
       </c>
       <c r="L17" s="58" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0703326999336146</v>
+        <v>0.0732857479916304</v>
       </c>
       <c r="M17" s="58" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0700537311383467</v>
+        <v>0.0730486664028592</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20080,39 +20080,39 @@
       </c>
       <c r="E19" s="57" t="n">
         <f aca="false">E16+E18</f>
-        <v>336.125</v>
+        <v>422.75</v>
       </c>
       <c r="F19" s="57" t="n">
         <f aca="false">F16+F18</f>
-        <v>826.75982</v>
+        <v>1026.78482</v>
       </c>
       <c r="G19" s="57" t="n">
         <f aca="false">G16+G18</f>
-        <v>1502.369892</v>
+        <v>1819.675692</v>
       </c>
       <c r="H19" s="57" t="n">
         <f aca="false">H16+H18</f>
-        <v>1481.0783</v>
+        <v>1759.5432</v>
       </c>
       <c r="I19" s="57" t="n">
         <f aca="false">I16+I18</f>
-        <v>1229.99607</v>
+        <v>1443.66057</v>
       </c>
       <c r="J19" s="57" t="n">
         <f aca="false">J16+J18</f>
-        <v>834.740460000001</v>
+        <v>980.396460000001</v>
       </c>
       <c r="K19" s="57" t="n">
         <f aca="false">K16+K18</f>
-        <v>439.48485</v>
+        <v>517.13235</v>
       </c>
       <c r="L19" s="57" t="n">
         <f aca="false">L16+L18</f>
-        <v>433.42299</v>
+        <v>509.99949</v>
       </c>
       <c r="M19" s="57" t="n">
         <f aca="false">M16+M18</f>
-        <v>427.36113</v>
+        <v>502.86663</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20125,27 +20125,27 @@
       </c>
       <c r="E20" s="58" t="n">
         <f aca="false">IF(E8=0,0,E19/E8)</f>
-        <v>0.716875499866702</v>
+        <v>0.550993809058325</v>
       </c>
       <c r="F20" s="58" t="n">
         <f aca="false">IF(F8=0,0,F19/F8)</f>
-        <v>0.439491646967079</v>
+        <v>0.399504160849881</v>
       </c>
       <c r="G20" s="58" t="n">
         <f aca="false">IF(G8=0,0,G19/G8)</f>
-        <v>0.391685988560788</v>
+        <v>0.390461633654762</v>
       </c>
       <c r="H20" s="58" t="n">
         <f aca="false">IF(H8=0,0,H19/H8)</f>
-        <v>0.319441965898515</v>
+        <v>0.318507693686208</v>
       </c>
       <c r="I20" s="58" t="n">
         <f aca="false">IF(I8=0,0,I19/I8)</f>
-        <v>0.245122997333731</v>
+        <v>0.244504936384131</v>
       </c>
       <c r="J20" s="58" t="n">
         <f aca="false">IF(J8=0,0,J19/J8)</f>
-        <v>0.168616757152129</v>
+        <v>0.168303522181073</v>
       </c>
       <c r="K20" s="58" t="n">
         <f aca="false">IF(K8=0,0,K19/K8)</f>
@@ -20153,11 +20153,11 @@
       </c>
       <c r="L20" s="58" t="n">
         <f aca="false">IF(L8=0,0,L19/L8)</f>
-        <v>0.0900000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="M20" s="58" t="n">
         <f aca="false">IF(M8=0,0,M19/M8)</f>
-        <v>0.0900000000000001</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20178,31 +20178,31 @@
       </c>
       <c r="G21" s="40" t="n">
         <f aca="false">G19-G15</f>
-        <v>346.049892</v>
+        <v>420.805692</v>
       </c>
       <c r="H21" s="40" t="n">
         <f aca="false">H19-H15</f>
-        <v>417.44705</v>
+        <v>497.46195</v>
       </c>
       <c r="I21" s="40" t="n">
         <f aca="false">I19-I15</f>
-        <v>451.60857</v>
+        <v>531.39807</v>
       </c>
       <c r="J21" s="40" t="n">
         <f aca="false">J19-J15</f>
-        <v>445.546710000001</v>
+        <v>524.265210000001</v>
       </c>
       <c r="K21" s="40" t="n">
         <f aca="false">K19-K15</f>
-        <v>439.48485</v>
+        <v>517.13235</v>
       </c>
       <c r="L21" s="40" t="n">
         <f aca="false">L19-L15</f>
-        <v>433.42299</v>
+        <v>509.99949</v>
       </c>
       <c r="M21" s="40" t="n">
         <f aca="false">M19-M15</f>
-        <v>427.36113</v>
+        <v>502.86663</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20215,19 +20215,19 @@
       </c>
       <c r="E22" s="58" t="n">
         <f aca="false">IF(E8=0,0,E21/E8)</f>
-        <v>0.426552919221541</v>
+        <v>0.260671228413164</v>
       </c>
       <c r="F22" s="58" t="n">
         <f aca="false">IF(F8=0,0,F21/F8)</f>
-        <v>0.144518776316692</v>
+        <v>0.10577788516459</v>
       </c>
       <c r="G22" s="58" t="n">
         <f aca="false">IF(G8=0,0,G21/G8)</f>
-        <v>0.0902193892204103</v>
+        <v>0.090295473348304</v>
       </c>
       <c r="H22" s="58" t="n">
         <f aca="false">IF(H8=0,0,H21/H8)</f>
-        <v>0.0900358247842371</v>
+        <v>0.090049200492005</v>
       </c>
       <c r="I22" s="58" t="n">
         <f aca="false">IF(I8=0,0,I21/I8)</f>
@@ -20243,11 +20243,11 @@
       </c>
       <c r="L22" s="58" t="n">
         <f aca="false">IF(L8=0,0,L21/L8)</f>
-        <v>0.0900000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="M22" s="58" t="n">
         <f aca="false">IF(M8=0,0,M21/M8)</f>
-        <v>0.0900000000000001</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20312,39 +20312,39 @@
       </c>
       <c r="E26" s="67" t="n">
         <f aca="false">SKBA!E38</f>
-        <v>81.693416</v>
+        <v>114.610916</v>
       </c>
       <c r="F26" s="67" t="n">
         <f aca="false">SKBA!F38</f>
-        <v>345.863394</v>
+        <v>466.629144</v>
       </c>
       <c r="G26" s="67" t="n">
         <f aca="false">SKBA!G38</f>
-        <v>423.6457176</v>
+        <v>692.4184008</v>
       </c>
       <c r="H26" s="67" t="n">
         <f aca="false">SKBA!H38</f>
-        <v>376.3357098</v>
+        <v>615.0020244</v>
       </c>
       <c r="I26" s="67" t="n">
         <f aca="false">SKBA!I38</f>
-        <v>289.798503</v>
+        <v>473.395686</v>
       </c>
       <c r="J26" s="67" t="n">
         <f aca="false">SKBA!J38</f>
-        <v>186.057921</v>
+        <v>303.63837</v>
       </c>
       <c r="K26" s="67" t="n">
         <f aca="false">SKBA!K38</f>
-        <v>79.8258390000002</v>
+        <v>129.804054</v>
       </c>
       <c r="L26" s="67" t="n">
         <f aca="false">SKBA!L38</f>
-        <v>78.7812570000001</v>
+        <v>128.094738</v>
       </c>
       <c r="M26" s="67" t="n">
         <f aca="false">SKBA!M38</f>
-        <v>77.7366750000001</v>
+        <v>126.385422</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20402,39 +20402,39 @@
       </c>
       <c r="E28" s="60" t="n">
         <f aca="false">E26+E27</f>
-        <v>-368.306584</v>
+        <v>-335.389084</v>
       </c>
       <c r="F28" s="60" t="n">
         <f aca="false">F26+F27</f>
-        <v>244.33099228</v>
+        <v>365.09674228</v>
       </c>
       <c r="G28" s="60" t="n">
         <f aca="false">G26+G27</f>
-        <v>1065.63890556</v>
+        <v>1334.41158876</v>
       </c>
       <c r="H28" s="60" t="n">
         <f aca="false">H26+H27</f>
-        <v>1165.6162793</v>
+        <v>1404.2825939</v>
       </c>
       <c r="I28" s="60" t="n">
         <f aca="false">I26+I27</f>
-        <v>958.0774169</v>
+        <v>1141.6745999</v>
       </c>
       <c r="J28" s="60" t="n">
         <f aca="false">J26+J27</f>
-        <v>633.2427827</v>
+        <v>750.8232317</v>
       </c>
       <c r="K28" s="60" t="n">
         <f aca="false">K26+K27</f>
-        <v>241.0923485</v>
+        <v>291.0705635</v>
       </c>
       <c r="L28" s="60" t="n">
         <f aca="false">L26+L27</f>
-        <v>238.1356643</v>
+        <v>287.4491453</v>
       </c>
       <c r="M28" s="60" t="n">
         <f aca="false">M26+M27</f>
-        <v>235.1789801</v>
+        <v>283.8277271</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20634,39 +20634,39 @@
       </c>
       <c r="E35" s="57" t="n">
         <f aca="false">E26+E32+E33+E34</f>
-        <v>39.050816</v>
+        <v>71.968316</v>
       </c>
       <c r="F35" s="57" t="n">
         <f aca="false">F26+F32+F33+F34</f>
-        <v>303.220794</v>
+        <v>423.986544</v>
       </c>
       <c r="G35" s="57" t="n">
         <f aca="false">G26+G32+G33+G34</f>
-        <v>381.0031176</v>
+        <v>649.7758008</v>
       </c>
       <c r="H35" s="57" t="n">
         <f aca="false">H26+H32+H33+H34</f>
-        <v>333.6931098</v>
+        <v>572.3594244</v>
       </c>
       <c r="I35" s="57" t="n">
         <f aca="false">I26+I32+I33+I34</f>
-        <v>247.155903</v>
+        <v>430.753086</v>
       </c>
       <c r="J35" s="57" t="n">
         <f aca="false">J26+J32+J33+J34</f>
-        <v>143.415321</v>
+        <v>260.99577</v>
       </c>
       <c r="K35" s="57" t="n">
         <f aca="false">K26+K32+K33+K34</f>
-        <v>37.1832390000002</v>
+        <v>87.1614540000001</v>
       </c>
       <c r="L35" s="57" t="n">
         <f aca="false">L26+L32+L33+L34</f>
-        <v>36.1386570000001</v>
+        <v>85.452138</v>
       </c>
       <c r="M35" s="57" t="n">
         <f aca="false">M26+M32+M33+M34</f>
-        <v>35.0940750000001</v>
+        <v>83.7428219999998</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21174,39 +21174,39 @@
       </c>
       <c r="E47" s="60" t="n">
         <f aca="false">E35+E43</f>
-        <v>-564.949184</v>
+        <v>-532.031684</v>
       </c>
       <c r="F47" s="60" t="n">
         <f aca="false">F35+F43</f>
-        <v>47.68839228</v>
+        <v>168.45414228</v>
       </c>
       <c r="G47" s="60" t="n">
         <f aca="false">G35+G43</f>
-        <v>868.99630556</v>
+        <v>1137.76898876</v>
       </c>
       <c r="H47" s="60" t="n">
         <f aca="false">H35+H43</f>
-        <v>968.9736793</v>
+        <v>1207.6399939</v>
       </c>
       <c r="I47" s="60" t="n">
         <f aca="false">I35+I43</f>
-        <v>761.4348169</v>
+        <v>945.0319999</v>
       </c>
       <c r="J47" s="60" t="n">
         <f aca="false">J35+J43</f>
-        <v>436.6001827</v>
+        <v>554.1806317</v>
       </c>
       <c r="K47" s="60" t="n">
         <f aca="false">K35+K43</f>
-        <v>44.4497485000001</v>
+        <v>94.4279635</v>
       </c>
       <c r="L47" s="60" t="n">
         <f aca="false">L35+L43</f>
-        <v>41.4930643000003</v>
+        <v>90.8065453000002</v>
       </c>
       <c r="M47" s="60" t="n">
         <f aca="false">M35+M43</f>
-        <v>38.5363801000002</v>
+        <v>87.1851270999999</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21264,39 +21264,39 @@
       </c>
       <c r="E49" s="40" t="n">
         <f aca="false">E47*E48</f>
-        <v>-470.318130057597</v>
+        <v>-442.914431663777</v>
       </c>
       <c r="F49" s="40" t="n">
         <f aca="false">F47*F48</f>
-        <v>35.1331081505672</v>
+        <v>124.103944716466</v>
       </c>
       <c r="G49" s="40" t="n">
         <f aca="false">G47*G48</f>
-        <v>566.556697524869</v>
+        <v>741.787550411592</v>
       </c>
       <c r="H49" s="40" t="n">
         <f aca="false">H47*H48</f>
-        <v>559.06072655291</v>
+        <v>696.762055386085</v>
       </c>
       <c r="I49" s="40" t="n">
         <f aca="false">I47*I48</f>
-        <v>388.777651566455</v>
+        <v>482.519729097867</v>
       </c>
       <c r="J49" s="40" t="n">
         <f aca="false">J47*J48</f>
-        <v>197.275898680788</v>
+        <v>250.404114524215</v>
       </c>
       <c r="K49" s="40" t="n">
         <f aca="false">K47*K48</f>
-        <v>17.7738283600304</v>
+        <v>37.7582882304995</v>
       </c>
       <c r="L49" s="40" t="n">
         <f aca="false">L47*L48</f>
-        <v>14.6827951417397</v>
+        <v>32.1329341339825</v>
       </c>
       <c r="M49" s="40" t="n">
         <f aca="false">M47*M48</f>
-        <v>12.0677333074644</v>
+        <v>27.3021715970717</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21456,39 +21456,39 @@
       </c>
       <c r="E56" s="40" t="n">
         <f aca="false">E28*E55</f>
-        <v>-317.077967396448</v>
+        <v>-288.73903878318</v>
       </c>
       <c r="F56" s="40" t="n">
         <f aca="false">F28*F55</f>
-        <v>190.358758495907</v>
+        <v>284.447592762507</v>
       </c>
       <c r="G56" s="40" t="n">
         <f aca="false">G28*G55</f>
-        <v>751.349660936006</v>
+        <v>940.853125324873</v>
       </c>
       <c r="H56" s="40" t="n">
         <f aca="false">H28*H55</f>
-        <v>743.747216160077</v>
+        <v>896.033530470594</v>
       </c>
       <c r="I56" s="40" t="n">
         <f aca="false">I28*I55</f>
-        <v>553.232995791486</v>
+        <v>659.249501115887</v>
       </c>
       <c r="J56" s="40" t="n">
         <f aca="false">J28*J55</f>
-        <v>330.914228790707</v>
+        <v>392.35834574661</v>
       </c>
       <c r="K56" s="40" t="n">
         <f aca="false">K28*K55</f>
-        <v>114.016142200041</v>
+        <v>137.65158025437</v>
       </c>
       <c r="L56" s="40" t="n">
         <f aca="false">L28*L55</f>
-        <v>101.91663570422</v>
+        <v>123.021681406457</v>
       </c>
       <c r="M56" s="40" t="n">
         <f aca="false">M28*M55</f>
-        <v>91.0870970752324</v>
+        <v>109.929228028829</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21505,7 +21505,7 @@
       </c>
       <c r="D59" s="39" t="n">
         <f aca="false">SUM(D56:M56)</f>
-        <v>2399.16805970109</v>
+        <v>3094.42883827081</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21514,7 +21514,7 @@
       </c>
       <c r="D60" s="39" t="n">
         <f aca="false">M28*(1+Assumptions!$C$93)/(Assumptions!$C$91-Assumptions!$C$93)</f>
-        <v>2822.1477612</v>
+        <v>3405.9327252</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21523,7 +21523,7 @@
       </c>
       <c r="D61" s="39" t="n">
         <f aca="false">D60*M55</f>
-        <v>1093.04516490279</v>
+        <v>1319.15073634594</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21532,7 +21532,7 @@
       </c>
       <c r="D62" s="74" t="n">
         <f aca="false">D59+D61</f>
-        <v>3492.21322460388</v>
+        <v>4413.57957461676</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21550,7 +21550,7 @@
       </c>
       <c r="D64" s="75" t="n">
         <f aca="false">D62-Assumptions!$C$94</f>
-        <v>-2907.78677539612</v>
+        <v>-1986.42042538325</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="D66" s="76" t="n">
         <f aca="false">D61/D62</f>
-        <v>0.312994967547198</v>
+        <v>0.298884548028227</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21576,7 +21576,7 @@
       </c>
       <c r="D69" s="39" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>977.431804817188</v>
+        <v>1606.27785202397</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21585,7 +21585,7 @@
       </c>
       <c r="D70" s="39" t="n">
         <f aca="false">M47*(1+Assumptions!$C$93)/(Assumptions!$C$92-Assumptions!$C$93)</f>
-        <v>357.337342745456</v>
+        <v>808.443905836363</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="D71" s="39" t="n">
         <f aca="false">D70*1/(1+Assumptions!$C$92)^((10)-Assumptions!$C$95)</f>
-        <v>111.900799760124</v>
+        <v>253.165591172847</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21603,7 +21603,7 @@
       </c>
       <c r="D72" s="74" t="n">
         <f aca="false">D69+D71</f>
-        <v>1089.33260457731</v>
+        <v>1859.44344319681</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21612,7 +21612,7 @@
       </c>
       <c r="D73" s="77" t="n">
         <f aca="false">D64</f>
-        <v>-2907.78677539612</v>
+        <v>-1986.42042538325</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21661,7 +21661,7 @@
       </c>
       <c r="D80" s="80" t="n">
         <f aca="false">D64</f>
-        <v>-2907.78677539612</v>
+        <v>-1986.42042538325</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21670,7 +21670,7 @@
       </c>
       <c r="D81" s="77" t="n">
         <f aca="false">(Assumptions!$C$119+Assumptions!$C$120)-D64</f>
-        <v>7907.78677539612</v>
+        <v>6986.42042538325</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21697,7 +21697,7 @@
       </c>
       <c r="D86" s="67" t="n">
         <f aca="false">G21</f>
-        <v>346.049892</v>
+        <v>420.805692</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21706,7 +21706,7 @@
       </c>
       <c r="D87" s="67" t="n">
         <f aca="false">AVERAGE(H21:J21)</f>
-        <v>438.200776666667</v>
+        <v>517.70841</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21734,15 +21734,15 @@
       </c>
       <c r="D90" s="80" t="n">
         <f aca="false">$D$86*D88</f>
-        <v>2768.399136</v>
+        <v>3366.445536</v>
       </c>
       <c r="E90" s="80" t="n">
         <f aca="false">$D$86*E88</f>
-        <v>3806.548812</v>
+        <v>4628.862612</v>
       </c>
       <c r="F90" s="80" t="n">
         <f aca="false">$D$86*F88</f>
-        <v>4844.698488</v>
+        <v>5891.279688</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21751,15 +21751,15 @@
       </c>
       <c r="D91" s="80" t="n">
         <f aca="false">$D$87*D88</f>
-        <v>3505.60621333333</v>
+        <v>4141.66728</v>
       </c>
       <c r="E91" s="80" t="n">
         <f aca="false">$D$87*E88</f>
-        <v>4820.20854333333</v>
+        <v>5694.79251</v>
       </c>
       <c r="F91" s="80" t="n">
         <f aca="false">$D$87*F88</f>
-        <v>6134.81087333334</v>
+        <v>7247.91774</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21768,7 +21768,7 @@
       </c>
       <c r="D92" s="77" t="n">
         <f aca="false">D62</f>
-        <v>3492.21322460388</v>
+        <v>4413.57957461676</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="D5" s="39" t="n">
         <f aca="false">Consolidated!D87</f>
-        <v>438.200776666667</v>
+        <v>517.70841</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21843,7 +21843,7 @@
       </c>
       <c r="D6" s="39" t="n">
         <f aca="false">Consolidated!D86</f>
-        <v>346.049892</v>
+        <v>420.805692</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21852,7 +21852,7 @@
       </c>
       <c r="D7" s="39" t="n">
         <f aca="false">AVERAGE(Consolidated!H8:J8)</f>
-        <v>4868.28233333333</v>
+        <v>5751.309</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21861,7 +21861,7 @@
       </c>
       <c r="D8" s="40" t="n">
         <f aca="false">Consolidated!D62</f>
-        <v>3492.21322460388</v>
+        <v>4413.57957461676</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21879,7 +21879,7 @@
       </c>
       <c r="D10" s="84" t="n">
         <f aca="false">D8/D5</f>
-        <v>7.9694364103338</v>
+        <v>8.52522286554463</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21888,7 +21888,7 @@
       </c>
       <c r="D11" s="86" t="n">
         <f aca="false">D8/D6</f>
-        <v>10.0916466247702</v>
+        <v>10.4884027438886</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22064,19 +22064,19 @@
       </c>
       <c r="D29" s="39" t="n">
         <f aca="false">C29*$D$5</f>
-        <v>3505.60621333333</v>
+        <v>4141.66728</v>
       </c>
       <c r="E29" s="93" t="n">
         <f aca="false">D29-$D$9</f>
-        <v>-2894.39378666667</v>
+        <v>-2258.33272</v>
       </c>
       <c r="F29" s="39" t="n">
         <f aca="false">C29*$D$6</f>
-        <v>2768.399136</v>
+        <v>3366.445536</v>
       </c>
       <c r="G29" s="93" t="n">
         <f aca="false">F29-$D$9</f>
-        <v>-3631.600864</v>
+        <v>-3033.554464</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22088,19 +22088,19 @@
       </c>
       <c r="D30" s="39" t="n">
         <f aca="false">C30*$D$5</f>
-        <v>4601.108155</v>
+        <v>5435.938305</v>
       </c>
       <c r="E30" s="93" t="n">
         <f aca="false">D30-$D$9</f>
-        <v>-1798.891845</v>
+        <v>-964.061694999999</v>
       </c>
       <c r="F30" s="39" t="n">
         <f aca="false">C30*$D$6</f>
-        <v>3633.523866</v>
+        <v>4418.459766</v>
       </c>
       <c r="G30" s="93" t="n">
         <f aca="false">F30-$D$9</f>
-        <v>-2766.476134</v>
+        <v>-1981.540234</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22112,19 +22112,19 @@
       </c>
       <c r="D31" s="39" t="n">
         <f aca="false">C31*$D$5</f>
-        <v>5696.61009666667</v>
+        <v>6730.20933</v>
       </c>
       <c r="E31" s="67" t="n">
         <f aca="false">D31-$D$9</f>
-        <v>-703.389903333333</v>
+        <v>330.209330000002</v>
       </c>
       <c r="F31" s="39" t="n">
         <f aca="false">C31*$D$6</f>
-        <v>4498.648596</v>
+        <v>5470.473996</v>
       </c>
       <c r="G31" s="93" t="n">
         <f aca="false">F31-$D$9</f>
-        <v>-1901.351404</v>
+        <v>-929.526003999999</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22136,19 +22136,19 @@
       </c>
       <c r="D32" s="39" t="n">
         <f aca="false">C32*$D$5</f>
-        <v>6573.01165</v>
+        <v>7765.62615</v>
       </c>
       <c r="E32" s="67" t="n">
         <f aca="false">D32-$D$9</f>
-        <v>173.011650000001</v>
+        <v>1365.62615</v>
       </c>
       <c r="F32" s="39" t="n">
         <f aca="false">C32*$D$6</f>
-        <v>5190.74838</v>
+        <v>6312.08538</v>
       </c>
       <c r="G32" s="67" t="n">
         <f aca="false">F32-$D$9</f>
-        <v>-1209.25162</v>
+        <v>-87.9146199999977</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22160,19 +22160,19 @@
       </c>
       <c r="D33" s="39" t="n">
         <f aca="false">C33*$D$5</f>
-        <v>8325.81475666667</v>
+        <v>9836.45979</v>
       </c>
       <c r="E33" s="67" t="n">
         <f aca="false">D33-$D$9</f>
-        <v>1925.81475666667</v>
+        <v>3436.45979</v>
       </c>
       <c r="F33" s="39" t="n">
         <f aca="false">C33*$D$6</f>
-        <v>6574.947948</v>
+        <v>7995.308148</v>
       </c>
       <c r="G33" s="67" t="n">
         <f aca="false">F33-$D$9</f>
-        <v>174.947947999995</v>
+        <v>1595.308148</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22253,11 +22253,11 @@
       </c>
       <c r="H39" s="84" t="n">
         <f aca="false">G39/$D$5</f>
-        <v>19.4659627600082</v>
+        <v>16.4764563125409</v>
       </c>
       <c r="I39" s="86" t="n">
         <f aca="false">G39/$D$6</f>
-        <v>24.6496248003453</v>
+        <v>20.270638354388</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22284,11 +22284,11 @@
       </c>
       <c r="H40" s="84" t="n">
         <f aca="false">G40/$D$5</f>
-        <v>17.8457009124577</v>
+        <v>15.1050279442051</v>
       </c>
       <c r="I40" s="86" t="n">
         <f aca="false">G40/$D$6</f>
-        <v>22.5978975309144</v>
+        <v>18.5833988196148</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22315,11 +22315,11 @@
       </c>
       <c r="H41" s="84" t="n">
         <f aca="false">G41/$D$5</f>
-        <v>17.8457009124577</v>
+        <v>15.1050279442051</v>
       </c>
       <c r="I41" s="86" t="n">
         <f aca="false">G41/$D$6</f>
-        <v>22.5978975309144</v>
+        <v>18.5833988196148</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22346,11 +22346,11 @@
       </c>
       <c r="H42" s="84" t="n">
         <f aca="false">G42/$D$5</f>
-        <v>16.5891713163981</v>
+        <v>14.0414712503937</v>
       </c>
       <c r="I42" s="86" t="n">
         <f aca="false">G42/$D$6</f>
-        <v>21.0067620974783</v>
+        <v>17.2749273436683</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22377,11 +22377,11 @@
       </c>
       <c r="H43" s="84" t="n">
         <f aca="false">G43/$D$5</f>
-        <v>15.927839950051</v>
+        <v>13.4817045694403</v>
       </c>
       <c r="I43" s="86" t="n">
         <f aca="false">G43/$D$6</f>
-        <v>20.1693223956698</v>
+        <v>16.5862581458016</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22418,7 +22418,7 @@
       </c>
       <c r="C48" s="94" t="n">
         <f aca="false">G39/($D$46*$D$7)</f>
-        <v>0.134781387197109</v>
+        <v>0.114087740052542</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22427,7 +22427,7 @@
       </c>
       <c r="C49" s="94" t="n">
         <f aca="false">G40/($D$46*$D$7)</f>
-        <v>0.123562772319038</v>
+        <v>0.104591574116164</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22436,7 +22436,7 @@
       </c>
       <c r="C50" s="94" t="n">
         <f aca="false">G41/($D$46*$D$7)</f>
-        <v>0.123562772319038</v>
+        <v>0.104591574116164</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="C51" s="94" t="n">
         <f aca="false">G42/($D$46*$D$7)</f>
-        <v>0.114862622005432</v>
+        <v>0.0972272005328505</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22454,7 +22454,7 @@
       </c>
       <c r="C52" s="94" t="n">
         <f aca="false">G43/($D$46*$D$7)</f>
-        <v>0.110283595524586</v>
+        <v>0.0933512144363696</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
model: run-rate ex-AMPC EBITDA 마진 9% → 13% 상향 반영
- gross margin 4곳(1-1동 20%·1-2동 18%·각형/파우치 19%) +4%p
- run-rate ex-AMPC EBITDA $518mm → $748mm (BA 295 + OT 452, 13.0%)
- DCF EV $6.0bn, AMPC PV 비중 76% → 55%, ex-AMPC 본질 EV $2.7bn
- FCFE 지분가치 +$3.1bn, 역산 시나리오 11.4x → 9.3x 전부 peer 밴드(8~13x) 내
- 덱 S2/S4/S5 갱신(멀티플 헤더 13%, peer 바 밴드 내), CLAUDE.md·펀딩구조_v2 동기화
- total_errors = 0

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWAFoC5mEReHSPt6vQXor
</commit_message>
<xml_diff>
--- a/sk_valuation_project/output/FCFF_model_lines.xlsx
+++ b/sk_valuation_project/output/FCFF_model_lines.xlsx
@@ -2561,18 +2561,18 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">·ex-AMPC EBITDA 9% (</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="8"/>
-        <color rgb="FF8C8473"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">지분 수익률 기준</t>
+      <t xml:space="preserve">·ex-AMPC EBITDA 13% (</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="8"/>
+        <color rgb="FF8C8473"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">마진 개선</t>
     </r>
     <r>
       <rPr>
@@ -2661,7 +2661,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(ex-AMPC EBITDA 9%)</t>
+      <t xml:space="preserve">(ex-AMPC EBITDA 13%)</t>
     </r>
   </si>
   <si>
@@ -13147,8 +13147,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="16082118"/>
-        <c:axId val="10905176"/>
+        <c:axId val="89734112"/>
+        <c:axId val="81998348"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -13261,28 +13261,28 @@
                   <c:v>-335.389084</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>365.09674228</c:v>
+                  <c:v>426.74986996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1334.41158876</c:v>
+                  <c:v>1487.67993132</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1404.2825939</c:v>
+                  <c:v>1591.2358751</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1141.6745999</c:v>
+                  <c:v>1340.3094203</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>750.8232317</c:v>
+                  <c:v>946.7918129</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>291.0705635</c:v>
+                  <c:v>484.3729055</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>287.4491453</c:v>
+                  <c:v>478.085248099999</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>283.8277271</c:v>
+                  <c:v>471.797590699999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13297,11 +13297,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="16082118"/>
-        <c:axId val="10905176"/>
+        <c:axId val="89734112"/>
+        <c:axId val="81998348"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="16082118"/>
+        <c:axId val="89734112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13333,7 +13333,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10905176"/>
+        <c:crossAx val="81998348"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13341,7 +13341,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10905176"/>
+        <c:axId val="81998348"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13383,7 +13383,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16082118"/>
+        <c:crossAx val="89734112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -15094,31 +15094,31 @@
         <v>0</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="G47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="H47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="I47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="J47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="K47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="L47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="M47" s="21" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15135,28 +15135,28 @@
         <v>0</v>
       </c>
       <c r="F48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="G48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="I48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="J48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="K48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="L48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="M48" s="21" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15172,39 +15172,39 @@
       </c>
       <c r="E49" s="39" t="n">
         <f aca="false">E46*(1-E47-E24)</f>
-        <v>130.2</v>
+        <v>124</v>
       </c>
       <c r="F49" s="39" t="n">
         <f aca="false">F46*(1-F47-F24)</f>
-        <v>130.2</v>
+        <v>124</v>
       </c>
       <c r="G49" s="39" t="n">
         <f aca="false">G46*(1-G47-G24)</f>
-        <v>128.52</v>
+        <v>122.4</v>
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">H46*(1-H47-H24)</f>
-        <v>126.84</v>
+        <v>120.8</v>
       </c>
       <c r="I49" s="39" t="n">
         <f aca="false">I46*(1-I47-I24)</f>
-        <v>125.16</v>
+        <v>119.2</v>
       </c>
       <c r="J49" s="39" t="n">
         <f aca="false">J46*(1-J47-J24)</f>
-        <v>123.48</v>
+        <v>117.6</v>
       </c>
       <c r="K49" s="39" t="n">
         <f aca="false">K46*(1-K47-K24)</f>
-        <v>121.8</v>
+        <v>116</v>
       </c>
       <c r="L49" s="39" t="n">
         <f aca="false">L46*(1-L47-L24)</f>
-        <v>120.12</v>
+        <v>114.4</v>
       </c>
       <c r="M49" s="39" t="n">
         <f aca="false">M46*(1-M47-M24)</f>
-        <v>118.44</v>
+        <v>112.8</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15224,35 +15224,35 @@
       </c>
       <c r="F50" s="39" t="n">
         <f aca="false">F46*(1-F48-F24)</f>
-        <v>133.3</v>
+        <v>127.1</v>
       </c>
       <c r="G50" s="39" t="n">
         <f aca="false">G46*(1-G48-G24)</f>
-        <v>131.58</v>
+        <v>125.46</v>
       </c>
       <c r="H50" s="39" t="n">
         <f aca="false">H46*(1-H48-H24)</f>
-        <v>129.86</v>
+        <v>123.82</v>
       </c>
       <c r="I50" s="39" t="n">
         <f aca="false">I46*(1-I48-I24)</f>
-        <v>128.14</v>
+        <v>122.18</v>
       </c>
       <c r="J50" s="39" t="n">
         <f aca="false">J46*(1-J48-J24)</f>
-        <v>126.42</v>
+        <v>120.54</v>
       </c>
       <c r="K50" s="39" t="n">
         <f aca="false">K46*(1-K48-K24)</f>
-        <v>124.7</v>
+        <v>118.9</v>
       </c>
       <c r="L50" s="39" t="n">
         <f aca="false">L46*(1-L48-L24)</f>
-        <v>122.98</v>
+        <v>117.26</v>
       </c>
       <c r="M50" s="39" t="n">
         <f aca="false">M46*(1-M48-M24)</f>
-        <v>121.26</v>
+        <v>115.62</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15999,28 +15999,28 @@
         <v>0</v>
       </c>
       <c r="F73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="G73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="H73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="I73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="J73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="K73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="L73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="M73" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16040,35 +16040,35 @@
       </c>
       <c r="F74" s="39" t="n">
         <f aca="false">F72*(1-F73-F24)</f>
-        <v>126.48</v>
+        <v>120.528</v>
       </c>
       <c r="G74" s="39" t="n">
         <f aca="false">G72*(1-G73-G24)</f>
-        <v>124.848</v>
+        <v>118.9728</v>
       </c>
       <c r="H74" s="39" t="n">
         <f aca="false">H72*(1-H73-H24)</f>
-        <v>123.216</v>
+        <v>117.4176</v>
       </c>
       <c r="I74" s="39" t="n">
         <f aca="false">I72*(1-I73-I24)</f>
-        <v>121.584</v>
+        <v>115.8624</v>
       </c>
       <c r="J74" s="39" t="n">
         <f aca="false">J72*(1-J73-J24)</f>
-        <v>119.952</v>
+        <v>114.3072</v>
       </c>
       <c r="K74" s="39" t="n">
         <f aca="false">K72*(1-K73-K24)</f>
-        <v>118.32</v>
+        <v>112.752</v>
       </c>
       <c r="L74" s="39" t="n">
         <f aca="false">L72*(1-L73-L24)</f>
-        <v>116.688</v>
+        <v>111.1968</v>
       </c>
       <c r="M74" s="39" t="n">
         <f aca="false">M72*(1-M73-M24)</f>
-        <v>115.056</v>
+        <v>109.6416</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16130,28 +16130,28 @@
         <v>0</v>
       </c>
       <c r="F76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="G76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="H76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="I76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="J76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="K76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="L76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="M76" s="21" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16171,35 +16171,35 @@
       </c>
       <c r="F77" s="39" t="n">
         <f aca="false">F75*(1-F76-F24)</f>
-        <v>131.75</v>
+        <v>125.55</v>
       </c>
       <c r="G77" s="39" t="n">
         <f aca="false">G75*(1-G76-G24)</f>
-        <v>130.05</v>
+        <v>123.93</v>
       </c>
       <c r="H77" s="39" t="n">
         <f aca="false">H75*(1-H76-H24)</f>
-        <v>128.35</v>
+        <v>122.31</v>
       </c>
       <c r="I77" s="39" t="n">
         <f aca="false">I75*(1-I76-I24)</f>
-        <v>126.65</v>
+        <v>120.69</v>
       </c>
       <c r="J77" s="39" t="n">
         <f aca="false">J75*(1-J76-J24)</f>
-        <v>124.95</v>
+        <v>119.07</v>
       </c>
       <c r="K77" s="39" t="n">
         <f aca="false">K75*(1-K76-K24)</f>
-        <v>123.25</v>
+        <v>117.45</v>
       </c>
       <c r="L77" s="39" t="n">
         <f aca="false">L75*(1-L76-L24)</f>
-        <v>121.55</v>
+        <v>115.83</v>
       </c>
       <c r="M77" s="39" t="n">
         <f aca="false">M75*(1-M76-M24)</f>
-        <v>119.85</v>
+        <v>114.21</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16856,39 +16856,39 @@
       </c>
       <c r="E9" s="39" t="n">
         <f aca="false">-(Assumptions!E43*Assumptions!E49+Assumptions!E44*Assumptions!E50)</f>
-        <v>-644.49</v>
+        <v>-613.8</v>
       </c>
       <c r="F9" s="39" t="n">
         <f aca="false">-(Assumptions!F43*Assumptions!F49+Assumptions!F44*Assumptions!F50)</f>
-        <v>-1503.531</v>
+        <v>-1432.665</v>
       </c>
       <c r="G9" s="39" t="n">
         <f aca="false">-(Assumptions!G43*Assumptions!G49+Assumptions!G44*Assumptions!G50)</f>
-        <v>-1801.116</v>
+        <v>-1716.2928</v>
       </c>
       <c r="H9" s="39" t="n">
         <f aca="false">-(Assumptions!H43*Assumptions!H49+Assumptions!H44*Assumptions!H50)</f>
-        <v>-1940.3802</v>
+        <v>-1849.0554</v>
       </c>
       <c r="I9" s="39" t="n">
         <f aca="false">-(Assumptions!I43*Assumptions!I49+Assumptions!I44*Assumptions!I50)</f>
-        <v>-1937.745</v>
+        <v>-1846.557</v>
       </c>
       <c r="J9" s="39" t="n">
         <f aca="false">-(Assumptions!J43*Assumptions!J49+Assumptions!J44*Assumptions!J50)</f>
-        <v>-1911.735</v>
+        <v>-1821.771</v>
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">-(Assumptions!K43*Assumptions!K49+Assumptions!K44*Assumptions!K50)</f>
-        <v>-1885.725</v>
+        <v>-1796.985</v>
       </c>
       <c r="L9" s="39" t="n">
         <f aca="false">-(Assumptions!L43*Assumptions!L49+Assumptions!L44*Assumptions!L50)</f>
-        <v>-1859.715</v>
+        <v>-1772.199</v>
       </c>
       <c r="M9" s="39" t="n">
         <f aca="false">-(Assumptions!M43*Assumptions!M49+Assumptions!M44*Assumptions!M50)</f>
-        <v>-1833.705</v>
+        <v>-1747.413</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16953,39 +16953,39 @@
       </c>
       <c r="E12" s="57" t="n">
         <f aca="false">E8+E9</f>
-        <v>122.76</v>
+        <v>153.45</v>
       </c>
       <c r="F12" s="57" t="n">
         <f aca="false">F8+F9</f>
-        <v>268.119</v>
+        <v>338.985</v>
       </c>
       <c r="G12" s="57" t="n">
         <f aca="false">G8+G9</f>
-        <v>319.464</v>
+        <v>404.2872</v>
       </c>
       <c r="H12" s="57" t="n">
         <f aca="false">H8+H9</f>
-        <v>342.7398</v>
+        <v>434.0646</v>
       </c>
       <c r="I12" s="57" t="n">
         <f aca="false">I8+I9</f>
-        <v>341.955</v>
+        <v>433.143</v>
       </c>
       <c r="J12" s="57" t="n">
         <f aca="false">J8+J9</f>
-        <v>337.365</v>
+        <v>427.329</v>
       </c>
       <c r="K12" s="57" t="n">
         <f aca="false">K8+K9</f>
-        <v>332.775</v>
+        <v>421.515</v>
       </c>
       <c r="L12" s="57" t="n">
         <f aca="false">L8+L9</f>
-        <v>328.185</v>
+        <v>415.701</v>
       </c>
       <c r="M12" s="57" t="n">
         <f aca="false">M8+M9</f>
-        <v>323.595</v>
+        <v>409.887</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17133,11 +17133,11 @@
       </c>
       <c r="E16" s="39" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(E12+E13))</f>
-        <v>123.275</v>
+        <v>92.5850000000001</v>
       </c>
       <c r="F16" s="39" t="n">
         <f aca="false">MAX(0,Assumptions!$C$85-(F12+F13))</f>
-        <v>38.1800000000001</v>
+        <v>0</v>
       </c>
       <c r="G16" s="39" t="n">
         <f aca="false">0</f>
@@ -17182,35 +17182,35 @@
       </c>
       <c r="F17" s="57" t="n">
         <f aca="false">F12+F13+F15+F16</f>
-        <v>171.986</v>
+        <v>204.672</v>
       </c>
       <c r="G17" s="57" t="n">
         <f aca="false">G12+G13+G15+G16</f>
-        <v>164.2152</v>
+        <v>249.0384</v>
       </c>
       <c r="H17" s="57" t="n">
         <f aca="false">H12+H13+H15+H16</f>
-        <v>177.7386</v>
+        <v>269.0634</v>
       </c>
       <c r="I17" s="57" t="n">
         <f aca="false">I12+I13+I15+I16</f>
-        <v>177.159</v>
+        <v>268.347</v>
       </c>
       <c r="J17" s="57" t="n">
         <f aca="false">J12+J13+J15+J16</f>
-        <v>174.405</v>
+        <v>264.369</v>
       </c>
       <c r="K17" s="57" t="n">
         <f aca="false">K12+K13+K15+K16</f>
-        <v>171.651</v>
+        <v>260.391</v>
       </c>
       <c r="L17" s="57" t="n">
         <f aca="false">L12+L13+L15+L16</f>
-        <v>168.897</v>
+        <v>256.413</v>
       </c>
       <c r="M17" s="57" t="n">
         <f aca="false">M12+M13+M15+M16</f>
-        <v>166.143</v>
+        <v>252.435</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17227,35 +17227,35 @@
       </c>
       <c r="F18" s="58" t="n">
         <f aca="false">IF(F8=0,0,F17/F8)</f>
-        <v>0.097076736375695</v>
+        <v>0.115526204385742</v>
       </c>
       <c r="G18" s="58" t="n">
         <f aca="false">IF(G8=0,0,G17/G8)</f>
-        <v>0.0774388139094023</v>
+        <v>0.117438813909402</v>
       </c>
       <c r="H18" s="58" t="n">
         <f aca="false">IF(H8=0,0,H17/H8)</f>
-        <v>0.0778489961105856</v>
+        <v>0.117848996110585</v>
       </c>
       <c r="I18" s="58" t="n">
         <f aca="false">IF(I8=0,0,I17/I8)</f>
-        <v>0.0777115409922358</v>
+        <v>0.117711540992236</v>
       </c>
       <c r="J18" s="58" t="n">
         <f aca="false">IF(J8=0,0,J17/J8)</f>
-        <v>0.0775443510737629</v>
+        <v>0.117544351073763</v>
       </c>
       <c r="K18" s="58" t="n">
         <f aca="false">IF(K8=0,0,K17/K8)</f>
-        <v>0.0773725490196079</v>
+        <v>0.117372549019608</v>
       </c>
       <c r="L18" s="58" t="n">
         <f aca="false">IF(L8=0,0,L17/L8)</f>
-        <v>0.0771959413135884</v>
+        <v>0.117195941313588</v>
       </c>
       <c r="M18" s="58" t="n">
         <f aca="false">IF(M8=0,0,M17/M8)</f>
-        <v>0.0770143234598803</v>
+        <v>0.11701432345988</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17317,35 +17317,35 @@
       </c>
       <c r="F20" s="57" t="n">
         <f aca="false">F17+F19</f>
-        <v>686.336</v>
+        <v>719.022</v>
       </c>
       <c r="G20" s="57" t="n">
         <f aca="false">G17+G19</f>
-        <v>787.9152</v>
+        <v>872.7384</v>
       </c>
       <c r="H20" s="57" t="n">
         <f aca="false">H17+H19</f>
-        <v>688.0386</v>
+        <v>779.3634</v>
       </c>
       <c r="I20" s="57" t="n">
         <f aca="false">I17+I19</f>
-        <v>521.409</v>
+        <v>612.597</v>
       </c>
       <c r="J20" s="57" t="n">
         <f aca="false">J17+J19</f>
-        <v>346.53</v>
+        <v>436.494</v>
       </c>
       <c r="K20" s="57" t="n">
         <f aca="false">K17+K19</f>
-        <v>171.651</v>
+        <v>260.391</v>
       </c>
       <c r="L20" s="57" t="n">
         <f aca="false">L17+L19</f>
-        <v>168.897</v>
+        <v>256.413</v>
       </c>
       <c r="M20" s="57" t="n">
         <f aca="false">M17+M19</f>
-        <v>166.143</v>
+        <v>252.435</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17414,35 +17414,35 @@
       </c>
       <c r="F24" s="39" t="n">
         <f aca="false">MAX(0,F17)</f>
-        <v>171.986</v>
+        <v>204.672</v>
       </c>
       <c r="G24" s="39" t="n">
         <f aca="false">MAX(0,G17)</f>
-        <v>164.2152</v>
+        <v>249.0384</v>
       </c>
       <c r="H24" s="39" t="n">
         <f aca="false">MAX(0,H17)</f>
-        <v>177.7386</v>
+        <v>269.0634</v>
       </c>
       <c r="I24" s="39" t="n">
         <f aca="false">MAX(0,I17)</f>
-        <v>177.159</v>
+        <v>268.347</v>
       </c>
       <c r="J24" s="39" t="n">
         <f aca="false">MAX(0,J17)</f>
-        <v>174.405</v>
+        <v>264.369</v>
       </c>
       <c r="K24" s="39" t="n">
         <f aca="false">MAX(0,K17)</f>
-        <v>171.651</v>
+        <v>260.391</v>
       </c>
       <c r="L24" s="39" t="n">
         <f aca="false">MAX(0,L17)</f>
-        <v>168.897</v>
+        <v>256.413</v>
       </c>
       <c r="M24" s="39" t="n">
         <f aca="false">MAX(0,M17)</f>
-        <v>166.143</v>
+        <v>252.435</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17463,31 +17463,31 @@
       </c>
       <c r="G25" s="39" t="n">
         <f aca="false">F28</f>
-        <v>3573.36</v>
+        <v>3547.2112</v>
       </c>
       <c r="H25" s="39" t="n">
         <f aca="false">G28</f>
-        <v>3441.98784</v>
+        <v>3347.98048</v>
       </c>
       <c r="I25" s="39" t="n">
         <f aca="false">H28</f>
-        <v>3299.79696</v>
+        <v>3132.72976</v>
       </c>
       <c r="J25" s="39" t="n">
         <f aca="false">I28</f>
-        <v>3158.06976</v>
+        <v>2918.05216</v>
       </c>
       <c r="K25" s="39" t="n">
         <f aca="false">J28</f>
-        <v>3018.54576</v>
+        <v>2706.55696</v>
       </c>
       <c r="L25" s="39" t="n">
         <f aca="false">K28</f>
-        <v>2881.22496</v>
+        <v>2498.24416</v>
       </c>
       <c r="M25" s="39" t="n">
         <f aca="false">L28</f>
-        <v>2746.10736</v>
+        <v>2293.11376</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17504,35 +17504,35 @@
       </c>
       <c r="F26" s="39" t="n">
         <f aca="false">MIN(F25,F24*Assumptions!$C$90)</f>
-        <v>137.5888</v>
+        <v>163.7376</v>
       </c>
       <c r="G26" s="39" t="n">
         <f aca="false">MIN(G25,G24*Assumptions!$C$90)</f>
-        <v>131.37216</v>
+        <v>199.23072</v>
       </c>
       <c r="H26" s="39" t="n">
         <f aca="false">MIN(H25,H24*Assumptions!$C$90)</f>
-        <v>142.19088</v>
+        <v>215.25072</v>
       </c>
       <c r="I26" s="39" t="n">
         <f aca="false">MIN(I25,I24*Assumptions!$C$90)</f>
-        <v>141.7272</v>
+        <v>214.6776</v>
       </c>
       <c r="J26" s="39" t="n">
         <f aca="false">MIN(J25,J24*Assumptions!$C$90)</f>
-        <v>139.524</v>
+        <v>211.4952</v>
       </c>
       <c r="K26" s="39" t="n">
         <f aca="false">MIN(K25,K24*Assumptions!$C$90)</f>
-        <v>137.3208</v>
+        <v>208.3128</v>
       </c>
       <c r="L26" s="39" t="n">
         <f aca="false">MIN(L25,L24*Assumptions!$C$90)</f>
-        <v>135.1176</v>
+        <v>205.1304</v>
       </c>
       <c r="M26" s="39" t="n">
         <f aca="false">MIN(M25,M24*Assumptions!$C$90)</f>
-        <v>132.9144</v>
+        <v>201.948</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17594,35 +17594,35 @@
       </c>
       <c r="F28" s="39" t="n">
         <f aca="false">F25-F26+F27</f>
-        <v>3573.36</v>
+        <v>3547.2112</v>
       </c>
       <c r="G28" s="39" t="n">
         <f aca="false">G25-G26+G27</f>
-        <v>3441.98784</v>
+        <v>3347.98048</v>
       </c>
       <c r="H28" s="39" t="n">
         <f aca="false">H25-H26+H27</f>
-        <v>3299.79696</v>
+        <v>3132.72976</v>
       </c>
       <c r="I28" s="39" t="n">
         <f aca="false">I25-I26+I27</f>
-        <v>3158.06976</v>
+        <v>2918.05216</v>
       </c>
       <c r="J28" s="39" t="n">
         <f aca="false">J25-J26+J27</f>
-        <v>3018.54576</v>
+        <v>2706.55696</v>
       </c>
       <c r="K28" s="39" t="n">
         <f aca="false">K25-K26+K27</f>
-        <v>2881.22496</v>
+        <v>2498.24416</v>
       </c>
       <c r="L28" s="39" t="n">
         <f aca="false">L25-L26+L27</f>
-        <v>2746.10736</v>
+        <v>2293.11376</v>
       </c>
       <c r="M28" s="39" t="n">
         <f aca="false">M25-M26+M27</f>
-        <v>2613.19296</v>
+        <v>2091.16576</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17639,35 +17639,35 @@
       </c>
       <c r="F29" s="39" t="n">
         <f aca="false">F24-F26</f>
-        <v>34.3972</v>
+        <v>40.9344</v>
       </c>
       <c r="G29" s="39" t="n">
         <f aca="false">G24-G26</f>
-        <v>32.8430400000001</v>
+        <v>49.80768</v>
       </c>
       <c r="H29" s="39" t="n">
         <f aca="false">H24-H26</f>
-        <v>35.5477200000001</v>
+        <v>53.8126799999999</v>
       </c>
       <c r="I29" s="39" t="n">
         <f aca="false">I24-I26</f>
-        <v>35.4318</v>
+        <v>53.6693999999999</v>
       </c>
       <c r="J29" s="39" t="n">
         <f aca="false">J24-J26</f>
-        <v>34.881</v>
+        <v>52.8738</v>
       </c>
       <c r="K29" s="39" t="n">
         <f aca="false">K24-K26</f>
-        <v>34.3302</v>
+        <v>52.0782</v>
       </c>
       <c r="L29" s="39" t="n">
         <f aca="false">L24-L26</f>
-        <v>33.7794</v>
+        <v>51.2825999999999</v>
       </c>
       <c r="M29" s="39" t="n">
         <f aca="false">M24-M26</f>
-        <v>33.2285999999999</v>
+        <v>50.4869999999999</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17684,35 +17684,35 @@
       </c>
       <c r="F30" s="39" t="n">
         <f aca="false">-F29*Assumptions!$C$87</f>
-        <v>-7.911356</v>
+        <v>-9.414912</v>
       </c>
       <c r="G30" s="39" t="n">
         <f aca="false">-G29*Assumptions!$C$87</f>
-        <v>-7.55389920000001</v>
+        <v>-11.4557664</v>
       </c>
       <c r="H30" s="39" t="n">
         <f aca="false">-H29*Assumptions!$C$87</f>
-        <v>-8.17597560000001</v>
+        <v>-12.3769164</v>
       </c>
       <c r="I30" s="39" t="n">
         <f aca="false">-I29*Assumptions!$C$87</f>
-        <v>-8.149314</v>
+        <v>-12.343962</v>
       </c>
       <c r="J30" s="39" t="n">
         <f aca="false">-J29*Assumptions!$C$87</f>
-        <v>-8.02263000000001</v>
+        <v>-12.160974</v>
       </c>
       <c r="K30" s="39" t="n">
         <f aca="false">-K29*Assumptions!$C$87</f>
-        <v>-7.89594600000001</v>
+        <v>-11.977986</v>
       </c>
       <c r="L30" s="39" t="n">
         <f aca="false">-L29*Assumptions!$C$87</f>
-        <v>-7.769262</v>
+        <v>-11.794998</v>
       </c>
       <c r="M30" s="39" t="n">
         <f aca="false">-M29*Assumptions!$C$87</f>
-        <v>-7.64257799999999</v>
+        <v>-11.61201</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17729,35 +17729,35 @@
       </c>
       <c r="F31" s="57" t="n">
         <f aca="false">F20+F30</f>
-        <v>678.424644</v>
+        <v>709.607088</v>
       </c>
       <c r="G31" s="57" t="n">
         <f aca="false">G20+G30</f>
-        <v>780.3613008</v>
+        <v>861.2826336</v>
       </c>
       <c r="H31" s="57" t="n">
         <f aca="false">H20+H30</f>
-        <v>679.8626244</v>
+        <v>766.9864836</v>
       </c>
       <c r="I31" s="57" t="n">
         <f aca="false">I20+I30</f>
-        <v>513.259686</v>
+        <v>600.253038</v>
       </c>
       <c r="J31" s="57" t="n">
         <f aca="false">J20+J30</f>
-        <v>338.50737</v>
+        <v>424.333026</v>
       </c>
       <c r="K31" s="57" t="n">
         <f aca="false">K20+K30</f>
-        <v>163.755054</v>
+        <v>248.413014</v>
       </c>
       <c r="L31" s="57" t="n">
         <f aca="false">L20+L30</f>
-        <v>161.127738</v>
+        <v>244.618002</v>
       </c>
       <c r="M31" s="57" t="n">
         <f aca="false">M20+M30</f>
-        <v>158.500422</v>
+        <v>240.82299</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18044,35 +18044,35 @@
       </c>
       <c r="F38" s="60" t="n">
         <f aca="false">F31+F32+F33+F34+F35+F37</f>
-        <v>466.629144</v>
+        <v>497.811588</v>
       </c>
       <c r="G38" s="60" t="n">
         <f aca="false">G31+G32+G33+G34+G35+G37</f>
-        <v>692.4184008</v>
+        <v>773.3397336</v>
       </c>
       <c r="H38" s="60" t="n">
         <f aca="false">H31+H32+H33+H34+H35+H37</f>
-        <v>615.0020244</v>
+        <v>702.1258836</v>
       </c>
       <c r="I38" s="60" t="n">
         <f aca="false">I31+I32+I33+I34+I35+I37</f>
-        <v>473.395686</v>
+        <v>560.389038</v>
       </c>
       <c r="J38" s="60" t="n">
         <f aca="false">J31+J32+J33+J34+J35+J37</f>
-        <v>303.63837</v>
+        <v>389.464026</v>
       </c>
       <c r="K38" s="60" t="n">
         <f aca="false">K31+K32+K33+K34+K35+K37</f>
-        <v>129.804054</v>
+        <v>214.462014</v>
       </c>
       <c r="L38" s="60" t="n">
         <f aca="false">L31+L32+L33+L34+L35+L37</f>
-        <v>128.094738</v>
+        <v>211.585002</v>
       </c>
       <c r="M38" s="60" t="n">
         <f aca="false">M31+M32+M33+M34+M35+M37</f>
-        <v>126.385422</v>
+        <v>208.70799</v>
       </c>
     </row>
   </sheetData>
@@ -18311,35 +18311,35 @@
       </c>
       <c r="F9" s="39" t="n">
         <f aca="false">-(Assumptions!F69*Assumptions!F74+Assumptions!F70*Assumptions!F77)</f>
-        <v>-678.7233</v>
+        <v>-646.78338</v>
       </c>
       <c r="G9" s="39" t="n">
         <f aca="false">-(Assumptions!G69*Assumptions!G74+Assumptions!G70*Assumptions!G77)</f>
-        <v>-2158.77798</v>
+        <v>-2057.188428</v>
       </c>
       <c r="H9" s="39" t="n">
         <f aca="false">-(Assumptions!H69*Assumptions!H74+Assumptions!H70*Assumptions!H77)</f>
-        <v>-2755.03275</v>
+        <v>-2625.38415</v>
       </c>
       <c r="I9" s="39" t="n">
         <f aca="false">-(Assumptions!I69*Assumptions!I74+Assumptions!I70*Assumptions!I77)</f>
-        <v>-3081.01455</v>
+        <v>-2936.02563</v>
       </c>
       <c r="J9" s="39" t="n">
         <f aca="false">-(Assumptions!J69*Assumptions!J74+Assumptions!J70*Assumptions!J77)</f>
-        <v>-3039.65865</v>
+        <v>-2896.61589</v>
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">-(Assumptions!K69*Assumptions!K74+Assumptions!K70*Assumptions!K77)</f>
-        <v>-2998.30275</v>
+        <v>-2857.20615</v>
       </c>
       <c r="L9" s="39" t="n">
         <f aca="false">-(Assumptions!L69*Assumptions!L74+Assumptions!L70*Assumptions!L77)</f>
-        <v>-2956.94685</v>
+        <v>-2817.79641</v>
       </c>
       <c r="M9" s="39" t="n">
         <f aca="false">-(Assumptions!M69*Assumptions!M74+Assumptions!M70*Assumptions!M77)</f>
-        <v>-2915.59095</v>
+        <v>-2778.38667</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18408,35 +18408,35 @@
       </c>
       <c r="F12" s="57" t="n">
         <f aca="false">F8+F9</f>
-        <v>119.7747</v>
+        <v>151.71462</v>
       </c>
       <c r="G12" s="57" t="n">
         <f aca="false">G8+G9</f>
-        <v>380.96082</v>
+        <v>482.550372</v>
       </c>
       <c r="H12" s="57" t="n">
         <f aca="false">H8+H9</f>
-        <v>486.18225</v>
+        <v>615.83085</v>
       </c>
       <c r="I12" s="57" t="n">
         <f aca="false">I8+I9</f>
-        <v>543.70845</v>
+        <v>688.697369999999</v>
       </c>
       <c r="J12" s="57" t="n">
         <f aca="false">J8+J9</f>
-        <v>536.410350000001</v>
+        <v>679.45311</v>
       </c>
       <c r="K12" s="57" t="n">
         <f aca="false">K8+K9</f>
-        <v>529.11225</v>
+        <v>670.20885</v>
       </c>
       <c r="L12" s="57" t="n">
         <f aca="false">L8+L9</f>
-        <v>521.81415</v>
+        <v>660.96459</v>
       </c>
       <c r="M12" s="57" t="n">
         <f aca="false">M8+M9</f>
-        <v>514.51605</v>
+        <v>651.72033</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18588,35 +18588,35 @@
       </c>
       <c r="F16" s="57" t="n">
         <f aca="false">F12+F13+F15</f>
-        <v>5.16482000000008</v>
+        <v>37.10474</v>
       </c>
       <c r="G16" s="57" t="n">
         <f aca="false">G12+G13+G15</f>
-        <v>161.876492</v>
+        <v>263.466044</v>
       </c>
       <c r="H16" s="57" t="n">
         <f aca="false">H12+H13+H15</f>
-        <v>225.00935</v>
+        <v>354.65795</v>
       </c>
       <c r="I16" s="57" t="n">
         <f aca="false">I12+I13+I15</f>
-        <v>259.52507</v>
+        <v>404.513989999999</v>
       </c>
       <c r="J16" s="57" t="n">
         <f aca="false">J12+J13+J15</f>
-        <v>255.146210000001</v>
+        <v>398.18897</v>
       </c>
       <c r="K16" s="57" t="n">
         <f aca="false">K12+K13+K15</f>
-        <v>250.76735</v>
+        <v>391.86395</v>
       </c>
       <c r="L16" s="57" t="n">
         <f aca="false">L12+L13+L15</f>
-        <v>246.38849</v>
+        <v>385.53893</v>
       </c>
       <c r="M16" s="57" t="n">
         <f aca="false">M12+M13+M15</f>
-        <v>242.00963</v>
+        <v>379.21391</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18633,35 +18633,35 @@
       </c>
       <c r="F17" s="58" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.0064681689872737</v>
+        <v>0.0464681689872736</v>
       </c>
       <c r="G17" s="58" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.0637374567809886</v>
+        <v>0.103737456780989</v>
       </c>
       <c r="H17" s="58" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.0694212972604409</v>
+        <v>0.109421297260441</v>
       </c>
       <c r="I17" s="58" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.0715985938787598</v>
+        <v>0.11159859387876</v>
       </c>
       <c r="J17" s="58" t="n">
         <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.0713482346118043</v>
+        <v>0.111348234611804</v>
       </c>
       <c r="K17" s="58" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0710909688823118</v>
+        <v>0.111090968882312</v>
       </c>
       <c r="L17" s="58" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0708265069086379</v>
+        <v>0.110826506908638</v>
       </c>
       <c r="M17" s="58" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0705545424676257</v>
+        <v>0.110554542467626</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18723,35 +18723,35 @@
       </c>
       <c r="F19" s="57" t="n">
         <f aca="false">F16+F18</f>
-        <v>245.73482</v>
+        <v>277.67474</v>
       </c>
       <c r="G19" s="57" t="n">
         <f aca="false">G16+G18</f>
-        <v>937.046492</v>
+        <v>1038.636044</v>
       </c>
       <c r="H19" s="57" t="n">
         <f aca="false">H16+H18</f>
-        <v>976.7906</v>
+        <v>1106.4392</v>
       </c>
       <c r="I19" s="57" t="n">
         <f aca="false">I16+I18</f>
-        <v>827.53757</v>
+        <v>972.526489999999</v>
       </c>
       <c r="J19" s="57" t="n">
         <f aca="false">J16+J18</f>
-        <v>539.152460000001</v>
+        <v>682.19522</v>
       </c>
       <c r="K19" s="57" t="n">
         <f aca="false">K16+K18</f>
-        <v>250.76735</v>
+        <v>391.86395</v>
       </c>
       <c r="L19" s="57" t="n">
         <f aca="false">L16+L18</f>
-        <v>246.38849</v>
+        <v>385.53893</v>
       </c>
       <c r="M19" s="57" t="n">
         <f aca="false">M16+M18</f>
-        <v>242.00963</v>
+        <v>379.21391</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18820,35 +18820,35 @@
       </c>
       <c r="F23" s="39" t="n">
         <f aca="false">MAX(0,F16)</f>
-        <v>5.16482000000008</v>
+        <v>37.10474</v>
       </c>
       <c r="G23" s="39" t="n">
         <f aca="false">MAX(0,G16)</f>
-        <v>161.876492</v>
+        <v>263.466044</v>
       </c>
       <c r="H23" s="39" t="n">
         <f aca="false">MAX(0,H16)</f>
-        <v>225.00935</v>
+        <v>354.65795</v>
       </c>
       <c r="I23" s="39" t="n">
         <f aca="false">MAX(0,I16)</f>
-        <v>259.52507</v>
+        <v>404.513989999999</v>
       </c>
       <c r="J23" s="39" t="n">
         <f aca="false">MAX(0,J16)</f>
-        <v>255.146210000001</v>
+        <v>398.18897</v>
       </c>
       <c r="K23" s="39" t="n">
         <f aca="false">MAX(0,K16)</f>
-        <v>250.76735</v>
+        <v>391.86395</v>
       </c>
       <c r="L23" s="39" t="n">
         <f aca="false">MAX(0,L16)</f>
-        <v>246.38849</v>
+        <v>385.53893</v>
       </c>
       <c r="M23" s="39" t="n">
         <f aca="false">MAX(0,M16)</f>
-        <v>242.00963</v>
+        <v>379.21391</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18869,7 +18869,7 @@
       </c>
       <c r="G24" s="39" t="n">
         <f aca="false">F27</f>
-        <v>55.8981439999999</v>
+        <v>30.346208</v>
       </c>
       <c r="H24" s="39" t="n">
         <f aca="false">G27</f>
@@ -18910,11 +18910,11 @@
       </c>
       <c r="F25" s="39" t="n">
         <f aca="false">MIN(F24,F23*Assumptions!$C$90)</f>
-        <v>4.13185600000006</v>
+        <v>29.683792</v>
       </c>
       <c r="G25" s="39" t="n">
         <f aca="false">MIN(G24,G23*Assumptions!$C$90)</f>
-        <v>55.8981439999999</v>
+        <v>30.346208</v>
       </c>
       <c r="H25" s="39" t="n">
         <f aca="false">MIN(H24,H23*Assumptions!$C$90)</f>
@@ -19000,7 +19000,7 @@
       </c>
       <c r="F27" s="39" t="n">
         <f aca="false">F24-F25+F26</f>
-        <v>55.8981439999999</v>
+        <v>30.346208</v>
       </c>
       <c r="G27" s="39" t="n">
         <f aca="false">G24-G25+G26</f>
@@ -19045,35 +19045,35 @@
       </c>
       <c r="F28" s="39" t="n">
         <f aca="false">F23-F25</f>
-        <v>1.03296400000001</v>
+        <v>7.420948</v>
       </c>
       <c r="G28" s="39" t="n">
         <f aca="false">G23-G25</f>
-        <v>105.978348</v>
+        <v>233.119836</v>
       </c>
       <c r="H28" s="39" t="n">
         <f aca="false">H23-H25</f>
-        <v>225.00935</v>
+        <v>354.65795</v>
       </c>
       <c r="I28" s="39" t="n">
         <f aca="false">I23-I25</f>
-        <v>259.52507</v>
+        <v>404.513989999999</v>
       </c>
       <c r="J28" s="39" t="n">
         <f aca="false">J23-J25</f>
-        <v>255.146210000001</v>
+        <v>398.18897</v>
       </c>
       <c r="K28" s="39" t="n">
         <f aca="false">K23-K25</f>
-        <v>250.76735</v>
+        <v>391.86395</v>
       </c>
       <c r="L28" s="39" t="n">
         <f aca="false">L23-L25</f>
-        <v>246.38849</v>
+        <v>385.53893</v>
       </c>
       <c r="M28" s="39" t="n">
         <f aca="false">M23-M25</f>
-        <v>242.00963</v>
+        <v>379.21391</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19090,35 +19090,35 @@
       </c>
       <c r="F29" s="39" t="n">
         <f aca="false">-F28*Assumptions!$C$87</f>
-        <v>-0.237581720000003</v>
+        <v>-1.70681804</v>
       </c>
       <c r="G29" s="39" t="n">
         <f aca="false">-G28*Assumptions!$C$87</f>
-        <v>-24.37502004</v>
+        <v>-53.6175622799999</v>
       </c>
       <c r="H29" s="39" t="n">
         <f aca="false">-H28*Assumptions!$C$87</f>
-        <v>-51.7521505</v>
+        <v>-81.5713285000001</v>
       </c>
       <c r="I29" s="39" t="n">
         <f aca="false">-I28*Assumptions!$C$87</f>
-        <v>-59.6907660999999</v>
+        <v>-93.0382176999999</v>
       </c>
       <c r="J29" s="39" t="n">
         <f aca="false">-J28*Assumptions!$C$87</f>
-        <v>-58.6836283000001</v>
+        <v>-91.5834631000001</v>
       </c>
       <c r="K29" s="39" t="n">
         <f aca="false">-K28*Assumptions!$C$87</f>
-        <v>-57.6764904999999</v>
+        <v>-90.1287084999999</v>
       </c>
       <c r="L29" s="39" t="n">
         <f aca="false">-L28*Assumptions!$C$87</f>
-        <v>-56.6693527000001</v>
+        <v>-88.6739538999999</v>
       </c>
       <c r="M29" s="39" t="n">
         <f aca="false">-M28*Assumptions!$C$87</f>
-        <v>-55.6622149</v>
+        <v>-87.2191992999999</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19135,35 +19135,35 @@
       </c>
       <c r="F30" s="57" t="n">
         <f aca="false">F19+F29</f>
-        <v>245.49723828</v>
+        <v>275.96792196</v>
       </c>
       <c r="G30" s="57" t="n">
         <f aca="false">G19+G29</f>
-        <v>912.67147196</v>
+        <v>985.01848172</v>
       </c>
       <c r="H30" s="57" t="n">
         <f aca="false">H19+H29</f>
-        <v>925.0384495</v>
+        <v>1024.8678715</v>
       </c>
       <c r="I30" s="57" t="n">
         <f aca="false">I19+I29</f>
-        <v>767.8468039</v>
+        <v>879.4882723</v>
       </c>
       <c r="J30" s="57" t="n">
         <f aca="false">J19+J29</f>
-        <v>480.4688317</v>
+        <v>590.6117569</v>
       </c>
       <c r="K30" s="57" t="n">
         <f aca="false">K19+K29</f>
-        <v>193.0908595</v>
+        <v>301.7352415</v>
       </c>
       <c r="L30" s="57" t="n">
         <f aca="false">L19+L29</f>
-        <v>189.7191373</v>
+        <v>296.8649761</v>
       </c>
       <c r="M30" s="57" t="n">
         <f aca="false">M19+M29</f>
-        <v>186.3474151</v>
+        <v>291.9947107</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19450,35 +19450,35 @@
       </c>
       <c r="F37" s="60" t="n">
         <f aca="false">F30+F31+F32+F33+F34+F36</f>
-        <v>-101.53240172</v>
+        <v>-71.06171804</v>
       </c>
       <c r="G37" s="60" t="n">
         <f aca="false">G30+G31+G32+G33+G34+G36</f>
-        <v>641.99318796</v>
+        <v>714.34019772</v>
       </c>
       <c r="H37" s="60" t="n">
         <f aca="false">H30+H31+H32+H33+H34+H36</f>
-        <v>789.2805695</v>
+        <v>889.1099915</v>
       </c>
       <c r="I37" s="60" t="n">
         <f aca="false">I30+I31+I32+I33+I34+I36</f>
-        <v>668.2789139</v>
+        <v>779.9203823</v>
       </c>
       <c r="J37" s="60" t="n">
         <f aca="false">J30+J31+J32+J33+J34+J36</f>
-        <v>447.1848617</v>
+        <v>557.3277869</v>
       </c>
       <c r="K37" s="60" t="n">
         <f aca="false">K30+K31+K32+K33+K34+K36</f>
-        <v>161.2665095</v>
+        <v>269.9108915</v>
       </c>
       <c r="L37" s="60" t="n">
         <f aca="false">L30+L31+L32+L33+L34+L36</f>
-        <v>159.3544073</v>
+        <v>266.5002461</v>
       </c>
       <c r="M37" s="60" t="n">
         <f aca="false">M30+M31+M32+M33+M34+M36</f>
-        <v>157.4423051</v>
+        <v>263.0896007</v>
       </c>
     </row>
   </sheetData>
@@ -19814,35 +19814,35 @@
       </c>
       <c r="F13" s="39" t="n">
         <f aca="false">SKBA!F17+SKOT!F16</f>
-        <v>177.15082</v>
+        <v>241.77674</v>
       </c>
       <c r="G13" s="39" t="n">
         <f aca="false">SKBA!G17+SKOT!G16</f>
-        <v>326.091692</v>
+        <v>512.504444</v>
       </c>
       <c r="H13" s="39" t="n">
         <f aca="false">SKBA!H17+SKOT!H16</f>
-        <v>402.74795</v>
+        <v>623.72135</v>
       </c>
       <c r="I13" s="39" t="n">
         <f aca="false">SKBA!I17+SKOT!I16</f>
-        <v>436.68407</v>
+        <v>672.860989999999</v>
       </c>
       <c r="J13" s="39" t="n">
         <f aca="false">SKBA!J17+SKOT!J16</f>
-        <v>429.551210000001</v>
+        <v>662.55797</v>
       </c>
       <c r="K13" s="39" t="n">
         <f aca="false">SKBA!K17+SKOT!K16</f>
-        <v>422.41835</v>
+        <v>652.254949999999</v>
       </c>
       <c r="L13" s="39" t="n">
         <f aca="false">SKBA!L17+SKOT!L16</f>
-        <v>415.28549</v>
+        <v>641.951929999999</v>
       </c>
       <c r="M13" s="39" t="n">
         <f aca="false">SKBA!M17+SKOT!M16</f>
-        <v>408.15263</v>
+        <v>631.648909999999</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19859,35 +19859,35 @@
       </c>
       <c r="F14" s="58" t="n">
         <f aca="false">IF(F8=0,0,F13/F8)</f>
-        <v>0.0689263108583631</v>
+        <v>0.0940711352031089</v>
       </c>
       <c r="G14" s="58" t="n">
         <f aca="false">IF(G8=0,0,G13/G8)</f>
-        <v>0.0699719710162318</v>
+        <v>0.109971971016232</v>
       </c>
       <c r="H14" s="58" t="n">
         <f aca="false">IF(H8=0,0,H13/H8)</f>
-        <v>0.0729043314715708</v>
+        <v>0.112904331471571</v>
       </c>
       <c r="I14" s="58" t="n">
         <f aca="false">IF(I8=0,0,I13/I8)</f>
-        <v>0.0739588051194841</v>
+        <v>0.113958805119484</v>
       </c>
       <c r="J14" s="58" t="n">
         <f aca="false">IF(J8=0,0,J13/J8)</f>
-        <v>0.0737405575700895</v>
+        <v>0.113740557570089</v>
       </c>
       <c r="K14" s="58" t="n">
         <f aca="false">IF(K8=0,0,K13/K8)</f>
-        <v>0.0735162893986423</v>
+        <v>0.113516289398642</v>
       </c>
       <c r="L14" s="58" t="n">
         <f aca="false">IF(L8=0,0,L13/L8)</f>
-        <v>0.0732857479916304</v>
+        <v>0.11328574799163</v>
       </c>
       <c r="M14" s="58" t="n">
         <f aca="false">IF(M8=0,0,M13/M8)</f>
-        <v>0.0730486664028592</v>
+        <v>0.113048666402859</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19949,35 +19949,35 @@
       </c>
       <c r="F16" s="57" t="n">
         <f aca="false">SKBA!F20+SKOT!F19</f>
-        <v>932.07082</v>
+        <v>996.69674</v>
       </c>
       <c r="G16" s="57" t="n">
         <f aca="false">SKBA!G20+SKOT!G19</f>
-        <v>1724.961692</v>
+        <v>1911.374444</v>
       </c>
       <c r="H16" s="57" t="n">
         <f aca="false">SKBA!H20+SKOT!H19</f>
-        <v>1664.8292</v>
+        <v>1885.8026</v>
       </c>
       <c r="I16" s="57" t="n">
         <f aca="false">SKBA!I20+SKOT!I19</f>
-        <v>1348.94657</v>
+        <v>1585.12349</v>
       </c>
       <c r="J16" s="57" t="n">
         <f aca="false">SKBA!J20+SKOT!J19</f>
-        <v>885.682460000001</v>
+        <v>1118.68922</v>
       </c>
       <c r="K16" s="57" t="n">
         <f aca="false">SKBA!K20+SKOT!K19</f>
-        <v>422.41835</v>
+        <v>652.254949999999</v>
       </c>
       <c r="L16" s="57" t="n">
         <f aca="false">SKBA!L20+SKOT!L19</f>
-        <v>415.28549</v>
+        <v>641.951929999999</v>
       </c>
       <c r="M16" s="57" t="n">
         <f aca="false">SKBA!M20+SKOT!M19</f>
-        <v>408.15263</v>
+        <v>631.648909999999</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19994,35 +19994,35 @@
       </c>
       <c r="F17" s="58" t="n">
         <f aca="false">IF(F8=0,0,F16/F8)</f>
-        <v>0.362652586543654</v>
+        <v>0.3877974108884</v>
       </c>
       <c r="G17" s="58" t="n">
         <f aca="false">IF(G8=0,0,G16/G8)</f>
-        <v>0.37013813132269</v>
+        <v>0.41013813132269</v>
       </c>
       <c r="H17" s="58" t="n">
         <f aca="false">IF(H8=0,0,H16/H8)</f>
-        <v>0.301362824665774</v>
+        <v>0.341362824665774</v>
       </c>
       <c r="I17" s="58" t="n">
         <f aca="false">IF(I8=0,0,I16/I8)</f>
-        <v>0.228463741503615</v>
+        <v>0.268463741503615</v>
       </c>
       <c r="J17" s="58" t="n">
         <f aca="false">IF(J8=0,0,J16/J8)</f>
-        <v>0.152044079751163</v>
+        <v>0.192044079751163</v>
       </c>
       <c r="K17" s="58" t="n">
         <f aca="false">IF(K8=0,0,K16/K8)</f>
-        <v>0.0735162893986423</v>
+        <v>0.113516289398642</v>
       </c>
       <c r="L17" s="58" t="n">
         <f aca="false">IF(L8=0,0,L16/L8)</f>
-        <v>0.0732857479916304</v>
+        <v>0.11328574799163</v>
       </c>
       <c r="M17" s="58" t="n">
         <f aca="false">IF(M8=0,0,M16/M8)</f>
-        <v>0.0730486664028592</v>
+        <v>0.113048666402859</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20084,35 +20084,35 @@
       </c>
       <c r="F19" s="57" t="n">
         <f aca="false">F16+F18</f>
-        <v>1026.78482</v>
+        <v>1091.41074</v>
       </c>
       <c r="G19" s="57" t="n">
         <f aca="false">G16+G18</f>
-        <v>1819.675692</v>
+        <v>2006.088444</v>
       </c>
       <c r="H19" s="57" t="n">
         <f aca="false">H16+H18</f>
-        <v>1759.5432</v>
+        <v>1980.5166</v>
       </c>
       <c r="I19" s="57" t="n">
         <f aca="false">I16+I18</f>
-        <v>1443.66057</v>
+        <v>1679.83749</v>
       </c>
       <c r="J19" s="57" t="n">
         <f aca="false">J16+J18</f>
-        <v>980.396460000001</v>
+        <v>1213.40322</v>
       </c>
       <c r="K19" s="57" t="n">
         <f aca="false">K16+K18</f>
-        <v>517.13235</v>
+        <v>746.968949999999</v>
       </c>
       <c r="L19" s="57" t="n">
         <f aca="false">L16+L18</f>
-        <v>509.99949</v>
+        <v>736.665929999999</v>
       </c>
       <c r="M19" s="57" t="n">
         <f aca="false">M16+M18</f>
-        <v>502.86663</v>
+        <v>726.362909999999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20129,35 +20129,35 @@
       </c>
       <c r="F20" s="58" t="n">
         <f aca="false">IF(F8=0,0,F19/F8)</f>
-        <v>0.399504160849881</v>
+        <v>0.424648985194627</v>
       </c>
       <c r="G20" s="58" t="n">
         <f aca="false">IF(G8=0,0,G19/G8)</f>
-        <v>0.390461633654762</v>
+        <v>0.430461633654762</v>
       </c>
       <c r="H20" s="58" t="n">
         <f aca="false">IF(H8=0,0,H19/H8)</f>
-        <v>0.318507693686208</v>
+        <v>0.358507693686208</v>
       </c>
       <c r="I20" s="58" t="n">
         <f aca="false">IF(I8=0,0,I19/I8)</f>
-        <v>0.244504936384131</v>
+        <v>0.284504936384131</v>
       </c>
       <c r="J20" s="58" t="n">
         <f aca="false">IF(J8=0,0,J19/J8)</f>
-        <v>0.168303522181073</v>
+        <v>0.208303522181073</v>
       </c>
       <c r="K20" s="58" t="n">
         <f aca="false">IF(K8=0,0,K19/K8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="L20" s="58" t="n">
         <f aca="false">IF(L8=0,0,L19/L8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="M20" s="58" t="n">
         <f aca="false">IF(M8=0,0,M19/M8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20174,35 +20174,35 @@
       </c>
       <c r="F21" s="40" t="n">
         <f aca="false">F19-F15</f>
-        <v>271.86482</v>
+        <v>336.49074</v>
       </c>
       <c r="G21" s="40" t="n">
         <f aca="false">G19-G15</f>
-        <v>420.805692</v>
+        <v>607.218443999999</v>
       </c>
       <c r="H21" s="40" t="n">
         <f aca="false">H19-H15</f>
-        <v>497.46195</v>
+        <v>718.43535</v>
       </c>
       <c r="I21" s="40" t="n">
         <f aca="false">I19-I15</f>
-        <v>531.39807</v>
+        <v>767.574989999999</v>
       </c>
       <c r="J21" s="40" t="n">
         <f aca="false">J19-J15</f>
-        <v>524.265210000001</v>
+        <v>757.27197</v>
       </c>
       <c r="K21" s="40" t="n">
         <f aca="false">K19-K15</f>
-        <v>517.13235</v>
+        <v>746.968949999999</v>
       </c>
       <c r="L21" s="40" t="n">
         <f aca="false">L19-L15</f>
-        <v>509.99949</v>
+        <v>736.665929999999</v>
       </c>
       <c r="M21" s="40" t="n">
         <f aca="false">M19-M15</f>
-        <v>502.86663</v>
+        <v>726.362909999999</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20219,35 +20219,35 @@
       </c>
       <c r="F22" s="58" t="n">
         <f aca="false">IF(F8=0,0,F21/F8)</f>
-        <v>0.10577788516459</v>
+        <v>0.130922709509336</v>
       </c>
       <c r="G22" s="58" t="n">
         <f aca="false">IF(G8=0,0,G21/G8)</f>
-        <v>0.090295473348304</v>
+        <v>0.130295473348304</v>
       </c>
       <c r="H22" s="58" t="n">
         <f aca="false">IF(H8=0,0,H21/H8)</f>
-        <v>0.090049200492005</v>
+        <v>0.130049200492005</v>
       </c>
       <c r="I22" s="58" t="n">
         <f aca="false">IF(I8=0,0,I21/I8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="J22" s="58" t="n">
         <f aca="false">IF(J8=0,0,J21/J8)</f>
-        <v>0.0900000000000001</v>
+        <v>0.13</v>
       </c>
       <c r="K22" s="58" t="n">
         <f aca="false">IF(K8=0,0,K21/K8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="L22" s="58" t="n">
         <f aca="false">IF(L8=0,0,L21/L8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="M22" s="58" t="n">
         <f aca="false">IF(M8=0,0,M21/M8)</f>
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20316,35 +20316,35 @@
       </c>
       <c r="F26" s="67" t="n">
         <f aca="false">SKBA!F38</f>
-        <v>466.629144</v>
+        <v>497.811588</v>
       </c>
       <c r="G26" s="67" t="n">
         <f aca="false">SKBA!G38</f>
-        <v>692.4184008</v>
+        <v>773.3397336</v>
       </c>
       <c r="H26" s="67" t="n">
         <f aca="false">SKBA!H38</f>
-        <v>615.0020244</v>
+        <v>702.1258836</v>
       </c>
       <c r="I26" s="67" t="n">
         <f aca="false">SKBA!I38</f>
-        <v>473.395686</v>
+        <v>560.389038</v>
       </c>
       <c r="J26" s="67" t="n">
         <f aca="false">SKBA!J38</f>
-        <v>303.63837</v>
+        <v>389.464026</v>
       </c>
       <c r="K26" s="67" t="n">
         <f aca="false">SKBA!K38</f>
-        <v>129.804054</v>
+        <v>214.462014</v>
       </c>
       <c r="L26" s="67" t="n">
         <f aca="false">SKBA!L38</f>
-        <v>128.094738</v>
+        <v>211.585002</v>
       </c>
       <c r="M26" s="67" t="n">
         <f aca="false">SKBA!M38</f>
-        <v>126.385422</v>
+        <v>208.70799</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20361,35 +20361,35 @@
       </c>
       <c r="F27" s="67" t="n">
         <f aca="false">SKOT!F37</f>
-        <v>-101.53240172</v>
+        <v>-71.06171804</v>
       </c>
       <c r="G27" s="67" t="n">
         <f aca="false">SKOT!G37</f>
-        <v>641.99318796</v>
+        <v>714.34019772</v>
       </c>
       <c r="H27" s="67" t="n">
         <f aca="false">SKOT!H37</f>
-        <v>789.2805695</v>
+        <v>889.1099915</v>
       </c>
       <c r="I27" s="67" t="n">
         <f aca="false">SKOT!I37</f>
-        <v>668.2789139</v>
+        <v>779.9203823</v>
       </c>
       <c r="J27" s="67" t="n">
         <f aca="false">SKOT!J37</f>
-        <v>447.1848617</v>
+        <v>557.3277869</v>
       </c>
       <c r="K27" s="67" t="n">
         <f aca="false">SKOT!K37</f>
-        <v>161.2665095</v>
+        <v>269.9108915</v>
       </c>
       <c r="L27" s="67" t="n">
         <f aca="false">SKOT!L37</f>
-        <v>159.3544073</v>
+        <v>266.5002461</v>
       </c>
       <c r="M27" s="67" t="n">
         <f aca="false">SKOT!M37</f>
-        <v>157.4423051</v>
+        <v>263.0896007</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20406,35 +20406,35 @@
       </c>
       <c r="F28" s="60" t="n">
         <f aca="false">F26+F27</f>
-        <v>365.09674228</v>
+        <v>426.74986996</v>
       </c>
       <c r="G28" s="60" t="n">
         <f aca="false">G26+G27</f>
-        <v>1334.41158876</v>
+        <v>1487.67993132</v>
       </c>
       <c r="H28" s="60" t="n">
         <f aca="false">H26+H27</f>
-        <v>1404.2825939</v>
+        <v>1591.2358751</v>
       </c>
       <c r="I28" s="60" t="n">
         <f aca="false">I26+I27</f>
-        <v>1141.6745999</v>
+        <v>1340.3094203</v>
       </c>
       <c r="J28" s="60" t="n">
         <f aca="false">J26+J27</f>
-        <v>750.8232317</v>
+        <v>946.7918129</v>
       </c>
       <c r="K28" s="60" t="n">
         <f aca="false">K26+K27</f>
-        <v>291.0705635</v>
+        <v>484.3729055</v>
       </c>
       <c r="L28" s="60" t="n">
         <f aca="false">L26+L27</f>
-        <v>287.4491453</v>
+        <v>478.085248099999</v>
       </c>
       <c r="M28" s="60" t="n">
         <f aca="false">M26+M27</f>
-        <v>283.8277271</v>
+        <v>471.797590699999</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20638,35 +20638,35 @@
       </c>
       <c r="F35" s="57" t="n">
         <f aca="false">F26+F32+F33+F34</f>
-        <v>423.986544</v>
+        <v>455.168988</v>
       </c>
       <c r="G35" s="57" t="n">
         <f aca="false">G26+G32+G33+G34</f>
-        <v>649.7758008</v>
+        <v>730.6971336</v>
       </c>
       <c r="H35" s="57" t="n">
         <f aca="false">H26+H32+H33+H34</f>
-        <v>572.3594244</v>
+        <v>659.4832836</v>
       </c>
       <c r="I35" s="57" t="n">
         <f aca="false">I26+I32+I33+I34</f>
-        <v>430.753086</v>
+        <v>517.746438</v>
       </c>
       <c r="J35" s="57" t="n">
         <f aca="false">J26+J32+J33+J34</f>
-        <v>260.99577</v>
+        <v>346.821426</v>
       </c>
       <c r="K35" s="57" t="n">
         <f aca="false">K26+K32+K33+K34</f>
-        <v>87.1614540000001</v>
+        <v>171.819414</v>
       </c>
       <c r="L35" s="57" t="n">
         <f aca="false">L26+L32+L33+L34</f>
-        <v>85.452138</v>
+        <v>168.942402</v>
       </c>
       <c r="M35" s="57" t="n">
         <f aca="false">M26+M32+M33+M34</f>
-        <v>83.7428219999998</v>
+        <v>166.06539</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20998,35 +20998,35 @@
       </c>
       <c r="F43" s="57" t="n">
         <f aca="false">F27+F36+F37+F41+F40+F42</f>
-        <v>-255.53240172</v>
+        <v>-225.06171804</v>
       </c>
       <c r="G43" s="57" t="n">
         <f aca="false">G27+G36+G37+G41+G40+G42</f>
-        <v>487.99318796</v>
+        <v>560.34019772</v>
       </c>
       <c r="H43" s="57" t="n">
         <f aca="false">H27+H36+H37+H41+H40+H42</f>
-        <v>635.2805695</v>
+        <v>735.1099915</v>
       </c>
       <c r="I43" s="57" t="n">
         <f aca="false">I27+I36+I37+I41+I40+I42</f>
-        <v>514.2789139</v>
+        <v>625.9203823</v>
       </c>
       <c r="J43" s="57" t="n">
         <f aca="false">J27+J36+J37+J41+J40+J42</f>
-        <v>293.1848617</v>
+        <v>403.3277869</v>
       </c>
       <c r="K43" s="57" t="n">
         <f aca="false">K27+K36+K37+K41+K40+K42</f>
-        <v>7.2665094999999</v>
+        <v>115.9108915</v>
       </c>
       <c r="L43" s="57" t="n">
         <f aca="false">L27+L36+L37+L41+L40+L42</f>
-        <v>5.35440730000016</v>
+        <v>112.5002461</v>
       </c>
       <c r="M43" s="57" t="n">
         <f aca="false">M27+M36+M37+M41+M40+M42</f>
-        <v>3.44230510000011</v>
+        <v>109.0896007</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21043,35 +21043,35 @@
       </c>
       <c r="F44" s="67" t="n">
         <f aca="false">SKOT!F19-SKOT!F15+SKOT!F32</f>
-        <v>288.47988</v>
+        <v>320.4198</v>
       </c>
       <c r="G44" s="67" t="n">
         <f aca="false">SKOT!G19-SKOT!G15+SKOT!G32</f>
-        <v>927.554328</v>
+        <v>1029.14388</v>
       </c>
       <c r="H44" s="67" t="n">
         <f aca="false">SKOT!H19-SKOT!H15+SKOT!H32</f>
-        <v>946.25415</v>
+        <v>1075.90275</v>
       </c>
       <c r="I44" s="67" t="n">
         <f aca="false">SKOT!I19-SKOT!I15+SKOT!I32</f>
-        <v>785.49588</v>
+        <v>930.484799999999</v>
       </c>
       <c r="J44" s="67" t="n">
         <f aca="false">SKOT!J19-SKOT!J15+SKOT!J32</f>
-        <v>498.570390000001</v>
+        <v>641.61315</v>
       </c>
       <c r="K44" s="67" t="n">
         <f aca="false">SKOT!K19-SKOT!K15+SKOT!K32</f>
-        <v>211.6449</v>
+        <v>352.7415</v>
       </c>
       <c r="L44" s="67" t="n">
         <f aca="false">SKOT!L19-SKOT!L15+SKOT!L32</f>
-        <v>208.72566</v>
+        <v>347.8761</v>
       </c>
       <c r="M44" s="67" t="n">
         <f aca="false">SKOT!M19-SKOT!M15+SKOT!M32</f>
-        <v>205.80642</v>
+        <v>343.0107</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21133,35 +21133,35 @@
       </c>
       <c r="F46" s="68" t="n">
         <f aca="false">IF(F45=0,0,F44/F45)</f>
-        <v>1.4423994</v>
+        <v>1.602099</v>
       </c>
       <c r="G46" s="68" t="n">
         <f aca="false">IF(G45=0,0,G44/G45)</f>
-        <v>4.63777164</v>
+        <v>5.1457194</v>
       </c>
       <c r="H46" s="68" t="n">
         <f aca="false">IF(H45=0,0,H44/H45)</f>
-        <v>4.73127075</v>
+        <v>5.37951375</v>
       </c>
       <c r="I46" s="68" t="n">
         <f aca="false">IF(I45=0,0,I44/I45)</f>
-        <v>3.9274794</v>
+        <v>4.652424</v>
       </c>
       <c r="J46" s="68" t="n">
         <f aca="false">IF(J45=0,0,J44/J45)</f>
-        <v>2.49285195</v>
+        <v>3.20806575</v>
       </c>
       <c r="K46" s="68" t="n">
         <f aca="false">IF(K45=0,0,K44/K45)</f>
-        <v>1.0582245</v>
+        <v>1.7637075</v>
       </c>
       <c r="L46" s="68" t="n">
         <f aca="false">IF(L45=0,0,L44/L45)</f>
-        <v>1.0436283</v>
+        <v>1.7393805</v>
       </c>
       <c r="M46" s="68" t="n">
         <f aca="false">IF(M45=0,0,M44/M45)</f>
-        <v>1.0290321</v>
+        <v>1.7150535</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21178,35 +21178,35 @@
       </c>
       <c r="F47" s="60" t="n">
         <f aca="false">F35+F43</f>
-        <v>168.45414228</v>
+        <v>230.10726996</v>
       </c>
       <c r="G47" s="60" t="n">
         <f aca="false">G35+G43</f>
-        <v>1137.76898876</v>
+        <v>1291.03733132</v>
       </c>
       <c r="H47" s="60" t="n">
         <f aca="false">H35+H43</f>
-        <v>1207.6399939</v>
+        <v>1394.5932751</v>
       </c>
       <c r="I47" s="60" t="n">
         <f aca="false">I35+I43</f>
-        <v>945.0319999</v>
+        <v>1143.6668203</v>
       </c>
       <c r="J47" s="60" t="n">
         <f aca="false">J35+J43</f>
-        <v>554.1806317</v>
+        <v>750.1492129</v>
       </c>
       <c r="K47" s="60" t="n">
         <f aca="false">K35+K43</f>
-        <v>94.4279635</v>
+        <v>287.7303055</v>
       </c>
       <c r="L47" s="60" t="n">
         <f aca="false">L35+L43</f>
-        <v>90.8065453000002</v>
+        <v>281.442648099999</v>
       </c>
       <c r="M47" s="60" t="n">
         <f aca="false">M35+M43</f>
-        <v>87.1851270999999</v>
+        <v>275.154990699999</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21268,35 +21268,35 @@
       </c>
       <c r="F49" s="40" t="n">
         <f aca="false">F47*F48</f>
-        <v>124.103944716466</v>
+        <v>169.525186638069</v>
       </c>
       <c r="G49" s="40" t="n">
         <f aca="false">G47*G48</f>
-        <v>741.787550411592</v>
+        <v>841.713413663617</v>
       </c>
       <c r="H49" s="40" t="n">
         <f aca="false">H47*H48</f>
-        <v>696.762055386085</v>
+        <v>804.626943207009</v>
       </c>
       <c r="I49" s="40" t="n">
         <f aca="false">I47*I48</f>
-        <v>482.519729097867</v>
+        <v>583.939807718436</v>
       </c>
       <c r="J49" s="40" t="n">
         <f aca="false">J47*J48</f>
-        <v>250.404114524215</v>
+        <v>338.951667872339</v>
       </c>
       <c r="K49" s="40" t="n">
         <f aca="false">K47*K48</f>
-        <v>37.7582882304995</v>
+        <v>115.052823390803</v>
       </c>
       <c r="L49" s="40" t="n">
         <f aca="false">L47*L48</f>
-        <v>32.1329341339825</v>
+        <v>99.591698417921</v>
       </c>
       <c r="M49" s="40" t="n">
         <f aca="false">M47*M48</f>
-        <v>27.3021715970717</v>
+        <v>86.1652557237834</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21460,35 +21460,35 @@
       </c>
       <c r="F56" s="40" t="n">
         <f aca="false">F28*F55</f>
-        <v>284.447592762507</v>
+        <v>332.481666266801</v>
       </c>
       <c r="G56" s="40" t="n">
         <f aca="false">G28*G55</f>
-        <v>940.853125324873</v>
+        <v>1048.91798351824</v>
       </c>
       <c r="H56" s="40" t="n">
         <f aca="false">H28*H55</f>
-        <v>896.033530470594</v>
+        <v>1015.32320144876</v>
       </c>
       <c r="I56" s="40" t="n">
         <f aca="false">I28*I55</f>
-        <v>659.249501115887</v>
+        <v>773.949351900352</v>
       </c>
       <c r="J56" s="40" t="n">
         <f aca="false">J28*J55</f>
-        <v>392.35834574661</v>
+        <v>494.765816761923</v>
       </c>
       <c r="K56" s="40" t="n">
         <f aca="false">K28*K55</f>
-        <v>137.65158025437</v>
+        <v>229.067120607252</v>
       </c>
       <c r="L56" s="40" t="n">
         <f aca="false">L28*L55</f>
-        <v>123.021681406457</v>
+        <v>204.609587603756</v>
       </c>
       <c r="M56" s="40" t="n">
         <f aca="false">M28*M55</f>
-        <v>109.929228028829</v>
+        <v>182.731776988226</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21505,7 +21505,7 @@
       </c>
       <c r="D59" s="39" t="n">
         <f aca="false">SUM(D56:M56)</f>
-        <v>3094.42883827081</v>
+        <v>3832.730758256</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21514,7 +21514,7 @@
       </c>
       <c r="D60" s="39" t="n">
         <f aca="false">M28*(1+Assumptions!$C$93)/(Assumptions!$C$91-Assumptions!$C$93)</f>
-        <v>3405.9327252</v>
+        <v>5661.57108839999</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21523,7 +21523,7 @@
       </c>
       <c r="D61" s="39" t="n">
         <f aca="false">D60*M55</f>
-        <v>1319.15073634594</v>
+        <v>2192.78132385871</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21532,7 +21532,7 @@
       </c>
       <c r="D62" s="74" t="n">
         <f aca="false">D59+D61</f>
-        <v>4413.57957461676</v>
+        <v>6025.51208211471</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21550,7 +21550,7 @@
       </c>
       <c r="D64" s="75" t="n">
         <f aca="false">D62-Assumptions!$C$94</f>
-        <v>-1986.42042538325</v>
+        <v>-374.487917885293</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="D66" s="76" t="n">
         <f aca="false">D61/D62</f>
-        <v>0.298884548028227</v>
+        <v>0.363916177409627</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21576,7 +21576,7 @@
       </c>
       <c r="D69" s="39" t="n">
         <f aca="false">SUM(D49:M49)</f>
-        <v>1606.27785202397</v>
+        <v>2253.07386055816</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21585,7 +21585,7 @@
       </c>
       <c r="D70" s="39" t="n">
         <f aca="false">M47*(1+Assumptions!$C$93)/(Assumptions!$C$92-Assumptions!$C$93)</f>
-        <v>808.443905836363</v>
+        <v>2551.4371864909</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="D71" s="39" t="n">
         <f aca="false">D70*1/(1+Assumptions!$C$92)^((10)-Assumptions!$C$95)</f>
-        <v>253.165591172847</v>
+        <v>798.986916711446</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21603,7 +21603,7 @@
       </c>
       <c r="D72" s="74" t="n">
         <f aca="false">D69+D71</f>
-        <v>1859.44344319681</v>
+        <v>3052.06077726961</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21612,7 +21612,7 @@
       </c>
       <c r="D73" s="77" t="n">
         <f aca="false">D64</f>
-        <v>-1986.42042538325</v>
+        <v>-374.487917885293</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21661,7 +21661,7 @@
       </c>
       <c r="D80" s="80" t="n">
         <f aca="false">D64</f>
-        <v>-1986.42042538325</v>
+        <v>-374.487917885293</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21670,7 +21670,7 @@
       </c>
       <c r="D81" s="77" t="n">
         <f aca="false">(Assumptions!$C$119+Assumptions!$C$120)-D64</f>
-        <v>6986.42042538325</v>
+        <v>5374.48791788529</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21697,7 +21697,7 @@
       </c>
       <c r="D86" s="67" t="n">
         <f aca="false">G21</f>
-        <v>420.805692</v>
+        <v>607.218443999999</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21706,7 +21706,7 @@
       </c>
       <c r="D87" s="67" t="n">
         <f aca="false">AVERAGE(H21:J21)</f>
-        <v>517.70841</v>
+        <v>747.76077</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21734,15 +21734,15 @@
       </c>
       <c r="D90" s="80" t="n">
         <f aca="false">$D$86*D88</f>
-        <v>3366.445536</v>
+        <v>4857.747552</v>
       </c>
       <c r="E90" s="80" t="n">
         <f aca="false">$D$86*E88</f>
-        <v>4628.862612</v>
+        <v>6679.40288399999</v>
       </c>
       <c r="F90" s="80" t="n">
         <f aca="false">$D$86*F88</f>
-        <v>5891.279688</v>
+        <v>8501.05821599999</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21751,15 +21751,15 @@
       </c>
       <c r="D91" s="80" t="n">
         <f aca="false">$D$87*D88</f>
-        <v>4141.66728</v>
+        <v>5982.08616</v>
       </c>
       <c r="E91" s="80" t="n">
         <f aca="false">$D$87*E88</f>
-        <v>5694.79251</v>
+        <v>8225.36847</v>
       </c>
       <c r="F91" s="80" t="n">
         <f aca="false">$D$87*F88</f>
-        <v>7247.91774</v>
+        <v>10468.65078</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21768,7 +21768,7 @@
       </c>
       <c r="D92" s="77" t="n">
         <f aca="false">D62</f>
-        <v>4413.57957461676</v>
+        <v>6025.51208211471</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="D5" s="39" t="n">
         <f aca="false">Consolidated!D87</f>
-        <v>517.70841</v>
+        <v>747.76077</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21843,7 +21843,7 @@
       </c>
       <c r="D6" s="39" t="n">
         <f aca="false">Consolidated!D86</f>
-        <v>420.805692</v>
+        <v>607.218443999999</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21861,7 +21861,7 @@
       </c>
       <c r="D8" s="40" t="n">
         <f aca="false">Consolidated!D62</f>
-        <v>4413.57957461676</v>
+        <v>6025.51208211471</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21879,7 +21879,7 @@
       </c>
       <c r="D10" s="84" t="n">
         <f aca="false">D8/D5</f>
-        <v>8.52522286554463</v>
+        <v>8.05807461939292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21888,7 +21888,7 @@
       </c>
       <c r="D11" s="86" t="n">
         <f aca="false">D8/D6</f>
-        <v>10.4884027438886</v>
+        <v>9.92313745021011</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22064,19 +22064,19 @@
       </c>
       <c r="D29" s="39" t="n">
         <f aca="false">C29*$D$5</f>
-        <v>4141.66728</v>
+        <v>5982.08616</v>
       </c>
       <c r="E29" s="93" t="n">
         <f aca="false">D29-$D$9</f>
-        <v>-2258.33272</v>
+        <v>-417.913840000002</v>
       </c>
       <c r="F29" s="39" t="n">
         <f aca="false">C29*$D$6</f>
-        <v>3366.445536</v>
+        <v>4857.747552</v>
       </c>
       <c r="G29" s="93" t="n">
         <f aca="false">F29-$D$9</f>
-        <v>-3033.554464</v>
+        <v>-1542.252448</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22088,19 +22088,19 @@
       </c>
       <c r="D30" s="39" t="n">
         <f aca="false">C30*$D$5</f>
-        <v>5435.938305</v>
+        <v>7851.488085</v>
       </c>
       <c r="E30" s="93" t="n">
         <f aca="false">D30-$D$9</f>
-        <v>-964.061694999999</v>
+        <v>1451.488085</v>
       </c>
       <c r="F30" s="39" t="n">
         <f aca="false">C30*$D$6</f>
-        <v>4418.459766</v>
+        <v>6375.79366199999</v>
       </c>
       <c r="G30" s="93" t="n">
         <f aca="false">F30-$D$9</f>
-        <v>-1981.540234</v>
+        <v>-24.2063380000063</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22112,19 +22112,19 @@
       </c>
       <c r="D31" s="39" t="n">
         <f aca="false">C31*$D$5</f>
-        <v>6730.20933</v>
+        <v>9720.89001</v>
       </c>
       <c r="E31" s="67" t="n">
         <f aca="false">D31-$D$9</f>
-        <v>330.209330000002</v>
+        <v>3320.89001</v>
       </c>
       <c r="F31" s="39" t="n">
         <f aca="false">C31*$D$6</f>
-        <v>5470.473996</v>
+        <v>7893.83977199999</v>
       </c>
       <c r="G31" s="93" t="n">
         <f aca="false">F31-$D$9</f>
-        <v>-929.526003999999</v>
+        <v>1493.83977199999</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22136,19 +22136,19 @@
       </c>
       <c r="D32" s="39" t="n">
         <f aca="false">C32*$D$5</f>
-        <v>7765.62615</v>
+        <v>11216.41155</v>
       </c>
       <c r="E32" s="67" t="n">
         <f aca="false">D32-$D$9</f>
-        <v>1365.62615</v>
+        <v>4816.41155</v>
       </c>
       <c r="F32" s="39" t="n">
         <f aca="false">C32*$D$6</f>
-        <v>6312.08538</v>
+        <v>9108.27665999999</v>
       </c>
       <c r="G32" s="67" t="n">
         <f aca="false">F32-$D$9</f>
-        <v>-87.9146199999977</v>
+        <v>2708.27665999999</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22160,19 +22160,19 @@
       </c>
       <c r="D33" s="39" t="n">
         <f aca="false">C33*$D$5</f>
-        <v>9836.45979</v>
+        <v>14207.45463</v>
       </c>
       <c r="E33" s="67" t="n">
         <f aca="false">D33-$D$9</f>
-        <v>3436.45979</v>
+        <v>7807.45463</v>
       </c>
       <c r="F33" s="39" t="n">
         <f aca="false">C33*$D$6</f>
-        <v>7995.308148</v>
+        <v>11537.150436</v>
       </c>
       <c r="G33" s="67" t="n">
         <f aca="false">F33-$D$9</f>
-        <v>1595.308148</v>
+        <v>5137.15043599999</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22253,11 +22253,11 @@
       </c>
       <c r="H39" s="84" t="n">
         <f aca="false">G39/$D$5</f>
-        <v>16.4764563125409</v>
+        <v>11.4073916982834</v>
       </c>
       <c r="I39" s="86" t="n">
         <f aca="false">G39/$D$6</f>
-        <v>20.270638354388</v>
+        <v>14.0476628868671</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22284,11 +22284,11 @@
       </c>
       <c r="H40" s="84" t="n">
         <f aca="false">G40/$D$5</f>
-        <v>15.1050279442051</v>
+        <v>10.4578901618495</v>
       </c>
       <c r="I40" s="86" t="n">
         <f aca="false">G40/$D$6</f>
-        <v>18.5833988196148</v>
+        <v>12.8783966911256</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22315,11 +22315,11 @@
       </c>
       <c r="H41" s="84" t="n">
         <f aca="false">G41/$D$5</f>
-        <v>15.1050279442051</v>
+        <v>10.4578901618495</v>
       </c>
       <c r="I41" s="86" t="n">
         <f aca="false">G41/$D$6</f>
-        <v>18.5833988196148</v>
+        <v>12.8783966911256</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22346,11 +22346,11 @@
       </c>
       <c r="H42" s="84" t="n">
         <f aca="false">G42/$D$5</f>
-        <v>14.0414712503937</v>
+        <v>9.72154203155381</v>
       </c>
       <c r="I42" s="86" t="n">
         <f aca="false">G42/$D$6</f>
-        <v>17.2749273436683</v>
+        <v>11.9716188250402</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22377,11 +22377,11 @@
       </c>
       <c r="H43" s="84" t="n">
         <f aca="false">G43/$D$5</f>
-        <v>13.4817045694403</v>
+        <v>9.33399038402977</v>
       </c>
       <c r="I43" s="86" t="n">
         <f aca="false">G43/$D$6</f>
-        <v>16.5862581458016</v>
+        <v>11.4943673165743</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>